<commit_message>
chore: update .gitignore to include .DS_Store and adjust crowners-app entry
</commit_message>
<xml_diff>
--- a/db/seeds/excel/seeds.xlsx
+++ b/db/seeds/excel/seeds.xlsx
@@ -4507,20 +4507,20 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="true"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="30.29"/>
-    <col customWidth="1" min="2" max="2" width="15.71"/>
-    <col customWidth="1" min="3" max="3" width="25.14"/>
-    <col customWidth="1" min="4" max="4" width="8.71"/>
-    <col customWidth="1" min="5" max="5" width="10.0"/>
-    <col customWidth="1" min="6" max="6" width="15.57"/>
-    <col customWidth="1" min="7" max="7" width="14.43"/>
-    <col customWidth="1" min="8" max="8" width="14.0"/>
-    <col customWidth="1" min="9" max="26" width="8.71"/>
+    <col customWidth="true" max="1" min="1" width="30.29"/>
+    <col customWidth="true" max="2" min="2" width="15.71"/>
+    <col customWidth="true" max="3" min="3" width="25.14"/>
+    <col customWidth="true" max="4" min="4" width="8.71"/>
+    <col customWidth="true" max="5" min="5" width="10"/>
+    <col customWidth="true" max="6" min="6" width="15.57"/>
+    <col customWidth="true" max="7" min="7" width="14.43"/>
+    <col customWidth="true" max="8" min="8" width="14"/>
+    <col customWidth="true" max="26" min="9" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
+    <row r="1" ht="14.25" customHeight="true">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4544,7 +4544,7 @@
       </c>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" ht="14.25" customHeight="1">
+    <row r="2" ht="14.25" customHeight="true">
       <c r="A2" s="2" t="s">
         <v>21</v>
       </c>
@@ -4568,7 +4568,7 @@
       </c>
       <c r="H2" s="4"/>
     </row>
-    <row r="3" ht="14.25" customHeight="1">
+    <row r="3" ht="14.25" customHeight="true">
       <c r="A3" s="2" t="s">
         <v>25</v>
       </c>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="H3" s="4"/>
     </row>
-    <row r="4" ht="14.25" customHeight="1">
+    <row r="4" ht="14.25" customHeight="true">
       <c r="A4" s="2" t="s">
         <v>28</v>
       </c>
@@ -4616,7 +4616,7 @@
       </c>
       <c r="H4" s="4"/>
     </row>
-    <row r="5" ht="14.25" customHeight="1">
+    <row r="5" ht="14.25" customHeight="true">
       <c r="A5" s="2" t="s">
         <v>31</v>
       </c>
@@ -4640,7 +4640,7 @@
       </c>
       <c r="H5" s="4"/>
     </row>
-    <row r="6" ht="14.25" customHeight="1">
+    <row r="6" ht="14.25" customHeight="true">
       <c r="A6" s="2" t="s">
         <v>35</v>
       </c>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="H6" s="4"/>
     </row>
-    <row r="7" ht="14.25" customHeight="1">
+    <row r="7" ht="14.25" customHeight="true">
       <c r="A7" s="2" t="s">
         <v>38</v>
       </c>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="H7" s="5"/>
     </row>
-    <row r="8" ht="14.25" customHeight="1">
+    <row r="8" ht="14.25" customHeight="true">
       <c r="A8" s="2" t="s">
         <v>42</v>
       </c>
@@ -4712,7 +4712,7 @@
       </c>
       <c r="H8" s="5"/>
     </row>
-    <row r="9" ht="14.25" customHeight="1">
+    <row r="9" ht="14.25" customHeight="true">
       <c r="A9" s="2" t="s">
         <v>45</v>
       </c>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="H9" s="5"/>
     </row>
-    <row r="10" ht="14.25" customHeight="1">
+    <row r="10" ht="14.25" customHeight="true">
       <c r="A10" s="2" t="s">
         <v>48</v>
       </c>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="H10" s="5"/>
     </row>
-    <row r="11" ht="14.25" customHeight="1">
+    <row r="11" ht="14.25" customHeight="true">
       <c r="A11" s="2" t="s">
         <v>51</v>
       </c>
@@ -4784,7 +4784,7 @@
       </c>
       <c r="H11" s="5"/>
     </row>
-    <row r="12" ht="14.25" customHeight="1">
+    <row r="12" ht="14.25" customHeight="true">
       <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="H12" s="5"/>
     </row>
-    <row r="13" ht="14.25" customHeight="1">
+    <row r="13" ht="14.25" customHeight="true">
       <c r="A13" s="2" t="s">
         <v>58</v>
       </c>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="H13" s="5"/>
     </row>
-    <row r="14" ht="14.25" customHeight="1">
+    <row r="14" ht="14.25" customHeight="true">
       <c r="A14" s="2" t="s">
         <v>61</v>
       </c>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="H14" s="5"/>
     </row>
-    <row r="15" ht="14.25" customHeight="1">
+    <row r="15" ht="14.25" customHeight="true">
       <c r="A15" s="2" t="s">
         <v>64</v>
       </c>
@@ -4880,7 +4880,7 @@
       </c>
       <c r="H15" s="5"/>
     </row>
-    <row r="16" ht="14.25" customHeight="1">
+    <row r="16" ht="14.25" customHeight="true">
       <c r="A16" s="2" t="s">
         <v>68</v>
       </c>
@@ -4904,993 +4904,993 @@
       </c>
       <c r="H16" s="5"/>
     </row>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
-    <row r="65" ht="14.25" customHeight="1"/>
-    <row r="66" ht="14.25" customHeight="1"/>
-    <row r="67" ht="14.25" customHeight="1"/>
-    <row r="68" ht="14.25" customHeight="1"/>
-    <row r="69" ht="14.25" customHeight="1"/>
-    <row r="70" ht="14.25" customHeight="1"/>
-    <row r="71" ht="14.25" customHeight="1"/>
-    <row r="72" ht="14.25" customHeight="1"/>
-    <row r="73" ht="14.25" customHeight="1"/>
-    <row r="74" ht="14.25" customHeight="1"/>
-    <row r="75" ht="14.25" customHeight="1"/>
-    <row r="76" ht="14.25" customHeight="1"/>
-    <row r="77" ht="14.25" customHeight="1"/>
-    <row r="78" ht="14.25" customHeight="1"/>
-    <row r="79" ht="14.25" customHeight="1"/>
-    <row r="80" ht="14.25" customHeight="1"/>
-    <row r="81" ht="14.25" customHeight="1"/>
-    <row r="82" ht="14.25" customHeight="1"/>
-    <row r="83" ht="14.25" customHeight="1"/>
-    <row r="84" ht="14.25" customHeight="1"/>
-    <row r="85" ht="14.25" customHeight="1"/>
-    <row r="86" ht="14.25" customHeight="1"/>
-    <row r="87" ht="14.25" customHeight="1"/>
-    <row r="88" ht="14.25" customHeight="1"/>
-    <row r="89" ht="14.25" customHeight="1"/>
-    <row r="90" ht="14.25" customHeight="1"/>
-    <row r="91" ht="14.25" customHeight="1"/>
-    <row r="92" ht="14.25" customHeight="1"/>
-    <row r="93" ht="14.25" customHeight="1"/>
-    <row r="94" ht="14.25" customHeight="1"/>
-    <row r="95" ht="14.25" customHeight="1"/>
-    <row r="96" ht="14.25" customHeight="1"/>
-    <row r="97" ht="14.25" customHeight="1"/>
-    <row r="98" ht="14.25" customHeight="1"/>
-    <row r="99" ht="14.25" customHeight="1"/>
-    <row r="100" ht="14.25" customHeight="1"/>
-    <row r="101" ht="14.25" customHeight="1"/>
-    <row r="102" ht="14.25" customHeight="1"/>
-    <row r="103" ht="14.25" customHeight="1"/>
-    <row r="104" ht="14.25" customHeight="1"/>
-    <row r="105" ht="14.25" customHeight="1"/>
-    <row r="106" ht="14.25" customHeight="1"/>
-    <row r="107" ht="14.25" customHeight="1"/>
-    <row r="108" ht="14.25" customHeight="1"/>
-    <row r="109" ht="14.25" customHeight="1"/>
-    <row r="110" ht="14.25" customHeight="1"/>
-    <row r="111" ht="14.25" customHeight="1"/>
-    <row r="112" ht="14.25" customHeight="1"/>
-    <row r="113" ht="14.25" customHeight="1"/>
-    <row r="114" ht="14.25" customHeight="1"/>
-    <row r="115" ht="14.25" customHeight="1"/>
-    <row r="116" ht="14.25" customHeight="1"/>
-    <row r="117" ht="14.25" customHeight="1"/>
-    <row r="118" ht="14.25" customHeight="1"/>
-    <row r="119" ht="14.25" customHeight="1"/>
-    <row r="120" ht="14.25" customHeight="1"/>
-    <row r="121" ht="14.25" customHeight="1"/>
-    <row r="122" ht="14.25" customHeight="1"/>
-    <row r="123" ht="14.25" customHeight="1"/>
-    <row r="124" ht="14.25" customHeight="1"/>
-    <row r="125" ht="14.25" customHeight="1"/>
-    <row r="126" ht="14.25" customHeight="1"/>
-    <row r="127" ht="14.25" customHeight="1"/>
-    <row r="128" ht="14.25" customHeight="1"/>
-    <row r="129" ht="14.25" customHeight="1"/>
-    <row r="130" ht="14.25" customHeight="1"/>
-    <row r="131" ht="14.25" customHeight="1"/>
-    <row r="132" ht="14.25" customHeight="1"/>
-    <row r="133" ht="14.25" customHeight="1"/>
-    <row r="134" ht="14.25" customHeight="1"/>
-    <row r="135" ht="14.25" customHeight="1"/>
-    <row r="136" ht="14.25" customHeight="1"/>
-    <row r="137" ht="14.25" customHeight="1"/>
-    <row r="138" ht="14.25" customHeight="1"/>
-    <row r="139" ht="14.25" customHeight="1"/>
-    <row r="140" ht="14.25" customHeight="1"/>
-    <row r="141" ht="14.25" customHeight="1"/>
-    <row r="142" ht="14.25" customHeight="1"/>
-    <row r="143" ht="14.25" customHeight="1"/>
-    <row r="144" ht="14.25" customHeight="1"/>
-    <row r="145" ht="14.25" customHeight="1"/>
-    <row r="146" ht="14.25" customHeight="1"/>
-    <row r="147" ht="14.25" customHeight="1"/>
-    <row r="148" ht="14.25" customHeight="1"/>
-    <row r="149" ht="14.25" customHeight="1"/>
-    <row r="150" ht="14.25" customHeight="1"/>
-    <row r="151" ht="14.25" customHeight="1"/>
-    <row r="152" ht="14.25" customHeight="1"/>
-    <row r="153" ht="14.25" customHeight="1"/>
-    <row r="154" ht="14.25" customHeight="1"/>
-    <row r="155" ht="14.25" customHeight="1"/>
-    <row r="156" ht="14.25" customHeight="1"/>
-    <row r="157" ht="14.25" customHeight="1"/>
-    <row r="158" ht="14.25" customHeight="1"/>
-    <row r="159" ht="14.25" customHeight="1"/>
-    <row r="160" ht="14.25" customHeight="1"/>
-    <row r="161" ht="14.25" customHeight="1"/>
-    <row r="162" ht="14.25" customHeight="1"/>
-    <row r="163" ht="14.25" customHeight="1"/>
-    <row r="164" ht="14.25" customHeight="1"/>
-    <row r="165" ht="14.25" customHeight="1"/>
-    <row r="166" ht="14.25" customHeight="1"/>
-    <row r="167" ht="14.25" customHeight="1"/>
-    <row r="168" ht="14.25" customHeight="1"/>
-    <row r="169" ht="14.25" customHeight="1"/>
-    <row r="170" ht="14.25" customHeight="1"/>
-    <row r="171" ht="14.25" customHeight="1"/>
-    <row r="172" ht="14.25" customHeight="1"/>
-    <row r="173" ht="14.25" customHeight="1"/>
-    <row r="174" ht="14.25" customHeight="1"/>
-    <row r="175" ht="14.25" customHeight="1"/>
-    <row r="176" ht="14.25" customHeight="1"/>
-    <row r="177" ht="14.25" customHeight="1"/>
-    <row r="178" ht="14.25" customHeight="1"/>
-    <row r="179" ht="14.25" customHeight="1"/>
-    <row r="180" ht="14.25" customHeight="1"/>
-    <row r="181" ht="14.25" customHeight="1"/>
-    <row r="182" ht="14.25" customHeight="1"/>
-    <row r="183" ht="14.25" customHeight="1"/>
-    <row r="184" ht="14.25" customHeight="1"/>
-    <row r="185" ht="14.25" customHeight="1"/>
-    <row r="186" ht="14.25" customHeight="1"/>
-    <row r="187" ht="14.25" customHeight="1"/>
-    <row r="188" ht="14.25" customHeight="1"/>
-    <row r="189" ht="14.25" customHeight="1"/>
-    <row r="190" ht="14.25" customHeight="1"/>
-    <row r="191" ht="14.25" customHeight="1"/>
-    <row r="192" ht="14.25" customHeight="1"/>
-    <row r="193" ht="14.25" customHeight="1"/>
-    <row r="194" ht="14.25" customHeight="1"/>
-    <row r="195" ht="14.25" customHeight="1"/>
-    <row r="196" ht="14.25" customHeight="1"/>
-    <row r="197" ht="14.25" customHeight="1"/>
-    <row r="198" ht="14.25" customHeight="1"/>
-    <row r="199" ht="14.25" customHeight="1"/>
-    <row r="200" ht="14.25" customHeight="1"/>
-    <row r="201" ht="14.25" customHeight="1"/>
-    <row r="202" ht="14.25" customHeight="1"/>
-    <row r="203" ht="14.25" customHeight="1"/>
-    <row r="204" ht="14.25" customHeight="1"/>
-    <row r="205" ht="14.25" customHeight="1"/>
-    <row r="206" ht="14.25" customHeight="1"/>
-    <row r="207" ht="14.25" customHeight="1"/>
-    <row r="208" ht="14.25" customHeight="1"/>
-    <row r="209" ht="14.25" customHeight="1"/>
-    <row r="210" ht="14.25" customHeight="1"/>
-    <row r="211" ht="14.25" customHeight="1"/>
-    <row r="212" ht="14.25" customHeight="1"/>
-    <row r="213" ht="14.25" customHeight="1"/>
-    <row r="214" ht="14.25" customHeight="1"/>
-    <row r="215" ht="14.25" customHeight="1"/>
-    <row r="216" ht="14.25" customHeight="1"/>
-    <row r="217" ht="14.25" customHeight="1"/>
-    <row r="218" ht="14.25" customHeight="1"/>
-    <row r="219" ht="14.25" customHeight="1"/>
-    <row r="220" ht="14.25" customHeight="1"/>
-    <row r="221" ht="14.25" customHeight="1"/>
-    <row r="222" ht="14.25" customHeight="1"/>
-    <row r="223" ht="14.25" customHeight="1"/>
-    <row r="224" ht="14.25" customHeight="1"/>
-    <row r="225" ht="14.25" customHeight="1"/>
-    <row r="226" ht="14.25" customHeight="1"/>
-    <row r="227" ht="14.25" customHeight="1"/>
-    <row r="228" ht="14.25" customHeight="1"/>
-    <row r="229" ht="14.25" customHeight="1"/>
-    <row r="230" ht="14.25" customHeight="1"/>
-    <row r="231" ht="14.25" customHeight="1"/>
-    <row r="232" ht="14.25" customHeight="1"/>
-    <row r="233" ht="14.25" customHeight="1"/>
-    <row r="234" ht="14.25" customHeight="1"/>
-    <row r="235" ht="14.25" customHeight="1"/>
-    <row r="236" ht="14.25" customHeight="1"/>
-    <row r="237" ht="14.25" customHeight="1"/>
-    <row r="238" ht="14.25" customHeight="1"/>
-    <row r="239" ht="14.25" customHeight="1"/>
-    <row r="240" ht="14.25" customHeight="1"/>
-    <row r="241" ht="14.25" customHeight="1"/>
-    <row r="242" ht="14.25" customHeight="1"/>
-    <row r="243" ht="14.25" customHeight="1"/>
-    <row r="244" ht="14.25" customHeight="1"/>
-    <row r="245" ht="14.25" customHeight="1"/>
-    <row r="246" ht="14.25" customHeight="1"/>
-    <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
-    <row r="249" ht="14.25" customHeight="1"/>
-    <row r="250" ht="14.25" customHeight="1"/>
-    <row r="251" ht="14.25" customHeight="1"/>
-    <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1"/>
-    <row r="254" ht="14.25" customHeight="1"/>
-    <row r="255" ht="14.25" customHeight="1"/>
-    <row r="256" ht="14.25" customHeight="1"/>
-    <row r="257" ht="14.25" customHeight="1"/>
-    <row r="258" ht="14.25" customHeight="1"/>
-    <row r="259" ht="14.25" customHeight="1"/>
-    <row r="260" ht="14.25" customHeight="1"/>
-    <row r="261" ht="14.25" customHeight="1"/>
-    <row r="262" ht="14.25" customHeight="1"/>
-    <row r="263" ht="14.25" customHeight="1"/>
-    <row r="264" ht="14.25" customHeight="1"/>
-    <row r="265" ht="14.25" customHeight="1"/>
-    <row r="266" ht="14.25" customHeight="1"/>
-    <row r="267" ht="14.25" customHeight="1"/>
-    <row r="268" ht="14.25" customHeight="1"/>
-    <row r="269" ht="14.25" customHeight="1"/>
-    <row r="270" ht="14.25" customHeight="1"/>
-    <row r="271" ht="14.25" customHeight="1"/>
-    <row r="272" ht="14.25" customHeight="1"/>
-    <row r="273" ht="14.25" customHeight="1"/>
-    <row r="274" ht="14.25" customHeight="1"/>
-    <row r="275" ht="14.25" customHeight="1"/>
-    <row r="276" ht="14.25" customHeight="1"/>
-    <row r="277" ht="14.25" customHeight="1"/>
-    <row r="278" ht="14.25" customHeight="1"/>
-    <row r="279" ht="14.25" customHeight="1"/>
-    <row r="280" ht="14.25" customHeight="1"/>
-    <row r="281" ht="14.25" customHeight="1"/>
-    <row r="282" ht="14.25" customHeight="1"/>
-    <row r="283" ht="14.25" customHeight="1"/>
-    <row r="284" ht="14.25" customHeight="1"/>
-    <row r="285" ht="14.25" customHeight="1"/>
-    <row r="286" ht="14.25" customHeight="1"/>
-    <row r="287" ht="14.25" customHeight="1"/>
-    <row r="288" ht="14.25" customHeight="1"/>
-    <row r="289" ht="14.25" customHeight="1"/>
-    <row r="290" ht="14.25" customHeight="1"/>
-    <row r="291" ht="14.25" customHeight="1"/>
-    <row r="292" ht="14.25" customHeight="1"/>
-    <row r="293" ht="14.25" customHeight="1"/>
-    <row r="294" ht="14.25" customHeight="1"/>
-    <row r="295" ht="14.25" customHeight="1"/>
-    <row r="296" ht="14.25" customHeight="1"/>
-    <row r="297" ht="14.25" customHeight="1"/>
-    <row r="298" ht="14.25" customHeight="1"/>
-    <row r="299" ht="14.25" customHeight="1"/>
-    <row r="300" ht="14.25" customHeight="1"/>
-    <row r="301" ht="14.25" customHeight="1"/>
-    <row r="302" ht="14.25" customHeight="1"/>
-    <row r="303" ht="14.25" customHeight="1"/>
-    <row r="304" ht="14.25" customHeight="1"/>
-    <row r="305" ht="14.25" customHeight="1"/>
-    <row r="306" ht="14.25" customHeight="1"/>
-    <row r="307" ht="14.25" customHeight="1"/>
-    <row r="308" ht="14.25" customHeight="1"/>
-    <row r="309" ht="14.25" customHeight="1"/>
-    <row r="310" ht="14.25" customHeight="1"/>
-    <row r="311" ht="14.25" customHeight="1"/>
-    <row r="312" ht="14.25" customHeight="1"/>
-    <row r="313" ht="14.25" customHeight="1"/>
-    <row r="314" ht="14.25" customHeight="1"/>
-    <row r="315" ht="14.25" customHeight="1"/>
-    <row r="316" ht="14.25" customHeight="1"/>
-    <row r="317" ht="14.25" customHeight="1"/>
-    <row r="318" ht="14.25" customHeight="1"/>
-    <row r="319" ht="14.25" customHeight="1"/>
-    <row r="320" ht="14.25" customHeight="1"/>
-    <row r="321" ht="14.25" customHeight="1"/>
-    <row r="322" ht="14.25" customHeight="1"/>
-    <row r="323" ht="14.25" customHeight="1"/>
-    <row r="324" ht="14.25" customHeight="1"/>
-    <row r="325" ht="14.25" customHeight="1"/>
-    <row r="326" ht="14.25" customHeight="1"/>
-    <row r="327" ht="14.25" customHeight="1"/>
-    <row r="328" ht="14.25" customHeight="1"/>
-    <row r="329" ht="14.25" customHeight="1"/>
-    <row r="330" ht="14.25" customHeight="1"/>
-    <row r="331" ht="14.25" customHeight="1"/>
-    <row r="332" ht="14.25" customHeight="1"/>
-    <row r="333" ht="14.25" customHeight="1"/>
-    <row r="334" ht="14.25" customHeight="1"/>
-    <row r="335" ht="14.25" customHeight="1"/>
-    <row r="336" ht="14.25" customHeight="1"/>
-    <row r="337" ht="14.25" customHeight="1"/>
-    <row r="338" ht="14.25" customHeight="1"/>
-    <row r="339" ht="14.25" customHeight="1"/>
-    <row r="340" ht="14.25" customHeight="1"/>
-    <row r="341" ht="14.25" customHeight="1"/>
-    <row r="342" ht="14.25" customHeight="1"/>
-    <row r="343" ht="14.25" customHeight="1"/>
-    <row r="344" ht="14.25" customHeight="1"/>
-    <row r="345" ht="14.25" customHeight="1"/>
-    <row r="346" ht="14.25" customHeight="1"/>
-    <row r="347" ht="14.25" customHeight="1"/>
-    <row r="348" ht="14.25" customHeight="1"/>
-    <row r="349" ht="14.25" customHeight="1"/>
-    <row r="350" ht="14.25" customHeight="1"/>
-    <row r="351" ht="14.25" customHeight="1"/>
-    <row r="352" ht="14.25" customHeight="1"/>
-    <row r="353" ht="14.25" customHeight="1"/>
-    <row r="354" ht="14.25" customHeight="1"/>
-    <row r="355" ht="14.25" customHeight="1"/>
-    <row r="356" ht="14.25" customHeight="1"/>
-    <row r="357" ht="14.25" customHeight="1"/>
-    <row r="358" ht="14.25" customHeight="1"/>
-    <row r="359" ht="14.25" customHeight="1"/>
-    <row r="360" ht="14.25" customHeight="1"/>
-    <row r="361" ht="14.25" customHeight="1"/>
-    <row r="362" ht="14.25" customHeight="1"/>
-    <row r="363" ht="14.25" customHeight="1"/>
-    <row r="364" ht="14.25" customHeight="1"/>
-    <row r="365" ht="14.25" customHeight="1"/>
-    <row r="366" ht="14.25" customHeight="1"/>
-    <row r="367" ht="14.25" customHeight="1"/>
-    <row r="368" ht="14.25" customHeight="1"/>
-    <row r="369" ht="14.25" customHeight="1"/>
-    <row r="370" ht="14.25" customHeight="1"/>
-    <row r="371" ht="14.25" customHeight="1"/>
-    <row r="372" ht="14.25" customHeight="1"/>
-    <row r="373" ht="14.25" customHeight="1"/>
-    <row r="374" ht="14.25" customHeight="1"/>
-    <row r="375" ht="14.25" customHeight="1"/>
-    <row r="376" ht="14.25" customHeight="1"/>
-    <row r="377" ht="14.25" customHeight="1"/>
-    <row r="378" ht="14.25" customHeight="1"/>
-    <row r="379" ht="14.25" customHeight="1"/>
-    <row r="380" ht="14.25" customHeight="1"/>
-    <row r="381" ht="14.25" customHeight="1"/>
-    <row r="382" ht="14.25" customHeight="1"/>
-    <row r="383" ht="14.25" customHeight="1"/>
-    <row r="384" ht="14.25" customHeight="1"/>
-    <row r="385" ht="14.25" customHeight="1"/>
-    <row r="386" ht="14.25" customHeight="1"/>
-    <row r="387" ht="14.25" customHeight="1"/>
-    <row r="388" ht="14.25" customHeight="1"/>
-    <row r="389" ht="14.25" customHeight="1"/>
-    <row r="390" ht="14.25" customHeight="1"/>
-    <row r="391" ht="14.25" customHeight="1"/>
-    <row r="392" ht="14.25" customHeight="1"/>
-    <row r="393" ht="14.25" customHeight="1"/>
-    <row r="394" ht="14.25" customHeight="1"/>
-    <row r="395" ht="14.25" customHeight="1"/>
-    <row r="396" ht="14.25" customHeight="1"/>
-    <row r="397" ht="14.25" customHeight="1"/>
-    <row r="398" ht="14.25" customHeight="1"/>
-    <row r="399" ht="14.25" customHeight="1"/>
-    <row r="400" ht="14.25" customHeight="1"/>
-    <row r="401" ht="14.25" customHeight="1"/>
-    <row r="402" ht="14.25" customHeight="1"/>
-    <row r="403" ht="14.25" customHeight="1"/>
-    <row r="404" ht="14.25" customHeight="1"/>
-    <row r="405" ht="14.25" customHeight="1"/>
-    <row r="406" ht="14.25" customHeight="1"/>
-    <row r="407" ht="14.25" customHeight="1"/>
-    <row r="408" ht="14.25" customHeight="1"/>
-    <row r="409" ht="14.25" customHeight="1"/>
-    <row r="410" ht="14.25" customHeight="1"/>
-    <row r="411" ht="14.25" customHeight="1"/>
-    <row r="412" ht="14.25" customHeight="1"/>
-    <row r="413" ht="14.25" customHeight="1"/>
-    <row r="414" ht="14.25" customHeight="1"/>
-    <row r="415" ht="14.25" customHeight="1"/>
-    <row r="416" ht="14.25" customHeight="1"/>
-    <row r="417" ht="14.25" customHeight="1"/>
-    <row r="418" ht="14.25" customHeight="1"/>
-    <row r="419" ht="14.25" customHeight="1"/>
-    <row r="420" ht="14.25" customHeight="1"/>
-    <row r="421" ht="14.25" customHeight="1"/>
-    <row r="422" ht="14.25" customHeight="1"/>
-    <row r="423" ht="14.25" customHeight="1"/>
-    <row r="424" ht="14.25" customHeight="1"/>
-    <row r="425" ht="14.25" customHeight="1"/>
-    <row r="426" ht="14.25" customHeight="1"/>
-    <row r="427" ht="14.25" customHeight="1"/>
-    <row r="428" ht="14.25" customHeight="1"/>
-    <row r="429" ht="14.25" customHeight="1"/>
-    <row r="430" ht="14.25" customHeight="1"/>
-    <row r="431" ht="14.25" customHeight="1"/>
-    <row r="432" ht="14.25" customHeight="1"/>
-    <row r="433" ht="14.25" customHeight="1"/>
-    <row r="434" ht="14.25" customHeight="1"/>
-    <row r="435" ht="14.25" customHeight="1"/>
-    <row r="436" ht="14.25" customHeight="1"/>
-    <row r="437" ht="14.25" customHeight="1"/>
-    <row r="438" ht="14.25" customHeight="1"/>
-    <row r="439" ht="14.25" customHeight="1"/>
-    <row r="440" ht="14.25" customHeight="1"/>
-    <row r="441" ht="14.25" customHeight="1"/>
-    <row r="442" ht="14.25" customHeight="1"/>
-    <row r="443" ht="14.25" customHeight="1"/>
-    <row r="444" ht="14.25" customHeight="1"/>
-    <row r="445" ht="14.25" customHeight="1"/>
-    <row r="446" ht="14.25" customHeight="1"/>
-    <row r="447" ht="14.25" customHeight="1"/>
-    <row r="448" ht="14.25" customHeight="1"/>
-    <row r="449" ht="14.25" customHeight="1"/>
-    <row r="450" ht="14.25" customHeight="1"/>
-    <row r="451" ht="14.25" customHeight="1"/>
-    <row r="452" ht="14.25" customHeight="1"/>
-    <row r="453" ht="14.25" customHeight="1"/>
-    <row r="454" ht="14.25" customHeight="1"/>
-    <row r="455" ht="14.25" customHeight="1"/>
-    <row r="456" ht="14.25" customHeight="1"/>
-    <row r="457" ht="14.25" customHeight="1"/>
-    <row r="458" ht="14.25" customHeight="1"/>
-    <row r="459" ht="14.25" customHeight="1"/>
-    <row r="460" ht="14.25" customHeight="1"/>
-    <row r="461" ht="14.25" customHeight="1"/>
-    <row r="462" ht="14.25" customHeight="1"/>
-    <row r="463" ht="14.25" customHeight="1"/>
-    <row r="464" ht="14.25" customHeight="1"/>
-    <row r="465" ht="14.25" customHeight="1"/>
-    <row r="466" ht="14.25" customHeight="1"/>
-    <row r="467" ht="14.25" customHeight="1"/>
-    <row r="468" ht="14.25" customHeight="1"/>
-    <row r="469" ht="14.25" customHeight="1"/>
-    <row r="470" ht="14.25" customHeight="1"/>
-    <row r="471" ht="14.25" customHeight="1"/>
-    <row r="472" ht="14.25" customHeight="1"/>
-    <row r="473" ht="14.25" customHeight="1"/>
-    <row r="474" ht="14.25" customHeight="1"/>
-    <row r="475" ht="14.25" customHeight="1"/>
-    <row r="476" ht="14.25" customHeight="1"/>
-    <row r="477" ht="14.25" customHeight="1"/>
-    <row r="478" ht="14.25" customHeight="1"/>
-    <row r="479" ht="14.25" customHeight="1"/>
-    <row r="480" ht="14.25" customHeight="1"/>
-    <row r="481" ht="14.25" customHeight="1"/>
-    <row r="482" ht="14.25" customHeight="1"/>
-    <row r="483" ht="14.25" customHeight="1"/>
-    <row r="484" ht="14.25" customHeight="1"/>
-    <row r="485" ht="14.25" customHeight="1"/>
-    <row r="486" ht="14.25" customHeight="1"/>
-    <row r="487" ht="14.25" customHeight="1"/>
-    <row r="488" ht="14.25" customHeight="1"/>
-    <row r="489" ht="14.25" customHeight="1"/>
-    <row r="490" ht="14.25" customHeight="1"/>
-    <row r="491" ht="14.25" customHeight="1"/>
-    <row r="492" ht="14.25" customHeight="1"/>
-    <row r="493" ht="14.25" customHeight="1"/>
-    <row r="494" ht="14.25" customHeight="1"/>
-    <row r="495" ht="14.25" customHeight="1"/>
-    <row r="496" ht="14.25" customHeight="1"/>
-    <row r="497" ht="14.25" customHeight="1"/>
-    <row r="498" ht="14.25" customHeight="1"/>
-    <row r="499" ht="14.25" customHeight="1"/>
-    <row r="500" ht="14.25" customHeight="1"/>
-    <row r="501" ht="14.25" customHeight="1"/>
-    <row r="502" ht="14.25" customHeight="1"/>
-    <row r="503" ht="14.25" customHeight="1"/>
-    <row r="504" ht="14.25" customHeight="1"/>
-    <row r="505" ht="14.25" customHeight="1"/>
-    <row r="506" ht="14.25" customHeight="1"/>
-    <row r="507" ht="14.25" customHeight="1"/>
-    <row r="508" ht="14.25" customHeight="1"/>
-    <row r="509" ht="14.25" customHeight="1"/>
-    <row r="510" ht="14.25" customHeight="1"/>
-    <row r="511" ht="14.25" customHeight="1"/>
-    <row r="512" ht="14.25" customHeight="1"/>
-    <row r="513" ht="14.25" customHeight="1"/>
-    <row r="514" ht="14.25" customHeight="1"/>
-    <row r="515" ht="14.25" customHeight="1"/>
-    <row r="516" ht="14.25" customHeight="1"/>
-    <row r="517" ht="14.25" customHeight="1"/>
-    <row r="518" ht="14.25" customHeight="1"/>
-    <row r="519" ht="14.25" customHeight="1"/>
-    <row r="520" ht="14.25" customHeight="1"/>
-    <row r="521" ht="14.25" customHeight="1"/>
-    <row r="522" ht="14.25" customHeight="1"/>
-    <row r="523" ht="14.25" customHeight="1"/>
-    <row r="524" ht="14.25" customHeight="1"/>
-    <row r="525" ht="14.25" customHeight="1"/>
-    <row r="526" ht="14.25" customHeight="1"/>
-    <row r="527" ht="14.25" customHeight="1"/>
-    <row r="528" ht="14.25" customHeight="1"/>
-    <row r="529" ht="14.25" customHeight="1"/>
-    <row r="530" ht="14.25" customHeight="1"/>
-    <row r="531" ht="14.25" customHeight="1"/>
-    <row r="532" ht="14.25" customHeight="1"/>
-    <row r="533" ht="14.25" customHeight="1"/>
-    <row r="534" ht="14.25" customHeight="1"/>
-    <row r="535" ht="14.25" customHeight="1"/>
-    <row r="536" ht="14.25" customHeight="1"/>
-    <row r="537" ht="14.25" customHeight="1"/>
-    <row r="538" ht="14.25" customHeight="1"/>
-    <row r="539" ht="14.25" customHeight="1"/>
-    <row r="540" ht="14.25" customHeight="1"/>
-    <row r="541" ht="14.25" customHeight="1"/>
-    <row r="542" ht="14.25" customHeight="1"/>
-    <row r="543" ht="14.25" customHeight="1"/>
-    <row r="544" ht="14.25" customHeight="1"/>
-    <row r="545" ht="14.25" customHeight="1"/>
-    <row r="546" ht="14.25" customHeight="1"/>
-    <row r="547" ht="14.25" customHeight="1"/>
-    <row r="548" ht="14.25" customHeight="1"/>
-    <row r="549" ht="14.25" customHeight="1"/>
-    <row r="550" ht="14.25" customHeight="1"/>
-    <row r="551" ht="14.25" customHeight="1"/>
-    <row r="552" ht="14.25" customHeight="1"/>
-    <row r="553" ht="14.25" customHeight="1"/>
-    <row r="554" ht="14.25" customHeight="1"/>
-    <row r="555" ht="14.25" customHeight="1"/>
-    <row r="556" ht="14.25" customHeight="1"/>
-    <row r="557" ht="14.25" customHeight="1"/>
-    <row r="558" ht="14.25" customHeight="1"/>
-    <row r="559" ht="14.25" customHeight="1"/>
-    <row r="560" ht="14.25" customHeight="1"/>
-    <row r="561" ht="14.25" customHeight="1"/>
-    <row r="562" ht="14.25" customHeight="1"/>
-    <row r="563" ht="14.25" customHeight="1"/>
-    <row r="564" ht="14.25" customHeight="1"/>
-    <row r="565" ht="14.25" customHeight="1"/>
-    <row r="566" ht="14.25" customHeight="1"/>
-    <row r="567" ht="14.25" customHeight="1"/>
-    <row r="568" ht="14.25" customHeight="1"/>
-    <row r="569" ht="14.25" customHeight="1"/>
-    <row r="570" ht="14.25" customHeight="1"/>
-    <row r="571" ht="14.25" customHeight="1"/>
-    <row r="572" ht="14.25" customHeight="1"/>
-    <row r="573" ht="14.25" customHeight="1"/>
-    <row r="574" ht="14.25" customHeight="1"/>
-    <row r="575" ht="14.25" customHeight="1"/>
-    <row r="576" ht="14.25" customHeight="1"/>
-    <row r="577" ht="14.25" customHeight="1"/>
-    <row r="578" ht="14.25" customHeight="1"/>
-    <row r="579" ht="14.25" customHeight="1"/>
-    <row r="580" ht="14.25" customHeight="1"/>
-    <row r="581" ht="14.25" customHeight="1"/>
-    <row r="582" ht="14.25" customHeight="1"/>
-    <row r="583" ht="14.25" customHeight="1"/>
-    <row r="584" ht="14.25" customHeight="1"/>
-    <row r="585" ht="14.25" customHeight="1"/>
-    <row r="586" ht="14.25" customHeight="1"/>
-    <row r="587" ht="14.25" customHeight="1"/>
-    <row r="588" ht="14.25" customHeight="1"/>
-    <row r="589" ht="14.25" customHeight="1"/>
-    <row r="590" ht="14.25" customHeight="1"/>
-    <row r="591" ht="14.25" customHeight="1"/>
-    <row r="592" ht="14.25" customHeight="1"/>
-    <row r="593" ht="14.25" customHeight="1"/>
-    <row r="594" ht="14.25" customHeight="1"/>
-    <row r="595" ht="14.25" customHeight="1"/>
-    <row r="596" ht="14.25" customHeight="1"/>
-    <row r="597" ht="14.25" customHeight="1"/>
-    <row r="598" ht="14.25" customHeight="1"/>
-    <row r="599" ht="14.25" customHeight="1"/>
-    <row r="600" ht="14.25" customHeight="1"/>
-    <row r="601" ht="14.25" customHeight="1"/>
-    <row r="602" ht="14.25" customHeight="1"/>
-    <row r="603" ht="14.25" customHeight="1"/>
-    <row r="604" ht="14.25" customHeight="1"/>
-    <row r="605" ht="14.25" customHeight="1"/>
-    <row r="606" ht="14.25" customHeight="1"/>
-    <row r="607" ht="14.25" customHeight="1"/>
-    <row r="608" ht="14.25" customHeight="1"/>
-    <row r="609" ht="14.25" customHeight="1"/>
-    <row r="610" ht="14.25" customHeight="1"/>
-    <row r="611" ht="14.25" customHeight="1"/>
-    <row r="612" ht="14.25" customHeight="1"/>
-    <row r="613" ht="14.25" customHeight="1"/>
-    <row r="614" ht="14.25" customHeight="1"/>
-    <row r="615" ht="14.25" customHeight="1"/>
-    <row r="616" ht="14.25" customHeight="1"/>
-    <row r="617" ht="14.25" customHeight="1"/>
-    <row r="618" ht="14.25" customHeight="1"/>
-    <row r="619" ht="14.25" customHeight="1"/>
-    <row r="620" ht="14.25" customHeight="1"/>
-    <row r="621" ht="14.25" customHeight="1"/>
-    <row r="622" ht="14.25" customHeight="1"/>
-    <row r="623" ht="14.25" customHeight="1"/>
-    <row r="624" ht="14.25" customHeight="1"/>
-    <row r="625" ht="14.25" customHeight="1"/>
-    <row r="626" ht="14.25" customHeight="1"/>
-    <row r="627" ht="14.25" customHeight="1"/>
-    <row r="628" ht="14.25" customHeight="1"/>
-    <row r="629" ht="14.25" customHeight="1"/>
-    <row r="630" ht="14.25" customHeight="1"/>
-    <row r="631" ht="14.25" customHeight="1"/>
-    <row r="632" ht="14.25" customHeight="1"/>
-    <row r="633" ht="14.25" customHeight="1"/>
-    <row r="634" ht="14.25" customHeight="1"/>
-    <row r="635" ht="14.25" customHeight="1"/>
-    <row r="636" ht="14.25" customHeight="1"/>
-    <row r="637" ht="14.25" customHeight="1"/>
-    <row r="638" ht="14.25" customHeight="1"/>
-    <row r="639" ht="14.25" customHeight="1"/>
-    <row r="640" ht="14.25" customHeight="1"/>
-    <row r="641" ht="14.25" customHeight="1"/>
-    <row r="642" ht="14.25" customHeight="1"/>
-    <row r="643" ht="14.25" customHeight="1"/>
-    <row r="644" ht="14.25" customHeight="1"/>
-    <row r="645" ht="14.25" customHeight="1"/>
-    <row r="646" ht="14.25" customHeight="1"/>
-    <row r="647" ht="14.25" customHeight="1"/>
-    <row r="648" ht="14.25" customHeight="1"/>
-    <row r="649" ht="14.25" customHeight="1"/>
-    <row r="650" ht="14.25" customHeight="1"/>
-    <row r="651" ht="14.25" customHeight="1"/>
-    <row r="652" ht="14.25" customHeight="1"/>
-    <row r="653" ht="14.25" customHeight="1"/>
-    <row r="654" ht="14.25" customHeight="1"/>
-    <row r="655" ht="14.25" customHeight="1"/>
-    <row r="656" ht="14.25" customHeight="1"/>
-    <row r="657" ht="14.25" customHeight="1"/>
-    <row r="658" ht="14.25" customHeight="1"/>
-    <row r="659" ht="14.25" customHeight="1"/>
-    <row r="660" ht="14.25" customHeight="1"/>
-    <row r="661" ht="14.25" customHeight="1"/>
-    <row r="662" ht="14.25" customHeight="1"/>
-    <row r="663" ht="14.25" customHeight="1"/>
-    <row r="664" ht="14.25" customHeight="1"/>
-    <row r="665" ht="14.25" customHeight="1"/>
-    <row r="666" ht="14.25" customHeight="1"/>
-    <row r="667" ht="14.25" customHeight="1"/>
-    <row r="668" ht="14.25" customHeight="1"/>
-    <row r="669" ht="14.25" customHeight="1"/>
-    <row r="670" ht="14.25" customHeight="1"/>
-    <row r="671" ht="14.25" customHeight="1"/>
-    <row r="672" ht="14.25" customHeight="1"/>
-    <row r="673" ht="14.25" customHeight="1"/>
-    <row r="674" ht="14.25" customHeight="1"/>
-    <row r="675" ht="14.25" customHeight="1"/>
-    <row r="676" ht="14.25" customHeight="1"/>
-    <row r="677" ht="14.25" customHeight="1"/>
-    <row r="678" ht="14.25" customHeight="1"/>
-    <row r="679" ht="14.25" customHeight="1"/>
-    <row r="680" ht="14.25" customHeight="1"/>
-    <row r="681" ht="14.25" customHeight="1"/>
-    <row r="682" ht="14.25" customHeight="1"/>
-    <row r="683" ht="14.25" customHeight="1"/>
-    <row r="684" ht="14.25" customHeight="1"/>
-    <row r="685" ht="14.25" customHeight="1"/>
-    <row r="686" ht="14.25" customHeight="1"/>
-    <row r="687" ht="14.25" customHeight="1"/>
-    <row r="688" ht="14.25" customHeight="1"/>
-    <row r="689" ht="14.25" customHeight="1"/>
-    <row r="690" ht="14.25" customHeight="1"/>
-    <row r="691" ht="14.25" customHeight="1"/>
-    <row r="692" ht="14.25" customHeight="1"/>
-    <row r="693" ht="14.25" customHeight="1"/>
-    <row r="694" ht="14.25" customHeight="1"/>
-    <row r="695" ht="14.25" customHeight="1"/>
-    <row r="696" ht="14.25" customHeight="1"/>
-    <row r="697" ht="14.25" customHeight="1"/>
-    <row r="698" ht="14.25" customHeight="1"/>
-    <row r="699" ht="14.25" customHeight="1"/>
-    <row r="700" ht="14.25" customHeight="1"/>
-    <row r="701" ht="14.25" customHeight="1"/>
-    <row r="702" ht="14.25" customHeight="1"/>
-    <row r="703" ht="14.25" customHeight="1"/>
-    <row r="704" ht="14.25" customHeight="1"/>
-    <row r="705" ht="14.25" customHeight="1"/>
-    <row r="706" ht="14.25" customHeight="1"/>
-    <row r="707" ht="14.25" customHeight="1"/>
-    <row r="708" ht="14.25" customHeight="1"/>
-    <row r="709" ht="14.25" customHeight="1"/>
-    <row r="710" ht="14.25" customHeight="1"/>
-    <row r="711" ht="14.25" customHeight="1"/>
-    <row r="712" ht="14.25" customHeight="1"/>
-    <row r="713" ht="14.25" customHeight="1"/>
-    <row r="714" ht="14.25" customHeight="1"/>
-    <row r="715" ht="14.25" customHeight="1"/>
-    <row r="716" ht="14.25" customHeight="1"/>
-    <row r="717" ht="14.25" customHeight="1"/>
-    <row r="718" ht="14.25" customHeight="1"/>
-    <row r="719" ht="14.25" customHeight="1"/>
-    <row r="720" ht="14.25" customHeight="1"/>
-    <row r="721" ht="14.25" customHeight="1"/>
-    <row r="722" ht="14.25" customHeight="1"/>
-    <row r="723" ht="14.25" customHeight="1"/>
-    <row r="724" ht="14.25" customHeight="1"/>
-    <row r="725" ht="14.25" customHeight="1"/>
-    <row r="726" ht="14.25" customHeight="1"/>
-    <row r="727" ht="14.25" customHeight="1"/>
-    <row r="728" ht="14.25" customHeight="1"/>
-    <row r="729" ht="14.25" customHeight="1"/>
-    <row r="730" ht="14.25" customHeight="1"/>
-    <row r="731" ht="14.25" customHeight="1"/>
-    <row r="732" ht="14.25" customHeight="1"/>
-    <row r="733" ht="14.25" customHeight="1"/>
-    <row r="734" ht="14.25" customHeight="1"/>
-    <row r="735" ht="14.25" customHeight="1"/>
-    <row r="736" ht="14.25" customHeight="1"/>
-    <row r="737" ht="14.25" customHeight="1"/>
-    <row r="738" ht="14.25" customHeight="1"/>
-    <row r="739" ht="14.25" customHeight="1"/>
-    <row r="740" ht="14.25" customHeight="1"/>
-    <row r="741" ht="14.25" customHeight="1"/>
-    <row r="742" ht="14.25" customHeight="1"/>
-    <row r="743" ht="14.25" customHeight="1"/>
-    <row r="744" ht="14.25" customHeight="1"/>
-    <row r="745" ht="14.25" customHeight="1"/>
-    <row r="746" ht="14.25" customHeight="1"/>
-    <row r="747" ht="14.25" customHeight="1"/>
-    <row r="748" ht="14.25" customHeight="1"/>
-    <row r="749" ht="14.25" customHeight="1"/>
-    <row r="750" ht="14.25" customHeight="1"/>
-    <row r="751" ht="14.25" customHeight="1"/>
-    <row r="752" ht="14.25" customHeight="1"/>
-    <row r="753" ht="14.25" customHeight="1"/>
-    <row r="754" ht="14.25" customHeight="1"/>
-    <row r="755" ht="14.25" customHeight="1"/>
-    <row r="756" ht="14.25" customHeight="1"/>
-    <row r="757" ht="14.25" customHeight="1"/>
-    <row r="758" ht="14.25" customHeight="1"/>
-    <row r="759" ht="14.25" customHeight="1"/>
-    <row r="760" ht="14.25" customHeight="1"/>
-    <row r="761" ht="14.25" customHeight="1"/>
-    <row r="762" ht="14.25" customHeight="1"/>
-    <row r="763" ht="14.25" customHeight="1"/>
-    <row r="764" ht="14.25" customHeight="1"/>
-    <row r="765" ht="14.25" customHeight="1"/>
-    <row r="766" ht="14.25" customHeight="1"/>
-    <row r="767" ht="14.25" customHeight="1"/>
-    <row r="768" ht="14.25" customHeight="1"/>
-    <row r="769" ht="14.25" customHeight="1"/>
-    <row r="770" ht="14.25" customHeight="1"/>
-    <row r="771" ht="14.25" customHeight="1"/>
-    <row r="772" ht="14.25" customHeight="1"/>
-    <row r="773" ht="14.25" customHeight="1"/>
-    <row r="774" ht="14.25" customHeight="1"/>
-    <row r="775" ht="14.25" customHeight="1"/>
-    <row r="776" ht="14.25" customHeight="1"/>
-    <row r="777" ht="14.25" customHeight="1"/>
-    <row r="778" ht="14.25" customHeight="1"/>
-    <row r="779" ht="14.25" customHeight="1"/>
-    <row r="780" ht="14.25" customHeight="1"/>
-    <row r="781" ht="14.25" customHeight="1"/>
-    <row r="782" ht="14.25" customHeight="1"/>
-    <row r="783" ht="14.25" customHeight="1"/>
-    <row r="784" ht="14.25" customHeight="1"/>
-    <row r="785" ht="14.25" customHeight="1"/>
-    <row r="786" ht="14.25" customHeight="1"/>
-    <row r="787" ht="14.25" customHeight="1"/>
-    <row r="788" ht="14.25" customHeight="1"/>
-    <row r="789" ht="14.25" customHeight="1"/>
-    <row r="790" ht="14.25" customHeight="1"/>
-    <row r="791" ht="14.25" customHeight="1"/>
-    <row r="792" ht="14.25" customHeight="1"/>
-    <row r="793" ht="14.25" customHeight="1"/>
-    <row r="794" ht="14.25" customHeight="1"/>
-    <row r="795" ht="14.25" customHeight="1"/>
-    <row r="796" ht="14.25" customHeight="1"/>
-    <row r="797" ht="14.25" customHeight="1"/>
-    <row r="798" ht="14.25" customHeight="1"/>
-    <row r="799" ht="14.25" customHeight="1"/>
-    <row r="800" ht="14.25" customHeight="1"/>
-    <row r="801" ht="14.25" customHeight="1"/>
-    <row r="802" ht="14.25" customHeight="1"/>
-    <row r="803" ht="14.25" customHeight="1"/>
-    <row r="804" ht="14.25" customHeight="1"/>
-    <row r="805" ht="14.25" customHeight="1"/>
-    <row r="806" ht="14.25" customHeight="1"/>
-    <row r="807" ht="14.25" customHeight="1"/>
-    <row r="808" ht="14.25" customHeight="1"/>
-    <row r="809" ht="14.25" customHeight="1"/>
-    <row r="810" ht="14.25" customHeight="1"/>
-    <row r="811" ht="14.25" customHeight="1"/>
-    <row r="812" ht="14.25" customHeight="1"/>
-    <row r="813" ht="14.25" customHeight="1"/>
-    <row r="814" ht="14.25" customHeight="1"/>
-    <row r="815" ht="14.25" customHeight="1"/>
-    <row r="816" ht="14.25" customHeight="1"/>
-    <row r="817" ht="14.25" customHeight="1"/>
-    <row r="818" ht="14.25" customHeight="1"/>
-    <row r="819" ht="14.25" customHeight="1"/>
-    <row r="820" ht="14.25" customHeight="1"/>
-    <row r="821" ht="14.25" customHeight="1"/>
-    <row r="822" ht="14.25" customHeight="1"/>
-    <row r="823" ht="14.25" customHeight="1"/>
-    <row r="824" ht="14.25" customHeight="1"/>
-    <row r="825" ht="14.25" customHeight="1"/>
-    <row r="826" ht="14.25" customHeight="1"/>
-    <row r="827" ht="14.25" customHeight="1"/>
-    <row r="828" ht="14.25" customHeight="1"/>
-    <row r="829" ht="14.25" customHeight="1"/>
-    <row r="830" ht="14.25" customHeight="1"/>
-    <row r="831" ht="14.25" customHeight="1"/>
-    <row r="832" ht="14.25" customHeight="1"/>
-    <row r="833" ht="14.25" customHeight="1"/>
-    <row r="834" ht="14.25" customHeight="1"/>
-    <row r="835" ht="14.25" customHeight="1"/>
-    <row r="836" ht="14.25" customHeight="1"/>
-    <row r="837" ht="14.25" customHeight="1"/>
-    <row r="838" ht="14.25" customHeight="1"/>
-    <row r="839" ht="14.25" customHeight="1"/>
-    <row r="840" ht="14.25" customHeight="1"/>
-    <row r="841" ht="14.25" customHeight="1"/>
-    <row r="842" ht="14.25" customHeight="1"/>
-    <row r="843" ht="14.25" customHeight="1"/>
-    <row r="844" ht="14.25" customHeight="1"/>
-    <row r="845" ht="14.25" customHeight="1"/>
-    <row r="846" ht="14.25" customHeight="1"/>
-    <row r="847" ht="14.25" customHeight="1"/>
-    <row r="848" ht="14.25" customHeight="1"/>
-    <row r="849" ht="14.25" customHeight="1"/>
-    <row r="850" ht="14.25" customHeight="1"/>
-    <row r="851" ht="14.25" customHeight="1"/>
-    <row r="852" ht="14.25" customHeight="1"/>
-    <row r="853" ht="14.25" customHeight="1"/>
-    <row r="854" ht="14.25" customHeight="1"/>
-    <row r="855" ht="14.25" customHeight="1"/>
-    <row r="856" ht="14.25" customHeight="1"/>
-    <row r="857" ht="14.25" customHeight="1"/>
-    <row r="858" ht="14.25" customHeight="1"/>
-    <row r="859" ht="14.25" customHeight="1"/>
-    <row r="860" ht="14.25" customHeight="1"/>
-    <row r="861" ht="14.25" customHeight="1"/>
-    <row r="862" ht="14.25" customHeight="1"/>
-    <row r="863" ht="14.25" customHeight="1"/>
-    <row r="864" ht="14.25" customHeight="1"/>
-    <row r="865" ht="14.25" customHeight="1"/>
-    <row r="866" ht="14.25" customHeight="1"/>
-    <row r="867" ht="14.25" customHeight="1"/>
-    <row r="868" ht="14.25" customHeight="1"/>
-    <row r="869" ht="14.25" customHeight="1"/>
-    <row r="870" ht="14.25" customHeight="1"/>
-    <row r="871" ht="14.25" customHeight="1"/>
-    <row r="872" ht="14.25" customHeight="1"/>
-    <row r="873" ht="14.25" customHeight="1"/>
-    <row r="874" ht="14.25" customHeight="1"/>
-    <row r="875" ht="14.25" customHeight="1"/>
-    <row r="876" ht="14.25" customHeight="1"/>
-    <row r="877" ht="14.25" customHeight="1"/>
-    <row r="878" ht="14.25" customHeight="1"/>
-    <row r="879" ht="14.25" customHeight="1"/>
-    <row r="880" ht="14.25" customHeight="1"/>
-    <row r="881" ht="14.25" customHeight="1"/>
-    <row r="882" ht="14.25" customHeight="1"/>
-    <row r="883" ht="14.25" customHeight="1"/>
-    <row r="884" ht="14.25" customHeight="1"/>
-    <row r="885" ht="14.25" customHeight="1"/>
-    <row r="886" ht="14.25" customHeight="1"/>
-    <row r="887" ht="14.25" customHeight="1"/>
-    <row r="888" ht="14.25" customHeight="1"/>
-    <row r="889" ht="14.25" customHeight="1"/>
-    <row r="890" ht="14.25" customHeight="1"/>
-    <row r="891" ht="14.25" customHeight="1"/>
-    <row r="892" ht="14.25" customHeight="1"/>
-    <row r="893" ht="14.25" customHeight="1"/>
-    <row r="894" ht="14.25" customHeight="1"/>
-    <row r="895" ht="14.25" customHeight="1"/>
-    <row r="896" ht="14.25" customHeight="1"/>
-    <row r="897" ht="14.25" customHeight="1"/>
-    <row r="898" ht="14.25" customHeight="1"/>
-    <row r="899" ht="14.25" customHeight="1"/>
-    <row r="900" ht="14.25" customHeight="1"/>
-    <row r="901" ht="14.25" customHeight="1"/>
-    <row r="902" ht="14.25" customHeight="1"/>
-    <row r="903" ht="14.25" customHeight="1"/>
-    <row r="904" ht="14.25" customHeight="1"/>
-    <row r="905" ht="14.25" customHeight="1"/>
-    <row r="906" ht="14.25" customHeight="1"/>
-    <row r="907" ht="14.25" customHeight="1"/>
-    <row r="908" ht="14.25" customHeight="1"/>
-    <row r="909" ht="14.25" customHeight="1"/>
-    <row r="910" ht="14.25" customHeight="1"/>
-    <row r="911" ht="14.25" customHeight="1"/>
-    <row r="912" ht="14.25" customHeight="1"/>
-    <row r="913" ht="14.25" customHeight="1"/>
-    <row r="914" ht="14.25" customHeight="1"/>
-    <row r="915" ht="14.25" customHeight="1"/>
-    <row r="916" ht="14.25" customHeight="1"/>
-    <row r="917" ht="14.25" customHeight="1"/>
-    <row r="918" ht="14.25" customHeight="1"/>
-    <row r="919" ht="14.25" customHeight="1"/>
-    <row r="920" ht="14.25" customHeight="1"/>
-    <row r="921" ht="14.25" customHeight="1"/>
-    <row r="922" ht="14.25" customHeight="1"/>
-    <row r="923" ht="14.25" customHeight="1"/>
-    <row r="924" ht="14.25" customHeight="1"/>
-    <row r="925" ht="14.25" customHeight="1"/>
-    <row r="926" ht="14.25" customHeight="1"/>
-    <row r="927" ht="14.25" customHeight="1"/>
-    <row r="928" ht="14.25" customHeight="1"/>
-    <row r="929" ht="14.25" customHeight="1"/>
-    <row r="930" ht="14.25" customHeight="1"/>
-    <row r="931" ht="14.25" customHeight="1"/>
-    <row r="932" ht="14.25" customHeight="1"/>
-    <row r="933" ht="14.25" customHeight="1"/>
-    <row r="934" ht="14.25" customHeight="1"/>
-    <row r="935" ht="14.25" customHeight="1"/>
-    <row r="936" ht="14.25" customHeight="1"/>
-    <row r="937" ht="14.25" customHeight="1"/>
-    <row r="938" ht="14.25" customHeight="1"/>
-    <row r="939" ht="14.25" customHeight="1"/>
-    <row r="940" ht="14.25" customHeight="1"/>
-    <row r="941" ht="14.25" customHeight="1"/>
-    <row r="942" ht="14.25" customHeight="1"/>
-    <row r="943" ht="14.25" customHeight="1"/>
-    <row r="944" ht="14.25" customHeight="1"/>
-    <row r="945" ht="14.25" customHeight="1"/>
-    <row r="946" ht="14.25" customHeight="1"/>
-    <row r="947" ht="14.25" customHeight="1"/>
-    <row r="948" ht="14.25" customHeight="1"/>
-    <row r="949" ht="14.25" customHeight="1"/>
-    <row r="950" ht="14.25" customHeight="1"/>
-    <row r="951" ht="14.25" customHeight="1"/>
-    <row r="952" ht="14.25" customHeight="1"/>
-    <row r="953" ht="14.25" customHeight="1"/>
-    <row r="954" ht="14.25" customHeight="1"/>
-    <row r="955" ht="14.25" customHeight="1"/>
-    <row r="956" ht="14.25" customHeight="1"/>
-    <row r="957" ht="14.25" customHeight="1"/>
-    <row r="958" ht="14.25" customHeight="1"/>
-    <row r="959" ht="14.25" customHeight="1"/>
-    <row r="960" ht="14.25" customHeight="1"/>
-    <row r="961" ht="14.25" customHeight="1"/>
-    <row r="962" ht="14.25" customHeight="1"/>
-    <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
-    <row r="973" ht="14.25" customHeight="1"/>
-    <row r="974" ht="14.25" customHeight="1"/>
-    <row r="975" ht="14.25" customHeight="1"/>
-    <row r="976" ht="14.25" customHeight="1"/>
-    <row r="977" ht="14.25" customHeight="1"/>
-    <row r="978" ht="14.25" customHeight="1"/>
-    <row r="979" ht="14.25" customHeight="1"/>
-    <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="17" ht="14.25" customHeight="true"/>
+    <row r="18" ht="14.25" customHeight="true"/>
+    <row r="19" ht="14.25" customHeight="true"/>
+    <row r="20" ht="14.25" customHeight="true"/>
+    <row r="21" ht="14.25" customHeight="true"/>
+    <row r="22" ht="14.25" customHeight="true"/>
+    <row r="23" ht="14.25" customHeight="true"/>
+    <row r="24" ht="14.25" customHeight="true"/>
+    <row r="25" ht="14.25" customHeight="true"/>
+    <row r="26" ht="14.25" customHeight="true"/>
+    <row r="27" ht="14.25" customHeight="true"/>
+    <row r="28" ht="14.25" customHeight="true"/>
+    <row r="29" ht="14.25" customHeight="true"/>
+    <row r="30" ht="14.25" customHeight="true"/>
+    <row r="31" ht="14.25" customHeight="true"/>
+    <row r="32" ht="14.25" customHeight="true"/>
+    <row r="33" ht="14.25" customHeight="true"/>
+    <row r="34" ht="14.25" customHeight="true"/>
+    <row r="35" ht="14.25" customHeight="true"/>
+    <row r="36" ht="14.25" customHeight="true"/>
+    <row r="37" ht="14.25" customHeight="true"/>
+    <row r="38" ht="14.25" customHeight="true"/>
+    <row r="39" ht="14.25" customHeight="true"/>
+    <row r="40" ht="14.25" customHeight="true"/>
+    <row r="41" ht="14.25" customHeight="true"/>
+    <row r="42" ht="14.25" customHeight="true"/>
+    <row r="43" ht="14.25" customHeight="true"/>
+    <row r="44" ht="14.25" customHeight="true"/>
+    <row r="45" ht="14.25" customHeight="true"/>
+    <row r="46" ht="14.25" customHeight="true"/>
+    <row r="47" ht="14.25" customHeight="true"/>
+    <row r="48" ht="14.25" customHeight="true"/>
+    <row r="49" ht="14.25" customHeight="true"/>
+    <row r="50" ht="14.25" customHeight="true"/>
+    <row r="51" ht="14.25" customHeight="true"/>
+    <row r="52" ht="14.25" customHeight="true"/>
+    <row r="53" ht="14.25" customHeight="true"/>
+    <row r="54" ht="14.25" customHeight="true"/>
+    <row r="55" ht="14.25" customHeight="true"/>
+    <row r="56" ht="14.25" customHeight="true"/>
+    <row r="57" ht="14.25" customHeight="true"/>
+    <row r="58" ht="14.25" customHeight="true"/>
+    <row r="59" ht="14.25" customHeight="true"/>
+    <row r="60" ht="14.25" customHeight="true"/>
+    <row r="61" ht="14.25" customHeight="true"/>
+    <row r="62" ht="14.25" customHeight="true"/>
+    <row r="63" ht="14.25" customHeight="true"/>
+    <row r="64" ht="14.25" customHeight="true"/>
+    <row r="65" ht="14.25" customHeight="true"/>
+    <row r="66" ht="14.25" customHeight="true"/>
+    <row r="67" ht="14.25" customHeight="true"/>
+    <row r="68" ht="14.25" customHeight="true"/>
+    <row r="69" ht="14.25" customHeight="true"/>
+    <row r="70" ht="14.25" customHeight="true"/>
+    <row r="71" ht="14.25" customHeight="true"/>
+    <row r="72" ht="14.25" customHeight="true"/>
+    <row r="73" ht="14.25" customHeight="true"/>
+    <row r="74" ht="14.25" customHeight="true"/>
+    <row r="75" ht="14.25" customHeight="true"/>
+    <row r="76" ht="14.25" customHeight="true"/>
+    <row r="77" ht="14.25" customHeight="true"/>
+    <row r="78" ht="14.25" customHeight="true"/>
+    <row r="79" ht="14.25" customHeight="true"/>
+    <row r="80" ht="14.25" customHeight="true"/>
+    <row r="81" ht="14.25" customHeight="true"/>
+    <row r="82" ht="14.25" customHeight="true"/>
+    <row r="83" ht="14.25" customHeight="true"/>
+    <row r="84" ht="14.25" customHeight="true"/>
+    <row r="85" ht="14.25" customHeight="true"/>
+    <row r="86" ht="14.25" customHeight="true"/>
+    <row r="87" ht="14.25" customHeight="true"/>
+    <row r="88" ht="14.25" customHeight="true"/>
+    <row r="89" ht="14.25" customHeight="true"/>
+    <row r="90" ht="14.25" customHeight="true"/>
+    <row r="91" ht="14.25" customHeight="true"/>
+    <row r="92" ht="14.25" customHeight="true"/>
+    <row r="93" ht="14.25" customHeight="true"/>
+    <row r="94" ht="14.25" customHeight="true"/>
+    <row r="95" ht="14.25" customHeight="true"/>
+    <row r="96" ht="14.25" customHeight="true"/>
+    <row r="97" ht="14.25" customHeight="true"/>
+    <row r="98" ht="14.25" customHeight="true"/>
+    <row r="99" ht="14.25" customHeight="true"/>
+    <row r="100" ht="14.25" customHeight="true"/>
+    <row r="101" ht="14.25" customHeight="true"/>
+    <row r="102" ht="14.25" customHeight="true"/>
+    <row r="103" ht="14.25" customHeight="true"/>
+    <row r="104" ht="14.25" customHeight="true"/>
+    <row r="105" ht="14.25" customHeight="true"/>
+    <row r="106" ht="14.25" customHeight="true"/>
+    <row r="107" ht="14.25" customHeight="true"/>
+    <row r="108" ht="14.25" customHeight="true"/>
+    <row r="109" ht="14.25" customHeight="true"/>
+    <row r="110" ht="14.25" customHeight="true"/>
+    <row r="111" ht="14.25" customHeight="true"/>
+    <row r="112" ht="14.25" customHeight="true"/>
+    <row r="113" ht="14.25" customHeight="true"/>
+    <row r="114" ht="14.25" customHeight="true"/>
+    <row r="115" ht="14.25" customHeight="true"/>
+    <row r="116" ht="14.25" customHeight="true"/>
+    <row r="117" ht="14.25" customHeight="true"/>
+    <row r="118" ht="14.25" customHeight="true"/>
+    <row r="119" ht="14.25" customHeight="true"/>
+    <row r="120" ht="14.25" customHeight="true"/>
+    <row r="121" ht="14.25" customHeight="true"/>
+    <row r="122" ht="14.25" customHeight="true"/>
+    <row r="123" ht="14.25" customHeight="true"/>
+    <row r="124" ht="14.25" customHeight="true"/>
+    <row r="125" ht="14.25" customHeight="true"/>
+    <row r="126" ht="14.25" customHeight="true"/>
+    <row r="127" ht="14.25" customHeight="true"/>
+    <row r="128" ht="14.25" customHeight="true"/>
+    <row r="129" ht="14.25" customHeight="true"/>
+    <row r="130" ht="14.25" customHeight="true"/>
+    <row r="131" ht="14.25" customHeight="true"/>
+    <row r="132" ht="14.25" customHeight="true"/>
+    <row r="133" ht="14.25" customHeight="true"/>
+    <row r="134" ht="14.25" customHeight="true"/>
+    <row r="135" ht="14.25" customHeight="true"/>
+    <row r="136" ht="14.25" customHeight="true"/>
+    <row r="137" ht="14.25" customHeight="true"/>
+    <row r="138" ht="14.25" customHeight="true"/>
+    <row r="139" ht="14.25" customHeight="true"/>
+    <row r="140" ht="14.25" customHeight="true"/>
+    <row r="141" ht="14.25" customHeight="true"/>
+    <row r="142" ht="14.25" customHeight="true"/>
+    <row r="143" ht="14.25" customHeight="true"/>
+    <row r="144" ht="14.25" customHeight="true"/>
+    <row r="145" ht="14.25" customHeight="true"/>
+    <row r="146" ht="14.25" customHeight="true"/>
+    <row r="147" ht="14.25" customHeight="true"/>
+    <row r="148" ht="14.25" customHeight="true"/>
+    <row r="149" ht="14.25" customHeight="true"/>
+    <row r="150" ht="14.25" customHeight="true"/>
+    <row r="151" ht="14.25" customHeight="true"/>
+    <row r="152" ht="14.25" customHeight="true"/>
+    <row r="153" ht="14.25" customHeight="true"/>
+    <row r="154" ht="14.25" customHeight="true"/>
+    <row r="155" ht="14.25" customHeight="true"/>
+    <row r="156" ht="14.25" customHeight="true"/>
+    <row r="157" ht="14.25" customHeight="true"/>
+    <row r="158" ht="14.25" customHeight="true"/>
+    <row r="159" ht="14.25" customHeight="true"/>
+    <row r="160" ht="14.25" customHeight="true"/>
+    <row r="161" ht="14.25" customHeight="true"/>
+    <row r="162" ht="14.25" customHeight="true"/>
+    <row r="163" ht="14.25" customHeight="true"/>
+    <row r="164" ht="14.25" customHeight="true"/>
+    <row r="165" ht="14.25" customHeight="true"/>
+    <row r="166" ht="14.25" customHeight="true"/>
+    <row r="167" ht="14.25" customHeight="true"/>
+    <row r="168" ht="14.25" customHeight="true"/>
+    <row r="169" ht="14.25" customHeight="true"/>
+    <row r="170" ht="14.25" customHeight="true"/>
+    <row r="171" ht="14.25" customHeight="true"/>
+    <row r="172" ht="14.25" customHeight="true"/>
+    <row r="173" ht="14.25" customHeight="true"/>
+    <row r="174" ht="14.25" customHeight="true"/>
+    <row r="175" ht="14.25" customHeight="true"/>
+    <row r="176" ht="14.25" customHeight="true"/>
+    <row r="177" ht="14.25" customHeight="true"/>
+    <row r="178" ht="14.25" customHeight="true"/>
+    <row r="179" ht="14.25" customHeight="true"/>
+    <row r="180" ht="14.25" customHeight="true"/>
+    <row r="181" ht="14.25" customHeight="true"/>
+    <row r="182" ht="14.25" customHeight="true"/>
+    <row r="183" ht="14.25" customHeight="true"/>
+    <row r="184" ht="14.25" customHeight="true"/>
+    <row r="185" ht="14.25" customHeight="true"/>
+    <row r="186" ht="14.25" customHeight="true"/>
+    <row r="187" ht="14.25" customHeight="true"/>
+    <row r="188" ht="14.25" customHeight="true"/>
+    <row r="189" ht="14.25" customHeight="true"/>
+    <row r="190" ht="14.25" customHeight="true"/>
+    <row r="191" ht="14.25" customHeight="true"/>
+    <row r="192" ht="14.25" customHeight="true"/>
+    <row r="193" ht="14.25" customHeight="true"/>
+    <row r="194" ht="14.25" customHeight="true"/>
+    <row r="195" ht="14.25" customHeight="true"/>
+    <row r="196" ht="14.25" customHeight="true"/>
+    <row r="197" ht="14.25" customHeight="true"/>
+    <row r="198" ht="14.25" customHeight="true"/>
+    <row r="199" ht="14.25" customHeight="true"/>
+    <row r="200" ht="14.25" customHeight="true"/>
+    <row r="201" ht="14.25" customHeight="true"/>
+    <row r="202" ht="14.25" customHeight="true"/>
+    <row r="203" ht="14.25" customHeight="true"/>
+    <row r="204" ht="14.25" customHeight="true"/>
+    <row r="205" ht="14.25" customHeight="true"/>
+    <row r="206" ht="14.25" customHeight="true"/>
+    <row r="207" ht="14.25" customHeight="true"/>
+    <row r="208" ht="14.25" customHeight="true"/>
+    <row r="209" ht="14.25" customHeight="true"/>
+    <row r="210" ht="14.25" customHeight="true"/>
+    <row r="211" ht="14.25" customHeight="true"/>
+    <row r="212" ht="14.25" customHeight="true"/>
+    <row r="213" ht="14.25" customHeight="true"/>
+    <row r="214" ht="14.25" customHeight="true"/>
+    <row r="215" ht="14.25" customHeight="true"/>
+    <row r="216" ht="14.25" customHeight="true"/>
+    <row r="217" ht="14.25" customHeight="true"/>
+    <row r="218" ht="14.25" customHeight="true"/>
+    <row r="219" ht="14.25" customHeight="true"/>
+    <row r="220" ht="14.25" customHeight="true"/>
+    <row r="221" ht="14.25" customHeight="true"/>
+    <row r="222" ht="14.25" customHeight="true"/>
+    <row r="223" ht="14.25" customHeight="true"/>
+    <row r="224" ht="14.25" customHeight="true"/>
+    <row r="225" ht="14.25" customHeight="true"/>
+    <row r="226" ht="14.25" customHeight="true"/>
+    <row r="227" ht="14.25" customHeight="true"/>
+    <row r="228" ht="14.25" customHeight="true"/>
+    <row r="229" ht="14.25" customHeight="true"/>
+    <row r="230" ht="14.25" customHeight="true"/>
+    <row r="231" ht="14.25" customHeight="true"/>
+    <row r="232" ht="14.25" customHeight="true"/>
+    <row r="233" ht="14.25" customHeight="true"/>
+    <row r="234" ht="14.25" customHeight="true"/>
+    <row r="235" ht="14.25" customHeight="true"/>
+    <row r="236" ht="14.25" customHeight="true"/>
+    <row r="237" ht="14.25" customHeight="true"/>
+    <row r="238" ht="14.25" customHeight="true"/>
+    <row r="239" ht="14.25" customHeight="true"/>
+    <row r="240" ht="14.25" customHeight="true"/>
+    <row r="241" ht="14.25" customHeight="true"/>
+    <row r="242" ht="14.25" customHeight="true"/>
+    <row r="243" ht="14.25" customHeight="true"/>
+    <row r="244" ht="14.25" customHeight="true"/>
+    <row r="245" ht="14.25" customHeight="true"/>
+    <row r="246" ht="14.25" customHeight="true"/>
+    <row r="247" ht="14.25" customHeight="true"/>
+    <row r="248" ht="14.25" customHeight="true"/>
+    <row r="249" ht="14.25" customHeight="true"/>
+    <row r="250" ht="14.25" customHeight="true"/>
+    <row r="251" ht="14.25" customHeight="true"/>
+    <row r="252" ht="14.25" customHeight="true"/>
+    <row r="253" ht="14.25" customHeight="true"/>
+    <row r="254" ht="14.25" customHeight="true"/>
+    <row r="255" ht="14.25" customHeight="true"/>
+    <row r="256" ht="14.25" customHeight="true"/>
+    <row r="257" ht="14.25" customHeight="true"/>
+    <row r="258" ht="14.25" customHeight="true"/>
+    <row r="259" ht="14.25" customHeight="true"/>
+    <row r="260" ht="14.25" customHeight="true"/>
+    <row r="261" ht="14.25" customHeight="true"/>
+    <row r="262" ht="14.25" customHeight="true"/>
+    <row r="263" ht="14.25" customHeight="true"/>
+    <row r="264" ht="14.25" customHeight="true"/>
+    <row r="265" ht="14.25" customHeight="true"/>
+    <row r="266" ht="14.25" customHeight="true"/>
+    <row r="267" ht="14.25" customHeight="true"/>
+    <row r="268" ht="14.25" customHeight="true"/>
+    <row r="269" ht="14.25" customHeight="true"/>
+    <row r="270" ht="14.25" customHeight="true"/>
+    <row r="271" ht="14.25" customHeight="true"/>
+    <row r="272" ht="14.25" customHeight="true"/>
+    <row r="273" ht="14.25" customHeight="true"/>
+    <row r="274" ht="14.25" customHeight="true"/>
+    <row r="275" ht="14.25" customHeight="true"/>
+    <row r="276" ht="14.25" customHeight="true"/>
+    <row r="277" ht="14.25" customHeight="true"/>
+    <row r="278" ht="14.25" customHeight="true"/>
+    <row r="279" ht="14.25" customHeight="true"/>
+    <row r="280" ht="14.25" customHeight="true"/>
+    <row r="281" ht="14.25" customHeight="true"/>
+    <row r="282" ht="14.25" customHeight="true"/>
+    <row r="283" ht="14.25" customHeight="true"/>
+    <row r="284" ht="14.25" customHeight="true"/>
+    <row r="285" ht="14.25" customHeight="true"/>
+    <row r="286" ht="14.25" customHeight="true"/>
+    <row r="287" ht="14.25" customHeight="true"/>
+    <row r="288" ht="14.25" customHeight="true"/>
+    <row r="289" ht="14.25" customHeight="true"/>
+    <row r="290" ht="14.25" customHeight="true"/>
+    <row r="291" ht="14.25" customHeight="true"/>
+    <row r="292" ht="14.25" customHeight="true"/>
+    <row r="293" ht="14.25" customHeight="true"/>
+    <row r="294" ht="14.25" customHeight="true"/>
+    <row r="295" ht="14.25" customHeight="true"/>
+    <row r="296" ht="14.25" customHeight="true"/>
+    <row r="297" ht="14.25" customHeight="true"/>
+    <row r="298" ht="14.25" customHeight="true"/>
+    <row r="299" ht="14.25" customHeight="true"/>
+    <row r="300" ht="14.25" customHeight="true"/>
+    <row r="301" ht="14.25" customHeight="true"/>
+    <row r="302" ht="14.25" customHeight="true"/>
+    <row r="303" ht="14.25" customHeight="true"/>
+    <row r="304" ht="14.25" customHeight="true"/>
+    <row r="305" ht="14.25" customHeight="true"/>
+    <row r="306" ht="14.25" customHeight="true"/>
+    <row r="307" ht="14.25" customHeight="true"/>
+    <row r="308" ht="14.25" customHeight="true"/>
+    <row r="309" ht="14.25" customHeight="true"/>
+    <row r="310" ht="14.25" customHeight="true"/>
+    <row r="311" ht="14.25" customHeight="true"/>
+    <row r="312" ht="14.25" customHeight="true"/>
+    <row r="313" ht="14.25" customHeight="true"/>
+    <row r="314" ht="14.25" customHeight="true"/>
+    <row r="315" ht="14.25" customHeight="true"/>
+    <row r="316" ht="14.25" customHeight="true"/>
+    <row r="317" ht="14.25" customHeight="true"/>
+    <row r="318" ht="14.25" customHeight="true"/>
+    <row r="319" ht="14.25" customHeight="true"/>
+    <row r="320" ht="14.25" customHeight="true"/>
+    <row r="321" ht="14.25" customHeight="true"/>
+    <row r="322" ht="14.25" customHeight="true"/>
+    <row r="323" ht="14.25" customHeight="true"/>
+    <row r="324" ht="14.25" customHeight="true"/>
+    <row r="325" ht="14.25" customHeight="true"/>
+    <row r="326" ht="14.25" customHeight="true"/>
+    <row r="327" ht="14.25" customHeight="true"/>
+    <row r="328" ht="14.25" customHeight="true"/>
+    <row r="329" ht="14.25" customHeight="true"/>
+    <row r="330" ht="14.25" customHeight="true"/>
+    <row r="331" ht="14.25" customHeight="true"/>
+    <row r="332" ht="14.25" customHeight="true"/>
+    <row r="333" ht="14.25" customHeight="true"/>
+    <row r="334" ht="14.25" customHeight="true"/>
+    <row r="335" ht="14.25" customHeight="true"/>
+    <row r="336" ht="14.25" customHeight="true"/>
+    <row r="337" ht="14.25" customHeight="true"/>
+    <row r="338" ht="14.25" customHeight="true"/>
+    <row r="339" ht="14.25" customHeight="true"/>
+    <row r="340" ht="14.25" customHeight="true"/>
+    <row r="341" ht="14.25" customHeight="true"/>
+    <row r="342" ht="14.25" customHeight="true"/>
+    <row r="343" ht="14.25" customHeight="true"/>
+    <row r="344" ht="14.25" customHeight="true"/>
+    <row r="345" ht="14.25" customHeight="true"/>
+    <row r="346" ht="14.25" customHeight="true"/>
+    <row r="347" ht="14.25" customHeight="true"/>
+    <row r="348" ht="14.25" customHeight="true"/>
+    <row r="349" ht="14.25" customHeight="true"/>
+    <row r="350" ht="14.25" customHeight="true"/>
+    <row r="351" ht="14.25" customHeight="true"/>
+    <row r="352" ht="14.25" customHeight="true"/>
+    <row r="353" ht="14.25" customHeight="true"/>
+    <row r="354" ht="14.25" customHeight="true"/>
+    <row r="355" ht="14.25" customHeight="true"/>
+    <row r="356" ht="14.25" customHeight="true"/>
+    <row r="357" ht="14.25" customHeight="true"/>
+    <row r="358" ht="14.25" customHeight="true"/>
+    <row r="359" ht="14.25" customHeight="true"/>
+    <row r="360" ht="14.25" customHeight="true"/>
+    <row r="361" ht="14.25" customHeight="true"/>
+    <row r="362" ht="14.25" customHeight="true"/>
+    <row r="363" ht="14.25" customHeight="true"/>
+    <row r="364" ht="14.25" customHeight="true"/>
+    <row r="365" ht="14.25" customHeight="true"/>
+    <row r="366" ht="14.25" customHeight="true"/>
+    <row r="367" ht="14.25" customHeight="true"/>
+    <row r="368" ht="14.25" customHeight="true"/>
+    <row r="369" ht="14.25" customHeight="true"/>
+    <row r="370" ht="14.25" customHeight="true"/>
+    <row r="371" ht="14.25" customHeight="true"/>
+    <row r="372" ht="14.25" customHeight="true"/>
+    <row r="373" ht="14.25" customHeight="true"/>
+    <row r="374" ht="14.25" customHeight="true"/>
+    <row r="375" ht="14.25" customHeight="true"/>
+    <row r="376" ht="14.25" customHeight="true"/>
+    <row r="377" ht="14.25" customHeight="true"/>
+    <row r="378" ht="14.25" customHeight="true"/>
+    <row r="379" ht="14.25" customHeight="true"/>
+    <row r="380" ht="14.25" customHeight="true"/>
+    <row r="381" ht="14.25" customHeight="true"/>
+    <row r="382" ht="14.25" customHeight="true"/>
+    <row r="383" ht="14.25" customHeight="true"/>
+    <row r="384" ht="14.25" customHeight="true"/>
+    <row r="385" ht="14.25" customHeight="true"/>
+    <row r="386" ht="14.25" customHeight="true"/>
+    <row r="387" ht="14.25" customHeight="true"/>
+    <row r="388" ht="14.25" customHeight="true"/>
+    <row r="389" ht="14.25" customHeight="true"/>
+    <row r="390" ht="14.25" customHeight="true"/>
+    <row r="391" ht="14.25" customHeight="true"/>
+    <row r="392" ht="14.25" customHeight="true"/>
+    <row r="393" ht="14.25" customHeight="true"/>
+    <row r="394" ht="14.25" customHeight="true"/>
+    <row r="395" ht="14.25" customHeight="true"/>
+    <row r="396" ht="14.25" customHeight="true"/>
+    <row r="397" ht="14.25" customHeight="true"/>
+    <row r="398" ht="14.25" customHeight="true"/>
+    <row r="399" ht="14.25" customHeight="true"/>
+    <row r="400" ht="14.25" customHeight="true"/>
+    <row r="401" ht="14.25" customHeight="true"/>
+    <row r="402" ht="14.25" customHeight="true"/>
+    <row r="403" ht="14.25" customHeight="true"/>
+    <row r="404" ht="14.25" customHeight="true"/>
+    <row r="405" ht="14.25" customHeight="true"/>
+    <row r="406" ht="14.25" customHeight="true"/>
+    <row r="407" ht="14.25" customHeight="true"/>
+    <row r="408" ht="14.25" customHeight="true"/>
+    <row r="409" ht="14.25" customHeight="true"/>
+    <row r="410" ht="14.25" customHeight="true"/>
+    <row r="411" ht="14.25" customHeight="true"/>
+    <row r="412" ht="14.25" customHeight="true"/>
+    <row r="413" ht="14.25" customHeight="true"/>
+    <row r="414" ht="14.25" customHeight="true"/>
+    <row r="415" ht="14.25" customHeight="true"/>
+    <row r="416" ht="14.25" customHeight="true"/>
+    <row r="417" ht="14.25" customHeight="true"/>
+    <row r="418" ht="14.25" customHeight="true"/>
+    <row r="419" ht="14.25" customHeight="true"/>
+    <row r="420" ht="14.25" customHeight="true"/>
+    <row r="421" ht="14.25" customHeight="true"/>
+    <row r="422" ht="14.25" customHeight="true"/>
+    <row r="423" ht="14.25" customHeight="true"/>
+    <row r="424" ht="14.25" customHeight="true"/>
+    <row r="425" ht="14.25" customHeight="true"/>
+    <row r="426" ht="14.25" customHeight="true"/>
+    <row r="427" ht="14.25" customHeight="true"/>
+    <row r="428" ht="14.25" customHeight="true"/>
+    <row r="429" ht="14.25" customHeight="true"/>
+    <row r="430" ht="14.25" customHeight="true"/>
+    <row r="431" ht="14.25" customHeight="true"/>
+    <row r="432" ht="14.25" customHeight="true"/>
+    <row r="433" ht="14.25" customHeight="true"/>
+    <row r="434" ht="14.25" customHeight="true"/>
+    <row r="435" ht="14.25" customHeight="true"/>
+    <row r="436" ht="14.25" customHeight="true"/>
+    <row r="437" ht="14.25" customHeight="true"/>
+    <row r="438" ht="14.25" customHeight="true"/>
+    <row r="439" ht="14.25" customHeight="true"/>
+    <row r="440" ht="14.25" customHeight="true"/>
+    <row r="441" ht="14.25" customHeight="true"/>
+    <row r="442" ht="14.25" customHeight="true"/>
+    <row r="443" ht="14.25" customHeight="true"/>
+    <row r="444" ht="14.25" customHeight="true"/>
+    <row r="445" ht="14.25" customHeight="true"/>
+    <row r="446" ht="14.25" customHeight="true"/>
+    <row r="447" ht="14.25" customHeight="true"/>
+    <row r="448" ht="14.25" customHeight="true"/>
+    <row r="449" ht="14.25" customHeight="true"/>
+    <row r="450" ht="14.25" customHeight="true"/>
+    <row r="451" ht="14.25" customHeight="true"/>
+    <row r="452" ht="14.25" customHeight="true"/>
+    <row r="453" ht="14.25" customHeight="true"/>
+    <row r="454" ht="14.25" customHeight="true"/>
+    <row r="455" ht="14.25" customHeight="true"/>
+    <row r="456" ht="14.25" customHeight="true"/>
+    <row r="457" ht="14.25" customHeight="true"/>
+    <row r="458" ht="14.25" customHeight="true"/>
+    <row r="459" ht="14.25" customHeight="true"/>
+    <row r="460" ht="14.25" customHeight="true"/>
+    <row r="461" ht="14.25" customHeight="true"/>
+    <row r="462" ht="14.25" customHeight="true"/>
+    <row r="463" ht="14.25" customHeight="true"/>
+    <row r="464" ht="14.25" customHeight="true"/>
+    <row r="465" ht="14.25" customHeight="true"/>
+    <row r="466" ht="14.25" customHeight="true"/>
+    <row r="467" ht="14.25" customHeight="true"/>
+    <row r="468" ht="14.25" customHeight="true"/>
+    <row r="469" ht="14.25" customHeight="true"/>
+    <row r="470" ht="14.25" customHeight="true"/>
+    <row r="471" ht="14.25" customHeight="true"/>
+    <row r="472" ht="14.25" customHeight="true"/>
+    <row r="473" ht="14.25" customHeight="true"/>
+    <row r="474" ht="14.25" customHeight="true"/>
+    <row r="475" ht="14.25" customHeight="true"/>
+    <row r="476" ht="14.25" customHeight="true"/>
+    <row r="477" ht="14.25" customHeight="true"/>
+    <row r="478" ht="14.25" customHeight="true"/>
+    <row r="479" ht="14.25" customHeight="true"/>
+    <row r="480" ht="14.25" customHeight="true"/>
+    <row r="481" ht="14.25" customHeight="true"/>
+    <row r="482" ht="14.25" customHeight="true"/>
+    <row r="483" ht="14.25" customHeight="true"/>
+    <row r="484" ht="14.25" customHeight="true"/>
+    <row r="485" ht="14.25" customHeight="true"/>
+    <row r="486" ht="14.25" customHeight="true"/>
+    <row r="487" ht="14.25" customHeight="true"/>
+    <row r="488" ht="14.25" customHeight="true"/>
+    <row r="489" ht="14.25" customHeight="true"/>
+    <row r="490" ht="14.25" customHeight="true"/>
+    <row r="491" ht="14.25" customHeight="true"/>
+    <row r="492" ht="14.25" customHeight="true"/>
+    <row r="493" ht="14.25" customHeight="true"/>
+    <row r="494" ht="14.25" customHeight="true"/>
+    <row r="495" ht="14.25" customHeight="true"/>
+    <row r="496" ht="14.25" customHeight="true"/>
+    <row r="497" ht="14.25" customHeight="true"/>
+    <row r="498" ht="14.25" customHeight="true"/>
+    <row r="499" ht="14.25" customHeight="true"/>
+    <row r="500" ht="14.25" customHeight="true"/>
+    <row r="501" ht="14.25" customHeight="true"/>
+    <row r="502" ht="14.25" customHeight="true"/>
+    <row r="503" ht="14.25" customHeight="true"/>
+    <row r="504" ht="14.25" customHeight="true"/>
+    <row r="505" ht="14.25" customHeight="true"/>
+    <row r="506" ht="14.25" customHeight="true"/>
+    <row r="507" ht="14.25" customHeight="true"/>
+    <row r="508" ht="14.25" customHeight="true"/>
+    <row r="509" ht="14.25" customHeight="true"/>
+    <row r="510" ht="14.25" customHeight="true"/>
+    <row r="511" ht="14.25" customHeight="true"/>
+    <row r="512" ht="14.25" customHeight="true"/>
+    <row r="513" ht="14.25" customHeight="true"/>
+    <row r="514" ht="14.25" customHeight="true"/>
+    <row r="515" ht="14.25" customHeight="true"/>
+    <row r="516" ht="14.25" customHeight="true"/>
+    <row r="517" ht="14.25" customHeight="true"/>
+    <row r="518" ht="14.25" customHeight="true"/>
+    <row r="519" ht="14.25" customHeight="true"/>
+    <row r="520" ht="14.25" customHeight="true"/>
+    <row r="521" ht="14.25" customHeight="true"/>
+    <row r="522" ht="14.25" customHeight="true"/>
+    <row r="523" ht="14.25" customHeight="true"/>
+    <row r="524" ht="14.25" customHeight="true"/>
+    <row r="525" ht="14.25" customHeight="true"/>
+    <row r="526" ht="14.25" customHeight="true"/>
+    <row r="527" ht="14.25" customHeight="true"/>
+    <row r="528" ht="14.25" customHeight="true"/>
+    <row r="529" ht="14.25" customHeight="true"/>
+    <row r="530" ht="14.25" customHeight="true"/>
+    <row r="531" ht="14.25" customHeight="true"/>
+    <row r="532" ht="14.25" customHeight="true"/>
+    <row r="533" ht="14.25" customHeight="true"/>
+    <row r="534" ht="14.25" customHeight="true"/>
+    <row r="535" ht="14.25" customHeight="true"/>
+    <row r="536" ht="14.25" customHeight="true"/>
+    <row r="537" ht="14.25" customHeight="true"/>
+    <row r="538" ht="14.25" customHeight="true"/>
+    <row r="539" ht="14.25" customHeight="true"/>
+    <row r="540" ht="14.25" customHeight="true"/>
+    <row r="541" ht="14.25" customHeight="true"/>
+    <row r="542" ht="14.25" customHeight="true"/>
+    <row r="543" ht="14.25" customHeight="true"/>
+    <row r="544" ht="14.25" customHeight="true"/>
+    <row r="545" ht="14.25" customHeight="true"/>
+    <row r="546" ht="14.25" customHeight="true"/>
+    <row r="547" ht="14.25" customHeight="true"/>
+    <row r="548" ht="14.25" customHeight="true"/>
+    <row r="549" ht="14.25" customHeight="true"/>
+    <row r="550" ht="14.25" customHeight="true"/>
+    <row r="551" ht="14.25" customHeight="true"/>
+    <row r="552" ht="14.25" customHeight="true"/>
+    <row r="553" ht="14.25" customHeight="true"/>
+    <row r="554" ht="14.25" customHeight="true"/>
+    <row r="555" ht="14.25" customHeight="true"/>
+    <row r="556" ht="14.25" customHeight="true"/>
+    <row r="557" ht="14.25" customHeight="true"/>
+    <row r="558" ht="14.25" customHeight="true"/>
+    <row r="559" ht="14.25" customHeight="true"/>
+    <row r="560" ht="14.25" customHeight="true"/>
+    <row r="561" ht="14.25" customHeight="true"/>
+    <row r="562" ht="14.25" customHeight="true"/>
+    <row r="563" ht="14.25" customHeight="true"/>
+    <row r="564" ht="14.25" customHeight="true"/>
+    <row r="565" ht="14.25" customHeight="true"/>
+    <row r="566" ht="14.25" customHeight="true"/>
+    <row r="567" ht="14.25" customHeight="true"/>
+    <row r="568" ht="14.25" customHeight="true"/>
+    <row r="569" ht="14.25" customHeight="true"/>
+    <row r="570" ht="14.25" customHeight="true"/>
+    <row r="571" ht="14.25" customHeight="true"/>
+    <row r="572" ht="14.25" customHeight="true"/>
+    <row r="573" ht="14.25" customHeight="true"/>
+    <row r="574" ht="14.25" customHeight="true"/>
+    <row r="575" ht="14.25" customHeight="true"/>
+    <row r="576" ht="14.25" customHeight="true"/>
+    <row r="577" ht="14.25" customHeight="true"/>
+    <row r="578" ht="14.25" customHeight="true"/>
+    <row r="579" ht="14.25" customHeight="true"/>
+    <row r="580" ht="14.25" customHeight="true"/>
+    <row r="581" ht="14.25" customHeight="true"/>
+    <row r="582" ht="14.25" customHeight="true"/>
+    <row r="583" ht="14.25" customHeight="true"/>
+    <row r="584" ht="14.25" customHeight="true"/>
+    <row r="585" ht="14.25" customHeight="true"/>
+    <row r="586" ht="14.25" customHeight="true"/>
+    <row r="587" ht="14.25" customHeight="true"/>
+    <row r="588" ht="14.25" customHeight="true"/>
+    <row r="589" ht="14.25" customHeight="true"/>
+    <row r="590" ht="14.25" customHeight="true"/>
+    <row r="591" ht="14.25" customHeight="true"/>
+    <row r="592" ht="14.25" customHeight="true"/>
+    <row r="593" ht="14.25" customHeight="true"/>
+    <row r="594" ht="14.25" customHeight="true"/>
+    <row r="595" ht="14.25" customHeight="true"/>
+    <row r="596" ht="14.25" customHeight="true"/>
+    <row r="597" ht="14.25" customHeight="true"/>
+    <row r="598" ht="14.25" customHeight="true"/>
+    <row r="599" ht="14.25" customHeight="true"/>
+    <row r="600" ht="14.25" customHeight="true"/>
+    <row r="601" ht="14.25" customHeight="true"/>
+    <row r="602" ht="14.25" customHeight="true"/>
+    <row r="603" ht="14.25" customHeight="true"/>
+    <row r="604" ht="14.25" customHeight="true"/>
+    <row r="605" ht="14.25" customHeight="true"/>
+    <row r="606" ht="14.25" customHeight="true"/>
+    <row r="607" ht="14.25" customHeight="true"/>
+    <row r="608" ht="14.25" customHeight="true"/>
+    <row r="609" ht="14.25" customHeight="true"/>
+    <row r="610" ht="14.25" customHeight="true"/>
+    <row r="611" ht="14.25" customHeight="true"/>
+    <row r="612" ht="14.25" customHeight="true"/>
+    <row r="613" ht="14.25" customHeight="true"/>
+    <row r="614" ht="14.25" customHeight="true"/>
+    <row r="615" ht="14.25" customHeight="true"/>
+    <row r="616" ht="14.25" customHeight="true"/>
+    <row r="617" ht="14.25" customHeight="true"/>
+    <row r="618" ht="14.25" customHeight="true"/>
+    <row r="619" ht="14.25" customHeight="true"/>
+    <row r="620" ht="14.25" customHeight="true"/>
+    <row r="621" ht="14.25" customHeight="true"/>
+    <row r="622" ht="14.25" customHeight="true"/>
+    <row r="623" ht="14.25" customHeight="true"/>
+    <row r="624" ht="14.25" customHeight="true"/>
+    <row r="625" ht="14.25" customHeight="true"/>
+    <row r="626" ht="14.25" customHeight="true"/>
+    <row r="627" ht="14.25" customHeight="true"/>
+    <row r="628" ht="14.25" customHeight="true"/>
+    <row r="629" ht="14.25" customHeight="true"/>
+    <row r="630" ht="14.25" customHeight="true"/>
+    <row r="631" ht="14.25" customHeight="true"/>
+    <row r="632" ht="14.25" customHeight="true"/>
+    <row r="633" ht="14.25" customHeight="true"/>
+    <row r="634" ht="14.25" customHeight="true"/>
+    <row r="635" ht="14.25" customHeight="true"/>
+    <row r="636" ht="14.25" customHeight="true"/>
+    <row r="637" ht="14.25" customHeight="true"/>
+    <row r="638" ht="14.25" customHeight="true"/>
+    <row r="639" ht="14.25" customHeight="true"/>
+    <row r="640" ht="14.25" customHeight="true"/>
+    <row r="641" ht="14.25" customHeight="true"/>
+    <row r="642" ht="14.25" customHeight="true"/>
+    <row r="643" ht="14.25" customHeight="true"/>
+    <row r="644" ht="14.25" customHeight="true"/>
+    <row r="645" ht="14.25" customHeight="true"/>
+    <row r="646" ht="14.25" customHeight="true"/>
+    <row r="647" ht="14.25" customHeight="true"/>
+    <row r="648" ht="14.25" customHeight="true"/>
+    <row r="649" ht="14.25" customHeight="true"/>
+    <row r="650" ht="14.25" customHeight="true"/>
+    <row r="651" ht="14.25" customHeight="true"/>
+    <row r="652" ht="14.25" customHeight="true"/>
+    <row r="653" ht="14.25" customHeight="true"/>
+    <row r="654" ht="14.25" customHeight="true"/>
+    <row r="655" ht="14.25" customHeight="true"/>
+    <row r="656" ht="14.25" customHeight="true"/>
+    <row r="657" ht="14.25" customHeight="true"/>
+    <row r="658" ht="14.25" customHeight="true"/>
+    <row r="659" ht="14.25" customHeight="true"/>
+    <row r="660" ht="14.25" customHeight="true"/>
+    <row r="661" ht="14.25" customHeight="true"/>
+    <row r="662" ht="14.25" customHeight="true"/>
+    <row r="663" ht="14.25" customHeight="true"/>
+    <row r="664" ht="14.25" customHeight="true"/>
+    <row r="665" ht="14.25" customHeight="true"/>
+    <row r="666" ht="14.25" customHeight="true"/>
+    <row r="667" ht="14.25" customHeight="true"/>
+    <row r="668" ht="14.25" customHeight="true"/>
+    <row r="669" ht="14.25" customHeight="true"/>
+    <row r="670" ht="14.25" customHeight="true"/>
+    <row r="671" ht="14.25" customHeight="true"/>
+    <row r="672" ht="14.25" customHeight="true"/>
+    <row r="673" ht="14.25" customHeight="true"/>
+    <row r="674" ht="14.25" customHeight="true"/>
+    <row r="675" ht="14.25" customHeight="true"/>
+    <row r="676" ht="14.25" customHeight="true"/>
+    <row r="677" ht="14.25" customHeight="true"/>
+    <row r="678" ht="14.25" customHeight="true"/>
+    <row r="679" ht="14.25" customHeight="true"/>
+    <row r="680" ht="14.25" customHeight="true"/>
+    <row r="681" ht="14.25" customHeight="true"/>
+    <row r="682" ht="14.25" customHeight="true"/>
+    <row r="683" ht="14.25" customHeight="true"/>
+    <row r="684" ht="14.25" customHeight="true"/>
+    <row r="685" ht="14.25" customHeight="true"/>
+    <row r="686" ht="14.25" customHeight="true"/>
+    <row r="687" ht="14.25" customHeight="true"/>
+    <row r="688" ht="14.25" customHeight="true"/>
+    <row r="689" ht="14.25" customHeight="true"/>
+    <row r="690" ht="14.25" customHeight="true"/>
+    <row r="691" ht="14.25" customHeight="true"/>
+    <row r="692" ht="14.25" customHeight="true"/>
+    <row r="693" ht="14.25" customHeight="true"/>
+    <row r="694" ht="14.25" customHeight="true"/>
+    <row r="695" ht="14.25" customHeight="true"/>
+    <row r="696" ht="14.25" customHeight="true"/>
+    <row r="697" ht="14.25" customHeight="true"/>
+    <row r="698" ht="14.25" customHeight="true"/>
+    <row r="699" ht="14.25" customHeight="true"/>
+    <row r="700" ht="14.25" customHeight="true"/>
+    <row r="701" ht="14.25" customHeight="true"/>
+    <row r="702" ht="14.25" customHeight="true"/>
+    <row r="703" ht="14.25" customHeight="true"/>
+    <row r="704" ht="14.25" customHeight="true"/>
+    <row r="705" ht="14.25" customHeight="true"/>
+    <row r="706" ht="14.25" customHeight="true"/>
+    <row r="707" ht="14.25" customHeight="true"/>
+    <row r="708" ht="14.25" customHeight="true"/>
+    <row r="709" ht="14.25" customHeight="true"/>
+    <row r="710" ht="14.25" customHeight="true"/>
+    <row r="711" ht="14.25" customHeight="true"/>
+    <row r="712" ht="14.25" customHeight="true"/>
+    <row r="713" ht="14.25" customHeight="true"/>
+    <row r="714" ht="14.25" customHeight="true"/>
+    <row r="715" ht="14.25" customHeight="true"/>
+    <row r="716" ht="14.25" customHeight="true"/>
+    <row r="717" ht="14.25" customHeight="true"/>
+    <row r="718" ht="14.25" customHeight="true"/>
+    <row r="719" ht="14.25" customHeight="true"/>
+    <row r="720" ht="14.25" customHeight="true"/>
+    <row r="721" ht="14.25" customHeight="true"/>
+    <row r="722" ht="14.25" customHeight="true"/>
+    <row r="723" ht="14.25" customHeight="true"/>
+    <row r="724" ht="14.25" customHeight="true"/>
+    <row r="725" ht="14.25" customHeight="true"/>
+    <row r="726" ht="14.25" customHeight="true"/>
+    <row r="727" ht="14.25" customHeight="true"/>
+    <row r="728" ht="14.25" customHeight="true"/>
+    <row r="729" ht="14.25" customHeight="true"/>
+    <row r="730" ht="14.25" customHeight="true"/>
+    <row r="731" ht="14.25" customHeight="true"/>
+    <row r="732" ht="14.25" customHeight="true"/>
+    <row r="733" ht="14.25" customHeight="true"/>
+    <row r="734" ht="14.25" customHeight="true"/>
+    <row r="735" ht="14.25" customHeight="true"/>
+    <row r="736" ht="14.25" customHeight="true"/>
+    <row r="737" ht="14.25" customHeight="true"/>
+    <row r="738" ht="14.25" customHeight="true"/>
+    <row r="739" ht="14.25" customHeight="true"/>
+    <row r="740" ht="14.25" customHeight="true"/>
+    <row r="741" ht="14.25" customHeight="true"/>
+    <row r="742" ht="14.25" customHeight="true"/>
+    <row r="743" ht="14.25" customHeight="true"/>
+    <row r="744" ht="14.25" customHeight="true"/>
+    <row r="745" ht="14.25" customHeight="true"/>
+    <row r="746" ht="14.25" customHeight="true"/>
+    <row r="747" ht="14.25" customHeight="true"/>
+    <row r="748" ht="14.25" customHeight="true"/>
+    <row r="749" ht="14.25" customHeight="true"/>
+    <row r="750" ht="14.25" customHeight="true"/>
+    <row r="751" ht="14.25" customHeight="true"/>
+    <row r="752" ht="14.25" customHeight="true"/>
+    <row r="753" ht="14.25" customHeight="true"/>
+    <row r="754" ht="14.25" customHeight="true"/>
+    <row r="755" ht="14.25" customHeight="true"/>
+    <row r="756" ht="14.25" customHeight="true"/>
+    <row r="757" ht="14.25" customHeight="true"/>
+    <row r="758" ht="14.25" customHeight="true"/>
+    <row r="759" ht="14.25" customHeight="true"/>
+    <row r="760" ht="14.25" customHeight="true"/>
+    <row r="761" ht="14.25" customHeight="true"/>
+    <row r="762" ht="14.25" customHeight="true"/>
+    <row r="763" ht="14.25" customHeight="true"/>
+    <row r="764" ht="14.25" customHeight="true"/>
+    <row r="765" ht="14.25" customHeight="true"/>
+    <row r="766" ht="14.25" customHeight="true"/>
+    <row r="767" ht="14.25" customHeight="true"/>
+    <row r="768" ht="14.25" customHeight="true"/>
+    <row r="769" ht="14.25" customHeight="true"/>
+    <row r="770" ht="14.25" customHeight="true"/>
+    <row r="771" ht="14.25" customHeight="true"/>
+    <row r="772" ht="14.25" customHeight="true"/>
+    <row r="773" ht="14.25" customHeight="true"/>
+    <row r="774" ht="14.25" customHeight="true"/>
+    <row r="775" ht="14.25" customHeight="true"/>
+    <row r="776" ht="14.25" customHeight="true"/>
+    <row r="777" ht="14.25" customHeight="true"/>
+    <row r="778" ht="14.25" customHeight="true"/>
+    <row r="779" ht="14.25" customHeight="true"/>
+    <row r="780" ht="14.25" customHeight="true"/>
+    <row r="781" ht="14.25" customHeight="true"/>
+    <row r="782" ht="14.25" customHeight="true"/>
+    <row r="783" ht="14.25" customHeight="true"/>
+    <row r="784" ht="14.25" customHeight="true"/>
+    <row r="785" ht="14.25" customHeight="true"/>
+    <row r="786" ht="14.25" customHeight="true"/>
+    <row r="787" ht="14.25" customHeight="true"/>
+    <row r="788" ht="14.25" customHeight="true"/>
+    <row r="789" ht="14.25" customHeight="true"/>
+    <row r="790" ht="14.25" customHeight="true"/>
+    <row r="791" ht="14.25" customHeight="true"/>
+    <row r="792" ht="14.25" customHeight="true"/>
+    <row r="793" ht="14.25" customHeight="true"/>
+    <row r="794" ht="14.25" customHeight="true"/>
+    <row r="795" ht="14.25" customHeight="true"/>
+    <row r="796" ht="14.25" customHeight="true"/>
+    <row r="797" ht="14.25" customHeight="true"/>
+    <row r="798" ht="14.25" customHeight="true"/>
+    <row r="799" ht="14.25" customHeight="true"/>
+    <row r="800" ht="14.25" customHeight="true"/>
+    <row r="801" ht="14.25" customHeight="true"/>
+    <row r="802" ht="14.25" customHeight="true"/>
+    <row r="803" ht="14.25" customHeight="true"/>
+    <row r="804" ht="14.25" customHeight="true"/>
+    <row r="805" ht="14.25" customHeight="true"/>
+    <row r="806" ht="14.25" customHeight="true"/>
+    <row r="807" ht="14.25" customHeight="true"/>
+    <row r="808" ht="14.25" customHeight="true"/>
+    <row r="809" ht="14.25" customHeight="true"/>
+    <row r="810" ht="14.25" customHeight="true"/>
+    <row r="811" ht="14.25" customHeight="true"/>
+    <row r="812" ht="14.25" customHeight="true"/>
+    <row r="813" ht="14.25" customHeight="true"/>
+    <row r="814" ht="14.25" customHeight="true"/>
+    <row r="815" ht="14.25" customHeight="true"/>
+    <row r="816" ht="14.25" customHeight="true"/>
+    <row r="817" ht="14.25" customHeight="true"/>
+    <row r="818" ht="14.25" customHeight="true"/>
+    <row r="819" ht="14.25" customHeight="true"/>
+    <row r="820" ht="14.25" customHeight="true"/>
+    <row r="821" ht="14.25" customHeight="true"/>
+    <row r="822" ht="14.25" customHeight="true"/>
+    <row r="823" ht="14.25" customHeight="true"/>
+    <row r="824" ht="14.25" customHeight="true"/>
+    <row r="825" ht="14.25" customHeight="true"/>
+    <row r="826" ht="14.25" customHeight="true"/>
+    <row r="827" ht="14.25" customHeight="true"/>
+    <row r="828" ht="14.25" customHeight="true"/>
+    <row r="829" ht="14.25" customHeight="true"/>
+    <row r="830" ht="14.25" customHeight="true"/>
+    <row r="831" ht="14.25" customHeight="true"/>
+    <row r="832" ht="14.25" customHeight="true"/>
+    <row r="833" ht="14.25" customHeight="true"/>
+    <row r="834" ht="14.25" customHeight="true"/>
+    <row r="835" ht="14.25" customHeight="true"/>
+    <row r="836" ht="14.25" customHeight="true"/>
+    <row r="837" ht="14.25" customHeight="true"/>
+    <row r="838" ht="14.25" customHeight="true"/>
+    <row r="839" ht="14.25" customHeight="true"/>
+    <row r="840" ht="14.25" customHeight="true"/>
+    <row r="841" ht="14.25" customHeight="true"/>
+    <row r="842" ht="14.25" customHeight="true"/>
+    <row r="843" ht="14.25" customHeight="true"/>
+    <row r="844" ht="14.25" customHeight="true"/>
+    <row r="845" ht="14.25" customHeight="true"/>
+    <row r="846" ht="14.25" customHeight="true"/>
+    <row r="847" ht="14.25" customHeight="true"/>
+    <row r="848" ht="14.25" customHeight="true"/>
+    <row r="849" ht="14.25" customHeight="true"/>
+    <row r="850" ht="14.25" customHeight="true"/>
+    <row r="851" ht="14.25" customHeight="true"/>
+    <row r="852" ht="14.25" customHeight="true"/>
+    <row r="853" ht="14.25" customHeight="true"/>
+    <row r="854" ht="14.25" customHeight="true"/>
+    <row r="855" ht="14.25" customHeight="true"/>
+    <row r="856" ht="14.25" customHeight="true"/>
+    <row r="857" ht="14.25" customHeight="true"/>
+    <row r="858" ht="14.25" customHeight="true"/>
+    <row r="859" ht="14.25" customHeight="true"/>
+    <row r="860" ht="14.25" customHeight="true"/>
+    <row r="861" ht="14.25" customHeight="true"/>
+    <row r="862" ht="14.25" customHeight="true"/>
+    <row r="863" ht="14.25" customHeight="true"/>
+    <row r="864" ht="14.25" customHeight="true"/>
+    <row r="865" ht="14.25" customHeight="true"/>
+    <row r="866" ht="14.25" customHeight="true"/>
+    <row r="867" ht="14.25" customHeight="true"/>
+    <row r="868" ht="14.25" customHeight="true"/>
+    <row r="869" ht="14.25" customHeight="true"/>
+    <row r="870" ht="14.25" customHeight="true"/>
+    <row r="871" ht="14.25" customHeight="true"/>
+    <row r="872" ht="14.25" customHeight="true"/>
+    <row r="873" ht="14.25" customHeight="true"/>
+    <row r="874" ht="14.25" customHeight="true"/>
+    <row r="875" ht="14.25" customHeight="true"/>
+    <row r="876" ht="14.25" customHeight="true"/>
+    <row r="877" ht="14.25" customHeight="true"/>
+    <row r="878" ht="14.25" customHeight="true"/>
+    <row r="879" ht="14.25" customHeight="true"/>
+    <row r="880" ht="14.25" customHeight="true"/>
+    <row r="881" ht="14.25" customHeight="true"/>
+    <row r="882" ht="14.25" customHeight="true"/>
+    <row r="883" ht="14.25" customHeight="true"/>
+    <row r="884" ht="14.25" customHeight="true"/>
+    <row r="885" ht="14.25" customHeight="true"/>
+    <row r="886" ht="14.25" customHeight="true"/>
+    <row r="887" ht="14.25" customHeight="true"/>
+    <row r="888" ht="14.25" customHeight="true"/>
+    <row r="889" ht="14.25" customHeight="true"/>
+    <row r="890" ht="14.25" customHeight="true"/>
+    <row r="891" ht="14.25" customHeight="true"/>
+    <row r="892" ht="14.25" customHeight="true"/>
+    <row r="893" ht="14.25" customHeight="true"/>
+    <row r="894" ht="14.25" customHeight="true"/>
+    <row r="895" ht="14.25" customHeight="true"/>
+    <row r="896" ht="14.25" customHeight="true"/>
+    <row r="897" ht="14.25" customHeight="true"/>
+    <row r="898" ht="14.25" customHeight="true"/>
+    <row r="899" ht="14.25" customHeight="true"/>
+    <row r="900" ht="14.25" customHeight="true"/>
+    <row r="901" ht="14.25" customHeight="true"/>
+    <row r="902" ht="14.25" customHeight="true"/>
+    <row r="903" ht="14.25" customHeight="true"/>
+    <row r="904" ht="14.25" customHeight="true"/>
+    <row r="905" ht="14.25" customHeight="true"/>
+    <row r="906" ht="14.25" customHeight="true"/>
+    <row r="907" ht="14.25" customHeight="true"/>
+    <row r="908" ht="14.25" customHeight="true"/>
+    <row r="909" ht="14.25" customHeight="true"/>
+    <row r="910" ht="14.25" customHeight="true"/>
+    <row r="911" ht="14.25" customHeight="true"/>
+    <row r="912" ht="14.25" customHeight="true"/>
+    <row r="913" ht="14.25" customHeight="true"/>
+    <row r="914" ht="14.25" customHeight="true"/>
+    <row r="915" ht="14.25" customHeight="true"/>
+    <row r="916" ht="14.25" customHeight="true"/>
+    <row r="917" ht="14.25" customHeight="true"/>
+    <row r="918" ht="14.25" customHeight="true"/>
+    <row r="919" ht="14.25" customHeight="true"/>
+    <row r="920" ht="14.25" customHeight="true"/>
+    <row r="921" ht="14.25" customHeight="true"/>
+    <row r="922" ht="14.25" customHeight="true"/>
+    <row r="923" ht="14.25" customHeight="true"/>
+    <row r="924" ht="14.25" customHeight="true"/>
+    <row r="925" ht="14.25" customHeight="true"/>
+    <row r="926" ht="14.25" customHeight="true"/>
+    <row r="927" ht="14.25" customHeight="true"/>
+    <row r="928" ht="14.25" customHeight="true"/>
+    <row r="929" ht="14.25" customHeight="true"/>
+    <row r="930" ht="14.25" customHeight="true"/>
+    <row r="931" ht="14.25" customHeight="true"/>
+    <row r="932" ht="14.25" customHeight="true"/>
+    <row r="933" ht="14.25" customHeight="true"/>
+    <row r="934" ht="14.25" customHeight="true"/>
+    <row r="935" ht="14.25" customHeight="true"/>
+    <row r="936" ht="14.25" customHeight="true"/>
+    <row r="937" ht="14.25" customHeight="true"/>
+    <row r="938" ht="14.25" customHeight="true"/>
+    <row r="939" ht="14.25" customHeight="true"/>
+    <row r="940" ht="14.25" customHeight="true"/>
+    <row r="941" ht="14.25" customHeight="true"/>
+    <row r="942" ht="14.25" customHeight="true"/>
+    <row r="943" ht="14.25" customHeight="true"/>
+    <row r="944" ht="14.25" customHeight="true"/>
+    <row r="945" ht="14.25" customHeight="true"/>
+    <row r="946" ht="14.25" customHeight="true"/>
+    <row r="947" ht="14.25" customHeight="true"/>
+    <row r="948" ht="14.25" customHeight="true"/>
+    <row r="949" ht="14.25" customHeight="true"/>
+    <row r="950" ht="14.25" customHeight="true"/>
+    <row r="951" ht="14.25" customHeight="true"/>
+    <row r="952" ht="14.25" customHeight="true"/>
+    <row r="953" ht="14.25" customHeight="true"/>
+    <row r="954" ht="14.25" customHeight="true"/>
+    <row r="955" ht="14.25" customHeight="true"/>
+    <row r="956" ht="14.25" customHeight="true"/>
+    <row r="957" ht="14.25" customHeight="true"/>
+    <row r="958" ht="14.25" customHeight="true"/>
+    <row r="959" ht="14.25" customHeight="true"/>
+    <row r="960" ht="14.25" customHeight="true"/>
+    <row r="961" ht="14.25" customHeight="true"/>
+    <row r="962" ht="14.25" customHeight="true"/>
+    <row r="963" ht="14.25" customHeight="true"/>
+    <row r="964" ht="14.25" customHeight="true"/>
+    <row r="965" ht="14.25" customHeight="true"/>
+    <row r="966" ht="14.25" customHeight="true"/>
+    <row r="967" ht="14.25" customHeight="true"/>
+    <row r="968" ht="14.25" customHeight="true"/>
+    <row r="969" ht="14.25" customHeight="true"/>
+    <row r="970" ht="14.25" customHeight="true"/>
+    <row r="971" ht="14.25" customHeight="true"/>
+    <row r="972" ht="14.25" customHeight="true"/>
+    <row r="973" ht="14.25" customHeight="true"/>
+    <row r="974" ht="14.25" customHeight="true"/>
+    <row r="975" ht="14.25" customHeight="true"/>
+    <row r="976" ht="14.25" customHeight="true"/>
+    <row r="977" ht="14.25" customHeight="true"/>
+    <row r="978" ht="14.25" customHeight="true"/>
+    <row r="979" ht="14.25" customHeight="true"/>
+    <row r="980" ht="14.25" customHeight="true"/>
+    <row r="981" ht="14.25" customHeight="true"/>
+    <row r="982" ht="14.25" customHeight="true"/>
+    <row r="983" ht="14.25" customHeight="true"/>
+    <row r="984" ht="14.25" customHeight="true"/>
+    <row r="985" ht="14.25" customHeight="true"/>
+    <row r="986" ht="14.25" customHeight="true"/>
+    <row r="987" ht="14.25" customHeight="true"/>
+    <row r="988" ht="14.25" customHeight="true"/>
+    <row r="989" ht="14.25" customHeight="true"/>
+    <row r="990" ht="14.25" customHeight="true"/>
+    <row r="991" ht="14.25" customHeight="true"/>
+    <row r="992" ht="14.25" customHeight="true"/>
+    <row r="993" ht="14.25" customHeight="true"/>
+    <row r="994" ht="14.25" customHeight="true"/>
+    <row r="995" ht="14.25" customHeight="true"/>
+    <row r="996" ht="14.25" customHeight="true"/>
+    <row r="997" ht="14.25" customHeight="true"/>
+    <row r="998" ht="14.25" customHeight="true"/>
+    <row r="999" ht="14.25" customHeight="true"/>
+    <row r="1000" ht="14.25" customHeight="true"/>
   </sheetData>
   <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -6942,14 +6942,14 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="true"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="33"/>
-    <col customWidth="true" max="2" min="2" width="30.29"/>
-    <col customWidth="true" max="27" min="3" width="8.71"/>
+    <col customWidth="1" min="1" max="1" width="33.0"/>
+    <col customWidth="1" min="2" max="2" width="30.29"/>
+    <col customWidth="1" min="3" max="27" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="true">
+    <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6966,7 +6966,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="true">
+    <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>77</v>
       </c>
@@ -6977,7 +6977,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="true">
+    <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>80</v>
       </c>
@@ -6988,7 +6988,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="true">
+    <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>83</v>
       </c>
@@ -6999,1005 +6999,1005 @@
         <v>85</v>
       </c>
     </row>
-    <row r="5" ht="14.25" customHeight="true"/>
-    <row r="6" ht="14.25" customHeight="true"/>
-    <row r="7" ht="14.25" customHeight="true"/>
-    <row r="8" ht="14.25" customHeight="true"/>
-    <row r="9" ht="14.25" customHeight="true"/>
-    <row r="10" ht="14.25" customHeight="true"/>
-    <row r="11" ht="14.25" customHeight="true"/>
-    <row r="12" ht="14.25" customHeight="true"/>
-    <row r="13" ht="14.25" customHeight="true"/>
-    <row r="14" ht="14.25" customHeight="true"/>
-    <row r="15" ht="14.25" customHeight="true"/>
-    <row r="16" ht="14.25" customHeight="true"/>
-    <row r="17" ht="14.25" customHeight="true"/>
-    <row r="18" ht="14.25" customHeight="true"/>
-    <row r="19" ht="14.25" customHeight="true"/>
-    <row r="20" ht="14.25" customHeight="true"/>
-    <row r="21" ht="14.25" customHeight="true"/>
-    <row r="22" ht="14.25" customHeight="true"/>
-    <row r="23" ht="14.25" customHeight="true"/>
-    <row r="24" ht="14.25" customHeight="true"/>
-    <row r="25" ht="14.25" customHeight="true"/>
-    <row r="26" ht="14.25" customHeight="true"/>
-    <row r="27" ht="14.25" customHeight="true"/>
-    <row r="28" ht="14.25" customHeight="true"/>
-    <row r="29" ht="14.25" customHeight="true"/>
-    <row r="30" ht="14.25" customHeight="true"/>
-    <row r="31" ht="14.25" customHeight="true"/>
-    <row r="32" ht="14.25" customHeight="true"/>
-    <row r="33" ht="14.25" customHeight="true"/>
-    <row r="34" ht="14.25" customHeight="true"/>
-    <row r="35" ht="14.25" customHeight="true"/>
-    <row r="36" ht="14.25" customHeight="true"/>
-    <row r="37" ht="14.25" customHeight="true"/>
-    <row r="38" ht="14.25" customHeight="true"/>
-    <row r="39" ht="14.25" customHeight="true"/>
-    <row r="40" ht="14.25" customHeight="true"/>
-    <row r="41" ht="14.25" customHeight="true"/>
-    <row r="42" ht="14.25" customHeight="true"/>
-    <row r="43" ht="14.25" customHeight="true"/>
-    <row r="44" ht="14.25" customHeight="true"/>
-    <row r="45" ht="14.25" customHeight="true"/>
-    <row r="46" ht="14.25" customHeight="true"/>
-    <row r="47" ht="14.25" customHeight="true"/>
-    <row r="48" ht="14.25" customHeight="true"/>
-    <row r="49" ht="14.25" customHeight="true"/>
-    <row r="50" ht="14.25" customHeight="true"/>
-    <row r="51" ht="14.25" customHeight="true"/>
-    <row r="52" ht="14.25" customHeight="true"/>
-    <row r="53" ht="14.25" customHeight="true"/>
-    <row r="54" ht="14.25" customHeight="true"/>
-    <row r="55" ht="14.25" customHeight="true"/>
-    <row r="56" ht="14.25" customHeight="true"/>
-    <row r="57" ht="14.25" customHeight="true"/>
-    <row r="58" ht="14.25" customHeight="true"/>
-    <row r="59" ht="14.25" customHeight="true"/>
-    <row r="60" ht="14.25" customHeight="true"/>
-    <row r="61" ht="14.25" customHeight="true"/>
-    <row r="62" ht="14.25" customHeight="true"/>
-    <row r="63" ht="14.25" customHeight="true"/>
-    <row r="64" ht="14.25" customHeight="true"/>
-    <row r="65" ht="14.25" customHeight="true"/>
-    <row r="66" ht="14.25" customHeight="true"/>
-    <row r="67" ht="14.25" customHeight="true"/>
-    <row r="68" ht="14.25" customHeight="true"/>
-    <row r="69" ht="14.25" customHeight="true"/>
-    <row r="70" ht="14.25" customHeight="true"/>
-    <row r="71" ht="14.25" customHeight="true"/>
-    <row r="72" ht="14.25" customHeight="true"/>
-    <row r="73" ht="14.25" customHeight="true"/>
-    <row r="74" ht="14.25" customHeight="true"/>
-    <row r="75" ht="14.25" customHeight="true"/>
-    <row r="76" ht="14.25" customHeight="true"/>
-    <row r="77" ht="14.25" customHeight="true"/>
-    <row r="78" ht="14.25" customHeight="true"/>
-    <row r="79" ht="14.25" customHeight="true"/>
-    <row r="80" ht="14.25" customHeight="true"/>
-    <row r="81" ht="14.25" customHeight="true"/>
-    <row r="82" ht="14.25" customHeight="true"/>
-    <row r="83" ht="14.25" customHeight="true"/>
-    <row r="84" ht="14.25" customHeight="true"/>
-    <row r="85" ht="14.25" customHeight="true"/>
-    <row r="86" ht="14.25" customHeight="true"/>
-    <row r="87" ht="14.25" customHeight="true"/>
-    <row r="88" ht="14.25" customHeight="true"/>
-    <row r="89" ht="14.25" customHeight="true"/>
-    <row r="90" ht="14.25" customHeight="true"/>
-    <row r="91" ht="14.25" customHeight="true"/>
-    <row r="92" ht="14.25" customHeight="true"/>
-    <row r="93" ht="14.25" customHeight="true"/>
-    <row r="94" ht="14.25" customHeight="true"/>
-    <row r="95" ht="14.25" customHeight="true"/>
-    <row r="96" ht="14.25" customHeight="true"/>
-    <row r="97" ht="14.25" customHeight="true"/>
-    <row r="98" ht="14.25" customHeight="true"/>
-    <row r="99" ht="14.25" customHeight="true"/>
-    <row r="100" ht="14.25" customHeight="true"/>
-    <row r="101" ht="14.25" customHeight="true"/>
-    <row r="102" ht="14.25" customHeight="true"/>
-    <row r="103" ht="14.25" customHeight="true"/>
-    <row r="104" ht="14.25" customHeight="true"/>
-    <row r="105" ht="14.25" customHeight="true"/>
-    <row r="106" ht="14.25" customHeight="true"/>
-    <row r="107" ht="14.25" customHeight="true"/>
-    <row r="108" ht="14.25" customHeight="true"/>
-    <row r="109" ht="14.25" customHeight="true"/>
-    <row r="110" ht="14.25" customHeight="true"/>
-    <row r="111" ht="14.25" customHeight="true"/>
-    <row r="112" ht="14.25" customHeight="true"/>
-    <row r="113" ht="14.25" customHeight="true"/>
-    <row r="114" ht="14.25" customHeight="true"/>
-    <row r="115" ht="14.25" customHeight="true"/>
-    <row r="116" ht="14.25" customHeight="true"/>
-    <row r="117" ht="14.25" customHeight="true"/>
-    <row r="118" ht="14.25" customHeight="true"/>
-    <row r="119" ht="14.25" customHeight="true"/>
-    <row r="120" ht="14.25" customHeight="true"/>
-    <row r="121" ht="14.25" customHeight="true"/>
-    <row r="122" ht="14.25" customHeight="true"/>
-    <row r="123" ht="14.25" customHeight="true"/>
-    <row r="124" ht="14.25" customHeight="true"/>
-    <row r="125" ht="14.25" customHeight="true"/>
-    <row r="126" ht="14.25" customHeight="true"/>
-    <row r="127" ht="14.25" customHeight="true"/>
-    <row r="128" ht="14.25" customHeight="true"/>
-    <row r="129" ht="14.25" customHeight="true"/>
-    <row r="130" ht="14.25" customHeight="true"/>
-    <row r="131" ht="14.25" customHeight="true"/>
-    <row r="132" ht="14.25" customHeight="true"/>
-    <row r="133" ht="14.25" customHeight="true"/>
-    <row r="134" ht="14.25" customHeight="true"/>
-    <row r="135" ht="14.25" customHeight="true"/>
-    <row r="136" ht="14.25" customHeight="true"/>
-    <row r="137" ht="14.25" customHeight="true"/>
-    <row r="138" ht="14.25" customHeight="true"/>
-    <row r="139" ht="14.25" customHeight="true"/>
-    <row r="140" ht="14.25" customHeight="true"/>
-    <row r="141" ht="14.25" customHeight="true"/>
-    <row r="142" ht="14.25" customHeight="true"/>
-    <row r="143" ht="14.25" customHeight="true"/>
-    <row r="144" ht="14.25" customHeight="true"/>
-    <row r="145" ht="14.25" customHeight="true"/>
-    <row r="146" ht="14.25" customHeight="true"/>
-    <row r="147" ht="14.25" customHeight="true"/>
-    <row r="148" ht="14.25" customHeight="true"/>
-    <row r="149" ht="14.25" customHeight="true"/>
-    <row r="150" ht="14.25" customHeight="true"/>
-    <row r="151" ht="14.25" customHeight="true"/>
-    <row r="152" ht="14.25" customHeight="true"/>
-    <row r="153" ht="14.25" customHeight="true"/>
-    <row r="154" ht="14.25" customHeight="true"/>
-    <row r="155" ht="14.25" customHeight="true"/>
-    <row r="156" ht="14.25" customHeight="true"/>
-    <row r="157" ht="14.25" customHeight="true"/>
-    <row r="158" ht="14.25" customHeight="true"/>
-    <row r="159" ht="14.25" customHeight="true"/>
-    <row r="160" ht="14.25" customHeight="true"/>
-    <row r="161" ht="14.25" customHeight="true"/>
-    <row r="162" ht="14.25" customHeight="true"/>
-    <row r="163" ht="14.25" customHeight="true"/>
-    <row r="164" ht="14.25" customHeight="true"/>
-    <row r="165" ht="14.25" customHeight="true"/>
-    <row r="166" ht="14.25" customHeight="true"/>
-    <row r="167" ht="14.25" customHeight="true"/>
-    <row r="168" ht="14.25" customHeight="true"/>
-    <row r="169" ht="14.25" customHeight="true"/>
-    <row r="170" ht="14.25" customHeight="true"/>
-    <row r="171" ht="14.25" customHeight="true"/>
-    <row r="172" ht="14.25" customHeight="true"/>
-    <row r="173" ht="14.25" customHeight="true"/>
-    <row r="174" ht="14.25" customHeight="true"/>
-    <row r="175" ht="14.25" customHeight="true"/>
-    <row r="176" ht="14.25" customHeight="true"/>
-    <row r="177" ht="14.25" customHeight="true"/>
-    <row r="178" ht="14.25" customHeight="true"/>
-    <row r="179" ht="14.25" customHeight="true"/>
-    <row r="180" ht="14.25" customHeight="true"/>
-    <row r="181" ht="14.25" customHeight="true"/>
-    <row r="182" ht="14.25" customHeight="true"/>
-    <row r="183" ht="14.25" customHeight="true"/>
-    <row r="184" ht="14.25" customHeight="true"/>
-    <row r="185" ht="14.25" customHeight="true"/>
-    <row r="186" ht="14.25" customHeight="true"/>
-    <row r="187" ht="14.25" customHeight="true"/>
-    <row r="188" ht="14.25" customHeight="true"/>
-    <row r="189" ht="14.25" customHeight="true"/>
-    <row r="190" ht="14.25" customHeight="true"/>
-    <row r="191" ht="14.25" customHeight="true"/>
-    <row r="192" ht="14.25" customHeight="true"/>
-    <row r="193" ht="14.25" customHeight="true"/>
-    <row r="194" ht="14.25" customHeight="true"/>
-    <row r="195" ht="14.25" customHeight="true"/>
-    <row r="196" ht="14.25" customHeight="true"/>
-    <row r="197" ht="14.25" customHeight="true"/>
-    <row r="198" ht="14.25" customHeight="true"/>
-    <row r="199" ht="14.25" customHeight="true"/>
-    <row r="200" ht="14.25" customHeight="true"/>
-    <row r="201" ht="14.25" customHeight="true"/>
-    <row r="202" ht="14.25" customHeight="true"/>
-    <row r="203" ht="14.25" customHeight="true"/>
-    <row r="204" ht="14.25" customHeight="true"/>
-    <row r="205" ht="14.25" customHeight="true"/>
-    <row r="206" ht="14.25" customHeight="true"/>
-    <row r="207" ht="14.25" customHeight="true"/>
-    <row r="208" ht="14.25" customHeight="true"/>
-    <row r="209" ht="14.25" customHeight="true"/>
-    <row r="210" ht="14.25" customHeight="true"/>
-    <row r="211" ht="14.25" customHeight="true"/>
-    <row r="212" ht="14.25" customHeight="true"/>
-    <row r="213" ht="14.25" customHeight="true"/>
-    <row r="214" ht="14.25" customHeight="true"/>
-    <row r="215" ht="14.25" customHeight="true"/>
-    <row r="216" ht="14.25" customHeight="true"/>
-    <row r="217" ht="14.25" customHeight="true"/>
-    <row r="218" ht="14.25" customHeight="true"/>
-    <row r="219" ht="14.25" customHeight="true"/>
-    <row r="220" ht="14.25" customHeight="true"/>
-    <row r="221" ht="14.25" customHeight="true"/>
-    <row r="222" ht="14.25" customHeight="true"/>
-    <row r="223" ht="14.25" customHeight="true"/>
-    <row r="224" ht="14.25" customHeight="true"/>
-    <row r="225" ht="14.25" customHeight="true"/>
-    <row r="226" ht="14.25" customHeight="true"/>
-    <row r="227" ht="14.25" customHeight="true"/>
-    <row r="228" ht="14.25" customHeight="true"/>
-    <row r="229" ht="14.25" customHeight="true"/>
-    <row r="230" ht="14.25" customHeight="true"/>
-    <row r="231" ht="14.25" customHeight="true"/>
-    <row r="232" ht="14.25" customHeight="true"/>
-    <row r="233" ht="14.25" customHeight="true"/>
-    <row r="234" ht="14.25" customHeight="true"/>
-    <row r="235" ht="14.25" customHeight="true"/>
-    <row r="236" ht="14.25" customHeight="true"/>
-    <row r="237" ht="14.25" customHeight="true"/>
-    <row r="238" ht="14.25" customHeight="true"/>
-    <row r="239" ht="14.25" customHeight="true"/>
-    <row r="240" ht="14.25" customHeight="true"/>
-    <row r="241" ht="14.25" customHeight="true"/>
-    <row r="242" ht="14.25" customHeight="true"/>
-    <row r="243" ht="14.25" customHeight="true"/>
-    <row r="244" ht="14.25" customHeight="true"/>
-    <row r="245" ht="14.25" customHeight="true"/>
-    <row r="246" ht="14.25" customHeight="true"/>
-    <row r="247" ht="14.25" customHeight="true"/>
-    <row r="248" ht="14.25" customHeight="true"/>
-    <row r="249" ht="14.25" customHeight="true"/>
-    <row r="250" ht="14.25" customHeight="true"/>
-    <row r="251" ht="14.25" customHeight="true"/>
-    <row r="252" ht="14.25" customHeight="true"/>
-    <row r="253" ht="14.25" customHeight="true"/>
-    <row r="254" ht="14.25" customHeight="true"/>
-    <row r="255" ht="14.25" customHeight="true"/>
-    <row r="256" ht="14.25" customHeight="true"/>
-    <row r="257" ht="14.25" customHeight="true"/>
-    <row r="258" ht="14.25" customHeight="true"/>
-    <row r="259" ht="14.25" customHeight="true"/>
-    <row r="260" ht="14.25" customHeight="true"/>
-    <row r="261" ht="14.25" customHeight="true"/>
-    <row r="262" ht="14.25" customHeight="true"/>
-    <row r="263" ht="14.25" customHeight="true"/>
-    <row r="264" ht="14.25" customHeight="true"/>
-    <row r="265" ht="14.25" customHeight="true"/>
-    <row r="266" ht="14.25" customHeight="true"/>
-    <row r="267" ht="14.25" customHeight="true"/>
-    <row r="268" ht="14.25" customHeight="true"/>
-    <row r="269" ht="14.25" customHeight="true"/>
-    <row r="270" ht="14.25" customHeight="true"/>
-    <row r="271" ht="14.25" customHeight="true"/>
-    <row r="272" ht="14.25" customHeight="true"/>
-    <row r="273" ht="14.25" customHeight="true"/>
-    <row r="274" ht="14.25" customHeight="true"/>
-    <row r="275" ht="14.25" customHeight="true"/>
-    <row r="276" ht="14.25" customHeight="true"/>
-    <row r="277" ht="14.25" customHeight="true"/>
-    <row r="278" ht="14.25" customHeight="true"/>
-    <row r="279" ht="14.25" customHeight="true"/>
-    <row r="280" ht="14.25" customHeight="true"/>
-    <row r="281" ht="14.25" customHeight="true"/>
-    <row r="282" ht="14.25" customHeight="true"/>
-    <row r="283" ht="14.25" customHeight="true"/>
-    <row r="284" ht="14.25" customHeight="true"/>
-    <row r="285" ht="14.25" customHeight="true"/>
-    <row r="286" ht="14.25" customHeight="true"/>
-    <row r="287" ht="14.25" customHeight="true"/>
-    <row r="288" ht="14.25" customHeight="true"/>
-    <row r="289" ht="14.25" customHeight="true"/>
-    <row r="290" ht="14.25" customHeight="true"/>
-    <row r="291" ht="14.25" customHeight="true"/>
-    <row r="292" ht="14.25" customHeight="true"/>
-    <row r="293" ht="14.25" customHeight="true"/>
-    <row r="294" ht="14.25" customHeight="true"/>
-    <row r="295" ht="14.25" customHeight="true"/>
-    <row r="296" ht="14.25" customHeight="true"/>
-    <row r="297" ht="14.25" customHeight="true"/>
-    <row r="298" ht="14.25" customHeight="true"/>
-    <row r="299" ht="14.25" customHeight="true"/>
-    <row r="300" ht="14.25" customHeight="true"/>
-    <row r="301" ht="14.25" customHeight="true"/>
-    <row r="302" ht="14.25" customHeight="true"/>
-    <row r="303" ht="14.25" customHeight="true"/>
-    <row r="304" ht="14.25" customHeight="true"/>
-    <row r="305" ht="14.25" customHeight="true"/>
-    <row r="306" ht="14.25" customHeight="true"/>
-    <row r="307" ht="14.25" customHeight="true"/>
-    <row r="308" ht="14.25" customHeight="true"/>
-    <row r="309" ht="14.25" customHeight="true"/>
-    <row r="310" ht="14.25" customHeight="true"/>
-    <row r="311" ht="14.25" customHeight="true"/>
-    <row r="312" ht="14.25" customHeight="true"/>
-    <row r="313" ht="14.25" customHeight="true"/>
-    <row r="314" ht="14.25" customHeight="true"/>
-    <row r="315" ht="14.25" customHeight="true"/>
-    <row r="316" ht="14.25" customHeight="true"/>
-    <row r="317" ht="14.25" customHeight="true"/>
-    <row r="318" ht="14.25" customHeight="true"/>
-    <row r="319" ht="14.25" customHeight="true"/>
-    <row r="320" ht="14.25" customHeight="true"/>
-    <row r="321" ht="14.25" customHeight="true"/>
-    <row r="322" ht="14.25" customHeight="true"/>
-    <row r="323" ht="14.25" customHeight="true"/>
-    <row r="324" ht="14.25" customHeight="true"/>
-    <row r="325" ht="14.25" customHeight="true"/>
-    <row r="326" ht="14.25" customHeight="true"/>
-    <row r="327" ht="14.25" customHeight="true"/>
-    <row r="328" ht="14.25" customHeight="true"/>
-    <row r="329" ht="14.25" customHeight="true"/>
-    <row r="330" ht="14.25" customHeight="true"/>
-    <row r="331" ht="14.25" customHeight="true"/>
-    <row r="332" ht="14.25" customHeight="true"/>
-    <row r="333" ht="14.25" customHeight="true"/>
-    <row r="334" ht="14.25" customHeight="true"/>
-    <row r="335" ht="14.25" customHeight="true"/>
-    <row r="336" ht="14.25" customHeight="true"/>
-    <row r="337" ht="14.25" customHeight="true"/>
-    <row r="338" ht="14.25" customHeight="true"/>
-    <row r="339" ht="14.25" customHeight="true"/>
-    <row r="340" ht="14.25" customHeight="true"/>
-    <row r="341" ht="14.25" customHeight="true"/>
-    <row r="342" ht="14.25" customHeight="true"/>
-    <row r="343" ht="14.25" customHeight="true"/>
-    <row r="344" ht="14.25" customHeight="true"/>
-    <row r="345" ht="14.25" customHeight="true"/>
-    <row r="346" ht="14.25" customHeight="true"/>
-    <row r="347" ht="14.25" customHeight="true"/>
-    <row r="348" ht="14.25" customHeight="true"/>
-    <row r="349" ht="14.25" customHeight="true"/>
-    <row r="350" ht="14.25" customHeight="true"/>
-    <row r="351" ht="14.25" customHeight="true"/>
-    <row r="352" ht="14.25" customHeight="true"/>
-    <row r="353" ht="14.25" customHeight="true"/>
-    <row r="354" ht="14.25" customHeight="true"/>
-    <row r="355" ht="14.25" customHeight="true"/>
-    <row r="356" ht="14.25" customHeight="true"/>
-    <row r="357" ht="14.25" customHeight="true"/>
-    <row r="358" ht="14.25" customHeight="true"/>
-    <row r="359" ht="14.25" customHeight="true"/>
-    <row r="360" ht="14.25" customHeight="true"/>
-    <row r="361" ht="14.25" customHeight="true"/>
-    <row r="362" ht="14.25" customHeight="true"/>
-    <row r="363" ht="14.25" customHeight="true"/>
-    <row r="364" ht="14.25" customHeight="true"/>
-    <row r="365" ht="14.25" customHeight="true"/>
-    <row r="366" ht="14.25" customHeight="true"/>
-    <row r="367" ht="14.25" customHeight="true"/>
-    <row r="368" ht="14.25" customHeight="true"/>
-    <row r="369" ht="14.25" customHeight="true"/>
-    <row r="370" ht="14.25" customHeight="true"/>
-    <row r="371" ht="14.25" customHeight="true"/>
-    <row r="372" ht="14.25" customHeight="true"/>
-    <row r="373" ht="14.25" customHeight="true"/>
-    <row r="374" ht="14.25" customHeight="true"/>
-    <row r="375" ht="14.25" customHeight="true"/>
-    <row r="376" ht="14.25" customHeight="true"/>
-    <row r="377" ht="14.25" customHeight="true"/>
-    <row r="378" ht="14.25" customHeight="true"/>
-    <row r="379" ht="14.25" customHeight="true"/>
-    <row r="380" ht="14.25" customHeight="true"/>
-    <row r="381" ht="14.25" customHeight="true"/>
-    <row r="382" ht="14.25" customHeight="true"/>
-    <row r="383" ht="14.25" customHeight="true"/>
-    <row r="384" ht="14.25" customHeight="true"/>
-    <row r="385" ht="14.25" customHeight="true"/>
-    <row r="386" ht="14.25" customHeight="true"/>
-    <row r="387" ht="14.25" customHeight="true"/>
-    <row r="388" ht="14.25" customHeight="true"/>
-    <row r="389" ht="14.25" customHeight="true"/>
-    <row r="390" ht="14.25" customHeight="true"/>
-    <row r="391" ht="14.25" customHeight="true"/>
-    <row r="392" ht="14.25" customHeight="true"/>
-    <row r="393" ht="14.25" customHeight="true"/>
-    <row r="394" ht="14.25" customHeight="true"/>
-    <row r="395" ht="14.25" customHeight="true"/>
-    <row r="396" ht="14.25" customHeight="true"/>
-    <row r="397" ht="14.25" customHeight="true"/>
-    <row r="398" ht="14.25" customHeight="true"/>
-    <row r="399" ht="14.25" customHeight="true"/>
-    <row r="400" ht="14.25" customHeight="true"/>
-    <row r="401" ht="14.25" customHeight="true"/>
-    <row r="402" ht="14.25" customHeight="true"/>
-    <row r="403" ht="14.25" customHeight="true"/>
-    <row r="404" ht="14.25" customHeight="true"/>
-    <row r="405" ht="14.25" customHeight="true"/>
-    <row r="406" ht="14.25" customHeight="true"/>
-    <row r="407" ht="14.25" customHeight="true"/>
-    <row r="408" ht="14.25" customHeight="true"/>
-    <row r="409" ht="14.25" customHeight="true"/>
-    <row r="410" ht="14.25" customHeight="true"/>
-    <row r="411" ht="14.25" customHeight="true"/>
-    <row r="412" ht="14.25" customHeight="true"/>
-    <row r="413" ht="14.25" customHeight="true"/>
-    <row r="414" ht="14.25" customHeight="true"/>
-    <row r="415" ht="14.25" customHeight="true"/>
-    <row r="416" ht="14.25" customHeight="true"/>
-    <row r="417" ht="14.25" customHeight="true"/>
-    <row r="418" ht="14.25" customHeight="true"/>
-    <row r="419" ht="14.25" customHeight="true"/>
-    <row r="420" ht="14.25" customHeight="true"/>
-    <row r="421" ht="14.25" customHeight="true"/>
-    <row r="422" ht="14.25" customHeight="true"/>
-    <row r="423" ht="14.25" customHeight="true"/>
-    <row r="424" ht="14.25" customHeight="true"/>
-    <row r="425" ht="14.25" customHeight="true"/>
-    <row r="426" ht="14.25" customHeight="true"/>
-    <row r="427" ht="14.25" customHeight="true"/>
-    <row r="428" ht="14.25" customHeight="true"/>
-    <row r="429" ht="14.25" customHeight="true"/>
-    <row r="430" ht="14.25" customHeight="true"/>
-    <row r="431" ht="14.25" customHeight="true"/>
-    <row r="432" ht="14.25" customHeight="true"/>
-    <row r="433" ht="14.25" customHeight="true"/>
-    <row r="434" ht="14.25" customHeight="true"/>
-    <row r="435" ht="14.25" customHeight="true"/>
-    <row r="436" ht="14.25" customHeight="true"/>
-    <row r="437" ht="14.25" customHeight="true"/>
-    <row r="438" ht="14.25" customHeight="true"/>
-    <row r="439" ht="14.25" customHeight="true"/>
-    <row r="440" ht="14.25" customHeight="true"/>
-    <row r="441" ht="14.25" customHeight="true"/>
-    <row r="442" ht="14.25" customHeight="true"/>
-    <row r="443" ht="14.25" customHeight="true"/>
-    <row r="444" ht="14.25" customHeight="true"/>
-    <row r="445" ht="14.25" customHeight="true"/>
-    <row r="446" ht="14.25" customHeight="true"/>
-    <row r="447" ht="14.25" customHeight="true"/>
-    <row r="448" ht="14.25" customHeight="true"/>
-    <row r="449" ht="14.25" customHeight="true"/>
-    <row r="450" ht="14.25" customHeight="true"/>
-    <row r="451" ht="14.25" customHeight="true"/>
-    <row r="452" ht="14.25" customHeight="true"/>
-    <row r="453" ht="14.25" customHeight="true"/>
-    <row r="454" ht="14.25" customHeight="true"/>
-    <row r="455" ht="14.25" customHeight="true"/>
-    <row r="456" ht="14.25" customHeight="true"/>
-    <row r="457" ht="14.25" customHeight="true"/>
-    <row r="458" ht="14.25" customHeight="true"/>
-    <row r="459" ht="14.25" customHeight="true"/>
-    <row r="460" ht="14.25" customHeight="true"/>
-    <row r="461" ht="14.25" customHeight="true"/>
-    <row r="462" ht="14.25" customHeight="true"/>
-    <row r="463" ht="14.25" customHeight="true"/>
-    <row r="464" ht="14.25" customHeight="true"/>
-    <row r="465" ht="14.25" customHeight="true"/>
-    <row r="466" ht="14.25" customHeight="true"/>
-    <row r="467" ht="14.25" customHeight="true"/>
-    <row r="468" ht="14.25" customHeight="true"/>
-    <row r="469" ht="14.25" customHeight="true"/>
-    <row r="470" ht="14.25" customHeight="true"/>
-    <row r="471" ht="14.25" customHeight="true"/>
-    <row r="472" ht="14.25" customHeight="true"/>
-    <row r="473" ht="14.25" customHeight="true"/>
-    <row r="474" ht="14.25" customHeight="true"/>
-    <row r="475" ht="14.25" customHeight="true"/>
-    <row r="476" ht="14.25" customHeight="true"/>
-    <row r="477" ht="14.25" customHeight="true"/>
-    <row r="478" ht="14.25" customHeight="true"/>
-    <row r="479" ht="14.25" customHeight="true"/>
-    <row r="480" ht="14.25" customHeight="true"/>
-    <row r="481" ht="14.25" customHeight="true"/>
-    <row r="482" ht="14.25" customHeight="true"/>
-    <row r="483" ht="14.25" customHeight="true"/>
-    <row r="484" ht="14.25" customHeight="true"/>
-    <row r="485" ht="14.25" customHeight="true"/>
-    <row r="486" ht="14.25" customHeight="true"/>
-    <row r="487" ht="14.25" customHeight="true"/>
-    <row r="488" ht="14.25" customHeight="true"/>
-    <row r="489" ht="14.25" customHeight="true"/>
-    <row r="490" ht="14.25" customHeight="true"/>
-    <row r="491" ht="14.25" customHeight="true"/>
-    <row r="492" ht="14.25" customHeight="true"/>
-    <row r="493" ht="14.25" customHeight="true"/>
-    <row r="494" ht="14.25" customHeight="true"/>
-    <row r="495" ht="14.25" customHeight="true"/>
-    <row r="496" ht="14.25" customHeight="true"/>
-    <row r="497" ht="14.25" customHeight="true"/>
-    <row r="498" ht="14.25" customHeight="true"/>
-    <row r="499" ht="14.25" customHeight="true"/>
-    <row r="500" ht="14.25" customHeight="true"/>
-    <row r="501" ht="14.25" customHeight="true"/>
-    <row r="502" ht="14.25" customHeight="true"/>
-    <row r="503" ht="14.25" customHeight="true"/>
-    <row r="504" ht="14.25" customHeight="true"/>
-    <row r="505" ht="14.25" customHeight="true"/>
-    <row r="506" ht="14.25" customHeight="true"/>
-    <row r="507" ht="14.25" customHeight="true"/>
-    <row r="508" ht="14.25" customHeight="true"/>
-    <row r="509" ht="14.25" customHeight="true"/>
-    <row r="510" ht="14.25" customHeight="true"/>
-    <row r="511" ht="14.25" customHeight="true"/>
-    <row r="512" ht="14.25" customHeight="true"/>
-    <row r="513" ht="14.25" customHeight="true"/>
-    <row r="514" ht="14.25" customHeight="true"/>
-    <row r="515" ht="14.25" customHeight="true"/>
-    <row r="516" ht="14.25" customHeight="true"/>
-    <row r="517" ht="14.25" customHeight="true"/>
-    <row r="518" ht="14.25" customHeight="true"/>
-    <row r="519" ht="14.25" customHeight="true"/>
-    <row r="520" ht="14.25" customHeight="true"/>
-    <row r="521" ht="14.25" customHeight="true"/>
-    <row r="522" ht="14.25" customHeight="true"/>
-    <row r="523" ht="14.25" customHeight="true"/>
-    <row r="524" ht="14.25" customHeight="true"/>
-    <row r="525" ht="14.25" customHeight="true"/>
-    <row r="526" ht="14.25" customHeight="true"/>
-    <row r="527" ht="14.25" customHeight="true"/>
-    <row r="528" ht="14.25" customHeight="true"/>
-    <row r="529" ht="14.25" customHeight="true"/>
-    <row r="530" ht="14.25" customHeight="true"/>
-    <row r="531" ht="14.25" customHeight="true"/>
-    <row r="532" ht="14.25" customHeight="true"/>
-    <row r="533" ht="14.25" customHeight="true"/>
-    <row r="534" ht="14.25" customHeight="true"/>
-    <row r="535" ht="14.25" customHeight="true"/>
-    <row r="536" ht="14.25" customHeight="true"/>
-    <row r="537" ht="14.25" customHeight="true"/>
-    <row r="538" ht="14.25" customHeight="true"/>
-    <row r="539" ht="14.25" customHeight="true"/>
-    <row r="540" ht="14.25" customHeight="true"/>
-    <row r="541" ht="14.25" customHeight="true"/>
-    <row r="542" ht="14.25" customHeight="true"/>
-    <row r="543" ht="14.25" customHeight="true"/>
-    <row r="544" ht="14.25" customHeight="true"/>
-    <row r="545" ht="14.25" customHeight="true"/>
-    <row r="546" ht="14.25" customHeight="true"/>
-    <row r="547" ht="14.25" customHeight="true"/>
-    <row r="548" ht="14.25" customHeight="true"/>
-    <row r="549" ht="14.25" customHeight="true"/>
-    <row r="550" ht="14.25" customHeight="true"/>
-    <row r="551" ht="14.25" customHeight="true"/>
-    <row r="552" ht="14.25" customHeight="true"/>
-    <row r="553" ht="14.25" customHeight="true"/>
-    <row r="554" ht="14.25" customHeight="true"/>
-    <row r="555" ht="14.25" customHeight="true"/>
-    <row r="556" ht="14.25" customHeight="true"/>
-    <row r="557" ht="14.25" customHeight="true"/>
-    <row r="558" ht="14.25" customHeight="true"/>
-    <row r="559" ht="14.25" customHeight="true"/>
-    <row r="560" ht="14.25" customHeight="true"/>
-    <row r="561" ht="14.25" customHeight="true"/>
-    <row r="562" ht="14.25" customHeight="true"/>
-    <row r="563" ht="14.25" customHeight="true"/>
-    <row r="564" ht="14.25" customHeight="true"/>
-    <row r="565" ht="14.25" customHeight="true"/>
-    <row r="566" ht="14.25" customHeight="true"/>
-    <row r="567" ht="14.25" customHeight="true"/>
-    <row r="568" ht="14.25" customHeight="true"/>
-    <row r="569" ht="14.25" customHeight="true"/>
-    <row r="570" ht="14.25" customHeight="true"/>
-    <row r="571" ht="14.25" customHeight="true"/>
-    <row r="572" ht="14.25" customHeight="true"/>
-    <row r="573" ht="14.25" customHeight="true"/>
-    <row r="574" ht="14.25" customHeight="true"/>
-    <row r="575" ht="14.25" customHeight="true"/>
-    <row r="576" ht="14.25" customHeight="true"/>
-    <row r="577" ht="14.25" customHeight="true"/>
-    <row r="578" ht="14.25" customHeight="true"/>
-    <row r="579" ht="14.25" customHeight="true"/>
-    <row r="580" ht="14.25" customHeight="true"/>
-    <row r="581" ht="14.25" customHeight="true"/>
-    <row r="582" ht="14.25" customHeight="true"/>
-    <row r="583" ht="14.25" customHeight="true"/>
-    <row r="584" ht="14.25" customHeight="true"/>
-    <row r="585" ht="14.25" customHeight="true"/>
-    <row r="586" ht="14.25" customHeight="true"/>
-    <row r="587" ht="14.25" customHeight="true"/>
-    <row r="588" ht="14.25" customHeight="true"/>
-    <row r="589" ht="14.25" customHeight="true"/>
-    <row r="590" ht="14.25" customHeight="true"/>
-    <row r="591" ht="14.25" customHeight="true"/>
-    <row r="592" ht="14.25" customHeight="true"/>
-    <row r="593" ht="14.25" customHeight="true"/>
-    <row r="594" ht="14.25" customHeight="true"/>
-    <row r="595" ht="14.25" customHeight="true"/>
-    <row r="596" ht="14.25" customHeight="true"/>
-    <row r="597" ht="14.25" customHeight="true"/>
-    <row r="598" ht="14.25" customHeight="true"/>
-    <row r="599" ht="14.25" customHeight="true"/>
-    <row r="600" ht="14.25" customHeight="true"/>
-    <row r="601" ht="14.25" customHeight="true"/>
-    <row r="602" ht="14.25" customHeight="true"/>
-    <row r="603" ht="14.25" customHeight="true"/>
-    <row r="604" ht="14.25" customHeight="true"/>
-    <row r="605" ht="14.25" customHeight="true"/>
-    <row r="606" ht="14.25" customHeight="true"/>
-    <row r="607" ht="14.25" customHeight="true"/>
-    <row r="608" ht="14.25" customHeight="true"/>
-    <row r="609" ht="14.25" customHeight="true"/>
-    <row r="610" ht="14.25" customHeight="true"/>
-    <row r="611" ht="14.25" customHeight="true"/>
-    <row r="612" ht="14.25" customHeight="true"/>
-    <row r="613" ht="14.25" customHeight="true"/>
-    <row r="614" ht="14.25" customHeight="true"/>
-    <row r="615" ht="14.25" customHeight="true"/>
-    <row r="616" ht="14.25" customHeight="true"/>
-    <row r="617" ht="14.25" customHeight="true"/>
-    <row r="618" ht="14.25" customHeight="true"/>
-    <row r="619" ht="14.25" customHeight="true"/>
-    <row r="620" ht="14.25" customHeight="true"/>
-    <row r="621" ht="14.25" customHeight="true"/>
-    <row r="622" ht="14.25" customHeight="true"/>
-    <row r="623" ht="14.25" customHeight="true"/>
-    <row r="624" ht="14.25" customHeight="true"/>
-    <row r="625" ht="14.25" customHeight="true"/>
-    <row r="626" ht="14.25" customHeight="true"/>
-    <row r="627" ht="14.25" customHeight="true"/>
-    <row r="628" ht="14.25" customHeight="true"/>
-    <row r="629" ht="14.25" customHeight="true"/>
-    <row r="630" ht="14.25" customHeight="true"/>
-    <row r="631" ht="14.25" customHeight="true"/>
-    <row r="632" ht="14.25" customHeight="true"/>
-    <row r="633" ht="14.25" customHeight="true"/>
-    <row r="634" ht="14.25" customHeight="true"/>
-    <row r="635" ht="14.25" customHeight="true"/>
-    <row r="636" ht="14.25" customHeight="true"/>
-    <row r="637" ht="14.25" customHeight="true"/>
-    <row r="638" ht="14.25" customHeight="true"/>
-    <row r="639" ht="14.25" customHeight="true"/>
-    <row r="640" ht="14.25" customHeight="true"/>
-    <row r="641" ht="14.25" customHeight="true"/>
-    <row r="642" ht="14.25" customHeight="true"/>
-    <row r="643" ht="14.25" customHeight="true"/>
-    <row r="644" ht="14.25" customHeight="true"/>
-    <row r="645" ht="14.25" customHeight="true"/>
-    <row r="646" ht="14.25" customHeight="true"/>
-    <row r="647" ht="14.25" customHeight="true"/>
-    <row r="648" ht="14.25" customHeight="true"/>
-    <row r="649" ht="14.25" customHeight="true"/>
-    <row r="650" ht="14.25" customHeight="true"/>
-    <row r="651" ht="14.25" customHeight="true"/>
-    <row r="652" ht="14.25" customHeight="true"/>
-    <row r="653" ht="14.25" customHeight="true"/>
-    <row r="654" ht="14.25" customHeight="true"/>
-    <row r="655" ht="14.25" customHeight="true"/>
-    <row r="656" ht="14.25" customHeight="true"/>
-    <row r="657" ht="14.25" customHeight="true"/>
-    <row r="658" ht="14.25" customHeight="true"/>
-    <row r="659" ht="14.25" customHeight="true"/>
-    <row r="660" ht="14.25" customHeight="true"/>
-    <row r="661" ht="14.25" customHeight="true"/>
-    <row r="662" ht="14.25" customHeight="true"/>
-    <row r="663" ht="14.25" customHeight="true"/>
-    <row r="664" ht="14.25" customHeight="true"/>
-    <row r="665" ht="14.25" customHeight="true"/>
-    <row r="666" ht="14.25" customHeight="true"/>
-    <row r="667" ht="14.25" customHeight="true"/>
-    <row r="668" ht="14.25" customHeight="true"/>
-    <row r="669" ht="14.25" customHeight="true"/>
-    <row r="670" ht="14.25" customHeight="true"/>
-    <row r="671" ht="14.25" customHeight="true"/>
-    <row r="672" ht="14.25" customHeight="true"/>
-    <row r="673" ht="14.25" customHeight="true"/>
-    <row r="674" ht="14.25" customHeight="true"/>
-    <row r="675" ht="14.25" customHeight="true"/>
-    <row r="676" ht="14.25" customHeight="true"/>
-    <row r="677" ht="14.25" customHeight="true"/>
-    <row r="678" ht="14.25" customHeight="true"/>
-    <row r="679" ht="14.25" customHeight="true"/>
-    <row r="680" ht="14.25" customHeight="true"/>
-    <row r="681" ht="14.25" customHeight="true"/>
-    <row r="682" ht="14.25" customHeight="true"/>
-    <row r="683" ht="14.25" customHeight="true"/>
-    <row r="684" ht="14.25" customHeight="true"/>
-    <row r="685" ht="14.25" customHeight="true"/>
-    <row r="686" ht="14.25" customHeight="true"/>
-    <row r="687" ht="14.25" customHeight="true"/>
-    <row r="688" ht="14.25" customHeight="true"/>
-    <row r="689" ht="14.25" customHeight="true"/>
-    <row r="690" ht="14.25" customHeight="true"/>
-    <row r="691" ht="14.25" customHeight="true"/>
-    <row r="692" ht="14.25" customHeight="true"/>
-    <row r="693" ht="14.25" customHeight="true"/>
-    <row r="694" ht="14.25" customHeight="true"/>
-    <row r="695" ht="14.25" customHeight="true"/>
-    <row r="696" ht="14.25" customHeight="true"/>
-    <row r="697" ht="14.25" customHeight="true"/>
-    <row r="698" ht="14.25" customHeight="true"/>
-    <row r="699" ht="14.25" customHeight="true"/>
-    <row r="700" ht="14.25" customHeight="true"/>
-    <row r="701" ht="14.25" customHeight="true"/>
-    <row r="702" ht="14.25" customHeight="true"/>
-    <row r="703" ht="14.25" customHeight="true"/>
-    <row r="704" ht="14.25" customHeight="true"/>
-    <row r="705" ht="14.25" customHeight="true"/>
-    <row r="706" ht="14.25" customHeight="true"/>
-    <row r="707" ht="14.25" customHeight="true"/>
-    <row r="708" ht="14.25" customHeight="true"/>
-    <row r="709" ht="14.25" customHeight="true"/>
-    <row r="710" ht="14.25" customHeight="true"/>
-    <row r="711" ht="14.25" customHeight="true"/>
-    <row r="712" ht="14.25" customHeight="true"/>
-    <row r="713" ht="14.25" customHeight="true"/>
-    <row r="714" ht="14.25" customHeight="true"/>
-    <row r="715" ht="14.25" customHeight="true"/>
-    <row r="716" ht="14.25" customHeight="true"/>
-    <row r="717" ht="14.25" customHeight="true"/>
-    <row r="718" ht="14.25" customHeight="true"/>
-    <row r="719" ht="14.25" customHeight="true"/>
-    <row r="720" ht="14.25" customHeight="true"/>
-    <row r="721" ht="14.25" customHeight="true"/>
-    <row r="722" ht="14.25" customHeight="true"/>
-    <row r="723" ht="14.25" customHeight="true"/>
-    <row r="724" ht="14.25" customHeight="true"/>
-    <row r="725" ht="14.25" customHeight="true"/>
-    <row r="726" ht="14.25" customHeight="true"/>
-    <row r="727" ht="14.25" customHeight="true"/>
-    <row r="728" ht="14.25" customHeight="true"/>
-    <row r="729" ht="14.25" customHeight="true"/>
-    <row r="730" ht="14.25" customHeight="true"/>
-    <row r="731" ht="14.25" customHeight="true"/>
-    <row r="732" ht="14.25" customHeight="true"/>
-    <row r="733" ht="14.25" customHeight="true"/>
-    <row r="734" ht="14.25" customHeight="true"/>
-    <row r="735" ht="14.25" customHeight="true"/>
-    <row r="736" ht="14.25" customHeight="true"/>
-    <row r="737" ht="14.25" customHeight="true"/>
-    <row r="738" ht="14.25" customHeight="true"/>
-    <row r="739" ht="14.25" customHeight="true"/>
-    <row r="740" ht="14.25" customHeight="true"/>
-    <row r="741" ht="14.25" customHeight="true"/>
-    <row r="742" ht="14.25" customHeight="true"/>
-    <row r="743" ht="14.25" customHeight="true"/>
-    <row r="744" ht="14.25" customHeight="true"/>
-    <row r="745" ht="14.25" customHeight="true"/>
-    <row r="746" ht="14.25" customHeight="true"/>
-    <row r="747" ht="14.25" customHeight="true"/>
-    <row r="748" ht="14.25" customHeight="true"/>
-    <row r="749" ht="14.25" customHeight="true"/>
-    <row r="750" ht="14.25" customHeight="true"/>
-    <row r="751" ht="14.25" customHeight="true"/>
-    <row r="752" ht="14.25" customHeight="true"/>
-    <row r="753" ht="14.25" customHeight="true"/>
-    <row r="754" ht="14.25" customHeight="true"/>
-    <row r="755" ht="14.25" customHeight="true"/>
-    <row r="756" ht="14.25" customHeight="true"/>
-    <row r="757" ht="14.25" customHeight="true"/>
-    <row r="758" ht="14.25" customHeight="true"/>
-    <row r="759" ht="14.25" customHeight="true"/>
-    <row r="760" ht="14.25" customHeight="true"/>
-    <row r="761" ht="14.25" customHeight="true"/>
-    <row r="762" ht="14.25" customHeight="true"/>
-    <row r="763" ht="14.25" customHeight="true"/>
-    <row r="764" ht="14.25" customHeight="true"/>
-    <row r="765" ht="14.25" customHeight="true"/>
-    <row r="766" ht="14.25" customHeight="true"/>
-    <row r="767" ht="14.25" customHeight="true"/>
-    <row r="768" ht="14.25" customHeight="true"/>
-    <row r="769" ht="14.25" customHeight="true"/>
-    <row r="770" ht="14.25" customHeight="true"/>
-    <row r="771" ht="14.25" customHeight="true"/>
-    <row r="772" ht="14.25" customHeight="true"/>
-    <row r="773" ht="14.25" customHeight="true"/>
-    <row r="774" ht="14.25" customHeight="true"/>
-    <row r="775" ht="14.25" customHeight="true"/>
-    <row r="776" ht="14.25" customHeight="true"/>
-    <row r="777" ht="14.25" customHeight="true"/>
-    <row r="778" ht="14.25" customHeight="true"/>
-    <row r="779" ht="14.25" customHeight="true"/>
-    <row r="780" ht="14.25" customHeight="true"/>
-    <row r="781" ht="14.25" customHeight="true"/>
-    <row r="782" ht="14.25" customHeight="true"/>
-    <row r="783" ht="14.25" customHeight="true"/>
-    <row r="784" ht="14.25" customHeight="true"/>
-    <row r="785" ht="14.25" customHeight="true"/>
-    <row r="786" ht="14.25" customHeight="true"/>
-    <row r="787" ht="14.25" customHeight="true"/>
-    <row r="788" ht="14.25" customHeight="true"/>
-    <row r="789" ht="14.25" customHeight="true"/>
-    <row r="790" ht="14.25" customHeight="true"/>
-    <row r="791" ht="14.25" customHeight="true"/>
-    <row r="792" ht="14.25" customHeight="true"/>
-    <row r="793" ht="14.25" customHeight="true"/>
-    <row r="794" ht="14.25" customHeight="true"/>
-    <row r="795" ht="14.25" customHeight="true"/>
-    <row r="796" ht="14.25" customHeight="true"/>
-    <row r="797" ht="14.25" customHeight="true"/>
-    <row r="798" ht="14.25" customHeight="true"/>
-    <row r="799" ht="14.25" customHeight="true"/>
-    <row r="800" ht="14.25" customHeight="true"/>
-    <row r="801" ht="14.25" customHeight="true"/>
-    <row r="802" ht="14.25" customHeight="true"/>
-    <row r="803" ht="14.25" customHeight="true"/>
-    <row r="804" ht="14.25" customHeight="true"/>
-    <row r="805" ht="14.25" customHeight="true"/>
-    <row r="806" ht="14.25" customHeight="true"/>
-    <row r="807" ht="14.25" customHeight="true"/>
-    <row r="808" ht="14.25" customHeight="true"/>
-    <row r="809" ht="14.25" customHeight="true"/>
-    <row r="810" ht="14.25" customHeight="true"/>
-    <row r="811" ht="14.25" customHeight="true"/>
-    <row r="812" ht="14.25" customHeight="true"/>
-    <row r="813" ht="14.25" customHeight="true"/>
-    <row r="814" ht="14.25" customHeight="true"/>
-    <row r="815" ht="14.25" customHeight="true"/>
-    <row r="816" ht="14.25" customHeight="true"/>
-    <row r="817" ht="14.25" customHeight="true"/>
-    <row r="818" ht="14.25" customHeight="true"/>
-    <row r="819" ht="14.25" customHeight="true"/>
-    <row r="820" ht="14.25" customHeight="true"/>
-    <row r="821" ht="14.25" customHeight="true"/>
-    <row r="822" ht="14.25" customHeight="true"/>
-    <row r="823" ht="14.25" customHeight="true"/>
-    <row r="824" ht="14.25" customHeight="true"/>
-    <row r="825" ht="14.25" customHeight="true"/>
-    <row r="826" ht="14.25" customHeight="true"/>
-    <row r="827" ht="14.25" customHeight="true"/>
-    <row r="828" ht="14.25" customHeight="true"/>
-    <row r="829" ht="14.25" customHeight="true"/>
-    <row r="830" ht="14.25" customHeight="true"/>
-    <row r="831" ht="14.25" customHeight="true"/>
-    <row r="832" ht="14.25" customHeight="true"/>
-    <row r="833" ht="14.25" customHeight="true"/>
-    <row r="834" ht="14.25" customHeight="true"/>
-    <row r="835" ht="14.25" customHeight="true"/>
-    <row r="836" ht="14.25" customHeight="true"/>
-    <row r="837" ht="14.25" customHeight="true"/>
-    <row r="838" ht="14.25" customHeight="true"/>
-    <row r="839" ht="14.25" customHeight="true"/>
-    <row r="840" ht="14.25" customHeight="true"/>
-    <row r="841" ht="14.25" customHeight="true"/>
-    <row r="842" ht="14.25" customHeight="true"/>
-    <row r="843" ht="14.25" customHeight="true"/>
-    <row r="844" ht="14.25" customHeight="true"/>
-    <row r="845" ht="14.25" customHeight="true"/>
-    <row r="846" ht="14.25" customHeight="true"/>
-    <row r="847" ht="14.25" customHeight="true"/>
-    <row r="848" ht="14.25" customHeight="true"/>
-    <row r="849" ht="14.25" customHeight="true"/>
-    <row r="850" ht="14.25" customHeight="true"/>
-    <row r="851" ht="14.25" customHeight="true"/>
-    <row r="852" ht="14.25" customHeight="true"/>
-    <row r="853" ht="14.25" customHeight="true"/>
-    <row r="854" ht="14.25" customHeight="true"/>
-    <row r="855" ht="14.25" customHeight="true"/>
-    <row r="856" ht="14.25" customHeight="true"/>
-    <row r="857" ht="14.25" customHeight="true"/>
-    <row r="858" ht="14.25" customHeight="true"/>
-    <row r="859" ht="14.25" customHeight="true"/>
-    <row r="860" ht="14.25" customHeight="true"/>
-    <row r="861" ht="14.25" customHeight="true"/>
-    <row r="862" ht="14.25" customHeight="true"/>
-    <row r="863" ht="14.25" customHeight="true"/>
-    <row r="864" ht="14.25" customHeight="true"/>
-    <row r="865" ht="14.25" customHeight="true"/>
-    <row r="866" ht="14.25" customHeight="true"/>
-    <row r="867" ht="14.25" customHeight="true"/>
-    <row r="868" ht="14.25" customHeight="true"/>
-    <row r="869" ht="14.25" customHeight="true"/>
-    <row r="870" ht="14.25" customHeight="true"/>
-    <row r="871" ht="14.25" customHeight="true"/>
-    <row r="872" ht="14.25" customHeight="true"/>
-    <row r="873" ht="14.25" customHeight="true"/>
-    <row r="874" ht="14.25" customHeight="true"/>
-    <row r="875" ht="14.25" customHeight="true"/>
-    <row r="876" ht="14.25" customHeight="true"/>
-    <row r="877" ht="14.25" customHeight="true"/>
-    <row r="878" ht="14.25" customHeight="true"/>
-    <row r="879" ht="14.25" customHeight="true"/>
-    <row r="880" ht="14.25" customHeight="true"/>
-    <row r="881" ht="14.25" customHeight="true"/>
-    <row r="882" ht="14.25" customHeight="true"/>
-    <row r="883" ht="14.25" customHeight="true"/>
-    <row r="884" ht="14.25" customHeight="true"/>
-    <row r="885" ht="14.25" customHeight="true"/>
-    <row r="886" ht="14.25" customHeight="true"/>
-    <row r="887" ht="14.25" customHeight="true"/>
-    <row r="888" ht="14.25" customHeight="true"/>
-    <row r="889" ht="14.25" customHeight="true"/>
-    <row r="890" ht="14.25" customHeight="true"/>
-    <row r="891" ht="14.25" customHeight="true"/>
-    <row r="892" ht="14.25" customHeight="true"/>
-    <row r="893" ht="14.25" customHeight="true"/>
-    <row r="894" ht="14.25" customHeight="true"/>
-    <row r="895" ht="14.25" customHeight="true"/>
-    <row r="896" ht="14.25" customHeight="true"/>
-    <row r="897" ht="14.25" customHeight="true"/>
-    <row r="898" ht="14.25" customHeight="true"/>
-    <row r="899" ht="14.25" customHeight="true"/>
-    <row r="900" ht="14.25" customHeight="true"/>
-    <row r="901" ht="14.25" customHeight="true"/>
-    <row r="902" ht="14.25" customHeight="true"/>
-    <row r="903" ht="14.25" customHeight="true"/>
-    <row r="904" ht="14.25" customHeight="true"/>
-    <row r="905" ht="14.25" customHeight="true"/>
-    <row r="906" ht="14.25" customHeight="true"/>
-    <row r="907" ht="14.25" customHeight="true"/>
-    <row r="908" ht="14.25" customHeight="true"/>
-    <row r="909" ht="14.25" customHeight="true"/>
-    <row r="910" ht="14.25" customHeight="true"/>
-    <row r="911" ht="14.25" customHeight="true"/>
-    <row r="912" ht="14.25" customHeight="true"/>
-    <row r="913" ht="14.25" customHeight="true"/>
-    <row r="914" ht="14.25" customHeight="true"/>
-    <row r="915" ht="14.25" customHeight="true"/>
-    <row r="916" ht="14.25" customHeight="true"/>
-    <row r="917" ht="14.25" customHeight="true"/>
-    <row r="918" ht="14.25" customHeight="true"/>
-    <row r="919" ht="14.25" customHeight="true"/>
-    <row r="920" ht="14.25" customHeight="true"/>
-    <row r="921" ht="14.25" customHeight="true"/>
-    <row r="922" ht="14.25" customHeight="true"/>
-    <row r="923" ht="14.25" customHeight="true"/>
-    <row r="924" ht="14.25" customHeight="true"/>
-    <row r="925" ht="14.25" customHeight="true"/>
-    <row r="926" ht="14.25" customHeight="true"/>
-    <row r="927" ht="14.25" customHeight="true"/>
-    <row r="928" ht="14.25" customHeight="true"/>
-    <row r="929" ht="14.25" customHeight="true"/>
-    <row r="930" ht="14.25" customHeight="true"/>
-    <row r="931" ht="14.25" customHeight="true"/>
-    <row r="932" ht="14.25" customHeight="true"/>
-    <row r="933" ht="14.25" customHeight="true"/>
-    <row r="934" ht="14.25" customHeight="true"/>
-    <row r="935" ht="14.25" customHeight="true"/>
-    <row r="936" ht="14.25" customHeight="true"/>
-    <row r="937" ht="14.25" customHeight="true"/>
-    <row r="938" ht="14.25" customHeight="true"/>
-    <row r="939" ht="14.25" customHeight="true"/>
-    <row r="940" ht="14.25" customHeight="true"/>
-    <row r="941" ht="14.25" customHeight="true"/>
-    <row r="942" ht="14.25" customHeight="true"/>
-    <row r="943" ht="14.25" customHeight="true"/>
-    <row r="944" ht="14.25" customHeight="true"/>
-    <row r="945" ht="14.25" customHeight="true"/>
-    <row r="946" ht="14.25" customHeight="true"/>
-    <row r="947" ht="14.25" customHeight="true"/>
-    <row r="948" ht="14.25" customHeight="true"/>
-    <row r="949" ht="14.25" customHeight="true"/>
-    <row r="950" ht="14.25" customHeight="true"/>
-    <row r="951" ht="14.25" customHeight="true"/>
-    <row r="952" ht="14.25" customHeight="true"/>
-    <row r="953" ht="14.25" customHeight="true"/>
-    <row r="954" ht="14.25" customHeight="true"/>
-    <row r="955" ht="14.25" customHeight="true"/>
-    <row r="956" ht="14.25" customHeight="true"/>
-    <row r="957" ht="14.25" customHeight="true"/>
-    <row r="958" ht="14.25" customHeight="true"/>
-    <row r="959" ht="14.25" customHeight="true"/>
-    <row r="960" ht="14.25" customHeight="true"/>
-    <row r="961" ht="14.25" customHeight="true"/>
-    <row r="962" ht="14.25" customHeight="true"/>
-    <row r="963" ht="14.25" customHeight="true"/>
-    <row r="964" ht="14.25" customHeight="true"/>
-    <row r="965" ht="14.25" customHeight="true"/>
-    <row r="966" ht="14.25" customHeight="true"/>
-    <row r="967" ht="14.25" customHeight="true"/>
-    <row r="968" ht="14.25" customHeight="true"/>
-    <row r="969" ht="14.25" customHeight="true"/>
-    <row r="970" ht="14.25" customHeight="true"/>
-    <row r="971" ht="14.25" customHeight="true"/>
-    <row r="972" ht="14.25" customHeight="true"/>
-    <row r="973" ht="14.25" customHeight="true"/>
-    <row r="974" ht="14.25" customHeight="true"/>
-    <row r="975" ht="14.25" customHeight="true"/>
-    <row r="976" ht="14.25" customHeight="true"/>
-    <row r="977" ht="14.25" customHeight="true"/>
-    <row r="978" ht="14.25" customHeight="true"/>
-    <row r="979" ht="14.25" customHeight="true"/>
-    <row r="980" ht="14.25" customHeight="true"/>
-    <row r="981" ht="14.25" customHeight="true"/>
-    <row r="982" ht="14.25" customHeight="true"/>
-    <row r="983" ht="14.25" customHeight="true"/>
-    <row r="984" ht="14.25" customHeight="true"/>
-    <row r="985" ht="14.25" customHeight="true"/>
-    <row r="986" ht="14.25" customHeight="true"/>
-    <row r="987" ht="14.25" customHeight="true"/>
-    <row r="988" ht="14.25" customHeight="true"/>
-    <row r="989" ht="14.25" customHeight="true"/>
-    <row r="990" ht="14.25" customHeight="true"/>
-    <row r="991" ht="14.25" customHeight="true"/>
-    <row r="992" ht="14.25" customHeight="true"/>
-    <row r="993" ht="14.25" customHeight="true"/>
-    <row r="994" ht="14.25" customHeight="true"/>
-    <row r="995" ht="14.25" customHeight="true"/>
-    <row r="996" ht="14.25" customHeight="true"/>
-    <row r="997" ht="14.25" customHeight="true"/>
-    <row r="998" ht="14.25" customHeight="true"/>
-    <row r="999" ht="14.25" customHeight="true"/>
-    <row r="1000" ht="14.25" customHeight="true"/>
+    <row r="5" ht="14.25" customHeight="1"/>
+    <row r="6" ht="14.25" customHeight="1"/>
+    <row r="7" ht="14.25" customHeight="1"/>
+    <row r="8" ht="14.25" customHeight="1"/>
+    <row r="9" ht="14.25" customHeight="1"/>
+    <row r="10" ht="14.25" customHeight="1"/>
+    <row r="11" ht="14.25" customHeight="1"/>
+    <row r="12" ht="14.25" customHeight="1"/>
+    <row r="13" ht="14.25" customHeight="1"/>
+    <row r="14" ht="14.25" customHeight="1"/>
+    <row r="15" ht="14.25" customHeight="1"/>
+    <row r="16" ht="14.25" customHeight="1"/>
+    <row r="17" ht="14.25" customHeight="1"/>
+    <row r="18" ht="14.25" customHeight="1"/>
+    <row r="19" ht="14.25" customHeight="1"/>
+    <row r="20" ht="14.25" customHeight="1"/>
+    <row r="21" ht="14.25" customHeight="1"/>
+    <row r="22" ht="14.25" customHeight="1"/>
+    <row r="23" ht="14.25" customHeight="1"/>
+    <row r="24" ht="14.25" customHeight="1"/>
+    <row r="25" ht="14.25" customHeight="1"/>
+    <row r="26" ht="14.25" customHeight="1"/>
+    <row r="27" ht="14.25" customHeight="1"/>
+    <row r="28" ht="14.25" customHeight="1"/>
+    <row r="29" ht="14.25" customHeight="1"/>
+    <row r="30" ht="14.25" customHeight="1"/>
+    <row r="31" ht="14.25" customHeight="1"/>
+    <row r="32" ht="14.25" customHeight="1"/>
+    <row r="33" ht="14.25" customHeight="1"/>
+    <row r="34" ht="14.25" customHeight="1"/>
+    <row r="35" ht="14.25" customHeight="1"/>
+    <row r="36" ht="14.25" customHeight="1"/>
+    <row r="37" ht="14.25" customHeight="1"/>
+    <row r="38" ht="14.25" customHeight="1"/>
+    <row r="39" ht="14.25" customHeight="1"/>
+    <row r="40" ht="14.25" customHeight="1"/>
+    <row r="41" ht="14.25" customHeight="1"/>
+    <row r="42" ht="14.25" customHeight="1"/>
+    <row r="43" ht="14.25" customHeight="1"/>
+    <row r="44" ht="14.25" customHeight="1"/>
+    <row r="45" ht="14.25" customHeight="1"/>
+    <row r="46" ht="14.25" customHeight="1"/>
+    <row r="47" ht="14.25" customHeight="1"/>
+    <row r="48" ht="14.25" customHeight="1"/>
+    <row r="49" ht="14.25" customHeight="1"/>
+    <row r="50" ht="14.25" customHeight="1"/>
+    <row r="51" ht="14.25" customHeight="1"/>
+    <row r="52" ht="14.25" customHeight="1"/>
+    <row r="53" ht="14.25" customHeight="1"/>
+    <row r="54" ht="14.25" customHeight="1"/>
+    <row r="55" ht="14.25" customHeight="1"/>
+    <row r="56" ht="14.25" customHeight="1"/>
+    <row r="57" ht="14.25" customHeight="1"/>
+    <row r="58" ht="14.25" customHeight="1"/>
+    <row r="59" ht="14.25" customHeight="1"/>
+    <row r="60" ht="14.25" customHeight="1"/>
+    <row r="61" ht="14.25" customHeight="1"/>
+    <row r="62" ht="14.25" customHeight="1"/>
+    <row r="63" ht="14.25" customHeight="1"/>
+    <row r="64" ht="14.25" customHeight="1"/>
+    <row r="65" ht="14.25" customHeight="1"/>
+    <row r="66" ht="14.25" customHeight="1"/>
+    <row r="67" ht="14.25" customHeight="1"/>
+    <row r="68" ht="14.25" customHeight="1"/>
+    <row r="69" ht="14.25" customHeight="1"/>
+    <row r="70" ht="14.25" customHeight="1"/>
+    <row r="71" ht="14.25" customHeight="1"/>
+    <row r="72" ht="14.25" customHeight="1"/>
+    <row r="73" ht="14.25" customHeight="1"/>
+    <row r="74" ht="14.25" customHeight="1"/>
+    <row r="75" ht="14.25" customHeight="1"/>
+    <row r="76" ht="14.25" customHeight="1"/>
+    <row r="77" ht="14.25" customHeight="1"/>
+    <row r="78" ht="14.25" customHeight="1"/>
+    <row r="79" ht="14.25" customHeight="1"/>
+    <row r="80" ht="14.25" customHeight="1"/>
+    <row r="81" ht="14.25" customHeight="1"/>
+    <row r="82" ht="14.25" customHeight="1"/>
+    <row r="83" ht="14.25" customHeight="1"/>
+    <row r="84" ht="14.25" customHeight="1"/>
+    <row r="85" ht="14.25" customHeight="1"/>
+    <row r="86" ht="14.25" customHeight="1"/>
+    <row r="87" ht="14.25" customHeight="1"/>
+    <row r="88" ht="14.25" customHeight="1"/>
+    <row r="89" ht="14.25" customHeight="1"/>
+    <row r="90" ht="14.25" customHeight="1"/>
+    <row r="91" ht="14.25" customHeight="1"/>
+    <row r="92" ht="14.25" customHeight="1"/>
+    <row r="93" ht="14.25" customHeight="1"/>
+    <row r="94" ht="14.25" customHeight="1"/>
+    <row r="95" ht="14.25" customHeight="1"/>
+    <row r="96" ht="14.25" customHeight="1"/>
+    <row r="97" ht="14.25" customHeight="1"/>
+    <row r="98" ht="14.25" customHeight="1"/>
+    <row r="99" ht="14.25" customHeight="1"/>
+    <row r="100" ht="14.25" customHeight="1"/>
+    <row r="101" ht="14.25" customHeight="1"/>
+    <row r="102" ht="14.25" customHeight="1"/>
+    <row r="103" ht="14.25" customHeight="1"/>
+    <row r="104" ht="14.25" customHeight="1"/>
+    <row r="105" ht="14.25" customHeight="1"/>
+    <row r="106" ht="14.25" customHeight="1"/>
+    <row r="107" ht="14.25" customHeight="1"/>
+    <row r="108" ht="14.25" customHeight="1"/>
+    <row r="109" ht="14.25" customHeight="1"/>
+    <row r="110" ht="14.25" customHeight="1"/>
+    <row r="111" ht="14.25" customHeight="1"/>
+    <row r="112" ht="14.25" customHeight="1"/>
+    <row r="113" ht="14.25" customHeight="1"/>
+    <row r="114" ht="14.25" customHeight="1"/>
+    <row r="115" ht="14.25" customHeight="1"/>
+    <row r="116" ht="14.25" customHeight="1"/>
+    <row r="117" ht="14.25" customHeight="1"/>
+    <row r="118" ht="14.25" customHeight="1"/>
+    <row r="119" ht="14.25" customHeight="1"/>
+    <row r="120" ht="14.25" customHeight="1"/>
+    <row r="121" ht="14.25" customHeight="1"/>
+    <row r="122" ht="14.25" customHeight="1"/>
+    <row r="123" ht="14.25" customHeight="1"/>
+    <row r="124" ht="14.25" customHeight="1"/>
+    <row r="125" ht="14.25" customHeight="1"/>
+    <row r="126" ht="14.25" customHeight="1"/>
+    <row r="127" ht="14.25" customHeight="1"/>
+    <row r="128" ht="14.25" customHeight="1"/>
+    <row r="129" ht="14.25" customHeight="1"/>
+    <row r="130" ht="14.25" customHeight="1"/>
+    <row r="131" ht="14.25" customHeight="1"/>
+    <row r="132" ht="14.25" customHeight="1"/>
+    <row r="133" ht="14.25" customHeight="1"/>
+    <row r="134" ht="14.25" customHeight="1"/>
+    <row r="135" ht="14.25" customHeight="1"/>
+    <row r="136" ht="14.25" customHeight="1"/>
+    <row r="137" ht="14.25" customHeight="1"/>
+    <row r="138" ht="14.25" customHeight="1"/>
+    <row r="139" ht="14.25" customHeight="1"/>
+    <row r="140" ht="14.25" customHeight="1"/>
+    <row r="141" ht="14.25" customHeight="1"/>
+    <row r="142" ht="14.25" customHeight="1"/>
+    <row r="143" ht="14.25" customHeight="1"/>
+    <row r="144" ht="14.25" customHeight="1"/>
+    <row r="145" ht="14.25" customHeight="1"/>
+    <row r="146" ht="14.25" customHeight="1"/>
+    <row r="147" ht="14.25" customHeight="1"/>
+    <row r="148" ht="14.25" customHeight="1"/>
+    <row r="149" ht="14.25" customHeight="1"/>
+    <row r="150" ht="14.25" customHeight="1"/>
+    <row r="151" ht="14.25" customHeight="1"/>
+    <row r="152" ht="14.25" customHeight="1"/>
+    <row r="153" ht="14.25" customHeight="1"/>
+    <row r="154" ht="14.25" customHeight="1"/>
+    <row r="155" ht="14.25" customHeight="1"/>
+    <row r="156" ht="14.25" customHeight="1"/>
+    <row r="157" ht="14.25" customHeight="1"/>
+    <row r="158" ht="14.25" customHeight="1"/>
+    <row r="159" ht="14.25" customHeight="1"/>
+    <row r="160" ht="14.25" customHeight="1"/>
+    <row r="161" ht="14.25" customHeight="1"/>
+    <row r="162" ht="14.25" customHeight="1"/>
+    <row r="163" ht="14.25" customHeight="1"/>
+    <row r="164" ht="14.25" customHeight="1"/>
+    <row r="165" ht="14.25" customHeight="1"/>
+    <row r="166" ht="14.25" customHeight="1"/>
+    <row r="167" ht="14.25" customHeight="1"/>
+    <row r="168" ht="14.25" customHeight="1"/>
+    <row r="169" ht="14.25" customHeight="1"/>
+    <row r="170" ht="14.25" customHeight="1"/>
+    <row r="171" ht="14.25" customHeight="1"/>
+    <row r="172" ht="14.25" customHeight="1"/>
+    <row r="173" ht="14.25" customHeight="1"/>
+    <row r="174" ht="14.25" customHeight="1"/>
+    <row r="175" ht="14.25" customHeight="1"/>
+    <row r="176" ht="14.25" customHeight="1"/>
+    <row r="177" ht="14.25" customHeight="1"/>
+    <row r="178" ht="14.25" customHeight="1"/>
+    <row r="179" ht="14.25" customHeight="1"/>
+    <row r="180" ht="14.25" customHeight="1"/>
+    <row r="181" ht="14.25" customHeight="1"/>
+    <row r="182" ht="14.25" customHeight="1"/>
+    <row r="183" ht="14.25" customHeight="1"/>
+    <row r="184" ht="14.25" customHeight="1"/>
+    <row r="185" ht="14.25" customHeight="1"/>
+    <row r="186" ht="14.25" customHeight="1"/>
+    <row r="187" ht="14.25" customHeight="1"/>
+    <row r="188" ht="14.25" customHeight="1"/>
+    <row r="189" ht="14.25" customHeight="1"/>
+    <row r="190" ht="14.25" customHeight="1"/>
+    <row r="191" ht="14.25" customHeight="1"/>
+    <row r="192" ht="14.25" customHeight="1"/>
+    <row r="193" ht="14.25" customHeight="1"/>
+    <row r="194" ht="14.25" customHeight="1"/>
+    <row r="195" ht="14.25" customHeight="1"/>
+    <row r="196" ht="14.25" customHeight="1"/>
+    <row r="197" ht="14.25" customHeight="1"/>
+    <row r="198" ht="14.25" customHeight="1"/>
+    <row r="199" ht="14.25" customHeight="1"/>
+    <row r="200" ht="14.25" customHeight="1"/>
+    <row r="201" ht="14.25" customHeight="1"/>
+    <row r="202" ht="14.25" customHeight="1"/>
+    <row r="203" ht="14.25" customHeight="1"/>
+    <row r="204" ht="14.25" customHeight="1"/>
+    <row r="205" ht="14.25" customHeight="1"/>
+    <row r="206" ht="14.25" customHeight="1"/>
+    <row r="207" ht="14.25" customHeight="1"/>
+    <row r="208" ht="14.25" customHeight="1"/>
+    <row r="209" ht="14.25" customHeight="1"/>
+    <row r="210" ht="14.25" customHeight="1"/>
+    <row r="211" ht="14.25" customHeight="1"/>
+    <row r="212" ht="14.25" customHeight="1"/>
+    <row r="213" ht="14.25" customHeight="1"/>
+    <row r="214" ht="14.25" customHeight="1"/>
+    <row r="215" ht="14.25" customHeight="1"/>
+    <row r="216" ht="14.25" customHeight="1"/>
+    <row r="217" ht="14.25" customHeight="1"/>
+    <row r="218" ht="14.25" customHeight="1"/>
+    <row r="219" ht="14.25" customHeight="1"/>
+    <row r="220" ht="14.25" customHeight="1"/>
+    <row r="221" ht="14.25" customHeight="1"/>
+    <row r="222" ht="14.25" customHeight="1"/>
+    <row r="223" ht="14.25" customHeight="1"/>
+    <row r="224" ht="14.25" customHeight="1"/>
+    <row r="225" ht="14.25" customHeight="1"/>
+    <row r="226" ht="14.25" customHeight="1"/>
+    <row r="227" ht="14.25" customHeight="1"/>
+    <row r="228" ht="14.25" customHeight="1"/>
+    <row r="229" ht="14.25" customHeight="1"/>
+    <row r="230" ht="14.25" customHeight="1"/>
+    <row r="231" ht="14.25" customHeight="1"/>
+    <row r="232" ht="14.25" customHeight="1"/>
+    <row r="233" ht="14.25" customHeight="1"/>
+    <row r="234" ht="14.25" customHeight="1"/>
+    <row r="235" ht="14.25" customHeight="1"/>
+    <row r="236" ht="14.25" customHeight="1"/>
+    <row r="237" ht="14.25" customHeight="1"/>
+    <row r="238" ht="14.25" customHeight="1"/>
+    <row r="239" ht="14.25" customHeight="1"/>
+    <row r="240" ht="14.25" customHeight="1"/>
+    <row r="241" ht="14.25" customHeight="1"/>
+    <row r="242" ht="14.25" customHeight="1"/>
+    <row r="243" ht="14.25" customHeight="1"/>
+    <row r="244" ht="14.25" customHeight="1"/>
+    <row r="245" ht="14.25" customHeight="1"/>
+    <row r="246" ht="14.25" customHeight="1"/>
+    <row r="247" ht="14.25" customHeight="1"/>
+    <row r="248" ht="14.25" customHeight="1"/>
+    <row r="249" ht="14.25" customHeight="1"/>
+    <row r="250" ht="14.25" customHeight="1"/>
+    <row r="251" ht="14.25" customHeight="1"/>
+    <row r="252" ht="14.25" customHeight="1"/>
+    <row r="253" ht="14.25" customHeight="1"/>
+    <row r="254" ht="14.25" customHeight="1"/>
+    <row r="255" ht="14.25" customHeight="1"/>
+    <row r="256" ht="14.25" customHeight="1"/>
+    <row r="257" ht="14.25" customHeight="1"/>
+    <row r="258" ht="14.25" customHeight="1"/>
+    <row r="259" ht="14.25" customHeight="1"/>
+    <row r="260" ht="14.25" customHeight="1"/>
+    <row r="261" ht="14.25" customHeight="1"/>
+    <row r="262" ht="14.25" customHeight="1"/>
+    <row r="263" ht="14.25" customHeight="1"/>
+    <row r="264" ht="14.25" customHeight="1"/>
+    <row r="265" ht="14.25" customHeight="1"/>
+    <row r="266" ht="14.25" customHeight="1"/>
+    <row r="267" ht="14.25" customHeight="1"/>
+    <row r="268" ht="14.25" customHeight="1"/>
+    <row r="269" ht="14.25" customHeight="1"/>
+    <row r="270" ht="14.25" customHeight="1"/>
+    <row r="271" ht="14.25" customHeight="1"/>
+    <row r="272" ht="14.25" customHeight="1"/>
+    <row r="273" ht="14.25" customHeight="1"/>
+    <row r="274" ht="14.25" customHeight="1"/>
+    <row r="275" ht="14.25" customHeight="1"/>
+    <row r="276" ht="14.25" customHeight="1"/>
+    <row r="277" ht="14.25" customHeight="1"/>
+    <row r="278" ht="14.25" customHeight="1"/>
+    <row r="279" ht="14.25" customHeight="1"/>
+    <row r="280" ht="14.25" customHeight="1"/>
+    <row r="281" ht="14.25" customHeight="1"/>
+    <row r="282" ht="14.25" customHeight="1"/>
+    <row r="283" ht="14.25" customHeight="1"/>
+    <row r="284" ht="14.25" customHeight="1"/>
+    <row r="285" ht="14.25" customHeight="1"/>
+    <row r="286" ht="14.25" customHeight="1"/>
+    <row r="287" ht="14.25" customHeight="1"/>
+    <row r="288" ht="14.25" customHeight="1"/>
+    <row r="289" ht="14.25" customHeight="1"/>
+    <row r="290" ht="14.25" customHeight="1"/>
+    <row r="291" ht="14.25" customHeight="1"/>
+    <row r="292" ht="14.25" customHeight="1"/>
+    <row r="293" ht="14.25" customHeight="1"/>
+    <row r="294" ht="14.25" customHeight="1"/>
+    <row r="295" ht="14.25" customHeight="1"/>
+    <row r="296" ht="14.25" customHeight="1"/>
+    <row r="297" ht="14.25" customHeight="1"/>
+    <row r="298" ht="14.25" customHeight="1"/>
+    <row r="299" ht="14.25" customHeight="1"/>
+    <row r="300" ht="14.25" customHeight="1"/>
+    <row r="301" ht="14.25" customHeight="1"/>
+    <row r="302" ht="14.25" customHeight="1"/>
+    <row r="303" ht="14.25" customHeight="1"/>
+    <row r="304" ht="14.25" customHeight="1"/>
+    <row r="305" ht="14.25" customHeight="1"/>
+    <row r="306" ht="14.25" customHeight="1"/>
+    <row r="307" ht="14.25" customHeight="1"/>
+    <row r="308" ht="14.25" customHeight="1"/>
+    <row r="309" ht="14.25" customHeight="1"/>
+    <row r="310" ht="14.25" customHeight="1"/>
+    <row r="311" ht="14.25" customHeight="1"/>
+    <row r="312" ht="14.25" customHeight="1"/>
+    <row r="313" ht="14.25" customHeight="1"/>
+    <row r="314" ht="14.25" customHeight="1"/>
+    <row r="315" ht="14.25" customHeight="1"/>
+    <row r="316" ht="14.25" customHeight="1"/>
+    <row r="317" ht="14.25" customHeight="1"/>
+    <row r="318" ht="14.25" customHeight="1"/>
+    <row r="319" ht="14.25" customHeight="1"/>
+    <row r="320" ht="14.25" customHeight="1"/>
+    <row r="321" ht="14.25" customHeight="1"/>
+    <row r="322" ht="14.25" customHeight="1"/>
+    <row r="323" ht="14.25" customHeight="1"/>
+    <row r="324" ht="14.25" customHeight="1"/>
+    <row r="325" ht="14.25" customHeight="1"/>
+    <row r="326" ht="14.25" customHeight="1"/>
+    <row r="327" ht="14.25" customHeight="1"/>
+    <row r="328" ht="14.25" customHeight="1"/>
+    <row r="329" ht="14.25" customHeight="1"/>
+    <row r="330" ht="14.25" customHeight="1"/>
+    <row r="331" ht="14.25" customHeight="1"/>
+    <row r="332" ht="14.25" customHeight="1"/>
+    <row r="333" ht="14.25" customHeight="1"/>
+    <row r="334" ht="14.25" customHeight="1"/>
+    <row r="335" ht="14.25" customHeight="1"/>
+    <row r="336" ht="14.25" customHeight="1"/>
+    <row r="337" ht="14.25" customHeight="1"/>
+    <row r="338" ht="14.25" customHeight="1"/>
+    <row r="339" ht="14.25" customHeight="1"/>
+    <row r="340" ht="14.25" customHeight="1"/>
+    <row r="341" ht="14.25" customHeight="1"/>
+    <row r="342" ht="14.25" customHeight="1"/>
+    <row r="343" ht="14.25" customHeight="1"/>
+    <row r="344" ht="14.25" customHeight="1"/>
+    <row r="345" ht="14.25" customHeight="1"/>
+    <row r="346" ht="14.25" customHeight="1"/>
+    <row r="347" ht="14.25" customHeight="1"/>
+    <row r="348" ht="14.25" customHeight="1"/>
+    <row r="349" ht="14.25" customHeight="1"/>
+    <row r="350" ht="14.25" customHeight="1"/>
+    <row r="351" ht="14.25" customHeight="1"/>
+    <row r="352" ht="14.25" customHeight="1"/>
+    <row r="353" ht="14.25" customHeight="1"/>
+    <row r="354" ht="14.25" customHeight="1"/>
+    <row r="355" ht="14.25" customHeight="1"/>
+    <row r="356" ht="14.25" customHeight="1"/>
+    <row r="357" ht="14.25" customHeight="1"/>
+    <row r="358" ht="14.25" customHeight="1"/>
+    <row r="359" ht="14.25" customHeight="1"/>
+    <row r="360" ht="14.25" customHeight="1"/>
+    <row r="361" ht="14.25" customHeight="1"/>
+    <row r="362" ht="14.25" customHeight="1"/>
+    <row r="363" ht="14.25" customHeight="1"/>
+    <row r="364" ht="14.25" customHeight="1"/>
+    <row r="365" ht="14.25" customHeight="1"/>
+    <row r="366" ht="14.25" customHeight="1"/>
+    <row r="367" ht="14.25" customHeight="1"/>
+    <row r="368" ht="14.25" customHeight="1"/>
+    <row r="369" ht="14.25" customHeight="1"/>
+    <row r="370" ht="14.25" customHeight="1"/>
+    <row r="371" ht="14.25" customHeight="1"/>
+    <row r="372" ht="14.25" customHeight="1"/>
+    <row r="373" ht="14.25" customHeight="1"/>
+    <row r="374" ht="14.25" customHeight="1"/>
+    <row r="375" ht="14.25" customHeight="1"/>
+    <row r="376" ht="14.25" customHeight="1"/>
+    <row r="377" ht="14.25" customHeight="1"/>
+    <row r="378" ht="14.25" customHeight="1"/>
+    <row r="379" ht="14.25" customHeight="1"/>
+    <row r="380" ht="14.25" customHeight="1"/>
+    <row r="381" ht="14.25" customHeight="1"/>
+    <row r="382" ht="14.25" customHeight="1"/>
+    <row r="383" ht="14.25" customHeight="1"/>
+    <row r="384" ht="14.25" customHeight="1"/>
+    <row r="385" ht="14.25" customHeight="1"/>
+    <row r="386" ht="14.25" customHeight="1"/>
+    <row r="387" ht="14.25" customHeight="1"/>
+    <row r="388" ht="14.25" customHeight="1"/>
+    <row r="389" ht="14.25" customHeight="1"/>
+    <row r="390" ht="14.25" customHeight="1"/>
+    <row r="391" ht="14.25" customHeight="1"/>
+    <row r="392" ht="14.25" customHeight="1"/>
+    <row r="393" ht="14.25" customHeight="1"/>
+    <row r="394" ht="14.25" customHeight="1"/>
+    <row r="395" ht="14.25" customHeight="1"/>
+    <row r="396" ht="14.25" customHeight="1"/>
+    <row r="397" ht="14.25" customHeight="1"/>
+    <row r="398" ht="14.25" customHeight="1"/>
+    <row r="399" ht="14.25" customHeight="1"/>
+    <row r="400" ht="14.25" customHeight="1"/>
+    <row r="401" ht="14.25" customHeight="1"/>
+    <row r="402" ht="14.25" customHeight="1"/>
+    <row r="403" ht="14.25" customHeight="1"/>
+    <row r="404" ht="14.25" customHeight="1"/>
+    <row r="405" ht="14.25" customHeight="1"/>
+    <row r="406" ht="14.25" customHeight="1"/>
+    <row r="407" ht="14.25" customHeight="1"/>
+    <row r="408" ht="14.25" customHeight="1"/>
+    <row r="409" ht="14.25" customHeight="1"/>
+    <row r="410" ht="14.25" customHeight="1"/>
+    <row r="411" ht="14.25" customHeight="1"/>
+    <row r="412" ht="14.25" customHeight="1"/>
+    <row r="413" ht="14.25" customHeight="1"/>
+    <row r="414" ht="14.25" customHeight="1"/>
+    <row r="415" ht="14.25" customHeight="1"/>
+    <row r="416" ht="14.25" customHeight="1"/>
+    <row r="417" ht="14.25" customHeight="1"/>
+    <row r="418" ht="14.25" customHeight="1"/>
+    <row r="419" ht="14.25" customHeight="1"/>
+    <row r="420" ht="14.25" customHeight="1"/>
+    <row r="421" ht="14.25" customHeight="1"/>
+    <row r="422" ht="14.25" customHeight="1"/>
+    <row r="423" ht="14.25" customHeight="1"/>
+    <row r="424" ht="14.25" customHeight="1"/>
+    <row r="425" ht="14.25" customHeight="1"/>
+    <row r="426" ht="14.25" customHeight="1"/>
+    <row r="427" ht="14.25" customHeight="1"/>
+    <row r="428" ht="14.25" customHeight="1"/>
+    <row r="429" ht="14.25" customHeight="1"/>
+    <row r="430" ht="14.25" customHeight="1"/>
+    <row r="431" ht="14.25" customHeight="1"/>
+    <row r="432" ht="14.25" customHeight="1"/>
+    <row r="433" ht="14.25" customHeight="1"/>
+    <row r="434" ht="14.25" customHeight="1"/>
+    <row r="435" ht="14.25" customHeight="1"/>
+    <row r="436" ht="14.25" customHeight="1"/>
+    <row r="437" ht="14.25" customHeight="1"/>
+    <row r="438" ht="14.25" customHeight="1"/>
+    <row r="439" ht="14.25" customHeight="1"/>
+    <row r="440" ht="14.25" customHeight="1"/>
+    <row r="441" ht="14.25" customHeight="1"/>
+    <row r="442" ht="14.25" customHeight="1"/>
+    <row r="443" ht="14.25" customHeight="1"/>
+    <row r="444" ht="14.25" customHeight="1"/>
+    <row r="445" ht="14.25" customHeight="1"/>
+    <row r="446" ht="14.25" customHeight="1"/>
+    <row r="447" ht="14.25" customHeight="1"/>
+    <row r="448" ht="14.25" customHeight="1"/>
+    <row r="449" ht="14.25" customHeight="1"/>
+    <row r="450" ht="14.25" customHeight="1"/>
+    <row r="451" ht="14.25" customHeight="1"/>
+    <row r="452" ht="14.25" customHeight="1"/>
+    <row r="453" ht="14.25" customHeight="1"/>
+    <row r="454" ht="14.25" customHeight="1"/>
+    <row r="455" ht="14.25" customHeight="1"/>
+    <row r="456" ht="14.25" customHeight="1"/>
+    <row r="457" ht="14.25" customHeight="1"/>
+    <row r="458" ht="14.25" customHeight="1"/>
+    <row r="459" ht="14.25" customHeight="1"/>
+    <row r="460" ht="14.25" customHeight="1"/>
+    <row r="461" ht="14.25" customHeight="1"/>
+    <row r="462" ht="14.25" customHeight="1"/>
+    <row r="463" ht="14.25" customHeight="1"/>
+    <row r="464" ht="14.25" customHeight="1"/>
+    <row r="465" ht="14.25" customHeight="1"/>
+    <row r="466" ht="14.25" customHeight="1"/>
+    <row r="467" ht="14.25" customHeight="1"/>
+    <row r="468" ht="14.25" customHeight="1"/>
+    <row r="469" ht="14.25" customHeight="1"/>
+    <row r="470" ht="14.25" customHeight="1"/>
+    <row r="471" ht="14.25" customHeight="1"/>
+    <row r="472" ht="14.25" customHeight="1"/>
+    <row r="473" ht="14.25" customHeight="1"/>
+    <row r="474" ht="14.25" customHeight="1"/>
+    <row r="475" ht="14.25" customHeight="1"/>
+    <row r="476" ht="14.25" customHeight="1"/>
+    <row r="477" ht="14.25" customHeight="1"/>
+    <row r="478" ht="14.25" customHeight="1"/>
+    <row r="479" ht="14.25" customHeight="1"/>
+    <row r="480" ht="14.25" customHeight="1"/>
+    <row r="481" ht="14.25" customHeight="1"/>
+    <row r="482" ht="14.25" customHeight="1"/>
+    <row r="483" ht="14.25" customHeight="1"/>
+    <row r="484" ht="14.25" customHeight="1"/>
+    <row r="485" ht="14.25" customHeight="1"/>
+    <row r="486" ht="14.25" customHeight="1"/>
+    <row r="487" ht="14.25" customHeight="1"/>
+    <row r="488" ht="14.25" customHeight="1"/>
+    <row r="489" ht="14.25" customHeight="1"/>
+    <row r="490" ht="14.25" customHeight="1"/>
+    <row r="491" ht="14.25" customHeight="1"/>
+    <row r="492" ht="14.25" customHeight="1"/>
+    <row r="493" ht="14.25" customHeight="1"/>
+    <row r="494" ht="14.25" customHeight="1"/>
+    <row r="495" ht="14.25" customHeight="1"/>
+    <row r="496" ht="14.25" customHeight="1"/>
+    <row r="497" ht="14.25" customHeight="1"/>
+    <row r="498" ht="14.25" customHeight="1"/>
+    <row r="499" ht="14.25" customHeight="1"/>
+    <row r="500" ht="14.25" customHeight="1"/>
+    <row r="501" ht="14.25" customHeight="1"/>
+    <row r="502" ht="14.25" customHeight="1"/>
+    <row r="503" ht="14.25" customHeight="1"/>
+    <row r="504" ht="14.25" customHeight="1"/>
+    <row r="505" ht="14.25" customHeight="1"/>
+    <row r="506" ht="14.25" customHeight="1"/>
+    <row r="507" ht="14.25" customHeight="1"/>
+    <row r="508" ht="14.25" customHeight="1"/>
+    <row r="509" ht="14.25" customHeight="1"/>
+    <row r="510" ht="14.25" customHeight="1"/>
+    <row r="511" ht="14.25" customHeight="1"/>
+    <row r="512" ht="14.25" customHeight="1"/>
+    <row r="513" ht="14.25" customHeight="1"/>
+    <row r="514" ht="14.25" customHeight="1"/>
+    <row r="515" ht="14.25" customHeight="1"/>
+    <row r="516" ht="14.25" customHeight="1"/>
+    <row r="517" ht="14.25" customHeight="1"/>
+    <row r="518" ht="14.25" customHeight="1"/>
+    <row r="519" ht="14.25" customHeight="1"/>
+    <row r="520" ht="14.25" customHeight="1"/>
+    <row r="521" ht="14.25" customHeight="1"/>
+    <row r="522" ht="14.25" customHeight="1"/>
+    <row r="523" ht="14.25" customHeight="1"/>
+    <row r="524" ht="14.25" customHeight="1"/>
+    <row r="525" ht="14.25" customHeight="1"/>
+    <row r="526" ht="14.25" customHeight="1"/>
+    <row r="527" ht="14.25" customHeight="1"/>
+    <row r="528" ht="14.25" customHeight="1"/>
+    <row r="529" ht="14.25" customHeight="1"/>
+    <row r="530" ht="14.25" customHeight="1"/>
+    <row r="531" ht="14.25" customHeight="1"/>
+    <row r="532" ht="14.25" customHeight="1"/>
+    <row r="533" ht="14.25" customHeight="1"/>
+    <row r="534" ht="14.25" customHeight="1"/>
+    <row r="535" ht="14.25" customHeight="1"/>
+    <row r="536" ht="14.25" customHeight="1"/>
+    <row r="537" ht="14.25" customHeight="1"/>
+    <row r="538" ht="14.25" customHeight="1"/>
+    <row r="539" ht="14.25" customHeight="1"/>
+    <row r="540" ht="14.25" customHeight="1"/>
+    <row r="541" ht="14.25" customHeight="1"/>
+    <row r="542" ht="14.25" customHeight="1"/>
+    <row r="543" ht="14.25" customHeight="1"/>
+    <row r="544" ht="14.25" customHeight="1"/>
+    <row r="545" ht="14.25" customHeight="1"/>
+    <row r="546" ht="14.25" customHeight="1"/>
+    <row r="547" ht="14.25" customHeight="1"/>
+    <row r="548" ht="14.25" customHeight="1"/>
+    <row r="549" ht="14.25" customHeight="1"/>
+    <row r="550" ht="14.25" customHeight="1"/>
+    <row r="551" ht="14.25" customHeight="1"/>
+    <row r="552" ht="14.25" customHeight="1"/>
+    <row r="553" ht="14.25" customHeight="1"/>
+    <row r="554" ht="14.25" customHeight="1"/>
+    <row r="555" ht="14.25" customHeight="1"/>
+    <row r="556" ht="14.25" customHeight="1"/>
+    <row r="557" ht="14.25" customHeight="1"/>
+    <row r="558" ht="14.25" customHeight="1"/>
+    <row r="559" ht="14.25" customHeight="1"/>
+    <row r="560" ht="14.25" customHeight="1"/>
+    <row r="561" ht="14.25" customHeight="1"/>
+    <row r="562" ht="14.25" customHeight="1"/>
+    <row r="563" ht="14.25" customHeight="1"/>
+    <row r="564" ht="14.25" customHeight="1"/>
+    <row r="565" ht="14.25" customHeight="1"/>
+    <row r="566" ht="14.25" customHeight="1"/>
+    <row r="567" ht="14.25" customHeight="1"/>
+    <row r="568" ht="14.25" customHeight="1"/>
+    <row r="569" ht="14.25" customHeight="1"/>
+    <row r="570" ht="14.25" customHeight="1"/>
+    <row r="571" ht="14.25" customHeight="1"/>
+    <row r="572" ht="14.25" customHeight="1"/>
+    <row r="573" ht="14.25" customHeight="1"/>
+    <row r="574" ht="14.25" customHeight="1"/>
+    <row r="575" ht="14.25" customHeight="1"/>
+    <row r="576" ht="14.25" customHeight="1"/>
+    <row r="577" ht="14.25" customHeight="1"/>
+    <row r="578" ht="14.25" customHeight="1"/>
+    <row r="579" ht="14.25" customHeight="1"/>
+    <row r="580" ht="14.25" customHeight="1"/>
+    <row r="581" ht="14.25" customHeight="1"/>
+    <row r="582" ht="14.25" customHeight="1"/>
+    <row r="583" ht="14.25" customHeight="1"/>
+    <row r="584" ht="14.25" customHeight="1"/>
+    <row r="585" ht="14.25" customHeight="1"/>
+    <row r="586" ht="14.25" customHeight="1"/>
+    <row r="587" ht="14.25" customHeight="1"/>
+    <row r="588" ht="14.25" customHeight="1"/>
+    <row r="589" ht="14.25" customHeight="1"/>
+    <row r="590" ht="14.25" customHeight="1"/>
+    <row r="591" ht="14.25" customHeight="1"/>
+    <row r="592" ht="14.25" customHeight="1"/>
+    <row r="593" ht="14.25" customHeight="1"/>
+    <row r="594" ht="14.25" customHeight="1"/>
+    <row r="595" ht="14.25" customHeight="1"/>
+    <row r="596" ht="14.25" customHeight="1"/>
+    <row r="597" ht="14.25" customHeight="1"/>
+    <row r="598" ht="14.25" customHeight="1"/>
+    <row r="599" ht="14.25" customHeight="1"/>
+    <row r="600" ht="14.25" customHeight="1"/>
+    <row r="601" ht="14.25" customHeight="1"/>
+    <row r="602" ht="14.25" customHeight="1"/>
+    <row r="603" ht="14.25" customHeight="1"/>
+    <row r="604" ht="14.25" customHeight="1"/>
+    <row r="605" ht="14.25" customHeight="1"/>
+    <row r="606" ht="14.25" customHeight="1"/>
+    <row r="607" ht="14.25" customHeight="1"/>
+    <row r="608" ht="14.25" customHeight="1"/>
+    <row r="609" ht="14.25" customHeight="1"/>
+    <row r="610" ht="14.25" customHeight="1"/>
+    <row r="611" ht="14.25" customHeight="1"/>
+    <row r="612" ht="14.25" customHeight="1"/>
+    <row r="613" ht="14.25" customHeight="1"/>
+    <row r="614" ht="14.25" customHeight="1"/>
+    <row r="615" ht="14.25" customHeight="1"/>
+    <row r="616" ht="14.25" customHeight="1"/>
+    <row r="617" ht="14.25" customHeight="1"/>
+    <row r="618" ht="14.25" customHeight="1"/>
+    <row r="619" ht="14.25" customHeight="1"/>
+    <row r="620" ht="14.25" customHeight="1"/>
+    <row r="621" ht="14.25" customHeight="1"/>
+    <row r="622" ht="14.25" customHeight="1"/>
+    <row r="623" ht="14.25" customHeight="1"/>
+    <row r="624" ht="14.25" customHeight="1"/>
+    <row r="625" ht="14.25" customHeight="1"/>
+    <row r="626" ht="14.25" customHeight="1"/>
+    <row r="627" ht="14.25" customHeight="1"/>
+    <row r="628" ht="14.25" customHeight="1"/>
+    <row r="629" ht="14.25" customHeight="1"/>
+    <row r="630" ht="14.25" customHeight="1"/>
+    <row r="631" ht="14.25" customHeight="1"/>
+    <row r="632" ht="14.25" customHeight="1"/>
+    <row r="633" ht="14.25" customHeight="1"/>
+    <row r="634" ht="14.25" customHeight="1"/>
+    <row r="635" ht="14.25" customHeight="1"/>
+    <row r="636" ht="14.25" customHeight="1"/>
+    <row r="637" ht="14.25" customHeight="1"/>
+    <row r="638" ht="14.25" customHeight="1"/>
+    <row r="639" ht="14.25" customHeight="1"/>
+    <row r="640" ht="14.25" customHeight="1"/>
+    <row r="641" ht="14.25" customHeight="1"/>
+    <row r="642" ht="14.25" customHeight="1"/>
+    <row r="643" ht="14.25" customHeight="1"/>
+    <row r="644" ht="14.25" customHeight="1"/>
+    <row r="645" ht="14.25" customHeight="1"/>
+    <row r="646" ht="14.25" customHeight="1"/>
+    <row r="647" ht="14.25" customHeight="1"/>
+    <row r="648" ht="14.25" customHeight="1"/>
+    <row r="649" ht="14.25" customHeight="1"/>
+    <row r="650" ht="14.25" customHeight="1"/>
+    <row r="651" ht="14.25" customHeight="1"/>
+    <row r="652" ht="14.25" customHeight="1"/>
+    <row r="653" ht="14.25" customHeight="1"/>
+    <row r="654" ht="14.25" customHeight="1"/>
+    <row r="655" ht="14.25" customHeight="1"/>
+    <row r="656" ht="14.25" customHeight="1"/>
+    <row r="657" ht="14.25" customHeight="1"/>
+    <row r="658" ht="14.25" customHeight="1"/>
+    <row r="659" ht="14.25" customHeight="1"/>
+    <row r="660" ht="14.25" customHeight="1"/>
+    <row r="661" ht="14.25" customHeight="1"/>
+    <row r="662" ht="14.25" customHeight="1"/>
+    <row r="663" ht="14.25" customHeight="1"/>
+    <row r="664" ht="14.25" customHeight="1"/>
+    <row r="665" ht="14.25" customHeight="1"/>
+    <row r="666" ht="14.25" customHeight="1"/>
+    <row r="667" ht="14.25" customHeight="1"/>
+    <row r="668" ht="14.25" customHeight="1"/>
+    <row r="669" ht="14.25" customHeight="1"/>
+    <row r="670" ht="14.25" customHeight="1"/>
+    <row r="671" ht="14.25" customHeight="1"/>
+    <row r="672" ht="14.25" customHeight="1"/>
+    <row r="673" ht="14.25" customHeight="1"/>
+    <row r="674" ht="14.25" customHeight="1"/>
+    <row r="675" ht="14.25" customHeight="1"/>
+    <row r="676" ht="14.25" customHeight="1"/>
+    <row r="677" ht="14.25" customHeight="1"/>
+    <row r="678" ht="14.25" customHeight="1"/>
+    <row r="679" ht="14.25" customHeight="1"/>
+    <row r="680" ht="14.25" customHeight="1"/>
+    <row r="681" ht="14.25" customHeight="1"/>
+    <row r="682" ht="14.25" customHeight="1"/>
+    <row r="683" ht="14.25" customHeight="1"/>
+    <row r="684" ht="14.25" customHeight="1"/>
+    <row r="685" ht="14.25" customHeight="1"/>
+    <row r="686" ht="14.25" customHeight="1"/>
+    <row r="687" ht="14.25" customHeight="1"/>
+    <row r="688" ht="14.25" customHeight="1"/>
+    <row r="689" ht="14.25" customHeight="1"/>
+    <row r="690" ht="14.25" customHeight="1"/>
+    <row r="691" ht="14.25" customHeight="1"/>
+    <row r="692" ht="14.25" customHeight="1"/>
+    <row r="693" ht="14.25" customHeight="1"/>
+    <row r="694" ht="14.25" customHeight="1"/>
+    <row r="695" ht="14.25" customHeight="1"/>
+    <row r="696" ht="14.25" customHeight="1"/>
+    <row r="697" ht="14.25" customHeight="1"/>
+    <row r="698" ht="14.25" customHeight="1"/>
+    <row r="699" ht="14.25" customHeight="1"/>
+    <row r="700" ht="14.25" customHeight="1"/>
+    <row r="701" ht="14.25" customHeight="1"/>
+    <row r="702" ht="14.25" customHeight="1"/>
+    <row r="703" ht="14.25" customHeight="1"/>
+    <row r="704" ht="14.25" customHeight="1"/>
+    <row r="705" ht="14.25" customHeight="1"/>
+    <row r="706" ht="14.25" customHeight="1"/>
+    <row r="707" ht="14.25" customHeight="1"/>
+    <row r="708" ht="14.25" customHeight="1"/>
+    <row r="709" ht="14.25" customHeight="1"/>
+    <row r="710" ht="14.25" customHeight="1"/>
+    <row r="711" ht="14.25" customHeight="1"/>
+    <row r="712" ht="14.25" customHeight="1"/>
+    <row r="713" ht="14.25" customHeight="1"/>
+    <row r="714" ht="14.25" customHeight="1"/>
+    <row r="715" ht="14.25" customHeight="1"/>
+    <row r="716" ht="14.25" customHeight="1"/>
+    <row r="717" ht="14.25" customHeight="1"/>
+    <row r="718" ht="14.25" customHeight="1"/>
+    <row r="719" ht="14.25" customHeight="1"/>
+    <row r="720" ht="14.25" customHeight="1"/>
+    <row r="721" ht="14.25" customHeight="1"/>
+    <row r="722" ht="14.25" customHeight="1"/>
+    <row r="723" ht="14.25" customHeight="1"/>
+    <row r="724" ht="14.25" customHeight="1"/>
+    <row r="725" ht="14.25" customHeight="1"/>
+    <row r="726" ht="14.25" customHeight="1"/>
+    <row r="727" ht="14.25" customHeight="1"/>
+    <row r="728" ht="14.25" customHeight="1"/>
+    <row r="729" ht="14.25" customHeight="1"/>
+    <row r="730" ht="14.25" customHeight="1"/>
+    <row r="731" ht="14.25" customHeight="1"/>
+    <row r="732" ht="14.25" customHeight="1"/>
+    <row r="733" ht="14.25" customHeight="1"/>
+    <row r="734" ht="14.25" customHeight="1"/>
+    <row r="735" ht="14.25" customHeight="1"/>
+    <row r="736" ht="14.25" customHeight="1"/>
+    <row r="737" ht="14.25" customHeight="1"/>
+    <row r="738" ht="14.25" customHeight="1"/>
+    <row r="739" ht="14.25" customHeight="1"/>
+    <row r="740" ht="14.25" customHeight="1"/>
+    <row r="741" ht="14.25" customHeight="1"/>
+    <row r="742" ht="14.25" customHeight="1"/>
+    <row r="743" ht="14.25" customHeight="1"/>
+    <row r="744" ht="14.25" customHeight="1"/>
+    <row r="745" ht="14.25" customHeight="1"/>
+    <row r="746" ht="14.25" customHeight="1"/>
+    <row r="747" ht="14.25" customHeight="1"/>
+    <row r="748" ht="14.25" customHeight="1"/>
+    <row r="749" ht="14.25" customHeight="1"/>
+    <row r="750" ht="14.25" customHeight="1"/>
+    <row r="751" ht="14.25" customHeight="1"/>
+    <row r="752" ht="14.25" customHeight="1"/>
+    <row r="753" ht="14.25" customHeight="1"/>
+    <row r="754" ht="14.25" customHeight="1"/>
+    <row r="755" ht="14.25" customHeight="1"/>
+    <row r="756" ht="14.25" customHeight="1"/>
+    <row r="757" ht="14.25" customHeight="1"/>
+    <row r="758" ht="14.25" customHeight="1"/>
+    <row r="759" ht="14.25" customHeight="1"/>
+    <row r="760" ht="14.25" customHeight="1"/>
+    <row r="761" ht="14.25" customHeight="1"/>
+    <row r="762" ht="14.25" customHeight="1"/>
+    <row r="763" ht="14.25" customHeight="1"/>
+    <row r="764" ht="14.25" customHeight="1"/>
+    <row r="765" ht="14.25" customHeight="1"/>
+    <row r="766" ht="14.25" customHeight="1"/>
+    <row r="767" ht="14.25" customHeight="1"/>
+    <row r="768" ht="14.25" customHeight="1"/>
+    <row r="769" ht="14.25" customHeight="1"/>
+    <row r="770" ht="14.25" customHeight="1"/>
+    <row r="771" ht="14.25" customHeight="1"/>
+    <row r="772" ht="14.25" customHeight="1"/>
+    <row r="773" ht="14.25" customHeight="1"/>
+    <row r="774" ht="14.25" customHeight="1"/>
+    <row r="775" ht="14.25" customHeight="1"/>
+    <row r="776" ht="14.25" customHeight="1"/>
+    <row r="777" ht="14.25" customHeight="1"/>
+    <row r="778" ht="14.25" customHeight="1"/>
+    <row r="779" ht="14.25" customHeight="1"/>
+    <row r="780" ht="14.25" customHeight="1"/>
+    <row r="781" ht="14.25" customHeight="1"/>
+    <row r="782" ht="14.25" customHeight="1"/>
+    <row r="783" ht="14.25" customHeight="1"/>
+    <row r="784" ht="14.25" customHeight="1"/>
+    <row r="785" ht="14.25" customHeight="1"/>
+    <row r="786" ht="14.25" customHeight="1"/>
+    <row r="787" ht="14.25" customHeight="1"/>
+    <row r="788" ht="14.25" customHeight="1"/>
+    <row r="789" ht="14.25" customHeight="1"/>
+    <row r="790" ht="14.25" customHeight="1"/>
+    <row r="791" ht="14.25" customHeight="1"/>
+    <row r="792" ht="14.25" customHeight="1"/>
+    <row r="793" ht="14.25" customHeight="1"/>
+    <row r="794" ht="14.25" customHeight="1"/>
+    <row r="795" ht="14.25" customHeight="1"/>
+    <row r="796" ht="14.25" customHeight="1"/>
+    <row r="797" ht="14.25" customHeight="1"/>
+    <row r="798" ht="14.25" customHeight="1"/>
+    <row r="799" ht="14.25" customHeight="1"/>
+    <row r="800" ht="14.25" customHeight="1"/>
+    <row r="801" ht="14.25" customHeight="1"/>
+    <row r="802" ht="14.25" customHeight="1"/>
+    <row r="803" ht="14.25" customHeight="1"/>
+    <row r="804" ht="14.25" customHeight="1"/>
+    <row r="805" ht="14.25" customHeight="1"/>
+    <row r="806" ht="14.25" customHeight="1"/>
+    <row r="807" ht="14.25" customHeight="1"/>
+    <row r="808" ht="14.25" customHeight="1"/>
+    <row r="809" ht="14.25" customHeight="1"/>
+    <row r="810" ht="14.25" customHeight="1"/>
+    <row r="811" ht="14.25" customHeight="1"/>
+    <row r="812" ht="14.25" customHeight="1"/>
+    <row r="813" ht="14.25" customHeight="1"/>
+    <row r="814" ht="14.25" customHeight="1"/>
+    <row r="815" ht="14.25" customHeight="1"/>
+    <row r="816" ht="14.25" customHeight="1"/>
+    <row r="817" ht="14.25" customHeight="1"/>
+    <row r="818" ht="14.25" customHeight="1"/>
+    <row r="819" ht="14.25" customHeight="1"/>
+    <row r="820" ht="14.25" customHeight="1"/>
+    <row r="821" ht="14.25" customHeight="1"/>
+    <row r="822" ht="14.25" customHeight="1"/>
+    <row r="823" ht="14.25" customHeight="1"/>
+    <row r="824" ht="14.25" customHeight="1"/>
+    <row r="825" ht="14.25" customHeight="1"/>
+    <row r="826" ht="14.25" customHeight="1"/>
+    <row r="827" ht="14.25" customHeight="1"/>
+    <row r="828" ht="14.25" customHeight="1"/>
+    <row r="829" ht="14.25" customHeight="1"/>
+    <row r="830" ht="14.25" customHeight="1"/>
+    <row r="831" ht="14.25" customHeight="1"/>
+    <row r="832" ht="14.25" customHeight="1"/>
+    <row r="833" ht="14.25" customHeight="1"/>
+    <row r="834" ht="14.25" customHeight="1"/>
+    <row r="835" ht="14.25" customHeight="1"/>
+    <row r="836" ht="14.25" customHeight="1"/>
+    <row r="837" ht="14.25" customHeight="1"/>
+    <row r="838" ht="14.25" customHeight="1"/>
+    <row r="839" ht="14.25" customHeight="1"/>
+    <row r="840" ht="14.25" customHeight="1"/>
+    <row r="841" ht="14.25" customHeight="1"/>
+    <row r="842" ht="14.25" customHeight="1"/>
+    <row r="843" ht="14.25" customHeight="1"/>
+    <row r="844" ht="14.25" customHeight="1"/>
+    <row r="845" ht="14.25" customHeight="1"/>
+    <row r="846" ht="14.25" customHeight="1"/>
+    <row r="847" ht="14.25" customHeight="1"/>
+    <row r="848" ht="14.25" customHeight="1"/>
+    <row r="849" ht="14.25" customHeight="1"/>
+    <row r="850" ht="14.25" customHeight="1"/>
+    <row r="851" ht="14.25" customHeight="1"/>
+    <row r="852" ht="14.25" customHeight="1"/>
+    <row r="853" ht="14.25" customHeight="1"/>
+    <row r="854" ht="14.25" customHeight="1"/>
+    <row r="855" ht="14.25" customHeight="1"/>
+    <row r="856" ht="14.25" customHeight="1"/>
+    <row r="857" ht="14.25" customHeight="1"/>
+    <row r="858" ht="14.25" customHeight="1"/>
+    <row r="859" ht="14.25" customHeight="1"/>
+    <row r="860" ht="14.25" customHeight="1"/>
+    <row r="861" ht="14.25" customHeight="1"/>
+    <row r="862" ht="14.25" customHeight="1"/>
+    <row r="863" ht="14.25" customHeight="1"/>
+    <row r="864" ht="14.25" customHeight="1"/>
+    <row r="865" ht="14.25" customHeight="1"/>
+    <row r="866" ht="14.25" customHeight="1"/>
+    <row r="867" ht="14.25" customHeight="1"/>
+    <row r="868" ht="14.25" customHeight="1"/>
+    <row r="869" ht="14.25" customHeight="1"/>
+    <row r="870" ht="14.25" customHeight="1"/>
+    <row r="871" ht="14.25" customHeight="1"/>
+    <row r="872" ht="14.25" customHeight="1"/>
+    <row r="873" ht="14.25" customHeight="1"/>
+    <row r="874" ht="14.25" customHeight="1"/>
+    <row r="875" ht="14.25" customHeight="1"/>
+    <row r="876" ht="14.25" customHeight="1"/>
+    <row r="877" ht="14.25" customHeight="1"/>
+    <row r="878" ht="14.25" customHeight="1"/>
+    <row r="879" ht="14.25" customHeight="1"/>
+    <row r="880" ht="14.25" customHeight="1"/>
+    <row r="881" ht="14.25" customHeight="1"/>
+    <row r="882" ht="14.25" customHeight="1"/>
+    <row r="883" ht="14.25" customHeight="1"/>
+    <row r="884" ht="14.25" customHeight="1"/>
+    <row r="885" ht="14.25" customHeight="1"/>
+    <row r="886" ht="14.25" customHeight="1"/>
+    <row r="887" ht="14.25" customHeight="1"/>
+    <row r="888" ht="14.25" customHeight="1"/>
+    <row r="889" ht="14.25" customHeight="1"/>
+    <row r="890" ht="14.25" customHeight="1"/>
+    <row r="891" ht="14.25" customHeight="1"/>
+    <row r="892" ht="14.25" customHeight="1"/>
+    <row r="893" ht="14.25" customHeight="1"/>
+    <row r="894" ht="14.25" customHeight="1"/>
+    <row r="895" ht="14.25" customHeight="1"/>
+    <row r="896" ht="14.25" customHeight="1"/>
+    <row r="897" ht="14.25" customHeight="1"/>
+    <row r="898" ht="14.25" customHeight="1"/>
+    <row r="899" ht="14.25" customHeight="1"/>
+    <row r="900" ht="14.25" customHeight="1"/>
+    <row r="901" ht="14.25" customHeight="1"/>
+    <row r="902" ht="14.25" customHeight="1"/>
+    <row r="903" ht="14.25" customHeight="1"/>
+    <row r="904" ht="14.25" customHeight="1"/>
+    <row r="905" ht="14.25" customHeight="1"/>
+    <row r="906" ht="14.25" customHeight="1"/>
+    <row r="907" ht="14.25" customHeight="1"/>
+    <row r="908" ht="14.25" customHeight="1"/>
+    <row r="909" ht="14.25" customHeight="1"/>
+    <row r="910" ht="14.25" customHeight="1"/>
+    <row r="911" ht="14.25" customHeight="1"/>
+    <row r="912" ht="14.25" customHeight="1"/>
+    <row r="913" ht="14.25" customHeight="1"/>
+    <row r="914" ht="14.25" customHeight="1"/>
+    <row r="915" ht="14.25" customHeight="1"/>
+    <row r="916" ht="14.25" customHeight="1"/>
+    <row r="917" ht="14.25" customHeight="1"/>
+    <row r="918" ht="14.25" customHeight="1"/>
+    <row r="919" ht="14.25" customHeight="1"/>
+    <row r="920" ht="14.25" customHeight="1"/>
+    <row r="921" ht="14.25" customHeight="1"/>
+    <row r="922" ht="14.25" customHeight="1"/>
+    <row r="923" ht="14.25" customHeight="1"/>
+    <row r="924" ht="14.25" customHeight="1"/>
+    <row r="925" ht="14.25" customHeight="1"/>
+    <row r="926" ht="14.25" customHeight="1"/>
+    <row r="927" ht="14.25" customHeight="1"/>
+    <row r="928" ht="14.25" customHeight="1"/>
+    <row r="929" ht="14.25" customHeight="1"/>
+    <row r="930" ht="14.25" customHeight="1"/>
+    <row r="931" ht="14.25" customHeight="1"/>
+    <row r="932" ht="14.25" customHeight="1"/>
+    <row r="933" ht="14.25" customHeight="1"/>
+    <row r="934" ht="14.25" customHeight="1"/>
+    <row r="935" ht="14.25" customHeight="1"/>
+    <row r="936" ht="14.25" customHeight="1"/>
+    <row r="937" ht="14.25" customHeight="1"/>
+    <row r="938" ht="14.25" customHeight="1"/>
+    <row r="939" ht="14.25" customHeight="1"/>
+    <row r="940" ht="14.25" customHeight="1"/>
+    <row r="941" ht="14.25" customHeight="1"/>
+    <row r="942" ht="14.25" customHeight="1"/>
+    <row r="943" ht="14.25" customHeight="1"/>
+    <row r="944" ht="14.25" customHeight="1"/>
+    <row r="945" ht="14.25" customHeight="1"/>
+    <row r="946" ht="14.25" customHeight="1"/>
+    <row r="947" ht="14.25" customHeight="1"/>
+    <row r="948" ht="14.25" customHeight="1"/>
+    <row r="949" ht="14.25" customHeight="1"/>
+    <row r="950" ht="14.25" customHeight="1"/>
+    <row r="951" ht="14.25" customHeight="1"/>
+    <row r="952" ht="14.25" customHeight="1"/>
+    <row r="953" ht="14.25" customHeight="1"/>
+    <row r="954" ht="14.25" customHeight="1"/>
+    <row r="955" ht="14.25" customHeight="1"/>
+    <row r="956" ht="14.25" customHeight="1"/>
+    <row r="957" ht="14.25" customHeight="1"/>
+    <row r="958" ht="14.25" customHeight="1"/>
+    <row r="959" ht="14.25" customHeight="1"/>
+    <row r="960" ht="14.25" customHeight="1"/>
+    <row r="961" ht="14.25" customHeight="1"/>
+    <row r="962" ht="14.25" customHeight="1"/>
+    <row r="963" ht="14.25" customHeight="1"/>
+    <row r="964" ht="14.25" customHeight="1"/>
+    <row r="965" ht="14.25" customHeight="1"/>
+    <row r="966" ht="14.25" customHeight="1"/>
+    <row r="967" ht="14.25" customHeight="1"/>
+    <row r="968" ht="14.25" customHeight="1"/>
+    <row r="969" ht="14.25" customHeight="1"/>
+    <row r="970" ht="14.25" customHeight="1"/>
+    <row r="971" ht="14.25" customHeight="1"/>
+    <row r="972" ht="14.25" customHeight="1"/>
+    <row r="973" ht="14.25" customHeight="1"/>
+    <row r="974" ht="14.25" customHeight="1"/>
+    <row r="975" ht="14.25" customHeight="1"/>
+    <row r="976" ht="14.25" customHeight="1"/>
+    <row r="977" ht="14.25" customHeight="1"/>
+    <row r="978" ht="14.25" customHeight="1"/>
+    <row r="979" ht="14.25" customHeight="1"/>
+    <row r="980" ht="14.25" customHeight="1"/>
+    <row r="981" ht="14.25" customHeight="1"/>
+    <row r="982" ht="14.25" customHeight="1"/>
+    <row r="983" ht="14.25" customHeight="1"/>
+    <row r="984" ht="14.25" customHeight="1"/>
+    <row r="985" ht="14.25" customHeight="1"/>
+    <row r="986" ht="14.25" customHeight="1"/>
+    <row r="987" ht="14.25" customHeight="1"/>
+    <row r="988" ht="14.25" customHeight="1"/>
+    <row r="989" ht="14.25" customHeight="1"/>
+    <row r="990" ht="14.25" customHeight="1"/>
+    <row r="991" ht="14.25" customHeight="1"/>
+    <row r="992" ht="14.25" customHeight="1"/>
+    <row r="993" ht="14.25" customHeight="1"/>
+    <row r="994" ht="14.25" customHeight="1"/>
+    <row r="995" ht="14.25" customHeight="1"/>
+    <row r="996" ht="14.25" customHeight="1"/>
+    <row r="997" ht="14.25" customHeight="1"/>
+    <row r="998" ht="14.25" customHeight="1"/>
+    <row r="999" ht="14.25" customHeight="1"/>
+    <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
   <printOptions/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: (report) add full_fee and program_fee_per_meeting fields to programs and program_registration_templates tables, and update related queries
</commit_message>
<xml_diff>
--- a/db/seeds/excel/seeds.xlsx
+++ b/db/seeds/excel/seeds.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="199">
   <si>
     <t>ID</t>
   </si>
@@ -83,6 +83,15 @@
   </si>
   <si>
     <t>LECTURER FEE</t>
+  </si>
+  <si>
+    <t>FEE PER MEETING</t>
+  </si>
+  <si>
+    <t>FULL FEE</t>
+  </si>
+  <si>
+    <t>ACQUISITION RIGHTS</t>
   </si>
   <si>
     <t>01JHC3YCRXPVRG5B009VKVFHC8</t>
@@ -614,7 +623,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -628,6 +637,12 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
@@ -672,28 +687,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyAlignment="true"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2025,450 +2048,450 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>119</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>123</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>124</v>
+      <c r="F3" s="11" t="s">
+        <v>127</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>130</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>128</v>
+        <v>122</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>131</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>131</v>
+        <v>133</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>134</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>132</v>
+        <v>122</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>135</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>138</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>136</v>
+        <v>122</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>139</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>142</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>140</v>
+        <v>122</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>143</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>143</v>
+        <v>145</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>146</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>144</v>
+        <v>122</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>147</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>147</v>
+        <v>149</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>150</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>148</v>
+        <v>122</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>151</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>151</v>
+        <v>153</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>154</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>153</v>
+        <v>155</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>156</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>158</v>
+      <c r="F11" s="11" t="s">
+        <v>161</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F20" s="10" t="s">
-        <v>194</v>
+      <c r="F20" s="12" t="s">
+        <v>197</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1"/>
@@ -4514,10 +4537,12 @@
     <col customWidth="true" max="3" min="3" width="25.14"/>
     <col customWidth="true" max="4" min="4" width="8.71"/>
     <col customWidth="true" max="5" min="5" width="10"/>
-    <col customWidth="true" max="6" min="6" width="15.57"/>
-    <col customWidth="true" max="7" min="7" width="14.43"/>
-    <col customWidth="true" max="8" min="8" width="14"/>
-    <col customWidth="true" max="26" min="9" width="8.71"/>
+    <col customWidth="true" max="6" min="6" width="24.43"/>
+    <col customWidth="true" max="7" min="7" width="23.86"/>
+    <col customWidth="true" max="8" min="8" width="18"/>
+    <col customWidth="true" max="9" min="9" width="20.86"/>
+    <col customWidth="true" max="10" min="10" width="21"/>
+    <col customWidth="true" max="26" min="11" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="true">
@@ -4542,367 +4567,495 @@
       <c r="G1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="1"/>
+      <c r="H1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="true">
       <c r="A2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="4">
+        <v>24</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="6">
         <v>720000.0</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="4">
+        <v>27</v>
+      </c>
+      <c r="F2" s="6">
         <v>100000.0</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="6">
         <v>485000.0</v>
       </c>
-      <c r="H2" s="4"/>
+      <c r="H2" s="7">
+        <v>34000.0</v>
+      </c>
+      <c r="I2" s="8">
+        <v>445000.0</v>
+      </c>
+      <c r="J2" s="9">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="6">
+        <v>1070000.0</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="4">
-        <v>1070000.0</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" s="4">
+      <c r="F3" s="6">
         <v>200000.0</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="6">
         <v>725000.0</v>
       </c>
-      <c r="H3" s="4"/>
+      <c r="H3" s="7">
+        <v>49500.0</v>
+      </c>
+      <c r="I3" s="8">
+        <v>645000.0</v>
+      </c>
+      <c r="J3" s="9">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" s="4">
+        <v>31</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="6">
         <v>1420000.0</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="4">
+        <v>27</v>
+      </c>
+      <c r="F4" s="6">
         <v>300000.0</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="6">
         <v>965000.0</v>
       </c>
-      <c r="H4" s="4"/>
+      <c r="H4" s="7">
+        <v>65000.0</v>
+      </c>
+      <c r="I4" s="8">
+        <v>845000.0</v>
+      </c>
+      <c r="J4" s="9">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="5" ht="14.25" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="4">
+        <v>34</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="6">
         <v>675000.0</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F5" s="4">
+        <v>37</v>
+      </c>
+      <c r="F5" s="6">
         <v>100000.0</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="6">
         <v>440000.0</v>
       </c>
-      <c r="H5" s="4"/>
+      <c r="H5" s="7">
+        <v>17000.0</v>
+      </c>
+      <c r="I5" s="8">
+        <v>400000.0</v>
+      </c>
+      <c r="J5" s="9">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="6" ht="14.25" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="6">
+        <v>475000.0</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="4">
-        <v>475000.0</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="4">
+      <c r="F6" s="6">
         <v>100000.0</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="6">
         <v>240000.0</v>
       </c>
-      <c r="H6" s="4"/>
+      <c r="H6" s="7">
+        <v>8500.0</v>
+      </c>
+      <c r="I6" s="8">
+        <v>200000.0</v>
+      </c>
+      <c r="J6" s="9">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="7" ht="14.25" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="4">
+        <v>41</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="6">
         <v>595000.0</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="4">
+        <v>44</v>
+      </c>
+      <c r="F7" s="6">
         <v>100000.0</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="6">
         <v>360000.0</v>
       </c>
-      <c r="H7" s="5"/>
+      <c r="H7" s="7">
+        <v>35500.0</v>
+      </c>
+      <c r="I7" s="8">
+        <v>320000.0</v>
+      </c>
+      <c r="J7" s="9">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="8" ht="14.25" customHeight="true">
       <c r="A8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="6">
+        <v>885000.0</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="4">
-        <v>885000.0</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" s="4">
+      <c r="F8" s="6">
         <v>200000.0</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="6">
         <v>540000.0</v>
       </c>
-      <c r="H8" s="5"/>
+      <c r="H8" s="7">
+        <v>51000.0</v>
+      </c>
+      <c r="I8" s="8">
+        <v>460000.0</v>
+      </c>
+      <c r="J8" s="9">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="true">
       <c r="A9" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="4">
+        <v>48</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="6">
         <v>1170000.0</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" s="4">
+        <v>44</v>
+      </c>
+      <c r="F9" s="6">
         <v>300000.0</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="6">
         <v>715000.0</v>
       </c>
-      <c r="H9" s="5"/>
+      <c r="H9" s="7">
+        <v>66000.0</v>
+      </c>
+      <c r="I9" s="8">
+        <v>595000.0</v>
+      </c>
+      <c r="J9" s="9">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="10" ht="14.25" customHeight="true">
       <c r="A10" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D10" s="4">
+        <v>51</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="6">
         <v>450000.0</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" s="4">
+        <v>44</v>
+      </c>
+      <c r="F10" s="6">
         <v>100000.0</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="6">
         <v>215000.0</v>
       </c>
-      <c r="H10" s="5"/>
+      <c r="H10" s="7">
+        <v>17500.0</v>
+      </c>
+      <c r="I10" s="8">
+        <v>175000.0</v>
+      </c>
+      <c r="J10" s="9">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="11" ht="14.25" customHeight="true">
       <c r="A11" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="4">
+        <v>54</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="6">
         <v>720000.0</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F11" s="4">
+        <v>57</v>
+      </c>
+      <c r="F11" s="6">
         <v>100000.0</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="6">
         <v>485000.0</v>
       </c>
-      <c r="H11" s="5"/>
+      <c r="H11" s="7">
+        <v>49000.0</v>
+      </c>
+      <c r="I11" s="8">
+        <v>445000.0</v>
+      </c>
+      <c r="J11" s="9">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="true">
       <c r="A12" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="6">
+        <v>970000.0</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D12" s="4">
-        <v>970000.0</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F12" s="4">
+      <c r="F12" s="6">
         <v>200000.0</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="6">
         <v>625000.0</v>
       </c>
-      <c r="H12" s="5"/>
+      <c r="H12" s="7">
+        <v>60500.0</v>
+      </c>
+      <c r="I12" s="8">
+        <v>545000.0</v>
+      </c>
+      <c r="J12" s="9">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="13" ht="14.25" customHeight="true">
       <c r="A13" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="4">
+        <v>61</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="6">
         <v>1220000.0</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F13" s="4">
+        <v>57</v>
+      </c>
+      <c r="F13" s="6">
         <v>300000.0</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="6">
         <v>765000.0</v>
       </c>
-      <c r="H13" s="5"/>
+      <c r="H13" s="7">
+        <v>71500.0</v>
+      </c>
+      <c r="I13" s="8">
+        <v>645000.0</v>
+      </c>
+      <c r="J13" s="9">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="14" ht="14.25" customHeight="true">
       <c r="A14" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D14" s="4">
+        <v>64</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="6">
         <v>600000.0</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="4">
+        <v>57</v>
+      </c>
+      <c r="F14" s="6">
         <v>100000.0</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="6">
         <v>365000.0</v>
       </c>
-      <c r="H14" s="5"/>
+      <c r="H14" s="7">
+        <v>36000.0</v>
+      </c>
+      <c r="I14" s="8">
+        <v>325000.0</v>
+      </c>
+      <c r="J14" s="9">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="true">
       <c r="A15" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D15" s="4">
+        <v>67</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="6">
         <v>550000.0</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F15" s="4">
+        <v>70</v>
+      </c>
+      <c r="F15" s="6">
         <v>100000.0</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="6">
         <v>315000.0</v>
       </c>
-      <c r="H15" s="5"/>
+      <c r="H15" s="7">
+        <v>18000.0</v>
+      </c>
+      <c r="I15" s="8">
+        <v>275000.0</v>
+      </c>
+      <c r="J15" s="9">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="16" ht="14.25" customHeight="true">
       <c r="A16" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="6">
+        <v>620000.0</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="4">
-        <v>620000.0</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F16" s="4">
+      <c r="F16" s="6">
         <v>100000.0</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="6">
         <v>385000.0</v>
       </c>
-      <c r="H16" s="5"/>
+      <c r="H16" s="7">
+        <v>23000.0</v>
+      </c>
+      <c r="I16" s="8">
+        <v>345000.0</v>
+      </c>
+      <c r="J16" s="9">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="17" ht="14.25" customHeight="true"/>
     <row r="18" ht="14.25" customHeight="true"/>
@@ -5919,18 +6072,18 @@
       <c r="D1" s="1"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="B2" s="6" t="s">
-        <v>71</v>
+      <c r="B2" s="9" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="B3" s="6" t="s">
-        <v>72</v>
+      <c r="B3" s="9" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="B4" s="6" t="s">
-        <v>73</v>
+      <c r="B4" s="9" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -6953,50 +7106,50 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>74</v>
+      <c r="B1" s="4" t="s">
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>81</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>84</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>87</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -8022,34 +8175,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -9073,49 +9226,49 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -10139,7 +10292,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -10149,35 +10302,35 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -11206,10 +11359,10 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
feat: (seeds) update seeds.xlsx with new data for improved testing
</commit_message>
<xml_diff>
--- a/db/seeds/excel/seeds.xlsx
+++ b/db/seeds/excel/seeds.xlsx
@@ -966,14 +966,14 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="true"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="29.71"/>
-    <col customWidth="1" min="2" max="2" width="13.86"/>
-    <col customWidth="1" min="3" max="26" width="8.71"/>
+    <col customWidth="true" max="1" min="1" width="29.71"/>
+    <col customWidth="true" max="2" min="2" width="13.86"/>
+    <col customWidth="true" max="26" min="3" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
+    <row r="1" ht="14.25" customHeight="true">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -981,7 +981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1">
+    <row r="2" ht="14.25" customHeight="true">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -989,7 +989,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1">
+    <row r="3" ht="14.25" customHeight="true">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -997,7 +997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1">
+    <row r="4" ht="14.25" customHeight="true">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="14.25" customHeight="1">
+    <row r="5" ht="14.25" customHeight="true">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" ht="14.25" customHeight="1">
+    <row r="6" ht="14.25" customHeight="true">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -1021,1003 +1021,1003 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="14.25" customHeight="1"/>
-    <row r="8" ht="14.25" customHeight="1"/>
-    <row r="9" ht="14.25" customHeight="1"/>
-    <row r="10" ht="14.25" customHeight="1"/>
-    <row r="11" ht="14.25" customHeight="1"/>
-    <row r="12" ht="14.25" customHeight="1"/>
-    <row r="13" ht="14.25" customHeight="1"/>
-    <row r="14" ht="14.25" customHeight="1"/>
-    <row r="15" ht="14.25" customHeight="1"/>
-    <row r="16" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
-    <row r="65" ht="14.25" customHeight="1"/>
-    <row r="66" ht="14.25" customHeight="1"/>
-    <row r="67" ht="14.25" customHeight="1"/>
-    <row r="68" ht="14.25" customHeight="1"/>
-    <row r="69" ht="14.25" customHeight="1"/>
-    <row r="70" ht="14.25" customHeight="1"/>
-    <row r="71" ht="14.25" customHeight="1"/>
-    <row r="72" ht="14.25" customHeight="1"/>
-    <row r="73" ht="14.25" customHeight="1"/>
-    <row r="74" ht="14.25" customHeight="1"/>
-    <row r="75" ht="14.25" customHeight="1"/>
-    <row r="76" ht="14.25" customHeight="1"/>
-    <row r="77" ht="14.25" customHeight="1"/>
-    <row r="78" ht="14.25" customHeight="1"/>
-    <row r="79" ht="14.25" customHeight="1"/>
-    <row r="80" ht="14.25" customHeight="1"/>
-    <row r="81" ht="14.25" customHeight="1"/>
-    <row r="82" ht="14.25" customHeight="1"/>
-    <row r="83" ht="14.25" customHeight="1"/>
-    <row r="84" ht="14.25" customHeight="1"/>
-    <row r="85" ht="14.25" customHeight="1"/>
-    <row r="86" ht="14.25" customHeight="1"/>
-    <row r="87" ht="14.25" customHeight="1"/>
-    <row r="88" ht="14.25" customHeight="1"/>
-    <row r="89" ht="14.25" customHeight="1"/>
-    <row r="90" ht="14.25" customHeight="1"/>
-    <row r="91" ht="14.25" customHeight="1"/>
-    <row r="92" ht="14.25" customHeight="1"/>
-    <row r="93" ht="14.25" customHeight="1"/>
-    <row r="94" ht="14.25" customHeight="1"/>
-    <row r="95" ht="14.25" customHeight="1"/>
-    <row r="96" ht="14.25" customHeight="1"/>
-    <row r="97" ht="14.25" customHeight="1"/>
-    <row r="98" ht="14.25" customHeight="1"/>
-    <row r="99" ht="14.25" customHeight="1"/>
-    <row r="100" ht="14.25" customHeight="1"/>
-    <row r="101" ht="14.25" customHeight="1"/>
-    <row r="102" ht="14.25" customHeight="1"/>
-    <row r="103" ht="14.25" customHeight="1"/>
-    <row r="104" ht="14.25" customHeight="1"/>
-    <row r="105" ht="14.25" customHeight="1"/>
-    <row r="106" ht="14.25" customHeight="1"/>
-    <row r="107" ht="14.25" customHeight="1"/>
-    <row r="108" ht="14.25" customHeight="1"/>
-    <row r="109" ht="14.25" customHeight="1"/>
-    <row r="110" ht="14.25" customHeight="1"/>
-    <row r="111" ht="14.25" customHeight="1"/>
-    <row r="112" ht="14.25" customHeight="1"/>
-    <row r="113" ht="14.25" customHeight="1"/>
-    <row r="114" ht="14.25" customHeight="1"/>
-    <row r="115" ht="14.25" customHeight="1"/>
-    <row r="116" ht="14.25" customHeight="1"/>
-    <row r="117" ht="14.25" customHeight="1"/>
-    <row r="118" ht="14.25" customHeight="1"/>
-    <row r="119" ht="14.25" customHeight="1"/>
-    <row r="120" ht="14.25" customHeight="1"/>
-    <row r="121" ht="14.25" customHeight="1"/>
-    <row r="122" ht="14.25" customHeight="1"/>
-    <row r="123" ht="14.25" customHeight="1"/>
-    <row r="124" ht="14.25" customHeight="1"/>
-    <row r="125" ht="14.25" customHeight="1"/>
-    <row r="126" ht="14.25" customHeight="1"/>
-    <row r="127" ht="14.25" customHeight="1"/>
-    <row r="128" ht="14.25" customHeight="1"/>
-    <row r="129" ht="14.25" customHeight="1"/>
-    <row r="130" ht="14.25" customHeight="1"/>
-    <row r="131" ht="14.25" customHeight="1"/>
-    <row r="132" ht="14.25" customHeight="1"/>
-    <row r="133" ht="14.25" customHeight="1"/>
-    <row r="134" ht="14.25" customHeight="1"/>
-    <row r="135" ht="14.25" customHeight="1"/>
-    <row r="136" ht="14.25" customHeight="1"/>
-    <row r="137" ht="14.25" customHeight="1"/>
-    <row r="138" ht="14.25" customHeight="1"/>
-    <row r="139" ht="14.25" customHeight="1"/>
-    <row r="140" ht="14.25" customHeight="1"/>
-    <row r="141" ht="14.25" customHeight="1"/>
-    <row r="142" ht="14.25" customHeight="1"/>
-    <row r="143" ht="14.25" customHeight="1"/>
-    <row r="144" ht="14.25" customHeight="1"/>
-    <row r="145" ht="14.25" customHeight="1"/>
-    <row r="146" ht="14.25" customHeight="1"/>
-    <row r="147" ht="14.25" customHeight="1"/>
-    <row r="148" ht="14.25" customHeight="1"/>
-    <row r="149" ht="14.25" customHeight="1"/>
-    <row r="150" ht="14.25" customHeight="1"/>
-    <row r="151" ht="14.25" customHeight="1"/>
-    <row r="152" ht="14.25" customHeight="1"/>
-    <row r="153" ht="14.25" customHeight="1"/>
-    <row r="154" ht="14.25" customHeight="1"/>
-    <row r="155" ht="14.25" customHeight="1"/>
-    <row r="156" ht="14.25" customHeight="1"/>
-    <row r="157" ht="14.25" customHeight="1"/>
-    <row r="158" ht="14.25" customHeight="1"/>
-    <row r="159" ht="14.25" customHeight="1"/>
-    <row r="160" ht="14.25" customHeight="1"/>
-    <row r="161" ht="14.25" customHeight="1"/>
-    <row r="162" ht="14.25" customHeight="1"/>
-    <row r="163" ht="14.25" customHeight="1"/>
-    <row r="164" ht="14.25" customHeight="1"/>
-    <row r="165" ht="14.25" customHeight="1"/>
-    <row r="166" ht="14.25" customHeight="1"/>
-    <row r="167" ht="14.25" customHeight="1"/>
-    <row r="168" ht="14.25" customHeight="1"/>
-    <row r="169" ht="14.25" customHeight="1"/>
-    <row r="170" ht="14.25" customHeight="1"/>
-    <row r="171" ht="14.25" customHeight="1"/>
-    <row r="172" ht="14.25" customHeight="1"/>
-    <row r="173" ht="14.25" customHeight="1"/>
-    <row r="174" ht="14.25" customHeight="1"/>
-    <row r="175" ht="14.25" customHeight="1"/>
-    <row r="176" ht="14.25" customHeight="1"/>
-    <row r="177" ht="14.25" customHeight="1"/>
-    <row r="178" ht="14.25" customHeight="1"/>
-    <row r="179" ht="14.25" customHeight="1"/>
-    <row r="180" ht="14.25" customHeight="1"/>
-    <row r="181" ht="14.25" customHeight="1"/>
-    <row r="182" ht="14.25" customHeight="1"/>
-    <row r="183" ht="14.25" customHeight="1"/>
-    <row r="184" ht="14.25" customHeight="1"/>
-    <row r="185" ht="14.25" customHeight="1"/>
-    <row r="186" ht="14.25" customHeight="1"/>
-    <row r="187" ht="14.25" customHeight="1"/>
-    <row r="188" ht="14.25" customHeight="1"/>
-    <row r="189" ht="14.25" customHeight="1"/>
-    <row r="190" ht="14.25" customHeight="1"/>
-    <row r="191" ht="14.25" customHeight="1"/>
-    <row r="192" ht="14.25" customHeight="1"/>
-    <row r="193" ht="14.25" customHeight="1"/>
-    <row r="194" ht="14.25" customHeight="1"/>
-    <row r="195" ht="14.25" customHeight="1"/>
-    <row r="196" ht="14.25" customHeight="1"/>
-    <row r="197" ht="14.25" customHeight="1"/>
-    <row r="198" ht="14.25" customHeight="1"/>
-    <row r="199" ht="14.25" customHeight="1"/>
-    <row r="200" ht="14.25" customHeight="1"/>
-    <row r="201" ht="14.25" customHeight="1"/>
-    <row r="202" ht="14.25" customHeight="1"/>
-    <row r="203" ht="14.25" customHeight="1"/>
-    <row r="204" ht="14.25" customHeight="1"/>
-    <row r="205" ht="14.25" customHeight="1"/>
-    <row r="206" ht="14.25" customHeight="1"/>
-    <row r="207" ht="14.25" customHeight="1"/>
-    <row r="208" ht="14.25" customHeight="1"/>
-    <row r="209" ht="14.25" customHeight="1"/>
-    <row r="210" ht="14.25" customHeight="1"/>
-    <row r="211" ht="14.25" customHeight="1"/>
-    <row r="212" ht="14.25" customHeight="1"/>
-    <row r="213" ht="14.25" customHeight="1"/>
-    <row r="214" ht="14.25" customHeight="1"/>
-    <row r="215" ht="14.25" customHeight="1"/>
-    <row r="216" ht="14.25" customHeight="1"/>
-    <row r="217" ht="14.25" customHeight="1"/>
-    <row r="218" ht="14.25" customHeight="1"/>
-    <row r="219" ht="14.25" customHeight="1"/>
-    <row r="220" ht="14.25" customHeight="1"/>
-    <row r="221" ht="14.25" customHeight="1"/>
-    <row r="222" ht="14.25" customHeight="1"/>
-    <row r="223" ht="14.25" customHeight="1"/>
-    <row r="224" ht="14.25" customHeight="1"/>
-    <row r="225" ht="14.25" customHeight="1"/>
-    <row r="226" ht="14.25" customHeight="1"/>
-    <row r="227" ht="14.25" customHeight="1"/>
-    <row r="228" ht="14.25" customHeight="1"/>
-    <row r="229" ht="14.25" customHeight="1"/>
-    <row r="230" ht="14.25" customHeight="1"/>
-    <row r="231" ht="14.25" customHeight="1"/>
-    <row r="232" ht="14.25" customHeight="1"/>
-    <row r="233" ht="14.25" customHeight="1"/>
-    <row r="234" ht="14.25" customHeight="1"/>
-    <row r="235" ht="14.25" customHeight="1"/>
-    <row r="236" ht="14.25" customHeight="1"/>
-    <row r="237" ht="14.25" customHeight="1"/>
-    <row r="238" ht="14.25" customHeight="1"/>
-    <row r="239" ht="14.25" customHeight="1"/>
-    <row r="240" ht="14.25" customHeight="1"/>
-    <row r="241" ht="14.25" customHeight="1"/>
-    <row r="242" ht="14.25" customHeight="1"/>
-    <row r="243" ht="14.25" customHeight="1"/>
-    <row r="244" ht="14.25" customHeight="1"/>
-    <row r="245" ht="14.25" customHeight="1"/>
-    <row r="246" ht="14.25" customHeight="1"/>
-    <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
-    <row r="249" ht="14.25" customHeight="1"/>
-    <row r="250" ht="14.25" customHeight="1"/>
-    <row r="251" ht="14.25" customHeight="1"/>
-    <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1"/>
-    <row r="254" ht="14.25" customHeight="1"/>
-    <row r="255" ht="14.25" customHeight="1"/>
-    <row r="256" ht="14.25" customHeight="1"/>
-    <row r="257" ht="14.25" customHeight="1"/>
-    <row r="258" ht="14.25" customHeight="1"/>
-    <row r="259" ht="14.25" customHeight="1"/>
-    <row r="260" ht="14.25" customHeight="1"/>
-    <row r="261" ht="14.25" customHeight="1"/>
-    <row r="262" ht="14.25" customHeight="1"/>
-    <row r="263" ht="14.25" customHeight="1"/>
-    <row r="264" ht="14.25" customHeight="1"/>
-    <row r="265" ht="14.25" customHeight="1"/>
-    <row r="266" ht="14.25" customHeight="1"/>
-    <row r="267" ht="14.25" customHeight="1"/>
-    <row r="268" ht="14.25" customHeight="1"/>
-    <row r="269" ht="14.25" customHeight="1"/>
-    <row r="270" ht="14.25" customHeight="1"/>
-    <row r="271" ht="14.25" customHeight="1"/>
-    <row r="272" ht="14.25" customHeight="1"/>
-    <row r="273" ht="14.25" customHeight="1"/>
-    <row r="274" ht="14.25" customHeight="1"/>
-    <row r="275" ht="14.25" customHeight="1"/>
-    <row r="276" ht="14.25" customHeight="1"/>
-    <row r="277" ht="14.25" customHeight="1"/>
-    <row r="278" ht="14.25" customHeight="1"/>
-    <row r="279" ht="14.25" customHeight="1"/>
-    <row r="280" ht="14.25" customHeight="1"/>
-    <row r="281" ht="14.25" customHeight="1"/>
-    <row r="282" ht="14.25" customHeight="1"/>
-    <row r="283" ht="14.25" customHeight="1"/>
-    <row r="284" ht="14.25" customHeight="1"/>
-    <row r="285" ht="14.25" customHeight="1"/>
-    <row r="286" ht="14.25" customHeight="1"/>
-    <row r="287" ht="14.25" customHeight="1"/>
-    <row r="288" ht="14.25" customHeight="1"/>
-    <row r="289" ht="14.25" customHeight="1"/>
-    <row r="290" ht="14.25" customHeight="1"/>
-    <row r="291" ht="14.25" customHeight="1"/>
-    <row r="292" ht="14.25" customHeight="1"/>
-    <row r="293" ht="14.25" customHeight="1"/>
-    <row r="294" ht="14.25" customHeight="1"/>
-    <row r="295" ht="14.25" customHeight="1"/>
-    <row r="296" ht="14.25" customHeight="1"/>
-    <row r="297" ht="14.25" customHeight="1"/>
-    <row r="298" ht="14.25" customHeight="1"/>
-    <row r="299" ht="14.25" customHeight="1"/>
-    <row r="300" ht="14.25" customHeight="1"/>
-    <row r="301" ht="14.25" customHeight="1"/>
-    <row r="302" ht="14.25" customHeight="1"/>
-    <row r="303" ht="14.25" customHeight="1"/>
-    <row r="304" ht="14.25" customHeight="1"/>
-    <row r="305" ht="14.25" customHeight="1"/>
-    <row r="306" ht="14.25" customHeight="1"/>
-    <row r="307" ht="14.25" customHeight="1"/>
-    <row r="308" ht="14.25" customHeight="1"/>
-    <row r="309" ht="14.25" customHeight="1"/>
-    <row r="310" ht="14.25" customHeight="1"/>
-    <row r="311" ht="14.25" customHeight="1"/>
-    <row r="312" ht="14.25" customHeight="1"/>
-    <row r="313" ht="14.25" customHeight="1"/>
-    <row r="314" ht="14.25" customHeight="1"/>
-    <row r="315" ht="14.25" customHeight="1"/>
-    <row r="316" ht="14.25" customHeight="1"/>
-    <row r="317" ht="14.25" customHeight="1"/>
-    <row r="318" ht="14.25" customHeight="1"/>
-    <row r="319" ht="14.25" customHeight="1"/>
-    <row r="320" ht="14.25" customHeight="1"/>
-    <row r="321" ht="14.25" customHeight="1"/>
-    <row r="322" ht="14.25" customHeight="1"/>
-    <row r="323" ht="14.25" customHeight="1"/>
-    <row r="324" ht="14.25" customHeight="1"/>
-    <row r="325" ht="14.25" customHeight="1"/>
-    <row r="326" ht="14.25" customHeight="1"/>
-    <row r="327" ht="14.25" customHeight="1"/>
-    <row r="328" ht="14.25" customHeight="1"/>
-    <row r="329" ht="14.25" customHeight="1"/>
-    <row r="330" ht="14.25" customHeight="1"/>
-    <row r="331" ht="14.25" customHeight="1"/>
-    <row r="332" ht="14.25" customHeight="1"/>
-    <row r="333" ht="14.25" customHeight="1"/>
-    <row r="334" ht="14.25" customHeight="1"/>
-    <row r="335" ht="14.25" customHeight="1"/>
-    <row r="336" ht="14.25" customHeight="1"/>
-    <row r="337" ht="14.25" customHeight="1"/>
-    <row r="338" ht="14.25" customHeight="1"/>
-    <row r="339" ht="14.25" customHeight="1"/>
-    <row r="340" ht="14.25" customHeight="1"/>
-    <row r="341" ht="14.25" customHeight="1"/>
-    <row r="342" ht="14.25" customHeight="1"/>
-    <row r="343" ht="14.25" customHeight="1"/>
-    <row r="344" ht="14.25" customHeight="1"/>
-    <row r="345" ht="14.25" customHeight="1"/>
-    <row r="346" ht="14.25" customHeight="1"/>
-    <row r="347" ht="14.25" customHeight="1"/>
-    <row r="348" ht="14.25" customHeight="1"/>
-    <row r="349" ht="14.25" customHeight="1"/>
-    <row r="350" ht="14.25" customHeight="1"/>
-    <row r="351" ht="14.25" customHeight="1"/>
-    <row r="352" ht="14.25" customHeight="1"/>
-    <row r="353" ht="14.25" customHeight="1"/>
-    <row r="354" ht="14.25" customHeight="1"/>
-    <row r="355" ht="14.25" customHeight="1"/>
-    <row r="356" ht="14.25" customHeight="1"/>
-    <row r="357" ht="14.25" customHeight="1"/>
-    <row r="358" ht="14.25" customHeight="1"/>
-    <row r="359" ht="14.25" customHeight="1"/>
-    <row r="360" ht="14.25" customHeight="1"/>
-    <row r="361" ht="14.25" customHeight="1"/>
-    <row r="362" ht="14.25" customHeight="1"/>
-    <row r="363" ht="14.25" customHeight="1"/>
-    <row r="364" ht="14.25" customHeight="1"/>
-    <row r="365" ht="14.25" customHeight="1"/>
-    <row r="366" ht="14.25" customHeight="1"/>
-    <row r="367" ht="14.25" customHeight="1"/>
-    <row r="368" ht="14.25" customHeight="1"/>
-    <row r="369" ht="14.25" customHeight="1"/>
-    <row r="370" ht="14.25" customHeight="1"/>
-    <row r="371" ht="14.25" customHeight="1"/>
-    <row r="372" ht="14.25" customHeight="1"/>
-    <row r="373" ht="14.25" customHeight="1"/>
-    <row r="374" ht="14.25" customHeight="1"/>
-    <row r="375" ht="14.25" customHeight="1"/>
-    <row r="376" ht="14.25" customHeight="1"/>
-    <row r="377" ht="14.25" customHeight="1"/>
-    <row r="378" ht="14.25" customHeight="1"/>
-    <row r="379" ht="14.25" customHeight="1"/>
-    <row r="380" ht="14.25" customHeight="1"/>
-    <row r="381" ht="14.25" customHeight="1"/>
-    <row r="382" ht="14.25" customHeight="1"/>
-    <row r="383" ht="14.25" customHeight="1"/>
-    <row r="384" ht="14.25" customHeight="1"/>
-    <row r="385" ht="14.25" customHeight="1"/>
-    <row r="386" ht="14.25" customHeight="1"/>
-    <row r="387" ht="14.25" customHeight="1"/>
-    <row r="388" ht="14.25" customHeight="1"/>
-    <row r="389" ht="14.25" customHeight="1"/>
-    <row r="390" ht="14.25" customHeight="1"/>
-    <row r="391" ht="14.25" customHeight="1"/>
-    <row r="392" ht="14.25" customHeight="1"/>
-    <row r="393" ht="14.25" customHeight="1"/>
-    <row r="394" ht="14.25" customHeight="1"/>
-    <row r="395" ht="14.25" customHeight="1"/>
-    <row r="396" ht="14.25" customHeight="1"/>
-    <row r="397" ht="14.25" customHeight="1"/>
-    <row r="398" ht="14.25" customHeight="1"/>
-    <row r="399" ht="14.25" customHeight="1"/>
-    <row r="400" ht="14.25" customHeight="1"/>
-    <row r="401" ht="14.25" customHeight="1"/>
-    <row r="402" ht="14.25" customHeight="1"/>
-    <row r="403" ht="14.25" customHeight="1"/>
-    <row r="404" ht="14.25" customHeight="1"/>
-    <row r="405" ht="14.25" customHeight="1"/>
-    <row r="406" ht="14.25" customHeight="1"/>
-    <row r="407" ht="14.25" customHeight="1"/>
-    <row r="408" ht="14.25" customHeight="1"/>
-    <row r="409" ht="14.25" customHeight="1"/>
-    <row r="410" ht="14.25" customHeight="1"/>
-    <row r="411" ht="14.25" customHeight="1"/>
-    <row r="412" ht="14.25" customHeight="1"/>
-    <row r="413" ht="14.25" customHeight="1"/>
-    <row r="414" ht="14.25" customHeight="1"/>
-    <row r="415" ht="14.25" customHeight="1"/>
-    <row r="416" ht="14.25" customHeight="1"/>
-    <row r="417" ht="14.25" customHeight="1"/>
-    <row r="418" ht="14.25" customHeight="1"/>
-    <row r="419" ht="14.25" customHeight="1"/>
-    <row r="420" ht="14.25" customHeight="1"/>
-    <row r="421" ht="14.25" customHeight="1"/>
-    <row r="422" ht="14.25" customHeight="1"/>
-    <row r="423" ht="14.25" customHeight="1"/>
-    <row r="424" ht="14.25" customHeight="1"/>
-    <row r="425" ht="14.25" customHeight="1"/>
-    <row r="426" ht="14.25" customHeight="1"/>
-    <row r="427" ht="14.25" customHeight="1"/>
-    <row r="428" ht="14.25" customHeight="1"/>
-    <row r="429" ht="14.25" customHeight="1"/>
-    <row r="430" ht="14.25" customHeight="1"/>
-    <row r="431" ht="14.25" customHeight="1"/>
-    <row r="432" ht="14.25" customHeight="1"/>
-    <row r="433" ht="14.25" customHeight="1"/>
-    <row r="434" ht="14.25" customHeight="1"/>
-    <row r="435" ht="14.25" customHeight="1"/>
-    <row r="436" ht="14.25" customHeight="1"/>
-    <row r="437" ht="14.25" customHeight="1"/>
-    <row r="438" ht="14.25" customHeight="1"/>
-    <row r="439" ht="14.25" customHeight="1"/>
-    <row r="440" ht="14.25" customHeight="1"/>
-    <row r="441" ht="14.25" customHeight="1"/>
-    <row r="442" ht="14.25" customHeight="1"/>
-    <row r="443" ht="14.25" customHeight="1"/>
-    <row r="444" ht="14.25" customHeight="1"/>
-    <row r="445" ht="14.25" customHeight="1"/>
-    <row r="446" ht="14.25" customHeight="1"/>
-    <row r="447" ht="14.25" customHeight="1"/>
-    <row r="448" ht="14.25" customHeight="1"/>
-    <row r="449" ht="14.25" customHeight="1"/>
-    <row r="450" ht="14.25" customHeight="1"/>
-    <row r="451" ht="14.25" customHeight="1"/>
-    <row r="452" ht="14.25" customHeight="1"/>
-    <row r="453" ht="14.25" customHeight="1"/>
-    <row r="454" ht="14.25" customHeight="1"/>
-    <row r="455" ht="14.25" customHeight="1"/>
-    <row r="456" ht="14.25" customHeight="1"/>
-    <row r="457" ht="14.25" customHeight="1"/>
-    <row r="458" ht="14.25" customHeight="1"/>
-    <row r="459" ht="14.25" customHeight="1"/>
-    <row r="460" ht="14.25" customHeight="1"/>
-    <row r="461" ht="14.25" customHeight="1"/>
-    <row r="462" ht="14.25" customHeight="1"/>
-    <row r="463" ht="14.25" customHeight="1"/>
-    <row r="464" ht="14.25" customHeight="1"/>
-    <row r="465" ht="14.25" customHeight="1"/>
-    <row r="466" ht="14.25" customHeight="1"/>
-    <row r="467" ht="14.25" customHeight="1"/>
-    <row r="468" ht="14.25" customHeight="1"/>
-    <row r="469" ht="14.25" customHeight="1"/>
-    <row r="470" ht="14.25" customHeight="1"/>
-    <row r="471" ht="14.25" customHeight="1"/>
-    <row r="472" ht="14.25" customHeight="1"/>
-    <row r="473" ht="14.25" customHeight="1"/>
-    <row r="474" ht="14.25" customHeight="1"/>
-    <row r="475" ht="14.25" customHeight="1"/>
-    <row r="476" ht="14.25" customHeight="1"/>
-    <row r="477" ht="14.25" customHeight="1"/>
-    <row r="478" ht="14.25" customHeight="1"/>
-    <row r="479" ht="14.25" customHeight="1"/>
-    <row r="480" ht="14.25" customHeight="1"/>
-    <row r="481" ht="14.25" customHeight="1"/>
-    <row r="482" ht="14.25" customHeight="1"/>
-    <row r="483" ht="14.25" customHeight="1"/>
-    <row r="484" ht="14.25" customHeight="1"/>
-    <row r="485" ht="14.25" customHeight="1"/>
-    <row r="486" ht="14.25" customHeight="1"/>
-    <row r="487" ht="14.25" customHeight="1"/>
-    <row r="488" ht="14.25" customHeight="1"/>
-    <row r="489" ht="14.25" customHeight="1"/>
-    <row r="490" ht="14.25" customHeight="1"/>
-    <row r="491" ht="14.25" customHeight="1"/>
-    <row r="492" ht="14.25" customHeight="1"/>
-    <row r="493" ht="14.25" customHeight="1"/>
-    <row r="494" ht="14.25" customHeight="1"/>
-    <row r="495" ht="14.25" customHeight="1"/>
-    <row r="496" ht="14.25" customHeight="1"/>
-    <row r="497" ht="14.25" customHeight="1"/>
-    <row r="498" ht="14.25" customHeight="1"/>
-    <row r="499" ht="14.25" customHeight="1"/>
-    <row r="500" ht="14.25" customHeight="1"/>
-    <row r="501" ht="14.25" customHeight="1"/>
-    <row r="502" ht="14.25" customHeight="1"/>
-    <row r="503" ht="14.25" customHeight="1"/>
-    <row r="504" ht="14.25" customHeight="1"/>
-    <row r="505" ht="14.25" customHeight="1"/>
-    <row r="506" ht="14.25" customHeight="1"/>
-    <row r="507" ht="14.25" customHeight="1"/>
-    <row r="508" ht="14.25" customHeight="1"/>
-    <row r="509" ht="14.25" customHeight="1"/>
-    <row r="510" ht="14.25" customHeight="1"/>
-    <row r="511" ht="14.25" customHeight="1"/>
-    <row r="512" ht="14.25" customHeight="1"/>
-    <row r="513" ht="14.25" customHeight="1"/>
-    <row r="514" ht="14.25" customHeight="1"/>
-    <row r="515" ht="14.25" customHeight="1"/>
-    <row r="516" ht="14.25" customHeight="1"/>
-    <row r="517" ht="14.25" customHeight="1"/>
-    <row r="518" ht="14.25" customHeight="1"/>
-    <row r="519" ht="14.25" customHeight="1"/>
-    <row r="520" ht="14.25" customHeight="1"/>
-    <row r="521" ht="14.25" customHeight="1"/>
-    <row r="522" ht="14.25" customHeight="1"/>
-    <row r="523" ht="14.25" customHeight="1"/>
-    <row r="524" ht="14.25" customHeight="1"/>
-    <row r="525" ht="14.25" customHeight="1"/>
-    <row r="526" ht="14.25" customHeight="1"/>
-    <row r="527" ht="14.25" customHeight="1"/>
-    <row r="528" ht="14.25" customHeight="1"/>
-    <row r="529" ht="14.25" customHeight="1"/>
-    <row r="530" ht="14.25" customHeight="1"/>
-    <row r="531" ht="14.25" customHeight="1"/>
-    <row r="532" ht="14.25" customHeight="1"/>
-    <row r="533" ht="14.25" customHeight="1"/>
-    <row r="534" ht="14.25" customHeight="1"/>
-    <row r="535" ht="14.25" customHeight="1"/>
-    <row r="536" ht="14.25" customHeight="1"/>
-    <row r="537" ht="14.25" customHeight="1"/>
-    <row r="538" ht="14.25" customHeight="1"/>
-    <row r="539" ht="14.25" customHeight="1"/>
-    <row r="540" ht="14.25" customHeight="1"/>
-    <row r="541" ht="14.25" customHeight="1"/>
-    <row r="542" ht="14.25" customHeight="1"/>
-    <row r="543" ht="14.25" customHeight="1"/>
-    <row r="544" ht="14.25" customHeight="1"/>
-    <row r="545" ht="14.25" customHeight="1"/>
-    <row r="546" ht="14.25" customHeight="1"/>
-    <row r="547" ht="14.25" customHeight="1"/>
-    <row r="548" ht="14.25" customHeight="1"/>
-    <row r="549" ht="14.25" customHeight="1"/>
-    <row r="550" ht="14.25" customHeight="1"/>
-    <row r="551" ht="14.25" customHeight="1"/>
-    <row r="552" ht="14.25" customHeight="1"/>
-    <row r="553" ht="14.25" customHeight="1"/>
-    <row r="554" ht="14.25" customHeight="1"/>
-    <row r="555" ht="14.25" customHeight="1"/>
-    <row r="556" ht="14.25" customHeight="1"/>
-    <row r="557" ht="14.25" customHeight="1"/>
-    <row r="558" ht="14.25" customHeight="1"/>
-    <row r="559" ht="14.25" customHeight="1"/>
-    <row r="560" ht="14.25" customHeight="1"/>
-    <row r="561" ht="14.25" customHeight="1"/>
-    <row r="562" ht="14.25" customHeight="1"/>
-    <row r="563" ht="14.25" customHeight="1"/>
-    <row r="564" ht="14.25" customHeight="1"/>
-    <row r="565" ht="14.25" customHeight="1"/>
-    <row r="566" ht="14.25" customHeight="1"/>
-    <row r="567" ht="14.25" customHeight="1"/>
-    <row r="568" ht="14.25" customHeight="1"/>
-    <row r="569" ht="14.25" customHeight="1"/>
-    <row r="570" ht="14.25" customHeight="1"/>
-    <row r="571" ht="14.25" customHeight="1"/>
-    <row r="572" ht="14.25" customHeight="1"/>
-    <row r="573" ht="14.25" customHeight="1"/>
-    <row r="574" ht="14.25" customHeight="1"/>
-    <row r="575" ht="14.25" customHeight="1"/>
-    <row r="576" ht="14.25" customHeight="1"/>
-    <row r="577" ht="14.25" customHeight="1"/>
-    <row r="578" ht="14.25" customHeight="1"/>
-    <row r="579" ht="14.25" customHeight="1"/>
-    <row r="580" ht="14.25" customHeight="1"/>
-    <row r="581" ht="14.25" customHeight="1"/>
-    <row r="582" ht="14.25" customHeight="1"/>
-    <row r="583" ht="14.25" customHeight="1"/>
-    <row r="584" ht="14.25" customHeight="1"/>
-    <row r="585" ht="14.25" customHeight="1"/>
-    <row r="586" ht="14.25" customHeight="1"/>
-    <row r="587" ht="14.25" customHeight="1"/>
-    <row r="588" ht="14.25" customHeight="1"/>
-    <row r="589" ht="14.25" customHeight="1"/>
-    <row r="590" ht="14.25" customHeight="1"/>
-    <row r="591" ht="14.25" customHeight="1"/>
-    <row r="592" ht="14.25" customHeight="1"/>
-    <row r="593" ht="14.25" customHeight="1"/>
-    <row r="594" ht="14.25" customHeight="1"/>
-    <row r="595" ht="14.25" customHeight="1"/>
-    <row r="596" ht="14.25" customHeight="1"/>
-    <row r="597" ht="14.25" customHeight="1"/>
-    <row r="598" ht="14.25" customHeight="1"/>
-    <row r="599" ht="14.25" customHeight="1"/>
-    <row r="600" ht="14.25" customHeight="1"/>
-    <row r="601" ht="14.25" customHeight="1"/>
-    <row r="602" ht="14.25" customHeight="1"/>
-    <row r="603" ht="14.25" customHeight="1"/>
-    <row r="604" ht="14.25" customHeight="1"/>
-    <row r="605" ht="14.25" customHeight="1"/>
-    <row r="606" ht="14.25" customHeight="1"/>
-    <row r="607" ht="14.25" customHeight="1"/>
-    <row r="608" ht="14.25" customHeight="1"/>
-    <row r="609" ht="14.25" customHeight="1"/>
-    <row r="610" ht="14.25" customHeight="1"/>
-    <row r="611" ht="14.25" customHeight="1"/>
-    <row r="612" ht="14.25" customHeight="1"/>
-    <row r="613" ht="14.25" customHeight="1"/>
-    <row r="614" ht="14.25" customHeight="1"/>
-    <row r="615" ht="14.25" customHeight="1"/>
-    <row r="616" ht="14.25" customHeight="1"/>
-    <row r="617" ht="14.25" customHeight="1"/>
-    <row r="618" ht="14.25" customHeight="1"/>
-    <row r="619" ht="14.25" customHeight="1"/>
-    <row r="620" ht="14.25" customHeight="1"/>
-    <row r="621" ht="14.25" customHeight="1"/>
-    <row r="622" ht="14.25" customHeight="1"/>
-    <row r="623" ht="14.25" customHeight="1"/>
-    <row r="624" ht="14.25" customHeight="1"/>
-    <row r="625" ht="14.25" customHeight="1"/>
-    <row r="626" ht="14.25" customHeight="1"/>
-    <row r="627" ht="14.25" customHeight="1"/>
-    <row r="628" ht="14.25" customHeight="1"/>
-    <row r="629" ht="14.25" customHeight="1"/>
-    <row r="630" ht="14.25" customHeight="1"/>
-    <row r="631" ht="14.25" customHeight="1"/>
-    <row r="632" ht="14.25" customHeight="1"/>
-    <row r="633" ht="14.25" customHeight="1"/>
-    <row r="634" ht="14.25" customHeight="1"/>
-    <row r="635" ht="14.25" customHeight="1"/>
-    <row r="636" ht="14.25" customHeight="1"/>
-    <row r="637" ht="14.25" customHeight="1"/>
-    <row r="638" ht="14.25" customHeight="1"/>
-    <row r="639" ht="14.25" customHeight="1"/>
-    <row r="640" ht="14.25" customHeight="1"/>
-    <row r="641" ht="14.25" customHeight="1"/>
-    <row r="642" ht="14.25" customHeight="1"/>
-    <row r="643" ht="14.25" customHeight="1"/>
-    <row r="644" ht="14.25" customHeight="1"/>
-    <row r="645" ht="14.25" customHeight="1"/>
-    <row r="646" ht="14.25" customHeight="1"/>
-    <row r="647" ht="14.25" customHeight="1"/>
-    <row r="648" ht="14.25" customHeight="1"/>
-    <row r="649" ht="14.25" customHeight="1"/>
-    <row r="650" ht="14.25" customHeight="1"/>
-    <row r="651" ht="14.25" customHeight="1"/>
-    <row r="652" ht="14.25" customHeight="1"/>
-    <row r="653" ht="14.25" customHeight="1"/>
-    <row r="654" ht="14.25" customHeight="1"/>
-    <row r="655" ht="14.25" customHeight="1"/>
-    <row r="656" ht="14.25" customHeight="1"/>
-    <row r="657" ht="14.25" customHeight="1"/>
-    <row r="658" ht="14.25" customHeight="1"/>
-    <row r="659" ht="14.25" customHeight="1"/>
-    <row r="660" ht="14.25" customHeight="1"/>
-    <row r="661" ht="14.25" customHeight="1"/>
-    <row r="662" ht="14.25" customHeight="1"/>
-    <row r="663" ht="14.25" customHeight="1"/>
-    <row r="664" ht="14.25" customHeight="1"/>
-    <row r="665" ht="14.25" customHeight="1"/>
-    <row r="666" ht="14.25" customHeight="1"/>
-    <row r="667" ht="14.25" customHeight="1"/>
-    <row r="668" ht="14.25" customHeight="1"/>
-    <row r="669" ht="14.25" customHeight="1"/>
-    <row r="670" ht="14.25" customHeight="1"/>
-    <row r="671" ht="14.25" customHeight="1"/>
-    <row r="672" ht="14.25" customHeight="1"/>
-    <row r="673" ht="14.25" customHeight="1"/>
-    <row r="674" ht="14.25" customHeight="1"/>
-    <row r="675" ht="14.25" customHeight="1"/>
-    <row r="676" ht="14.25" customHeight="1"/>
-    <row r="677" ht="14.25" customHeight="1"/>
-    <row r="678" ht="14.25" customHeight="1"/>
-    <row r="679" ht="14.25" customHeight="1"/>
-    <row r="680" ht="14.25" customHeight="1"/>
-    <row r="681" ht="14.25" customHeight="1"/>
-    <row r="682" ht="14.25" customHeight="1"/>
-    <row r="683" ht="14.25" customHeight="1"/>
-    <row r="684" ht="14.25" customHeight="1"/>
-    <row r="685" ht="14.25" customHeight="1"/>
-    <row r="686" ht="14.25" customHeight="1"/>
-    <row r="687" ht="14.25" customHeight="1"/>
-    <row r="688" ht="14.25" customHeight="1"/>
-    <row r="689" ht="14.25" customHeight="1"/>
-    <row r="690" ht="14.25" customHeight="1"/>
-    <row r="691" ht="14.25" customHeight="1"/>
-    <row r="692" ht="14.25" customHeight="1"/>
-    <row r="693" ht="14.25" customHeight="1"/>
-    <row r="694" ht="14.25" customHeight="1"/>
-    <row r="695" ht="14.25" customHeight="1"/>
-    <row r="696" ht="14.25" customHeight="1"/>
-    <row r="697" ht="14.25" customHeight="1"/>
-    <row r="698" ht="14.25" customHeight="1"/>
-    <row r="699" ht="14.25" customHeight="1"/>
-    <row r="700" ht="14.25" customHeight="1"/>
-    <row r="701" ht="14.25" customHeight="1"/>
-    <row r="702" ht="14.25" customHeight="1"/>
-    <row r="703" ht="14.25" customHeight="1"/>
-    <row r="704" ht="14.25" customHeight="1"/>
-    <row r="705" ht="14.25" customHeight="1"/>
-    <row r="706" ht="14.25" customHeight="1"/>
-    <row r="707" ht="14.25" customHeight="1"/>
-    <row r="708" ht="14.25" customHeight="1"/>
-    <row r="709" ht="14.25" customHeight="1"/>
-    <row r="710" ht="14.25" customHeight="1"/>
-    <row r="711" ht="14.25" customHeight="1"/>
-    <row r="712" ht="14.25" customHeight="1"/>
-    <row r="713" ht="14.25" customHeight="1"/>
-    <row r="714" ht="14.25" customHeight="1"/>
-    <row r="715" ht="14.25" customHeight="1"/>
-    <row r="716" ht="14.25" customHeight="1"/>
-    <row r="717" ht="14.25" customHeight="1"/>
-    <row r="718" ht="14.25" customHeight="1"/>
-    <row r="719" ht="14.25" customHeight="1"/>
-    <row r="720" ht="14.25" customHeight="1"/>
-    <row r="721" ht="14.25" customHeight="1"/>
-    <row r="722" ht="14.25" customHeight="1"/>
-    <row r="723" ht="14.25" customHeight="1"/>
-    <row r="724" ht="14.25" customHeight="1"/>
-    <row r="725" ht="14.25" customHeight="1"/>
-    <row r="726" ht="14.25" customHeight="1"/>
-    <row r="727" ht="14.25" customHeight="1"/>
-    <row r="728" ht="14.25" customHeight="1"/>
-    <row r="729" ht="14.25" customHeight="1"/>
-    <row r="730" ht="14.25" customHeight="1"/>
-    <row r="731" ht="14.25" customHeight="1"/>
-    <row r="732" ht="14.25" customHeight="1"/>
-    <row r="733" ht="14.25" customHeight="1"/>
-    <row r="734" ht="14.25" customHeight="1"/>
-    <row r="735" ht="14.25" customHeight="1"/>
-    <row r="736" ht="14.25" customHeight="1"/>
-    <row r="737" ht="14.25" customHeight="1"/>
-    <row r="738" ht="14.25" customHeight="1"/>
-    <row r="739" ht="14.25" customHeight="1"/>
-    <row r="740" ht="14.25" customHeight="1"/>
-    <row r="741" ht="14.25" customHeight="1"/>
-    <row r="742" ht="14.25" customHeight="1"/>
-    <row r="743" ht="14.25" customHeight="1"/>
-    <row r="744" ht="14.25" customHeight="1"/>
-    <row r="745" ht="14.25" customHeight="1"/>
-    <row r="746" ht="14.25" customHeight="1"/>
-    <row r="747" ht="14.25" customHeight="1"/>
-    <row r="748" ht="14.25" customHeight="1"/>
-    <row r="749" ht="14.25" customHeight="1"/>
-    <row r="750" ht="14.25" customHeight="1"/>
-    <row r="751" ht="14.25" customHeight="1"/>
-    <row r="752" ht="14.25" customHeight="1"/>
-    <row r="753" ht="14.25" customHeight="1"/>
-    <row r="754" ht="14.25" customHeight="1"/>
-    <row r="755" ht="14.25" customHeight="1"/>
-    <row r="756" ht="14.25" customHeight="1"/>
-    <row r="757" ht="14.25" customHeight="1"/>
-    <row r="758" ht="14.25" customHeight="1"/>
-    <row r="759" ht="14.25" customHeight="1"/>
-    <row r="760" ht="14.25" customHeight="1"/>
-    <row r="761" ht="14.25" customHeight="1"/>
-    <row r="762" ht="14.25" customHeight="1"/>
-    <row r="763" ht="14.25" customHeight="1"/>
-    <row r="764" ht="14.25" customHeight="1"/>
-    <row r="765" ht="14.25" customHeight="1"/>
-    <row r="766" ht="14.25" customHeight="1"/>
-    <row r="767" ht="14.25" customHeight="1"/>
-    <row r="768" ht="14.25" customHeight="1"/>
-    <row r="769" ht="14.25" customHeight="1"/>
-    <row r="770" ht="14.25" customHeight="1"/>
-    <row r="771" ht="14.25" customHeight="1"/>
-    <row r="772" ht="14.25" customHeight="1"/>
-    <row r="773" ht="14.25" customHeight="1"/>
-    <row r="774" ht="14.25" customHeight="1"/>
-    <row r="775" ht="14.25" customHeight="1"/>
-    <row r="776" ht="14.25" customHeight="1"/>
-    <row r="777" ht="14.25" customHeight="1"/>
-    <row r="778" ht="14.25" customHeight="1"/>
-    <row r="779" ht="14.25" customHeight="1"/>
-    <row r="780" ht="14.25" customHeight="1"/>
-    <row r="781" ht="14.25" customHeight="1"/>
-    <row r="782" ht="14.25" customHeight="1"/>
-    <row r="783" ht="14.25" customHeight="1"/>
-    <row r="784" ht="14.25" customHeight="1"/>
-    <row r="785" ht="14.25" customHeight="1"/>
-    <row r="786" ht="14.25" customHeight="1"/>
-    <row r="787" ht="14.25" customHeight="1"/>
-    <row r="788" ht="14.25" customHeight="1"/>
-    <row r="789" ht="14.25" customHeight="1"/>
-    <row r="790" ht="14.25" customHeight="1"/>
-    <row r="791" ht="14.25" customHeight="1"/>
-    <row r="792" ht="14.25" customHeight="1"/>
-    <row r="793" ht="14.25" customHeight="1"/>
-    <row r="794" ht="14.25" customHeight="1"/>
-    <row r="795" ht="14.25" customHeight="1"/>
-    <row r="796" ht="14.25" customHeight="1"/>
-    <row r="797" ht="14.25" customHeight="1"/>
-    <row r="798" ht="14.25" customHeight="1"/>
-    <row r="799" ht="14.25" customHeight="1"/>
-    <row r="800" ht="14.25" customHeight="1"/>
-    <row r="801" ht="14.25" customHeight="1"/>
-    <row r="802" ht="14.25" customHeight="1"/>
-    <row r="803" ht="14.25" customHeight="1"/>
-    <row r="804" ht="14.25" customHeight="1"/>
-    <row r="805" ht="14.25" customHeight="1"/>
-    <row r="806" ht="14.25" customHeight="1"/>
-    <row r="807" ht="14.25" customHeight="1"/>
-    <row r="808" ht="14.25" customHeight="1"/>
-    <row r="809" ht="14.25" customHeight="1"/>
-    <row r="810" ht="14.25" customHeight="1"/>
-    <row r="811" ht="14.25" customHeight="1"/>
-    <row r="812" ht="14.25" customHeight="1"/>
-    <row r="813" ht="14.25" customHeight="1"/>
-    <row r="814" ht="14.25" customHeight="1"/>
-    <row r="815" ht="14.25" customHeight="1"/>
-    <row r="816" ht="14.25" customHeight="1"/>
-    <row r="817" ht="14.25" customHeight="1"/>
-    <row r="818" ht="14.25" customHeight="1"/>
-    <row r="819" ht="14.25" customHeight="1"/>
-    <row r="820" ht="14.25" customHeight="1"/>
-    <row r="821" ht="14.25" customHeight="1"/>
-    <row r="822" ht="14.25" customHeight="1"/>
-    <row r="823" ht="14.25" customHeight="1"/>
-    <row r="824" ht="14.25" customHeight="1"/>
-    <row r="825" ht="14.25" customHeight="1"/>
-    <row r="826" ht="14.25" customHeight="1"/>
-    <row r="827" ht="14.25" customHeight="1"/>
-    <row r="828" ht="14.25" customHeight="1"/>
-    <row r="829" ht="14.25" customHeight="1"/>
-    <row r="830" ht="14.25" customHeight="1"/>
-    <row r="831" ht="14.25" customHeight="1"/>
-    <row r="832" ht="14.25" customHeight="1"/>
-    <row r="833" ht="14.25" customHeight="1"/>
-    <row r="834" ht="14.25" customHeight="1"/>
-    <row r="835" ht="14.25" customHeight="1"/>
-    <row r="836" ht="14.25" customHeight="1"/>
-    <row r="837" ht="14.25" customHeight="1"/>
-    <row r="838" ht="14.25" customHeight="1"/>
-    <row r="839" ht="14.25" customHeight="1"/>
-    <row r="840" ht="14.25" customHeight="1"/>
-    <row r="841" ht="14.25" customHeight="1"/>
-    <row r="842" ht="14.25" customHeight="1"/>
-    <row r="843" ht="14.25" customHeight="1"/>
-    <row r="844" ht="14.25" customHeight="1"/>
-    <row r="845" ht="14.25" customHeight="1"/>
-    <row r="846" ht="14.25" customHeight="1"/>
-    <row r="847" ht="14.25" customHeight="1"/>
-    <row r="848" ht="14.25" customHeight="1"/>
-    <row r="849" ht="14.25" customHeight="1"/>
-    <row r="850" ht="14.25" customHeight="1"/>
-    <row r="851" ht="14.25" customHeight="1"/>
-    <row r="852" ht="14.25" customHeight="1"/>
-    <row r="853" ht="14.25" customHeight="1"/>
-    <row r="854" ht="14.25" customHeight="1"/>
-    <row r="855" ht="14.25" customHeight="1"/>
-    <row r="856" ht="14.25" customHeight="1"/>
-    <row r="857" ht="14.25" customHeight="1"/>
-    <row r="858" ht="14.25" customHeight="1"/>
-    <row r="859" ht="14.25" customHeight="1"/>
-    <row r="860" ht="14.25" customHeight="1"/>
-    <row r="861" ht="14.25" customHeight="1"/>
-    <row r="862" ht="14.25" customHeight="1"/>
-    <row r="863" ht="14.25" customHeight="1"/>
-    <row r="864" ht="14.25" customHeight="1"/>
-    <row r="865" ht="14.25" customHeight="1"/>
-    <row r="866" ht="14.25" customHeight="1"/>
-    <row r="867" ht="14.25" customHeight="1"/>
-    <row r="868" ht="14.25" customHeight="1"/>
-    <row r="869" ht="14.25" customHeight="1"/>
-    <row r="870" ht="14.25" customHeight="1"/>
-    <row r="871" ht="14.25" customHeight="1"/>
-    <row r="872" ht="14.25" customHeight="1"/>
-    <row r="873" ht="14.25" customHeight="1"/>
-    <row r="874" ht="14.25" customHeight="1"/>
-    <row r="875" ht="14.25" customHeight="1"/>
-    <row r="876" ht="14.25" customHeight="1"/>
-    <row r="877" ht="14.25" customHeight="1"/>
-    <row r="878" ht="14.25" customHeight="1"/>
-    <row r="879" ht="14.25" customHeight="1"/>
-    <row r="880" ht="14.25" customHeight="1"/>
-    <row r="881" ht="14.25" customHeight="1"/>
-    <row r="882" ht="14.25" customHeight="1"/>
-    <row r="883" ht="14.25" customHeight="1"/>
-    <row r="884" ht="14.25" customHeight="1"/>
-    <row r="885" ht="14.25" customHeight="1"/>
-    <row r="886" ht="14.25" customHeight="1"/>
-    <row r="887" ht="14.25" customHeight="1"/>
-    <row r="888" ht="14.25" customHeight="1"/>
-    <row r="889" ht="14.25" customHeight="1"/>
-    <row r="890" ht="14.25" customHeight="1"/>
-    <row r="891" ht="14.25" customHeight="1"/>
-    <row r="892" ht="14.25" customHeight="1"/>
-    <row r="893" ht="14.25" customHeight="1"/>
-    <row r="894" ht="14.25" customHeight="1"/>
-    <row r="895" ht="14.25" customHeight="1"/>
-    <row r="896" ht="14.25" customHeight="1"/>
-    <row r="897" ht="14.25" customHeight="1"/>
-    <row r="898" ht="14.25" customHeight="1"/>
-    <row r="899" ht="14.25" customHeight="1"/>
-    <row r="900" ht="14.25" customHeight="1"/>
-    <row r="901" ht="14.25" customHeight="1"/>
-    <row r="902" ht="14.25" customHeight="1"/>
-    <row r="903" ht="14.25" customHeight="1"/>
-    <row r="904" ht="14.25" customHeight="1"/>
-    <row r="905" ht="14.25" customHeight="1"/>
-    <row r="906" ht="14.25" customHeight="1"/>
-    <row r="907" ht="14.25" customHeight="1"/>
-    <row r="908" ht="14.25" customHeight="1"/>
-    <row r="909" ht="14.25" customHeight="1"/>
-    <row r="910" ht="14.25" customHeight="1"/>
-    <row r="911" ht="14.25" customHeight="1"/>
-    <row r="912" ht="14.25" customHeight="1"/>
-    <row r="913" ht="14.25" customHeight="1"/>
-    <row r="914" ht="14.25" customHeight="1"/>
-    <row r="915" ht="14.25" customHeight="1"/>
-    <row r="916" ht="14.25" customHeight="1"/>
-    <row r="917" ht="14.25" customHeight="1"/>
-    <row r="918" ht="14.25" customHeight="1"/>
-    <row r="919" ht="14.25" customHeight="1"/>
-    <row r="920" ht="14.25" customHeight="1"/>
-    <row r="921" ht="14.25" customHeight="1"/>
-    <row r="922" ht="14.25" customHeight="1"/>
-    <row r="923" ht="14.25" customHeight="1"/>
-    <row r="924" ht="14.25" customHeight="1"/>
-    <row r="925" ht="14.25" customHeight="1"/>
-    <row r="926" ht="14.25" customHeight="1"/>
-    <row r="927" ht="14.25" customHeight="1"/>
-    <row r="928" ht="14.25" customHeight="1"/>
-    <row r="929" ht="14.25" customHeight="1"/>
-    <row r="930" ht="14.25" customHeight="1"/>
-    <row r="931" ht="14.25" customHeight="1"/>
-    <row r="932" ht="14.25" customHeight="1"/>
-    <row r="933" ht="14.25" customHeight="1"/>
-    <row r="934" ht="14.25" customHeight="1"/>
-    <row r="935" ht="14.25" customHeight="1"/>
-    <row r="936" ht="14.25" customHeight="1"/>
-    <row r="937" ht="14.25" customHeight="1"/>
-    <row r="938" ht="14.25" customHeight="1"/>
-    <row r="939" ht="14.25" customHeight="1"/>
-    <row r="940" ht="14.25" customHeight="1"/>
-    <row r="941" ht="14.25" customHeight="1"/>
-    <row r="942" ht="14.25" customHeight="1"/>
-    <row r="943" ht="14.25" customHeight="1"/>
-    <row r="944" ht="14.25" customHeight="1"/>
-    <row r="945" ht="14.25" customHeight="1"/>
-    <row r="946" ht="14.25" customHeight="1"/>
-    <row r="947" ht="14.25" customHeight="1"/>
-    <row r="948" ht="14.25" customHeight="1"/>
-    <row r="949" ht="14.25" customHeight="1"/>
-    <row r="950" ht="14.25" customHeight="1"/>
-    <row r="951" ht="14.25" customHeight="1"/>
-    <row r="952" ht="14.25" customHeight="1"/>
-    <row r="953" ht="14.25" customHeight="1"/>
-    <row r="954" ht="14.25" customHeight="1"/>
-    <row r="955" ht="14.25" customHeight="1"/>
-    <row r="956" ht="14.25" customHeight="1"/>
-    <row r="957" ht="14.25" customHeight="1"/>
-    <row r="958" ht="14.25" customHeight="1"/>
-    <row r="959" ht="14.25" customHeight="1"/>
-    <row r="960" ht="14.25" customHeight="1"/>
-    <row r="961" ht="14.25" customHeight="1"/>
-    <row r="962" ht="14.25" customHeight="1"/>
-    <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
-    <row r="973" ht="14.25" customHeight="1"/>
-    <row r="974" ht="14.25" customHeight="1"/>
-    <row r="975" ht="14.25" customHeight="1"/>
-    <row r="976" ht="14.25" customHeight="1"/>
-    <row r="977" ht="14.25" customHeight="1"/>
-    <row r="978" ht="14.25" customHeight="1"/>
-    <row r="979" ht="14.25" customHeight="1"/>
-    <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="7" ht="14.25" customHeight="true"/>
+    <row r="8" ht="14.25" customHeight="true"/>
+    <row r="9" ht="14.25" customHeight="true"/>
+    <row r="10" ht="14.25" customHeight="true"/>
+    <row r="11" ht="14.25" customHeight="true"/>
+    <row r="12" ht="14.25" customHeight="true"/>
+    <row r="13" ht="14.25" customHeight="true"/>
+    <row r="14" ht="14.25" customHeight="true"/>
+    <row r="15" ht="14.25" customHeight="true"/>
+    <row r="16" ht="14.25" customHeight="true"/>
+    <row r="17" ht="14.25" customHeight="true"/>
+    <row r="18" ht="14.25" customHeight="true"/>
+    <row r="19" ht="14.25" customHeight="true"/>
+    <row r="20" ht="14.25" customHeight="true"/>
+    <row r="21" ht="14.25" customHeight="true"/>
+    <row r="22" ht="14.25" customHeight="true"/>
+    <row r="23" ht="14.25" customHeight="true"/>
+    <row r="24" ht="14.25" customHeight="true"/>
+    <row r="25" ht="14.25" customHeight="true"/>
+    <row r="26" ht="14.25" customHeight="true"/>
+    <row r="27" ht="14.25" customHeight="true"/>
+    <row r="28" ht="14.25" customHeight="true"/>
+    <row r="29" ht="14.25" customHeight="true"/>
+    <row r="30" ht="14.25" customHeight="true"/>
+    <row r="31" ht="14.25" customHeight="true"/>
+    <row r="32" ht="14.25" customHeight="true"/>
+    <row r="33" ht="14.25" customHeight="true"/>
+    <row r="34" ht="14.25" customHeight="true"/>
+    <row r="35" ht="14.25" customHeight="true"/>
+    <row r="36" ht="14.25" customHeight="true"/>
+    <row r="37" ht="14.25" customHeight="true"/>
+    <row r="38" ht="14.25" customHeight="true"/>
+    <row r="39" ht="14.25" customHeight="true"/>
+    <row r="40" ht="14.25" customHeight="true"/>
+    <row r="41" ht="14.25" customHeight="true"/>
+    <row r="42" ht="14.25" customHeight="true"/>
+    <row r="43" ht="14.25" customHeight="true"/>
+    <row r="44" ht="14.25" customHeight="true"/>
+    <row r="45" ht="14.25" customHeight="true"/>
+    <row r="46" ht="14.25" customHeight="true"/>
+    <row r="47" ht="14.25" customHeight="true"/>
+    <row r="48" ht="14.25" customHeight="true"/>
+    <row r="49" ht="14.25" customHeight="true"/>
+    <row r="50" ht="14.25" customHeight="true"/>
+    <row r="51" ht="14.25" customHeight="true"/>
+    <row r="52" ht="14.25" customHeight="true"/>
+    <row r="53" ht="14.25" customHeight="true"/>
+    <row r="54" ht="14.25" customHeight="true"/>
+    <row r="55" ht="14.25" customHeight="true"/>
+    <row r="56" ht="14.25" customHeight="true"/>
+    <row r="57" ht="14.25" customHeight="true"/>
+    <row r="58" ht="14.25" customHeight="true"/>
+    <row r="59" ht="14.25" customHeight="true"/>
+    <row r="60" ht="14.25" customHeight="true"/>
+    <row r="61" ht="14.25" customHeight="true"/>
+    <row r="62" ht="14.25" customHeight="true"/>
+    <row r="63" ht="14.25" customHeight="true"/>
+    <row r="64" ht="14.25" customHeight="true"/>
+    <row r="65" ht="14.25" customHeight="true"/>
+    <row r="66" ht="14.25" customHeight="true"/>
+    <row r="67" ht="14.25" customHeight="true"/>
+    <row r="68" ht="14.25" customHeight="true"/>
+    <row r="69" ht="14.25" customHeight="true"/>
+    <row r="70" ht="14.25" customHeight="true"/>
+    <row r="71" ht="14.25" customHeight="true"/>
+    <row r="72" ht="14.25" customHeight="true"/>
+    <row r="73" ht="14.25" customHeight="true"/>
+    <row r="74" ht="14.25" customHeight="true"/>
+    <row r="75" ht="14.25" customHeight="true"/>
+    <row r="76" ht="14.25" customHeight="true"/>
+    <row r="77" ht="14.25" customHeight="true"/>
+    <row r="78" ht="14.25" customHeight="true"/>
+    <row r="79" ht="14.25" customHeight="true"/>
+    <row r="80" ht="14.25" customHeight="true"/>
+    <row r="81" ht="14.25" customHeight="true"/>
+    <row r="82" ht="14.25" customHeight="true"/>
+    <row r="83" ht="14.25" customHeight="true"/>
+    <row r="84" ht="14.25" customHeight="true"/>
+    <row r="85" ht="14.25" customHeight="true"/>
+    <row r="86" ht="14.25" customHeight="true"/>
+    <row r="87" ht="14.25" customHeight="true"/>
+    <row r="88" ht="14.25" customHeight="true"/>
+    <row r="89" ht="14.25" customHeight="true"/>
+    <row r="90" ht="14.25" customHeight="true"/>
+    <row r="91" ht="14.25" customHeight="true"/>
+    <row r="92" ht="14.25" customHeight="true"/>
+    <row r="93" ht="14.25" customHeight="true"/>
+    <row r="94" ht="14.25" customHeight="true"/>
+    <row r="95" ht="14.25" customHeight="true"/>
+    <row r="96" ht="14.25" customHeight="true"/>
+    <row r="97" ht="14.25" customHeight="true"/>
+    <row r="98" ht="14.25" customHeight="true"/>
+    <row r="99" ht="14.25" customHeight="true"/>
+    <row r="100" ht="14.25" customHeight="true"/>
+    <row r="101" ht="14.25" customHeight="true"/>
+    <row r="102" ht="14.25" customHeight="true"/>
+    <row r="103" ht="14.25" customHeight="true"/>
+    <row r="104" ht="14.25" customHeight="true"/>
+    <row r="105" ht="14.25" customHeight="true"/>
+    <row r="106" ht="14.25" customHeight="true"/>
+    <row r="107" ht="14.25" customHeight="true"/>
+    <row r="108" ht="14.25" customHeight="true"/>
+    <row r="109" ht="14.25" customHeight="true"/>
+    <row r="110" ht="14.25" customHeight="true"/>
+    <row r="111" ht="14.25" customHeight="true"/>
+    <row r="112" ht="14.25" customHeight="true"/>
+    <row r="113" ht="14.25" customHeight="true"/>
+    <row r="114" ht="14.25" customHeight="true"/>
+    <row r="115" ht="14.25" customHeight="true"/>
+    <row r="116" ht="14.25" customHeight="true"/>
+    <row r="117" ht="14.25" customHeight="true"/>
+    <row r="118" ht="14.25" customHeight="true"/>
+    <row r="119" ht="14.25" customHeight="true"/>
+    <row r="120" ht="14.25" customHeight="true"/>
+    <row r="121" ht="14.25" customHeight="true"/>
+    <row r="122" ht="14.25" customHeight="true"/>
+    <row r="123" ht="14.25" customHeight="true"/>
+    <row r="124" ht="14.25" customHeight="true"/>
+    <row r="125" ht="14.25" customHeight="true"/>
+    <row r="126" ht="14.25" customHeight="true"/>
+    <row r="127" ht="14.25" customHeight="true"/>
+    <row r="128" ht="14.25" customHeight="true"/>
+    <row r="129" ht="14.25" customHeight="true"/>
+    <row r="130" ht="14.25" customHeight="true"/>
+    <row r="131" ht="14.25" customHeight="true"/>
+    <row r="132" ht="14.25" customHeight="true"/>
+    <row r="133" ht="14.25" customHeight="true"/>
+    <row r="134" ht="14.25" customHeight="true"/>
+    <row r="135" ht="14.25" customHeight="true"/>
+    <row r="136" ht="14.25" customHeight="true"/>
+    <row r="137" ht="14.25" customHeight="true"/>
+    <row r="138" ht="14.25" customHeight="true"/>
+    <row r="139" ht="14.25" customHeight="true"/>
+    <row r="140" ht="14.25" customHeight="true"/>
+    <row r="141" ht="14.25" customHeight="true"/>
+    <row r="142" ht="14.25" customHeight="true"/>
+    <row r="143" ht="14.25" customHeight="true"/>
+    <row r="144" ht="14.25" customHeight="true"/>
+    <row r="145" ht="14.25" customHeight="true"/>
+    <row r="146" ht="14.25" customHeight="true"/>
+    <row r="147" ht="14.25" customHeight="true"/>
+    <row r="148" ht="14.25" customHeight="true"/>
+    <row r="149" ht="14.25" customHeight="true"/>
+    <row r="150" ht="14.25" customHeight="true"/>
+    <row r="151" ht="14.25" customHeight="true"/>
+    <row r="152" ht="14.25" customHeight="true"/>
+    <row r="153" ht="14.25" customHeight="true"/>
+    <row r="154" ht="14.25" customHeight="true"/>
+    <row r="155" ht="14.25" customHeight="true"/>
+    <row r="156" ht="14.25" customHeight="true"/>
+    <row r="157" ht="14.25" customHeight="true"/>
+    <row r="158" ht="14.25" customHeight="true"/>
+    <row r="159" ht="14.25" customHeight="true"/>
+    <row r="160" ht="14.25" customHeight="true"/>
+    <row r="161" ht="14.25" customHeight="true"/>
+    <row r="162" ht="14.25" customHeight="true"/>
+    <row r="163" ht="14.25" customHeight="true"/>
+    <row r="164" ht="14.25" customHeight="true"/>
+    <row r="165" ht="14.25" customHeight="true"/>
+    <row r="166" ht="14.25" customHeight="true"/>
+    <row r="167" ht="14.25" customHeight="true"/>
+    <row r="168" ht="14.25" customHeight="true"/>
+    <row r="169" ht="14.25" customHeight="true"/>
+    <row r="170" ht="14.25" customHeight="true"/>
+    <row r="171" ht="14.25" customHeight="true"/>
+    <row r="172" ht="14.25" customHeight="true"/>
+    <row r="173" ht="14.25" customHeight="true"/>
+    <row r="174" ht="14.25" customHeight="true"/>
+    <row r="175" ht="14.25" customHeight="true"/>
+    <row r="176" ht="14.25" customHeight="true"/>
+    <row r="177" ht="14.25" customHeight="true"/>
+    <row r="178" ht="14.25" customHeight="true"/>
+    <row r="179" ht="14.25" customHeight="true"/>
+    <row r="180" ht="14.25" customHeight="true"/>
+    <row r="181" ht="14.25" customHeight="true"/>
+    <row r="182" ht="14.25" customHeight="true"/>
+    <row r="183" ht="14.25" customHeight="true"/>
+    <row r="184" ht="14.25" customHeight="true"/>
+    <row r="185" ht="14.25" customHeight="true"/>
+    <row r="186" ht="14.25" customHeight="true"/>
+    <row r="187" ht="14.25" customHeight="true"/>
+    <row r="188" ht="14.25" customHeight="true"/>
+    <row r="189" ht="14.25" customHeight="true"/>
+    <row r="190" ht="14.25" customHeight="true"/>
+    <row r="191" ht="14.25" customHeight="true"/>
+    <row r="192" ht="14.25" customHeight="true"/>
+    <row r="193" ht="14.25" customHeight="true"/>
+    <row r="194" ht="14.25" customHeight="true"/>
+    <row r="195" ht="14.25" customHeight="true"/>
+    <row r="196" ht="14.25" customHeight="true"/>
+    <row r="197" ht="14.25" customHeight="true"/>
+    <row r="198" ht="14.25" customHeight="true"/>
+    <row r="199" ht="14.25" customHeight="true"/>
+    <row r="200" ht="14.25" customHeight="true"/>
+    <row r="201" ht="14.25" customHeight="true"/>
+    <row r="202" ht="14.25" customHeight="true"/>
+    <row r="203" ht="14.25" customHeight="true"/>
+    <row r="204" ht="14.25" customHeight="true"/>
+    <row r="205" ht="14.25" customHeight="true"/>
+    <row r="206" ht="14.25" customHeight="true"/>
+    <row r="207" ht="14.25" customHeight="true"/>
+    <row r="208" ht="14.25" customHeight="true"/>
+    <row r="209" ht="14.25" customHeight="true"/>
+    <row r="210" ht="14.25" customHeight="true"/>
+    <row r="211" ht="14.25" customHeight="true"/>
+    <row r="212" ht="14.25" customHeight="true"/>
+    <row r="213" ht="14.25" customHeight="true"/>
+    <row r="214" ht="14.25" customHeight="true"/>
+    <row r="215" ht="14.25" customHeight="true"/>
+    <row r="216" ht="14.25" customHeight="true"/>
+    <row r="217" ht="14.25" customHeight="true"/>
+    <row r="218" ht="14.25" customHeight="true"/>
+    <row r="219" ht="14.25" customHeight="true"/>
+    <row r="220" ht="14.25" customHeight="true"/>
+    <row r="221" ht="14.25" customHeight="true"/>
+    <row r="222" ht="14.25" customHeight="true"/>
+    <row r="223" ht="14.25" customHeight="true"/>
+    <row r="224" ht="14.25" customHeight="true"/>
+    <row r="225" ht="14.25" customHeight="true"/>
+    <row r="226" ht="14.25" customHeight="true"/>
+    <row r="227" ht="14.25" customHeight="true"/>
+    <row r="228" ht="14.25" customHeight="true"/>
+    <row r="229" ht="14.25" customHeight="true"/>
+    <row r="230" ht="14.25" customHeight="true"/>
+    <row r="231" ht="14.25" customHeight="true"/>
+    <row r="232" ht="14.25" customHeight="true"/>
+    <row r="233" ht="14.25" customHeight="true"/>
+    <row r="234" ht="14.25" customHeight="true"/>
+    <row r="235" ht="14.25" customHeight="true"/>
+    <row r="236" ht="14.25" customHeight="true"/>
+    <row r="237" ht="14.25" customHeight="true"/>
+    <row r="238" ht="14.25" customHeight="true"/>
+    <row r="239" ht="14.25" customHeight="true"/>
+    <row r="240" ht="14.25" customHeight="true"/>
+    <row r="241" ht="14.25" customHeight="true"/>
+    <row r="242" ht="14.25" customHeight="true"/>
+    <row r="243" ht="14.25" customHeight="true"/>
+    <row r="244" ht="14.25" customHeight="true"/>
+    <row r="245" ht="14.25" customHeight="true"/>
+    <row r="246" ht="14.25" customHeight="true"/>
+    <row r="247" ht="14.25" customHeight="true"/>
+    <row r="248" ht="14.25" customHeight="true"/>
+    <row r="249" ht="14.25" customHeight="true"/>
+    <row r="250" ht="14.25" customHeight="true"/>
+    <row r="251" ht="14.25" customHeight="true"/>
+    <row r="252" ht="14.25" customHeight="true"/>
+    <row r="253" ht="14.25" customHeight="true"/>
+    <row r="254" ht="14.25" customHeight="true"/>
+    <row r="255" ht="14.25" customHeight="true"/>
+    <row r="256" ht="14.25" customHeight="true"/>
+    <row r="257" ht="14.25" customHeight="true"/>
+    <row r="258" ht="14.25" customHeight="true"/>
+    <row r="259" ht="14.25" customHeight="true"/>
+    <row r="260" ht="14.25" customHeight="true"/>
+    <row r="261" ht="14.25" customHeight="true"/>
+    <row r="262" ht="14.25" customHeight="true"/>
+    <row r="263" ht="14.25" customHeight="true"/>
+    <row r="264" ht="14.25" customHeight="true"/>
+    <row r="265" ht="14.25" customHeight="true"/>
+    <row r="266" ht="14.25" customHeight="true"/>
+    <row r="267" ht="14.25" customHeight="true"/>
+    <row r="268" ht="14.25" customHeight="true"/>
+    <row r="269" ht="14.25" customHeight="true"/>
+    <row r="270" ht="14.25" customHeight="true"/>
+    <row r="271" ht="14.25" customHeight="true"/>
+    <row r="272" ht="14.25" customHeight="true"/>
+    <row r="273" ht="14.25" customHeight="true"/>
+    <row r="274" ht="14.25" customHeight="true"/>
+    <row r="275" ht="14.25" customHeight="true"/>
+    <row r="276" ht="14.25" customHeight="true"/>
+    <row r="277" ht="14.25" customHeight="true"/>
+    <row r="278" ht="14.25" customHeight="true"/>
+    <row r="279" ht="14.25" customHeight="true"/>
+    <row r="280" ht="14.25" customHeight="true"/>
+    <row r="281" ht="14.25" customHeight="true"/>
+    <row r="282" ht="14.25" customHeight="true"/>
+    <row r="283" ht="14.25" customHeight="true"/>
+    <row r="284" ht="14.25" customHeight="true"/>
+    <row r="285" ht="14.25" customHeight="true"/>
+    <row r="286" ht="14.25" customHeight="true"/>
+    <row r="287" ht="14.25" customHeight="true"/>
+    <row r="288" ht="14.25" customHeight="true"/>
+    <row r="289" ht="14.25" customHeight="true"/>
+    <row r="290" ht="14.25" customHeight="true"/>
+    <row r="291" ht="14.25" customHeight="true"/>
+    <row r="292" ht="14.25" customHeight="true"/>
+    <row r="293" ht="14.25" customHeight="true"/>
+    <row r="294" ht="14.25" customHeight="true"/>
+    <row r="295" ht="14.25" customHeight="true"/>
+    <row r="296" ht="14.25" customHeight="true"/>
+    <row r="297" ht="14.25" customHeight="true"/>
+    <row r="298" ht="14.25" customHeight="true"/>
+    <row r="299" ht="14.25" customHeight="true"/>
+    <row r="300" ht="14.25" customHeight="true"/>
+    <row r="301" ht="14.25" customHeight="true"/>
+    <row r="302" ht="14.25" customHeight="true"/>
+    <row r="303" ht="14.25" customHeight="true"/>
+    <row r="304" ht="14.25" customHeight="true"/>
+    <row r="305" ht="14.25" customHeight="true"/>
+    <row r="306" ht="14.25" customHeight="true"/>
+    <row r="307" ht="14.25" customHeight="true"/>
+    <row r="308" ht="14.25" customHeight="true"/>
+    <row r="309" ht="14.25" customHeight="true"/>
+    <row r="310" ht="14.25" customHeight="true"/>
+    <row r="311" ht="14.25" customHeight="true"/>
+    <row r="312" ht="14.25" customHeight="true"/>
+    <row r="313" ht="14.25" customHeight="true"/>
+    <row r="314" ht="14.25" customHeight="true"/>
+    <row r="315" ht="14.25" customHeight="true"/>
+    <row r="316" ht="14.25" customHeight="true"/>
+    <row r="317" ht="14.25" customHeight="true"/>
+    <row r="318" ht="14.25" customHeight="true"/>
+    <row r="319" ht="14.25" customHeight="true"/>
+    <row r="320" ht="14.25" customHeight="true"/>
+    <row r="321" ht="14.25" customHeight="true"/>
+    <row r="322" ht="14.25" customHeight="true"/>
+    <row r="323" ht="14.25" customHeight="true"/>
+    <row r="324" ht="14.25" customHeight="true"/>
+    <row r="325" ht="14.25" customHeight="true"/>
+    <row r="326" ht="14.25" customHeight="true"/>
+    <row r="327" ht="14.25" customHeight="true"/>
+    <row r="328" ht="14.25" customHeight="true"/>
+    <row r="329" ht="14.25" customHeight="true"/>
+    <row r="330" ht="14.25" customHeight="true"/>
+    <row r="331" ht="14.25" customHeight="true"/>
+    <row r="332" ht="14.25" customHeight="true"/>
+    <row r="333" ht="14.25" customHeight="true"/>
+    <row r="334" ht="14.25" customHeight="true"/>
+    <row r="335" ht="14.25" customHeight="true"/>
+    <row r="336" ht="14.25" customHeight="true"/>
+    <row r="337" ht="14.25" customHeight="true"/>
+    <row r="338" ht="14.25" customHeight="true"/>
+    <row r="339" ht="14.25" customHeight="true"/>
+    <row r="340" ht="14.25" customHeight="true"/>
+    <row r="341" ht="14.25" customHeight="true"/>
+    <row r="342" ht="14.25" customHeight="true"/>
+    <row r="343" ht="14.25" customHeight="true"/>
+    <row r="344" ht="14.25" customHeight="true"/>
+    <row r="345" ht="14.25" customHeight="true"/>
+    <row r="346" ht="14.25" customHeight="true"/>
+    <row r="347" ht="14.25" customHeight="true"/>
+    <row r="348" ht="14.25" customHeight="true"/>
+    <row r="349" ht="14.25" customHeight="true"/>
+    <row r="350" ht="14.25" customHeight="true"/>
+    <row r="351" ht="14.25" customHeight="true"/>
+    <row r="352" ht="14.25" customHeight="true"/>
+    <row r="353" ht="14.25" customHeight="true"/>
+    <row r="354" ht="14.25" customHeight="true"/>
+    <row r="355" ht="14.25" customHeight="true"/>
+    <row r="356" ht="14.25" customHeight="true"/>
+    <row r="357" ht="14.25" customHeight="true"/>
+    <row r="358" ht="14.25" customHeight="true"/>
+    <row r="359" ht="14.25" customHeight="true"/>
+    <row r="360" ht="14.25" customHeight="true"/>
+    <row r="361" ht="14.25" customHeight="true"/>
+    <row r="362" ht="14.25" customHeight="true"/>
+    <row r="363" ht="14.25" customHeight="true"/>
+    <row r="364" ht="14.25" customHeight="true"/>
+    <row r="365" ht="14.25" customHeight="true"/>
+    <row r="366" ht="14.25" customHeight="true"/>
+    <row r="367" ht="14.25" customHeight="true"/>
+    <row r="368" ht="14.25" customHeight="true"/>
+    <row r="369" ht="14.25" customHeight="true"/>
+    <row r="370" ht="14.25" customHeight="true"/>
+    <row r="371" ht="14.25" customHeight="true"/>
+    <row r="372" ht="14.25" customHeight="true"/>
+    <row r="373" ht="14.25" customHeight="true"/>
+    <row r="374" ht="14.25" customHeight="true"/>
+    <row r="375" ht="14.25" customHeight="true"/>
+    <row r="376" ht="14.25" customHeight="true"/>
+    <row r="377" ht="14.25" customHeight="true"/>
+    <row r="378" ht="14.25" customHeight="true"/>
+    <row r="379" ht="14.25" customHeight="true"/>
+    <row r="380" ht="14.25" customHeight="true"/>
+    <row r="381" ht="14.25" customHeight="true"/>
+    <row r="382" ht="14.25" customHeight="true"/>
+    <row r="383" ht="14.25" customHeight="true"/>
+    <row r="384" ht="14.25" customHeight="true"/>
+    <row r="385" ht="14.25" customHeight="true"/>
+    <row r="386" ht="14.25" customHeight="true"/>
+    <row r="387" ht="14.25" customHeight="true"/>
+    <row r="388" ht="14.25" customHeight="true"/>
+    <row r="389" ht="14.25" customHeight="true"/>
+    <row r="390" ht="14.25" customHeight="true"/>
+    <row r="391" ht="14.25" customHeight="true"/>
+    <row r="392" ht="14.25" customHeight="true"/>
+    <row r="393" ht="14.25" customHeight="true"/>
+    <row r="394" ht="14.25" customHeight="true"/>
+    <row r="395" ht="14.25" customHeight="true"/>
+    <row r="396" ht="14.25" customHeight="true"/>
+    <row r="397" ht="14.25" customHeight="true"/>
+    <row r="398" ht="14.25" customHeight="true"/>
+    <row r="399" ht="14.25" customHeight="true"/>
+    <row r="400" ht="14.25" customHeight="true"/>
+    <row r="401" ht="14.25" customHeight="true"/>
+    <row r="402" ht="14.25" customHeight="true"/>
+    <row r="403" ht="14.25" customHeight="true"/>
+    <row r="404" ht="14.25" customHeight="true"/>
+    <row r="405" ht="14.25" customHeight="true"/>
+    <row r="406" ht="14.25" customHeight="true"/>
+    <row r="407" ht="14.25" customHeight="true"/>
+    <row r="408" ht="14.25" customHeight="true"/>
+    <row r="409" ht="14.25" customHeight="true"/>
+    <row r="410" ht="14.25" customHeight="true"/>
+    <row r="411" ht="14.25" customHeight="true"/>
+    <row r="412" ht="14.25" customHeight="true"/>
+    <row r="413" ht="14.25" customHeight="true"/>
+    <row r="414" ht="14.25" customHeight="true"/>
+    <row r="415" ht="14.25" customHeight="true"/>
+    <row r="416" ht="14.25" customHeight="true"/>
+    <row r="417" ht="14.25" customHeight="true"/>
+    <row r="418" ht="14.25" customHeight="true"/>
+    <row r="419" ht="14.25" customHeight="true"/>
+    <row r="420" ht="14.25" customHeight="true"/>
+    <row r="421" ht="14.25" customHeight="true"/>
+    <row r="422" ht="14.25" customHeight="true"/>
+    <row r="423" ht="14.25" customHeight="true"/>
+    <row r="424" ht="14.25" customHeight="true"/>
+    <row r="425" ht="14.25" customHeight="true"/>
+    <row r="426" ht="14.25" customHeight="true"/>
+    <row r="427" ht="14.25" customHeight="true"/>
+    <row r="428" ht="14.25" customHeight="true"/>
+    <row r="429" ht="14.25" customHeight="true"/>
+    <row r="430" ht="14.25" customHeight="true"/>
+    <row r="431" ht="14.25" customHeight="true"/>
+    <row r="432" ht="14.25" customHeight="true"/>
+    <row r="433" ht="14.25" customHeight="true"/>
+    <row r="434" ht="14.25" customHeight="true"/>
+    <row r="435" ht="14.25" customHeight="true"/>
+    <row r="436" ht="14.25" customHeight="true"/>
+    <row r="437" ht="14.25" customHeight="true"/>
+    <row r="438" ht="14.25" customHeight="true"/>
+    <row r="439" ht="14.25" customHeight="true"/>
+    <row r="440" ht="14.25" customHeight="true"/>
+    <row r="441" ht="14.25" customHeight="true"/>
+    <row r="442" ht="14.25" customHeight="true"/>
+    <row r="443" ht="14.25" customHeight="true"/>
+    <row r="444" ht="14.25" customHeight="true"/>
+    <row r="445" ht="14.25" customHeight="true"/>
+    <row r="446" ht="14.25" customHeight="true"/>
+    <row r="447" ht="14.25" customHeight="true"/>
+    <row r="448" ht="14.25" customHeight="true"/>
+    <row r="449" ht="14.25" customHeight="true"/>
+    <row r="450" ht="14.25" customHeight="true"/>
+    <row r="451" ht="14.25" customHeight="true"/>
+    <row r="452" ht="14.25" customHeight="true"/>
+    <row r="453" ht="14.25" customHeight="true"/>
+    <row r="454" ht="14.25" customHeight="true"/>
+    <row r="455" ht="14.25" customHeight="true"/>
+    <row r="456" ht="14.25" customHeight="true"/>
+    <row r="457" ht="14.25" customHeight="true"/>
+    <row r="458" ht="14.25" customHeight="true"/>
+    <row r="459" ht="14.25" customHeight="true"/>
+    <row r="460" ht="14.25" customHeight="true"/>
+    <row r="461" ht="14.25" customHeight="true"/>
+    <row r="462" ht="14.25" customHeight="true"/>
+    <row r="463" ht="14.25" customHeight="true"/>
+    <row r="464" ht="14.25" customHeight="true"/>
+    <row r="465" ht="14.25" customHeight="true"/>
+    <row r="466" ht="14.25" customHeight="true"/>
+    <row r="467" ht="14.25" customHeight="true"/>
+    <row r="468" ht="14.25" customHeight="true"/>
+    <row r="469" ht="14.25" customHeight="true"/>
+    <row r="470" ht="14.25" customHeight="true"/>
+    <row r="471" ht="14.25" customHeight="true"/>
+    <row r="472" ht="14.25" customHeight="true"/>
+    <row r="473" ht="14.25" customHeight="true"/>
+    <row r="474" ht="14.25" customHeight="true"/>
+    <row r="475" ht="14.25" customHeight="true"/>
+    <row r="476" ht="14.25" customHeight="true"/>
+    <row r="477" ht="14.25" customHeight="true"/>
+    <row r="478" ht="14.25" customHeight="true"/>
+    <row r="479" ht="14.25" customHeight="true"/>
+    <row r="480" ht="14.25" customHeight="true"/>
+    <row r="481" ht="14.25" customHeight="true"/>
+    <row r="482" ht="14.25" customHeight="true"/>
+    <row r="483" ht="14.25" customHeight="true"/>
+    <row r="484" ht="14.25" customHeight="true"/>
+    <row r="485" ht="14.25" customHeight="true"/>
+    <row r="486" ht="14.25" customHeight="true"/>
+    <row r="487" ht="14.25" customHeight="true"/>
+    <row r="488" ht="14.25" customHeight="true"/>
+    <row r="489" ht="14.25" customHeight="true"/>
+    <row r="490" ht="14.25" customHeight="true"/>
+    <row r="491" ht="14.25" customHeight="true"/>
+    <row r="492" ht="14.25" customHeight="true"/>
+    <row r="493" ht="14.25" customHeight="true"/>
+    <row r="494" ht="14.25" customHeight="true"/>
+    <row r="495" ht="14.25" customHeight="true"/>
+    <row r="496" ht="14.25" customHeight="true"/>
+    <row r="497" ht="14.25" customHeight="true"/>
+    <row r="498" ht="14.25" customHeight="true"/>
+    <row r="499" ht="14.25" customHeight="true"/>
+    <row r="500" ht="14.25" customHeight="true"/>
+    <row r="501" ht="14.25" customHeight="true"/>
+    <row r="502" ht="14.25" customHeight="true"/>
+    <row r="503" ht="14.25" customHeight="true"/>
+    <row r="504" ht="14.25" customHeight="true"/>
+    <row r="505" ht="14.25" customHeight="true"/>
+    <row r="506" ht="14.25" customHeight="true"/>
+    <row r="507" ht="14.25" customHeight="true"/>
+    <row r="508" ht="14.25" customHeight="true"/>
+    <row r="509" ht="14.25" customHeight="true"/>
+    <row r="510" ht="14.25" customHeight="true"/>
+    <row r="511" ht="14.25" customHeight="true"/>
+    <row r="512" ht="14.25" customHeight="true"/>
+    <row r="513" ht="14.25" customHeight="true"/>
+    <row r="514" ht="14.25" customHeight="true"/>
+    <row r="515" ht="14.25" customHeight="true"/>
+    <row r="516" ht="14.25" customHeight="true"/>
+    <row r="517" ht="14.25" customHeight="true"/>
+    <row r="518" ht="14.25" customHeight="true"/>
+    <row r="519" ht="14.25" customHeight="true"/>
+    <row r="520" ht="14.25" customHeight="true"/>
+    <row r="521" ht="14.25" customHeight="true"/>
+    <row r="522" ht="14.25" customHeight="true"/>
+    <row r="523" ht="14.25" customHeight="true"/>
+    <row r="524" ht="14.25" customHeight="true"/>
+    <row r="525" ht="14.25" customHeight="true"/>
+    <row r="526" ht="14.25" customHeight="true"/>
+    <row r="527" ht="14.25" customHeight="true"/>
+    <row r="528" ht="14.25" customHeight="true"/>
+    <row r="529" ht="14.25" customHeight="true"/>
+    <row r="530" ht="14.25" customHeight="true"/>
+    <row r="531" ht="14.25" customHeight="true"/>
+    <row r="532" ht="14.25" customHeight="true"/>
+    <row r="533" ht="14.25" customHeight="true"/>
+    <row r="534" ht="14.25" customHeight="true"/>
+    <row r="535" ht="14.25" customHeight="true"/>
+    <row r="536" ht="14.25" customHeight="true"/>
+    <row r="537" ht="14.25" customHeight="true"/>
+    <row r="538" ht="14.25" customHeight="true"/>
+    <row r="539" ht="14.25" customHeight="true"/>
+    <row r="540" ht="14.25" customHeight="true"/>
+    <row r="541" ht="14.25" customHeight="true"/>
+    <row r="542" ht="14.25" customHeight="true"/>
+    <row r="543" ht="14.25" customHeight="true"/>
+    <row r="544" ht="14.25" customHeight="true"/>
+    <row r="545" ht="14.25" customHeight="true"/>
+    <row r="546" ht="14.25" customHeight="true"/>
+    <row r="547" ht="14.25" customHeight="true"/>
+    <row r="548" ht="14.25" customHeight="true"/>
+    <row r="549" ht="14.25" customHeight="true"/>
+    <row r="550" ht="14.25" customHeight="true"/>
+    <row r="551" ht="14.25" customHeight="true"/>
+    <row r="552" ht="14.25" customHeight="true"/>
+    <row r="553" ht="14.25" customHeight="true"/>
+    <row r="554" ht="14.25" customHeight="true"/>
+    <row r="555" ht="14.25" customHeight="true"/>
+    <row r="556" ht="14.25" customHeight="true"/>
+    <row r="557" ht="14.25" customHeight="true"/>
+    <row r="558" ht="14.25" customHeight="true"/>
+    <row r="559" ht="14.25" customHeight="true"/>
+    <row r="560" ht="14.25" customHeight="true"/>
+    <row r="561" ht="14.25" customHeight="true"/>
+    <row r="562" ht="14.25" customHeight="true"/>
+    <row r="563" ht="14.25" customHeight="true"/>
+    <row r="564" ht="14.25" customHeight="true"/>
+    <row r="565" ht="14.25" customHeight="true"/>
+    <row r="566" ht="14.25" customHeight="true"/>
+    <row r="567" ht="14.25" customHeight="true"/>
+    <row r="568" ht="14.25" customHeight="true"/>
+    <row r="569" ht="14.25" customHeight="true"/>
+    <row r="570" ht="14.25" customHeight="true"/>
+    <row r="571" ht="14.25" customHeight="true"/>
+    <row r="572" ht="14.25" customHeight="true"/>
+    <row r="573" ht="14.25" customHeight="true"/>
+    <row r="574" ht="14.25" customHeight="true"/>
+    <row r="575" ht="14.25" customHeight="true"/>
+    <row r="576" ht="14.25" customHeight="true"/>
+    <row r="577" ht="14.25" customHeight="true"/>
+    <row r="578" ht="14.25" customHeight="true"/>
+    <row r="579" ht="14.25" customHeight="true"/>
+    <row r="580" ht="14.25" customHeight="true"/>
+    <row r="581" ht="14.25" customHeight="true"/>
+    <row r="582" ht="14.25" customHeight="true"/>
+    <row r="583" ht="14.25" customHeight="true"/>
+    <row r="584" ht="14.25" customHeight="true"/>
+    <row r="585" ht="14.25" customHeight="true"/>
+    <row r="586" ht="14.25" customHeight="true"/>
+    <row r="587" ht="14.25" customHeight="true"/>
+    <row r="588" ht="14.25" customHeight="true"/>
+    <row r="589" ht="14.25" customHeight="true"/>
+    <row r="590" ht="14.25" customHeight="true"/>
+    <row r="591" ht="14.25" customHeight="true"/>
+    <row r="592" ht="14.25" customHeight="true"/>
+    <row r="593" ht="14.25" customHeight="true"/>
+    <row r="594" ht="14.25" customHeight="true"/>
+    <row r="595" ht="14.25" customHeight="true"/>
+    <row r="596" ht="14.25" customHeight="true"/>
+    <row r="597" ht="14.25" customHeight="true"/>
+    <row r="598" ht="14.25" customHeight="true"/>
+    <row r="599" ht="14.25" customHeight="true"/>
+    <row r="600" ht="14.25" customHeight="true"/>
+    <row r="601" ht="14.25" customHeight="true"/>
+    <row r="602" ht="14.25" customHeight="true"/>
+    <row r="603" ht="14.25" customHeight="true"/>
+    <row r="604" ht="14.25" customHeight="true"/>
+    <row r="605" ht="14.25" customHeight="true"/>
+    <row r="606" ht="14.25" customHeight="true"/>
+    <row r="607" ht="14.25" customHeight="true"/>
+    <row r="608" ht="14.25" customHeight="true"/>
+    <row r="609" ht="14.25" customHeight="true"/>
+    <row r="610" ht="14.25" customHeight="true"/>
+    <row r="611" ht="14.25" customHeight="true"/>
+    <row r="612" ht="14.25" customHeight="true"/>
+    <row r="613" ht="14.25" customHeight="true"/>
+    <row r="614" ht="14.25" customHeight="true"/>
+    <row r="615" ht="14.25" customHeight="true"/>
+    <row r="616" ht="14.25" customHeight="true"/>
+    <row r="617" ht="14.25" customHeight="true"/>
+    <row r="618" ht="14.25" customHeight="true"/>
+    <row r="619" ht="14.25" customHeight="true"/>
+    <row r="620" ht="14.25" customHeight="true"/>
+    <row r="621" ht="14.25" customHeight="true"/>
+    <row r="622" ht="14.25" customHeight="true"/>
+    <row r="623" ht="14.25" customHeight="true"/>
+    <row r="624" ht="14.25" customHeight="true"/>
+    <row r="625" ht="14.25" customHeight="true"/>
+    <row r="626" ht="14.25" customHeight="true"/>
+    <row r="627" ht="14.25" customHeight="true"/>
+    <row r="628" ht="14.25" customHeight="true"/>
+    <row r="629" ht="14.25" customHeight="true"/>
+    <row r="630" ht="14.25" customHeight="true"/>
+    <row r="631" ht="14.25" customHeight="true"/>
+    <row r="632" ht="14.25" customHeight="true"/>
+    <row r="633" ht="14.25" customHeight="true"/>
+    <row r="634" ht="14.25" customHeight="true"/>
+    <row r="635" ht="14.25" customHeight="true"/>
+    <row r="636" ht="14.25" customHeight="true"/>
+    <row r="637" ht="14.25" customHeight="true"/>
+    <row r="638" ht="14.25" customHeight="true"/>
+    <row r="639" ht="14.25" customHeight="true"/>
+    <row r="640" ht="14.25" customHeight="true"/>
+    <row r="641" ht="14.25" customHeight="true"/>
+    <row r="642" ht="14.25" customHeight="true"/>
+    <row r="643" ht="14.25" customHeight="true"/>
+    <row r="644" ht="14.25" customHeight="true"/>
+    <row r="645" ht="14.25" customHeight="true"/>
+    <row r="646" ht="14.25" customHeight="true"/>
+    <row r="647" ht="14.25" customHeight="true"/>
+    <row r="648" ht="14.25" customHeight="true"/>
+    <row r="649" ht="14.25" customHeight="true"/>
+    <row r="650" ht="14.25" customHeight="true"/>
+    <row r="651" ht="14.25" customHeight="true"/>
+    <row r="652" ht="14.25" customHeight="true"/>
+    <row r="653" ht="14.25" customHeight="true"/>
+    <row r="654" ht="14.25" customHeight="true"/>
+    <row r="655" ht="14.25" customHeight="true"/>
+    <row r="656" ht="14.25" customHeight="true"/>
+    <row r="657" ht="14.25" customHeight="true"/>
+    <row r="658" ht="14.25" customHeight="true"/>
+    <row r="659" ht="14.25" customHeight="true"/>
+    <row r="660" ht="14.25" customHeight="true"/>
+    <row r="661" ht="14.25" customHeight="true"/>
+    <row r="662" ht="14.25" customHeight="true"/>
+    <row r="663" ht="14.25" customHeight="true"/>
+    <row r="664" ht="14.25" customHeight="true"/>
+    <row r="665" ht="14.25" customHeight="true"/>
+    <row r="666" ht="14.25" customHeight="true"/>
+    <row r="667" ht="14.25" customHeight="true"/>
+    <row r="668" ht="14.25" customHeight="true"/>
+    <row r="669" ht="14.25" customHeight="true"/>
+    <row r="670" ht="14.25" customHeight="true"/>
+    <row r="671" ht="14.25" customHeight="true"/>
+    <row r="672" ht="14.25" customHeight="true"/>
+    <row r="673" ht="14.25" customHeight="true"/>
+    <row r="674" ht="14.25" customHeight="true"/>
+    <row r="675" ht="14.25" customHeight="true"/>
+    <row r="676" ht="14.25" customHeight="true"/>
+    <row r="677" ht="14.25" customHeight="true"/>
+    <row r="678" ht="14.25" customHeight="true"/>
+    <row r="679" ht="14.25" customHeight="true"/>
+    <row r="680" ht="14.25" customHeight="true"/>
+    <row r="681" ht="14.25" customHeight="true"/>
+    <row r="682" ht="14.25" customHeight="true"/>
+    <row r="683" ht="14.25" customHeight="true"/>
+    <row r="684" ht="14.25" customHeight="true"/>
+    <row r="685" ht="14.25" customHeight="true"/>
+    <row r="686" ht="14.25" customHeight="true"/>
+    <row r="687" ht="14.25" customHeight="true"/>
+    <row r="688" ht="14.25" customHeight="true"/>
+    <row r="689" ht="14.25" customHeight="true"/>
+    <row r="690" ht="14.25" customHeight="true"/>
+    <row r="691" ht="14.25" customHeight="true"/>
+    <row r="692" ht="14.25" customHeight="true"/>
+    <row r="693" ht="14.25" customHeight="true"/>
+    <row r="694" ht="14.25" customHeight="true"/>
+    <row r="695" ht="14.25" customHeight="true"/>
+    <row r="696" ht="14.25" customHeight="true"/>
+    <row r="697" ht="14.25" customHeight="true"/>
+    <row r="698" ht="14.25" customHeight="true"/>
+    <row r="699" ht="14.25" customHeight="true"/>
+    <row r="700" ht="14.25" customHeight="true"/>
+    <row r="701" ht="14.25" customHeight="true"/>
+    <row r="702" ht="14.25" customHeight="true"/>
+    <row r="703" ht="14.25" customHeight="true"/>
+    <row r="704" ht="14.25" customHeight="true"/>
+    <row r="705" ht="14.25" customHeight="true"/>
+    <row r="706" ht="14.25" customHeight="true"/>
+    <row r="707" ht="14.25" customHeight="true"/>
+    <row r="708" ht="14.25" customHeight="true"/>
+    <row r="709" ht="14.25" customHeight="true"/>
+    <row r="710" ht="14.25" customHeight="true"/>
+    <row r="711" ht="14.25" customHeight="true"/>
+    <row r="712" ht="14.25" customHeight="true"/>
+    <row r="713" ht="14.25" customHeight="true"/>
+    <row r="714" ht="14.25" customHeight="true"/>
+    <row r="715" ht="14.25" customHeight="true"/>
+    <row r="716" ht="14.25" customHeight="true"/>
+    <row r="717" ht="14.25" customHeight="true"/>
+    <row r="718" ht="14.25" customHeight="true"/>
+    <row r="719" ht="14.25" customHeight="true"/>
+    <row r="720" ht="14.25" customHeight="true"/>
+    <row r="721" ht="14.25" customHeight="true"/>
+    <row r="722" ht="14.25" customHeight="true"/>
+    <row r="723" ht="14.25" customHeight="true"/>
+    <row r="724" ht="14.25" customHeight="true"/>
+    <row r="725" ht="14.25" customHeight="true"/>
+    <row r="726" ht="14.25" customHeight="true"/>
+    <row r="727" ht="14.25" customHeight="true"/>
+    <row r="728" ht="14.25" customHeight="true"/>
+    <row r="729" ht="14.25" customHeight="true"/>
+    <row r="730" ht="14.25" customHeight="true"/>
+    <row r="731" ht="14.25" customHeight="true"/>
+    <row r="732" ht="14.25" customHeight="true"/>
+    <row r="733" ht="14.25" customHeight="true"/>
+    <row r="734" ht="14.25" customHeight="true"/>
+    <row r="735" ht="14.25" customHeight="true"/>
+    <row r="736" ht="14.25" customHeight="true"/>
+    <row r="737" ht="14.25" customHeight="true"/>
+    <row r="738" ht="14.25" customHeight="true"/>
+    <row r="739" ht="14.25" customHeight="true"/>
+    <row r="740" ht="14.25" customHeight="true"/>
+    <row r="741" ht="14.25" customHeight="true"/>
+    <row r="742" ht="14.25" customHeight="true"/>
+    <row r="743" ht="14.25" customHeight="true"/>
+    <row r="744" ht="14.25" customHeight="true"/>
+    <row r="745" ht="14.25" customHeight="true"/>
+    <row r="746" ht="14.25" customHeight="true"/>
+    <row r="747" ht="14.25" customHeight="true"/>
+    <row r="748" ht="14.25" customHeight="true"/>
+    <row r="749" ht="14.25" customHeight="true"/>
+    <row r="750" ht="14.25" customHeight="true"/>
+    <row r="751" ht="14.25" customHeight="true"/>
+    <row r="752" ht="14.25" customHeight="true"/>
+    <row r="753" ht="14.25" customHeight="true"/>
+    <row r="754" ht="14.25" customHeight="true"/>
+    <row r="755" ht="14.25" customHeight="true"/>
+    <row r="756" ht="14.25" customHeight="true"/>
+    <row r="757" ht="14.25" customHeight="true"/>
+    <row r="758" ht="14.25" customHeight="true"/>
+    <row r="759" ht="14.25" customHeight="true"/>
+    <row r="760" ht="14.25" customHeight="true"/>
+    <row r="761" ht="14.25" customHeight="true"/>
+    <row r="762" ht="14.25" customHeight="true"/>
+    <row r="763" ht="14.25" customHeight="true"/>
+    <row r="764" ht="14.25" customHeight="true"/>
+    <row r="765" ht="14.25" customHeight="true"/>
+    <row r="766" ht="14.25" customHeight="true"/>
+    <row r="767" ht="14.25" customHeight="true"/>
+    <row r="768" ht="14.25" customHeight="true"/>
+    <row r="769" ht="14.25" customHeight="true"/>
+    <row r="770" ht="14.25" customHeight="true"/>
+    <row r="771" ht="14.25" customHeight="true"/>
+    <row r="772" ht="14.25" customHeight="true"/>
+    <row r="773" ht="14.25" customHeight="true"/>
+    <row r="774" ht="14.25" customHeight="true"/>
+    <row r="775" ht="14.25" customHeight="true"/>
+    <row r="776" ht="14.25" customHeight="true"/>
+    <row r="777" ht="14.25" customHeight="true"/>
+    <row r="778" ht="14.25" customHeight="true"/>
+    <row r="779" ht="14.25" customHeight="true"/>
+    <row r="780" ht="14.25" customHeight="true"/>
+    <row r="781" ht="14.25" customHeight="true"/>
+    <row r="782" ht="14.25" customHeight="true"/>
+    <row r="783" ht="14.25" customHeight="true"/>
+    <row r="784" ht="14.25" customHeight="true"/>
+    <row r="785" ht="14.25" customHeight="true"/>
+    <row r="786" ht="14.25" customHeight="true"/>
+    <row r="787" ht="14.25" customHeight="true"/>
+    <row r="788" ht="14.25" customHeight="true"/>
+    <row r="789" ht="14.25" customHeight="true"/>
+    <row r="790" ht="14.25" customHeight="true"/>
+    <row r="791" ht="14.25" customHeight="true"/>
+    <row r="792" ht="14.25" customHeight="true"/>
+    <row r="793" ht="14.25" customHeight="true"/>
+    <row r="794" ht="14.25" customHeight="true"/>
+    <row r="795" ht="14.25" customHeight="true"/>
+    <row r="796" ht="14.25" customHeight="true"/>
+    <row r="797" ht="14.25" customHeight="true"/>
+    <row r="798" ht="14.25" customHeight="true"/>
+    <row r="799" ht="14.25" customHeight="true"/>
+    <row r="800" ht="14.25" customHeight="true"/>
+    <row r="801" ht="14.25" customHeight="true"/>
+    <row r="802" ht="14.25" customHeight="true"/>
+    <row r="803" ht="14.25" customHeight="true"/>
+    <row r="804" ht="14.25" customHeight="true"/>
+    <row r="805" ht="14.25" customHeight="true"/>
+    <row r="806" ht="14.25" customHeight="true"/>
+    <row r="807" ht="14.25" customHeight="true"/>
+    <row r="808" ht="14.25" customHeight="true"/>
+    <row r="809" ht="14.25" customHeight="true"/>
+    <row r="810" ht="14.25" customHeight="true"/>
+    <row r="811" ht="14.25" customHeight="true"/>
+    <row r="812" ht="14.25" customHeight="true"/>
+    <row r="813" ht="14.25" customHeight="true"/>
+    <row r="814" ht="14.25" customHeight="true"/>
+    <row r="815" ht="14.25" customHeight="true"/>
+    <row r="816" ht="14.25" customHeight="true"/>
+    <row r="817" ht="14.25" customHeight="true"/>
+    <row r="818" ht="14.25" customHeight="true"/>
+    <row r="819" ht="14.25" customHeight="true"/>
+    <row r="820" ht="14.25" customHeight="true"/>
+    <row r="821" ht="14.25" customHeight="true"/>
+    <row r="822" ht="14.25" customHeight="true"/>
+    <row r="823" ht="14.25" customHeight="true"/>
+    <row r="824" ht="14.25" customHeight="true"/>
+    <row r="825" ht="14.25" customHeight="true"/>
+    <row r="826" ht="14.25" customHeight="true"/>
+    <row r="827" ht="14.25" customHeight="true"/>
+    <row r="828" ht="14.25" customHeight="true"/>
+    <row r="829" ht="14.25" customHeight="true"/>
+    <row r="830" ht="14.25" customHeight="true"/>
+    <row r="831" ht="14.25" customHeight="true"/>
+    <row r="832" ht="14.25" customHeight="true"/>
+    <row r="833" ht="14.25" customHeight="true"/>
+    <row r="834" ht="14.25" customHeight="true"/>
+    <row r="835" ht="14.25" customHeight="true"/>
+    <row r="836" ht="14.25" customHeight="true"/>
+    <row r="837" ht="14.25" customHeight="true"/>
+    <row r="838" ht="14.25" customHeight="true"/>
+    <row r="839" ht="14.25" customHeight="true"/>
+    <row r="840" ht="14.25" customHeight="true"/>
+    <row r="841" ht="14.25" customHeight="true"/>
+    <row r="842" ht="14.25" customHeight="true"/>
+    <row r="843" ht="14.25" customHeight="true"/>
+    <row r="844" ht="14.25" customHeight="true"/>
+    <row r="845" ht="14.25" customHeight="true"/>
+    <row r="846" ht="14.25" customHeight="true"/>
+    <row r="847" ht="14.25" customHeight="true"/>
+    <row r="848" ht="14.25" customHeight="true"/>
+    <row r="849" ht="14.25" customHeight="true"/>
+    <row r="850" ht="14.25" customHeight="true"/>
+    <row r="851" ht="14.25" customHeight="true"/>
+    <row r="852" ht="14.25" customHeight="true"/>
+    <row r="853" ht="14.25" customHeight="true"/>
+    <row r="854" ht="14.25" customHeight="true"/>
+    <row r="855" ht="14.25" customHeight="true"/>
+    <row r="856" ht="14.25" customHeight="true"/>
+    <row r="857" ht="14.25" customHeight="true"/>
+    <row r="858" ht="14.25" customHeight="true"/>
+    <row r="859" ht="14.25" customHeight="true"/>
+    <row r="860" ht="14.25" customHeight="true"/>
+    <row r="861" ht="14.25" customHeight="true"/>
+    <row r="862" ht="14.25" customHeight="true"/>
+    <row r="863" ht="14.25" customHeight="true"/>
+    <row r="864" ht="14.25" customHeight="true"/>
+    <row r="865" ht="14.25" customHeight="true"/>
+    <row r="866" ht="14.25" customHeight="true"/>
+    <row r="867" ht="14.25" customHeight="true"/>
+    <row r="868" ht="14.25" customHeight="true"/>
+    <row r="869" ht="14.25" customHeight="true"/>
+    <row r="870" ht="14.25" customHeight="true"/>
+    <row r="871" ht="14.25" customHeight="true"/>
+    <row r="872" ht="14.25" customHeight="true"/>
+    <row r="873" ht="14.25" customHeight="true"/>
+    <row r="874" ht="14.25" customHeight="true"/>
+    <row r="875" ht="14.25" customHeight="true"/>
+    <row r="876" ht="14.25" customHeight="true"/>
+    <row r="877" ht="14.25" customHeight="true"/>
+    <row r="878" ht="14.25" customHeight="true"/>
+    <row r="879" ht="14.25" customHeight="true"/>
+    <row r="880" ht="14.25" customHeight="true"/>
+    <row r="881" ht="14.25" customHeight="true"/>
+    <row r="882" ht="14.25" customHeight="true"/>
+    <row r="883" ht="14.25" customHeight="true"/>
+    <row r="884" ht="14.25" customHeight="true"/>
+    <row r="885" ht="14.25" customHeight="true"/>
+    <row r="886" ht="14.25" customHeight="true"/>
+    <row r="887" ht="14.25" customHeight="true"/>
+    <row r="888" ht="14.25" customHeight="true"/>
+    <row r="889" ht="14.25" customHeight="true"/>
+    <row r="890" ht="14.25" customHeight="true"/>
+    <row r="891" ht="14.25" customHeight="true"/>
+    <row r="892" ht="14.25" customHeight="true"/>
+    <row r="893" ht="14.25" customHeight="true"/>
+    <row r="894" ht="14.25" customHeight="true"/>
+    <row r="895" ht="14.25" customHeight="true"/>
+    <row r="896" ht="14.25" customHeight="true"/>
+    <row r="897" ht="14.25" customHeight="true"/>
+    <row r="898" ht="14.25" customHeight="true"/>
+    <row r="899" ht="14.25" customHeight="true"/>
+    <row r="900" ht="14.25" customHeight="true"/>
+    <row r="901" ht="14.25" customHeight="true"/>
+    <row r="902" ht="14.25" customHeight="true"/>
+    <row r="903" ht="14.25" customHeight="true"/>
+    <row r="904" ht="14.25" customHeight="true"/>
+    <row r="905" ht="14.25" customHeight="true"/>
+    <row r="906" ht="14.25" customHeight="true"/>
+    <row r="907" ht="14.25" customHeight="true"/>
+    <row r="908" ht="14.25" customHeight="true"/>
+    <row r="909" ht="14.25" customHeight="true"/>
+    <row r="910" ht="14.25" customHeight="true"/>
+    <row r="911" ht="14.25" customHeight="true"/>
+    <row r="912" ht="14.25" customHeight="true"/>
+    <row r="913" ht="14.25" customHeight="true"/>
+    <row r="914" ht="14.25" customHeight="true"/>
+    <row r="915" ht="14.25" customHeight="true"/>
+    <row r="916" ht="14.25" customHeight="true"/>
+    <row r="917" ht="14.25" customHeight="true"/>
+    <row r="918" ht="14.25" customHeight="true"/>
+    <row r="919" ht="14.25" customHeight="true"/>
+    <row r="920" ht="14.25" customHeight="true"/>
+    <row r="921" ht="14.25" customHeight="true"/>
+    <row r="922" ht="14.25" customHeight="true"/>
+    <row r="923" ht="14.25" customHeight="true"/>
+    <row r="924" ht="14.25" customHeight="true"/>
+    <row r="925" ht="14.25" customHeight="true"/>
+    <row r="926" ht="14.25" customHeight="true"/>
+    <row r="927" ht="14.25" customHeight="true"/>
+    <row r="928" ht="14.25" customHeight="true"/>
+    <row r="929" ht="14.25" customHeight="true"/>
+    <row r="930" ht="14.25" customHeight="true"/>
+    <row r="931" ht="14.25" customHeight="true"/>
+    <row r="932" ht="14.25" customHeight="true"/>
+    <row r="933" ht="14.25" customHeight="true"/>
+    <row r="934" ht="14.25" customHeight="true"/>
+    <row r="935" ht="14.25" customHeight="true"/>
+    <row r="936" ht="14.25" customHeight="true"/>
+    <row r="937" ht="14.25" customHeight="true"/>
+    <row r="938" ht="14.25" customHeight="true"/>
+    <row r="939" ht="14.25" customHeight="true"/>
+    <row r="940" ht="14.25" customHeight="true"/>
+    <row r="941" ht="14.25" customHeight="true"/>
+    <row r="942" ht="14.25" customHeight="true"/>
+    <row r="943" ht="14.25" customHeight="true"/>
+    <row r="944" ht="14.25" customHeight="true"/>
+    <row r="945" ht="14.25" customHeight="true"/>
+    <row r="946" ht="14.25" customHeight="true"/>
+    <row r="947" ht="14.25" customHeight="true"/>
+    <row r="948" ht="14.25" customHeight="true"/>
+    <row r="949" ht="14.25" customHeight="true"/>
+    <row r="950" ht="14.25" customHeight="true"/>
+    <row r="951" ht="14.25" customHeight="true"/>
+    <row r="952" ht="14.25" customHeight="true"/>
+    <row r="953" ht="14.25" customHeight="true"/>
+    <row r="954" ht="14.25" customHeight="true"/>
+    <row r="955" ht="14.25" customHeight="true"/>
+    <row r="956" ht="14.25" customHeight="true"/>
+    <row r="957" ht="14.25" customHeight="true"/>
+    <row r="958" ht="14.25" customHeight="true"/>
+    <row r="959" ht="14.25" customHeight="true"/>
+    <row r="960" ht="14.25" customHeight="true"/>
+    <row r="961" ht="14.25" customHeight="true"/>
+    <row r="962" ht="14.25" customHeight="true"/>
+    <row r="963" ht="14.25" customHeight="true"/>
+    <row r="964" ht="14.25" customHeight="true"/>
+    <row r="965" ht="14.25" customHeight="true"/>
+    <row r="966" ht="14.25" customHeight="true"/>
+    <row r="967" ht="14.25" customHeight="true"/>
+    <row r="968" ht="14.25" customHeight="true"/>
+    <row r="969" ht="14.25" customHeight="true"/>
+    <row r="970" ht="14.25" customHeight="true"/>
+    <row r="971" ht="14.25" customHeight="true"/>
+    <row r="972" ht="14.25" customHeight="true"/>
+    <row r="973" ht="14.25" customHeight="true"/>
+    <row r="974" ht="14.25" customHeight="true"/>
+    <row r="975" ht="14.25" customHeight="true"/>
+    <row r="976" ht="14.25" customHeight="true"/>
+    <row r="977" ht="14.25" customHeight="true"/>
+    <row r="978" ht="14.25" customHeight="true"/>
+    <row r="979" ht="14.25" customHeight="true"/>
+    <row r="980" ht="14.25" customHeight="true"/>
+    <row r="981" ht="14.25" customHeight="true"/>
+    <row r="982" ht="14.25" customHeight="true"/>
+    <row r="983" ht="14.25" customHeight="true"/>
+    <row r="984" ht="14.25" customHeight="true"/>
+    <row r="985" ht="14.25" customHeight="true"/>
+    <row r="986" ht="14.25" customHeight="true"/>
+    <row r="987" ht="14.25" customHeight="true"/>
+    <row r="988" ht="14.25" customHeight="true"/>
+    <row r="989" ht="14.25" customHeight="true"/>
+    <row r="990" ht="14.25" customHeight="true"/>
+    <row r="991" ht="14.25" customHeight="true"/>
+    <row r="992" ht="14.25" customHeight="true"/>
+    <row r="993" ht="14.25" customHeight="true"/>
+    <row r="994" ht="14.25" customHeight="true"/>
+    <row r="995" ht="14.25" customHeight="true"/>
+    <row r="996" ht="14.25" customHeight="true"/>
+    <row r="997" ht="14.25" customHeight="true"/>
+    <row r="998" ht="14.25" customHeight="true"/>
+    <row r="999" ht="14.25" customHeight="true"/>
+    <row r="1000" ht="14.25" customHeight="true"/>
   </sheetData>
   <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -3490,14 +3490,14 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="true"/>
   <cols>
-    <col customWidth="1" min="1" max="2" width="8.71"/>
-    <col customWidth="1" min="3" max="3" width="26.71"/>
-    <col customWidth="1" min="4" max="26" width="8.71"/>
+    <col customWidth="true" max="2" min="1" width="8.71"/>
+    <col customWidth="true" max="3" min="3" width="26.71"/>
+    <col customWidth="true" max="26" min="4" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
+    <row r="1" ht="14.25" customHeight="true">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1">
+    <row r="2" ht="14.25" customHeight="true">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -3519,1007 +3519,1007 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1"/>
-    <row r="4" ht="14.25" customHeight="1"/>
-    <row r="5" ht="14.25" customHeight="1"/>
-    <row r="6" ht="14.25" customHeight="1"/>
-    <row r="7" ht="14.25" customHeight="1"/>
-    <row r="8" ht="14.25" customHeight="1"/>
-    <row r="9" ht="14.25" customHeight="1"/>
-    <row r="10" ht="14.25" customHeight="1"/>
-    <row r="11" ht="14.25" customHeight="1"/>
-    <row r="12" ht="14.25" customHeight="1"/>
-    <row r="13" ht="14.25" customHeight="1"/>
-    <row r="14" ht="14.25" customHeight="1"/>
-    <row r="15" ht="14.25" customHeight="1"/>
-    <row r="16" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
-    <row r="65" ht="14.25" customHeight="1"/>
-    <row r="66" ht="14.25" customHeight="1"/>
-    <row r="67" ht="14.25" customHeight="1"/>
-    <row r="68" ht="14.25" customHeight="1"/>
-    <row r="69" ht="14.25" customHeight="1"/>
-    <row r="70" ht="14.25" customHeight="1"/>
-    <row r="71" ht="14.25" customHeight="1"/>
-    <row r="72" ht="14.25" customHeight="1"/>
-    <row r="73" ht="14.25" customHeight="1"/>
-    <row r="74" ht="14.25" customHeight="1"/>
-    <row r="75" ht="14.25" customHeight="1"/>
-    <row r="76" ht="14.25" customHeight="1"/>
-    <row r="77" ht="14.25" customHeight="1"/>
-    <row r="78" ht="14.25" customHeight="1"/>
-    <row r="79" ht="14.25" customHeight="1"/>
-    <row r="80" ht="14.25" customHeight="1"/>
-    <row r="81" ht="14.25" customHeight="1"/>
-    <row r="82" ht="14.25" customHeight="1"/>
-    <row r="83" ht="14.25" customHeight="1"/>
-    <row r="84" ht="14.25" customHeight="1"/>
-    <row r="85" ht="14.25" customHeight="1"/>
-    <row r="86" ht="14.25" customHeight="1"/>
-    <row r="87" ht="14.25" customHeight="1"/>
-    <row r="88" ht="14.25" customHeight="1"/>
-    <row r="89" ht="14.25" customHeight="1"/>
-    <row r="90" ht="14.25" customHeight="1"/>
-    <row r="91" ht="14.25" customHeight="1"/>
-    <row r="92" ht="14.25" customHeight="1"/>
-    <row r="93" ht="14.25" customHeight="1"/>
-    <row r="94" ht="14.25" customHeight="1"/>
-    <row r="95" ht="14.25" customHeight="1"/>
-    <row r="96" ht="14.25" customHeight="1"/>
-    <row r="97" ht="14.25" customHeight="1"/>
-    <row r="98" ht="14.25" customHeight="1"/>
-    <row r="99" ht="14.25" customHeight="1"/>
-    <row r="100" ht="14.25" customHeight="1"/>
-    <row r="101" ht="14.25" customHeight="1"/>
-    <row r="102" ht="14.25" customHeight="1"/>
-    <row r="103" ht="14.25" customHeight="1"/>
-    <row r="104" ht="14.25" customHeight="1"/>
-    <row r="105" ht="14.25" customHeight="1"/>
-    <row r="106" ht="14.25" customHeight="1"/>
-    <row r="107" ht="14.25" customHeight="1"/>
-    <row r="108" ht="14.25" customHeight="1"/>
-    <row r="109" ht="14.25" customHeight="1"/>
-    <row r="110" ht="14.25" customHeight="1"/>
-    <row r="111" ht="14.25" customHeight="1"/>
-    <row r="112" ht="14.25" customHeight="1"/>
-    <row r="113" ht="14.25" customHeight="1"/>
-    <row r="114" ht="14.25" customHeight="1"/>
-    <row r="115" ht="14.25" customHeight="1"/>
-    <row r="116" ht="14.25" customHeight="1"/>
-    <row r="117" ht="14.25" customHeight="1"/>
-    <row r="118" ht="14.25" customHeight="1"/>
-    <row r="119" ht="14.25" customHeight="1"/>
-    <row r="120" ht="14.25" customHeight="1"/>
-    <row r="121" ht="14.25" customHeight="1"/>
-    <row r="122" ht="14.25" customHeight="1"/>
-    <row r="123" ht="14.25" customHeight="1"/>
-    <row r="124" ht="14.25" customHeight="1"/>
-    <row r="125" ht="14.25" customHeight="1"/>
-    <row r="126" ht="14.25" customHeight="1"/>
-    <row r="127" ht="14.25" customHeight="1"/>
-    <row r="128" ht="14.25" customHeight="1"/>
-    <row r="129" ht="14.25" customHeight="1"/>
-    <row r="130" ht="14.25" customHeight="1"/>
-    <row r="131" ht="14.25" customHeight="1"/>
-    <row r="132" ht="14.25" customHeight="1"/>
-    <row r="133" ht="14.25" customHeight="1"/>
-    <row r="134" ht="14.25" customHeight="1"/>
-    <row r="135" ht="14.25" customHeight="1"/>
-    <row r="136" ht="14.25" customHeight="1"/>
-    <row r="137" ht="14.25" customHeight="1"/>
-    <row r="138" ht="14.25" customHeight="1"/>
-    <row r="139" ht="14.25" customHeight="1"/>
-    <row r="140" ht="14.25" customHeight="1"/>
-    <row r="141" ht="14.25" customHeight="1"/>
-    <row r="142" ht="14.25" customHeight="1"/>
-    <row r="143" ht="14.25" customHeight="1"/>
-    <row r="144" ht="14.25" customHeight="1"/>
-    <row r="145" ht="14.25" customHeight="1"/>
-    <row r="146" ht="14.25" customHeight="1"/>
-    <row r="147" ht="14.25" customHeight="1"/>
-    <row r="148" ht="14.25" customHeight="1"/>
-    <row r="149" ht="14.25" customHeight="1"/>
-    <row r="150" ht="14.25" customHeight="1"/>
-    <row r="151" ht="14.25" customHeight="1"/>
-    <row r="152" ht="14.25" customHeight="1"/>
-    <row r="153" ht="14.25" customHeight="1"/>
-    <row r="154" ht="14.25" customHeight="1"/>
-    <row r="155" ht="14.25" customHeight="1"/>
-    <row r="156" ht="14.25" customHeight="1"/>
-    <row r="157" ht="14.25" customHeight="1"/>
-    <row r="158" ht="14.25" customHeight="1"/>
-    <row r="159" ht="14.25" customHeight="1"/>
-    <row r="160" ht="14.25" customHeight="1"/>
-    <row r="161" ht="14.25" customHeight="1"/>
-    <row r="162" ht="14.25" customHeight="1"/>
-    <row r="163" ht="14.25" customHeight="1"/>
-    <row r="164" ht="14.25" customHeight="1"/>
-    <row r="165" ht="14.25" customHeight="1"/>
-    <row r="166" ht="14.25" customHeight="1"/>
-    <row r="167" ht="14.25" customHeight="1"/>
-    <row r="168" ht="14.25" customHeight="1"/>
-    <row r="169" ht="14.25" customHeight="1"/>
-    <row r="170" ht="14.25" customHeight="1"/>
-    <row r="171" ht="14.25" customHeight="1"/>
-    <row r="172" ht="14.25" customHeight="1"/>
-    <row r="173" ht="14.25" customHeight="1"/>
-    <row r="174" ht="14.25" customHeight="1"/>
-    <row r="175" ht="14.25" customHeight="1"/>
-    <row r="176" ht="14.25" customHeight="1"/>
-    <row r="177" ht="14.25" customHeight="1"/>
-    <row r="178" ht="14.25" customHeight="1"/>
-    <row r="179" ht="14.25" customHeight="1"/>
-    <row r="180" ht="14.25" customHeight="1"/>
-    <row r="181" ht="14.25" customHeight="1"/>
-    <row r="182" ht="14.25" customHeight="1"/>
-    <row r="183" ht="14.25" customHeight="1"/>
-    <row r="184" ht="14.25" customHeight="1"/>
-    <row r="185" ht="14.25" customHeight="1"/>
-    <row r="186" ht="14.25" customHeight="1"/>
-    <row r="187" ht="14.25" customHeight="1"/>
-    <row r="188" ht="14.25" customHeight="1"/>
-    <row r="189" ht="14.25" customHeight="1"/>
-    <row r="190" ht="14.25" customHeight="1"/>
-    <row r="191" ht="14.25" customHeight="1"/>
-    <row r="192" ht="14.25" customHeight="1"/>
-    <row r="193" ht="14.25" customHeight="1"/>
-    <row r="194" ht="14.25" customHeight="1"/>
-    <row r="195" ht="14.25" customHeight="1"/>
-    <row r="196" ht="14.25" customHeight="1"/>
-    <row r="197" ht="14.25" customHeight="1"/>
-    <row r="198" ht="14.25" customHeight="1"/>
-    <row r="199" ht="14.25" customHeight="1"/>
-    <row r="200" ht="14.25" customHeight="1"/>
-    <row r="201" ht="14.25" customHeight="1"/>
-    <row r="202" ht="14.25" customHeight="1"/>
-    <row r="203" ht="14.25" customHeight="1"/>
-    <row r="204" ht="14.25" customHeight="1"/>
-    <row r="205" ht="14.25" customHeight="1"/>
-    <row r="206" ht="14.25" customHeight="1"/>
-    <row r="207" ht="14.25" customHeight="1"/>
-    <row r="208" ht="14.25" customHeight="1"/>
-    <row r="209" ht="14.25" customHeight="1"/>
-    <row r="210" ht="14.25" customHeight="1"/>
-    <row r="211" ht="14.25" customHeight="1"/>
-    <row r="212" ht="14.25" customHeight="1"/>
-    <row r="213" ht="14.25" customHeight="1"/>
-    <row r="214" ht="14.25" customHeight="1"/>
-    <row r="215" ht="14.25" customHeight="1"/>
-    <row r="216" ht="14.25" customHeight="1"/>
-    <row r="217" ht="14.25" customHeight="1"/>
-    <row r="218" ht="14.25" customHeight="1"/>
-    <row r="219" ht="14.25" customHeight="1"/>
-    <row r="220" ht="14.25" customHeight="1"/>
-    <row r="221" ht="14.25" customHeight="1"/>
-    <row r="222" ht="14.25" customHeight="1"/>
-    <row r="223" ht="14.25" customHeight="1"/>
-    <row r="224" ht="14.25" customHeight="1"/>
-    <row r="225" ht="14.25" customHeight="1"/>
-    <row r="226" ht="14.25" customHeight="1"/>
-    <row r="227" ht="14.25" customHeight="1"/>
-    <row r="228" ht="14.25" customHeight="1"/>
-    <row r="229" ht="14.25" customHeight="1"/>
-    <row r="230" ht="14.25" customHeight="1"/>
-    <row r="231" ht="14.25" customHeight="1"/>
-    <row r="232" ht="14.25" customHeight="1"/>
-    <row r="233" ht="14.25" customHeight="1"/>
-    <row r="234" ht="14.25" customHeight="1"/>
-    <row r="235" ht="14.25" customHeight="1"/>
-    <row r="236" ht="14.25" customHeight="1"/>
-    <row r="237" ht="14.25" customHeight="1"/>
-    <row r="238" ht="14.25" customHeight="1"/>
-    <row r="239" ht="14.25" customHeight="1"/>
-    <row r="240" ht="14.25" customHeight="1"/>
-    <row r="241" ht="14.25" customHeight="1"/>
-    <row r="242" ht="14.25" customHeight="1"/>
-    <row r="243" ht="14.25" customHeight="1"/>
-    <row r="244" ht="14.25" customHeight="1"/>
-    <row r="245" ht="14.25" customHeight="1"/>
-    <row r="246" ht="14.25" customHeight="1"/>
-    <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
-    <row r="249" ht="14.25" customHeight="1"/>
-    <row r="250" ht="14.25" customHeight="1"/>
-    <row r="251" ht="14.25" customHeight="1"/>
-    <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1"/>
-    <row r="254" ht="14.25" customHeight="1"/>
-    <row r="255" ht="14.25" customHeight="1"/>
-    <row r="256" ht="14.25" customHeight="1"/>
-    <row r="257" ht="14.25" customHeight="1"/>
-    <row r="258" ht="14.25" customHeight="1"/>
-    <row r="259" ht="14.25" customHeight="1"/>
-    <row r="260" ht="14.25" customHeight="1"/>
-    <row r="261" ht="14.25" customHeight="1"/>
-    <row r="262" ht="14.25" customHeight="1"/>
-    <row r="263" ht="14.25" customHeight="1"/>
-    <row r="264" ht="14.25" customHeight="1"/>
-    <row r="265" ht="14.25" customHeight="1"/>
-    <row r="266" ht="14.25" customHeight="1"/>
-    <row r="267" ht="14.25" customHeight="1"/>
-    <row r="268" ht="14.25" customHeight="1"/>
-    <row r="269" ht="14.25" customHeight="1"/>
-    <row r="270" ht="14.25" customHeight="1"/>
-    <row r="271" ht="14.25" customHeight="1"/>
-    <row r="272" ht="14.25" customHeight="1"/>
-    <row r="273" ht="14.25" customHeight="1"/>
-    <row r="274" ht="14.25" customHeight="1"/>
-    <row r="275" ht="14.25" customHeight="1"/>
-    <row r="276" ht="14.25" customHeight="1"/>
-    <row r="277" ht="14.25" customHeight="1"/>
-    <row r="278" ht="14.25" customHeight="1"/>
-    <row r="279" ht="14.25" customHeight="1"/>
-    <row r="280" ht="14.25" customHeight="1"/>
-    <row r="281" ht="14.25" customHeight="1"/>
-    <row r="282" ht="14.25" customHeight="1"/>
-    <row r="283" ht="14.25" customHeight="1"/>
-    <row r="284" ht="14.25" customHeight="1"/>
-    <row r="285" ht="14.25" customHeight="1"/>
-    <row r="286" ht="14.25" customHeight="1"/>
-    <row r="287" ht="14.25" customHeight="1"/>
-    <row r="288" ht="14.25" customHeight="1"/>
-    <row r="289" ht="14.25" customHeight="1"/>
-    <row r="290" ht="14.25" customHeight="1"/>
-    <row r="291" ht="14.25" customHeight="1"/>
-    <row r="292" ht="14.25" customHeight="1"/>
-    <row r="293" ht="14.25" customHeight="1"/>
-    <row r="294" ht="14.25" customHeight="1"/>
-    <row r="295" ht="14.25" customHeight="1"/>
-    <row r="296" ht="14.25" customHeight="1"/>
-    <row r="297" ht="14.25" customHeight="1"/>
-    <row r="298" ht="14.25" customHeight="1"/>
-    <row r="299" ht="14.25" customHeight="1"/>
-    <row r="300" ht="14.25" customHeight="1"/>
-    <row r="301" ht="14.25" customHeight="1"/>
-    <row r="302" ht="14.25" customHeight="1"/>
-    <row r="303" ht="14.25" customHeight="1"/>
-    <row r="304" ht="14.25" customHeight="1"/>
-    <row r="305" ht="14.25" customHeight="1"/>
-    <row r="306" ht="14.25" customHeight="1"/>
-    <row r="307" ht="14.25" customHeight="1"/>
-    <row r="308" ht="14.25" customHeight="1"/>
-    <row r="309" ht="14.25" customHeight="1"/>
-    <row r="310" ht="14.25" customHeight="1"/>
-    <row r="311" ht="14.25" customHeight="1"/>
-    <row r="312" ht="14.25" customHeight="1"/>
-    <row r="313" ht="14.25" customHeight="1"/>
-    <row r="314" ht="14.25" customHeight="1"/>
-    <row r="315" ht="14.25" customHeight="1"/>
-    <row r="316" ht="14.25" customHeight="1"/>
-    <row r="317" ht="14.25" customHeight="1"/>
-    <row r="318" ht="14.25" customHeight="1"/>
-    <row r="319" ht="14.25" customHeight="1"/>
-    <row r="320" ht="14.25" customHeight="1"/>
-    <row r="321" ht="14.25" customHeight="1"/>
-    <row r="322" ht="14.25" customHeight="1"/>
-    <row r="323" ht="14.25" customHeight="1"/>
-    <row r="324" ht="14.25" customHeight="1"/>
-    <row r="325" ht="14.25" customHeight="1"/>
-    <row r="326" ht="14.25" customHeight="1"/>
-    <row r="327" ht="14.25" customHeight="1"/>
-    <row r="328" ht="14.25" customHeight="1"/>
-    <row r="329" ht="14.25" customHeight="1"/>
-    <row r="330" ht="14.25" customHeight="1"/>
-    <row r="331" ht="14.25" customHeight="1"/>
-    <row r="332" ht="14.25" customHeight="1"/>
-    <row r="333" ht="14.25" customHeight="1"/>
-    <row r="334" ht="14.25" customHeight="1"/>
-    <row r="335" ht="14.25" customHeight="1"/>
-    <row r="336" ht="14.25" customHeight="1"/>
-    <row r="337" ht="14.25" customHeight="1"/>
-    <row r="338" ht="14.25" customHeight="1"/>
-    <row r="339" ht="14.25" customHeight="1"/>
-    <row r="340" ht="14.25" customHeight="1"/>
-    <row r="341" ht="14.25" customHeight="1"/>
-    <row r="342" ht="14.25" customHeight="1"/>
-    <row r="343" ht="14.25" customHeight="1"/>
-    <row r="344" ht="14.25" customHeight="1"/>
-    <row r="345" ht="14.25" customHeight="1"/>
-    <row r="346" ht="14.25" customHeight="1"/>
-    <row r="347" ht="14.25" customHeight="1"/>
-    <row r="348" ht="14.25" customHeight="1"/>
-    <row r="349" ht="14.25" customHeight="1"/>
-    <row r="350" ht="14.25" customHeight="1"/>
-    <row r="351" ht="14.25" customHeight="1"/>
-    <row r="352" ht="14.25" customHeight="1"/>
-    <row r="353" ht="14.25" customHeight="1"/>
-    <row r="354" ht="14.25" customHeight="1"/>
-    <row r="355" ht="14.25" customHeight="1"/>
-    <row r="356" ht="14.25" customHeight="1"/>
-    <row r="357" ht="14.25" customHeight="1"/>
-    <row r="358" ht="14.25" customHeight="1"/>
-    <row r="359" ht="14.25" customHeight="1"/>
-    <row r="360" ht="14.25" customHeight="1"/>
-    <row r="361" ht="14.25" customHeight="1"/>
-    <row r="362" ht="14.25" customHeight="1"/>
-    <row r="363" ht="14.25" customHeight="1"/>
-    <row r="364" ht="14.25" customHeight="1"/>
-    <row r="365" ht="14.25" customHeight="1"/>
-    <row r="366" ht="14.25" customHeight="1"/>
-    <row r="367" ht="14.25" customHeight="1"/>
-    <row r="368" ht="14.25" customHeight="1"/>
-    <row r="369" ht="14.25" customHeight="1"/>
-    <row r="370" ht="14.25" customHeight="1"/>
-    <row r="371" ht="14.25" customHeight="1"/>
-    <row r="372" ht="14.25" customHeight="1"/>
-    <row r="373" ht="14.25" customHeight="1"/>
-    <row r="374" ht="14.25" customHeight="1"/>
-    <row r="375" ht="14.25" customHeight="1"/>
-    <row r="376" ht="14.25" customHeight="1"/>
-    <row r="377" ht="14.25" customHeight="1"/>
-    <row r="378" ht="14.25" customHeight="1"/>
-    <row r="379" ht="14.25" customHeight="1"/>
-    <row r="380" ht="14.25" customHeight="1"/>
-    <row r="381" ht="14.25" customHeight="1"/>
-    <row r="382" ht="14.25" customHeight="1"/>
-    <row r="383" ht="14.25" customHeight="1"/>
-    <row r="384" ht="14.25" customHeight="1"/>
-    <row r="385" ht="14.25" customHeight="1"/>
-    <row r="386" ht="14.25" customHeight="1"/>
-    <row r="387" ht="14.25" customHeight="1"/>
-    <row r="388" ht="14.25" customHeight="1"/>
-    <row r="389" ht="14.25" customHeight="1"/>
-    <row r="390" ht="14.25" customHeight="1"/>
-    <row r="391" ht="14.25" customHeight="1"/>
-    <row r="392" ht="14.25" customHeight="1"/>
-    <row r="393" ht="14.25" customHeight="1"/>
-    <row r="394" ht="14.25" customHeight="1"/>
-    <row r="395" ht="14.25" customHeight="1"/>
-    <row r="396" ht="14.25" customHeight="1"/>
-    <row r="397" ht="14.25" customHeight="1"/>
-    <row r="398" ht="14.25" customHeight="1"/>
-    <row r="399" ht="14.25" customHeight="1"/>
-    <row r="400" ht="14.25" customHeight="1"/>
-    <row r="401" ht="14.25" customHeight="1"/>
-    <row r="402" ht="14.25" customHeight="1"/>
-    <row r="403" ht="14.25" customHeight="1"/>
-    <row r="404" ht="14.25" customHeight="1"/>
-    <row r="405" ht="14.25" customHeight="1"/>
-    <row r="406" ht="14.25" customHeight="1"/>
-    <row r="407" ht="14.25" customHeight="1"/>
-    <row r="408" ht="14.25" customHeight="1"/>
-    <row r="409" ht="14.25" customHeight="1"/>
-    <row r="410" ht="14.25" customHeight="1"/>
-    <row r="411" ht="14.25" customHeight="1"/>
-    <row r="412" ht="14.25" customHeight="1"/>
-    <row r="413" ht="14.25" customHeight="1"/>
-    <row r="414" ht="14.25" customHeight="1"/>
-    <row r="415" ht="14.25" customHeight="1"/>
-    <row r="416" ht="14.25" customHeight="1"/>
-    <row r="417" ht="14.25" customHeight="1"/>
-    <row r="418" ht="14.25" customHeight="1"/>
-    <row r="419" ht="14.25" customHeight="1"/>
-    <row r="420" ht="14.25" customHeight="1"/>
-    <row r="421" ht="14.25" customHeight="1"/>
-    <row r="422" ht="14.25" customHeight="1"/>
-    <row r="423" ht="14.25" customHeight="1"/>
-    <row r="424" ht="14.25" customHeight="1"/>
-    <row r="425" ht="14.25" customHeight="1"/>
-    <row r="426" ht="14.25" customHeight="1"/>
-    <row r="427" ht="14.25" customHeight="1"/>
-    <row r="428" ht="14.25" customHeight="1"/>
-    <row r="429" ht="14.25" customHeight="1"/>
-    <row r="430" ht="14.25" customHeight="1"/>
-    <row r="431" ht="14.25" customHeight="1"/>
-    <row r="432" ht="14.25" customHeight="1"/>
-    <row r="433" ht="14.25" customHeight="1"/>
-    <row r="434" ht="14.25" customHeight="1"/>
-    <row r="435" ht="14.25" customHeight="1"/>
-    <row r="436" ht="14.25" customHeight="1"/>
-    <row r="437" ht="14.25" customHeight="1"/>
-    <row r="438" ht="14.25" customHeight="1"/>
-    <row r="439" ht="14.25" customHeight="1"/>
-    <row r="440" ht="14.25" customHeight="1"/>
-    <row r="441" ht="14.25" customHeight="1"/>
-    <row r="442" ht="14.25" customHeight="1"/>
-    <row r="443" ht="14.25" customHeight="1"/>
-    <row r="444" ht="14.25" customHeight="1"/>
-    <row r="445" ht="14.25" customHeight="1"/>
-    <row r="446" ht="14.25" customHeight="1"/>
-    <row r="447" ht="14.25" customHeight="1"/>
-    <row r="448" ht="14.25" customHeight="1"/>
-    <row r="449" ht="14.25" customHeight="1"/>
-    <row r="450" ht="14.25" customHeight="1"/>
-    <row r="451" ht="14.25" customHeight="1"/>
-    <row r="452" ht="14.25" customHeight="1"/>
-    <row r="453" ht="14.25" customHeight="1"/>
-    <row r="454" ht="14.25" customHeight="1"/>
-    <row r="455" ht="14.25" customHeight="1"/>
-    <row r="456" ht="14.25" customHeight="1"/>
-    <row r="457" ht="14.25" customHeight="1"/>
-    <row r="458" ht="14.25" customHeight="1"/>
-    <row r="459" ht="14.25" customHeight="1"/>
-    <row r="460" ht="14.25" customHeight="1"/>
-    <row r="461" ht="14.25" customHeight="1"/>
-    <row r="462" ht="14.25" customHeight="1"/>
-    <row r="463" ht="14.25" customHeight="1"/>
-    <row r="464" ht="14.25" customHeight="1"/>
-    <row r="465" ht="14.25" customHeight="1"/>
-    <row r="466" ht="14.25" customHeight="1"/>
-    <row r="467" ht="14.25" customHeight="1"/>
-    <row r="468" ht="14.25" customHeight="1"/>
-    <row r="469" ht="14.25" customHeight="1"/>
-    <row r="470" ht="14.25" customHeight="1"/>
-    <row r="471" ht="14.25" customHeight="1"/>
-    <row r="472" ht="14.25" customHeight="1"/>
-    <row r="473" ht="14.25" customHeight="1"/>
-    <row r="474" ht="14.25" customHeight="1"/>
-    <row r="475" ht="14.25" customHeight="1"/>
-    <row r="476" ht="14.25" customHeight="1"/>
-    <row r="477" ht="14.25" customHeight="1"/>
-    <row r="478" ht="14.25" customHeight="1"/>
-    <row r="479" ht="14.25" customHeight="1"/>
-    <row r="480" ht="14.25" customHeight="1"/>
-    <row r="481" ht="14.25" customHeight="1"/>
-    <row r="482" ht="14.25" customHeight="1"/>
-    <row r="483" ht="14.25" customHeight="1"/>
-    <row r="484" ht="14.25" customHeight="1"/>
-    <row r="485" ht="14.25" customHeight="1"/>
-    <row r="486" ht="14.25" customHeight="1"/>
-    <row r="487" ht="14.25" customHeight="1"/>
-    <row r="488" ht="14.25" customHeight="1"/>
-    <row r="489" ht="14.25" customHeight="1"/>
-    <row r="490" ht="14.25" customHeight="1"/>
-    <row r="491" ht="14.25" customHeight="1"/>
-    <row r="492" ht="14.25" customHeight="1"/>
-    <row r="493" ht="14.25" customHeight="1"/>
-    <row r="494" ht="14.25" customHeight="1"/>
-    <row r="495" ht="14.25" customHeight="1"/>
-    <row r="496" ht="14.25" customHeight="1"/>
-    <row r="497" ht="14.25" customHeight="1"/>
-    <row r="498" ht="14.25" customHeight="1"/>
-    <row r="499" ht="14.25" customHeight="1"/>
-    <row r="500" ht="14.25" customHeight="1"/>
-    <row r="501" ht="14.25" customHeight="1"/>
-    <row r="502" ht="14.25" customHeight="1"/>
-    <row r="503" ht="14.25" customHeight="1"/>
-    <row r="504" ht="14.25" customHeight="1"/>
-    <row r="505" ht="14.25" customHeight="1"/>
-    <row r="506" ht="14.25" customHeight="1"/>
-    <row r="507" ht="14.25" customHeight="1"/>
-    <row r="508" ht="14.25" customHeight="1"/>
-    <row r="509" ht="14.25" customHeight="1"/>
-    <row r="510" ht="14.25" customHeight="1"/>
-    <row r="511" ht="14.25" customHeight="1"/>
-    <row r="512" ht="14.25" customHeight="1"/>
-    <row r="513" ht="14.25" customHeight="1"/>
-    <row r="514" ht="14.25" customHeight="1"/>
-    <row r="515" ht="14.25" customHeight="1"/>
-    <row r="516" ht="14.25" customHeight="1"/>
-    <row r="517" ht="14.25" customHeight="1"/>
-    <row r="518" ht="14.25" customHeight="1"/>
-    <row r="519" ht="14.25" customHeight="1"/>
-    <row r="520" ht="14.25" customHeight="1"/>
-    <row r="521" ht="14.25" customHeight="1"/>
-    <row r="522" ht="14.25" customHeight="1"/>
-    <row r="523" ht="14.25" customHeight="1"/>
-    <row r="524" ht="14.25" customHeight="1"/>
-    <row r="525" ht="14.25" customHeight="1"/>
-    <row r="526" ht="14.25" customHeight="1"/>
-    <row r="527" ht="14.25" customHeight="1"/>
-    <row r="528" ht="14.25" customHeight="1"/>
-    <row r="529" ht="14.25" customHeight="1"/>
-    <row r="530" ht="14.25" customHeight="1"/>
-    <row r="531" ht="14.25" customHeight="1"/>
-    <row r="532" ht="14.25" customHeight="1"/>
-    <row r="533" ht="14.25" customHeight="1"/>
-    <row r="534" ht="14.25" customHeight="1"/>
-    <row r="535" ht="14.25" customHeight="1"/>
-    <row r="536" ht="14.25" customHeight="1"/>
-    <row r="537" ht="14.25" customHeight="1"/>
-    <row r="538" ht="14.25" customHeight="1"/>
-    <row r="539" ht="14.25" customHeight="1"/>
-    <row r="540" ht="14.25" customHeight="1"/>
-    <row r="541" ht="14.25" customHeight="1"/>
-    <row r="542" ht="14.25" customHeight="1"/>
-    <row r="543" ht="14.25" customHeight="1"/>
-    <row r="544" ht="14.25" customHeight="1"/>
-    <row r="545" ht="14.25" customHeight="1"/>
-    <row r="546" ht="14.25" customHeight="1"/>
-    <row r="547" ht="14.25" customHeight="1"/>
-    <row r="548" ht="14.25" customHeight="1"/>
-    <row r="549" ht="14.25" customHeight="1"/>
-    <row r="550" ht="14.25" customHeight="1"/>
-    <row r="551" ht="14.25" customHeight="1"/>
-    <row r="552" ht="14.25" customHeight="1"/>
-    <row r="553" ht="14.25" customHeight="1"/>
-    <row r="554" ht="14.25" customHeight="1"/>
-    <row r="555" ht="14.25" customHeight="1"/>
-    <row r="556" ht="14.25" customHeight="1"/>
-    <row r="557" ht="14.25" customHeight="1"/>
-    <row r="558" ht="14.25" customHeight="1"/>
-    <row r="559" ht="14.25" customHeight="1"/>
-    <row r="560" ht="14.25" customHeight="1"/>
-    <row r="561" ht="14.25" customHeight="1"/>
-    <row r="562" ht="14.25" customHeight="1"/>
-    <row r="563" ht="14.25" customHeight="1"/>
-    <row r="564" ht="14.25" customHeight="1"/>
-    <row r="565" ht="14.25" customHeight="1"/>
-    <row r="566" ht="14.25" customHeight="1"/>
-    <row r="567" ht="14.25" customHeight="1"/>
-    <row r="568" ht="14.25" customHeight="1"/>
-    <row r="569" ht="14.25" customHeight="1"/>
-    <row r="570" ht="14.25" customHeight="1"/>
-    <row r="571" ht="14.25" customHeight="1"/>
-    <row r="572" ht="14.25" customHeight="1"/>
-    <row r="573" ht="14.25" customHeight="1"/>
-    <row r="574" ht="14.25" customHeight="1"/>
-    <row r="575" ht="14.25" customHeight="1"/>
-    <row r="576" ht="14.25" customHeight="1"/>
-    <row r="577" ht="14.25" customHeight="1"/>
-    <row r="578" ht="14.25" customHeight="1"/>
-    <row r="579" ht="14.25" customHeight="1"/>
-    <row r="580" ht="14.25" customHeight="1"/>
-    <row r="581" ht="14.25" customHeight="1"/>
-    <row r="582" ht="14.25" customHeight="1"/>
-    <row r="583" ht="14.25" customHeight="1"/>
-    <row r="584" ht="14.25" customHeight="1"/>
-    <row r="585" ht="14.25" customHeight="1"/>
-    <row r="586" ht="14.25" customHeight="1"/>
-    <row r="587" ht="14.25" customHeight="1"/>
-    <row r="588" ht="14.25" customHeight="1"/>
-    <row r="589" ht="14.25" customHeight="1"/>
-    <row r="590" ht="14.25" customHeight="1"/>
-    <row r="591" ht="14.25" customHeight="1"/>
-    <row r="592" ht="14.25" customHeight="1"/>
-    <row r="593" ht="14.25" customHeight="1"/>
-    <row r="594" ht="14.25" customHeight="1"/>
-    <row r="595" ht="14.25" customHeight="1"/>
-    <row r="596" ht="14.25" customHeight="1"/>
-    <row r="597" ht="14.25" customHeight="1"/>
-    <row r="598" ht="14.25" customHeight="1"/>
-    <row r="599" ht="14.25" customHeight="1"/>
-    <row r="600" ht="14.25" customHeight="1"/>
-    <row r="601" ht="14.25" customHeight="1"/>
-    <row r="602" ht="14.25" customHeight="1"/>
-    <row r="603" ht="14.25" customHeight="1"/>
-    <row r="604" ht="14.25" customHeight="1"/>
-    <row r="605" ht="14.25" customHeight="1"/>
-    <row r="606" ht="14.25" customHeight="1"/>
-    <row r="607" ht="14.25" customHeight="1"/>
-    <row r="608" ht="14.25" customHeight="1"/>
-    <row r="609" ht="14.25" customHeight="1"/>
-    <row r="610" ht="14.25" customHeight="1"/>
-    <row r="611" ht="14.25" customHeight="1"/>
-    <row r="612" ht="14.25" customHeight="1"/>
-    <row r="613" ht="14.25" customHeight="1"/>
-    <row r="614" ht="14.25" customHeight="1"/>
-    <row r="615" ht="14.25" customHeight="1"/>
-    <row r="616" ht="14.25" customHeight="1"/>
-    <row r="617" ht="14.25" customHeight="1"/>
-    <row r="618" ht="14.25" customHeight="1"/>
-    <row r="619" ht="14.25" customHeight="1"/>
-    <row r="620" ht="14.25" customHeight="1"/>
-    <row r="621" ht="14.25" customHeight="1"/>
-    <row r="622" ht="14.25" customHeight="1"/>
-    <row r="623" ht="14.25" customHeight="1"/>
-    <row r="624" ht="14.25" customHeight="1"/>
-    <row r="625" ht="14.25" customHeight="1"/>
-    <row r="626" ht="14.25" customHeight="1"/>
-    <row r="627" ht="14.25" customHeight="1"/>
-    <row r="628" ht="14.25" customHeight="1"/>
-    <row r="629" ht="14.25" customHeight="1"/>
-    <row r="630" ht="14.25" customHeight="1"/>
-    <row r="631" ht="14.25" customHeight="1"/>
-    <row r="632" ht="14.25" customHeight="1"/>
-    <row r="633" ht="14.25" customHeight="1"/>
-    <row r="634" ht="14.25" customHeight="1"/>
-    <row r="635" ht="14.25" customHeight="1"/>
-    <row r="636" ht="14.25" customHeight="1"/>
-    <row r="637" ht="14.25" customHeight="1"/>
-    <row r="638" ht="14.25" customHeight="1"/>
-    <row r="639" ht="14.25" customHeight="1"/>
-    <row r="640" ht="14.25" customHeight="1"/>
-    <row r="641" ht="14.25" customHeight="1"/>
-    <row r="642" ht="14.25" customHeight="1"/>
-    <row r="643" ht="14.25" customHeight="1"/>
-    <row r="644" ht="14.25" customHeight="1"/>
-    <row r="645" ht="14.25" customHeight="1"/>
-    <row r="646" ht="14.25" customHeight="1"/>
-    <row r="647" ht="14.25" customHeight="1"/>
-    <row r="648" ht="14.25" customHeight="1"/>
-    <row r="649" ht="14.25" customHeight="1"/>
-    <row r="650" ht="14.25" customHeight="1"/>
-    <row r="651" ht="14.25" customHeight="1"/>
-    <row r="652" ht="14.25" customHeight="1"/>
-    <row r="653" ht="14.25" customHeight="1"/>
-    <row r="654" ht="14.25" customHeight="1"/>
-    <row r="655" ht="14.25" customHeight="1"/>
-    <row r="656" ht="14.25" customHeight="1"/>
-    <row r="657" ht="14.25" customHeight="1"/>
-    <row r="658" ht="14.25" customHeight="1"/>
-    <row r="659" ht="14.25" customHeight="1"/>
-    <row r="660" ht="14.25" customHeight="1"/>
-    <row r="661" ht="14.25" customHeight="1"/>
-    <row r="662" ht="14.25" customHeight="1"/>
-    <row r="663" ht="14.25" customHeight="1"/>
-    <row r="664" ht="14.25" customHeight="1"/>
-    <row r="665" ht="14.25" customHeight="1"/>
-    <row r="666" ht="14.25" customHeight="1"/>
-    <row r="667" ht="14.25" customHeight="1"/>
-    <row r="668" ht="14.25" customHeight="1"/>
-    <row r="669" ht="14.25" customHeight="1"/>
-    <row r="670" ht="14.25" customHeight="1"/>
-    <row r="671" ht="14.25" customHeight="1"/>
-    <row r="672" ht="14.25" customHeight="1"/>
-    <row r="673" ht="14.25" customHeight="1"/>
-    <row r="674" ht="14.25" customHeight="1"/>
-    <row r="675" ht="14.25" customHeight="1"/>
-    <row r="676" ht="14.25" customHeight="1"/>
-    <row r="677" ht="14.25" customHeight="1"/>
-    <row r="678" ht="14.25" customHeight="1"/>
-    <row r="679" ht="14.25" customHeight="1"/>
-    <row r="680" ht="14.25" customHeight="1"/>
-    <row r="681" ht="14.25" customHeight="1"/>
-    <row r="682" ht="14.25" customHeight="1"/>
-    <row r="683" ht="14.25" customHeight="1"/>
-    <row r="684" ht="14.25" customHeight="1"/>
-    <row r="685" ht="14.25" customHeight="1"/>
-    <row r="686" ht="14.25" customHeight="1"/>
-    <row r="687" ht="14.25" customHeight="1"/>
-    <row r="688" ht="14.25" customHeight="1"/>
-    <row r="689" ht="14.25" customHeight="1"/>
-    <row r="690" ht="14.25" customHeight="1"/>
-    <row r="691" ht="14.25" customHeight="1"/>
-    <row r="692" ht="14.25" customHeight="1"/>
-    <row r="693" ht="14.25" customHeight="1"/>
-    <row r="694" ht="14.25" customHeight="1"/>
-    <row r="695" ht="14.25" customHeight="1"/>
-    <row r="696" ht="14.25" customHeight="1"/>
-    <row r="697" ht="14.25" customHeight="1"/>
-    <row r="698" ht="14.25" customHeight="1"/>
-    <row r="699" ht="14.25" customHeight="1"/>
-    <row r="700" ht="14.25" customHeight="1"/>
-    <row r="701" ht="14.25" customHeight="1"/>
-    <row r="702" ht="14.25" customHeight="1"/>
-    <row r="703" ht="14.25" customHeight="1"/>
-    <row r="704" ht="14.25" customHeight="1"/>
-    <row r="705" ht="14.25" customHeight="1"/>
-    <row r="706" ht="14.25" customHeight="1"/>
-    <row r="707" ht="14.25" customHeight="1"/>
-    <row r="708" ht="14.25" customHeight="1"/>
-    <row r="709" ht="14.25" customHeight="1"/>
-    <row r="710" ht="14.25" customHeight="1"/>
-    <row r="711" ht="14.25" customHeight="1"/>
-    <row r="712" ht="14.25" customHeight="1"/>
-    <row r="713" ht="14.25" customHeight="1"/>
-    <row r="714" ht="14.25" customHeight="1"/>
-    <row r="715" ht="14.25" customHeight="1"/>
-    <row r="716" ht="14.25" customHeight="1"/>
-    <row r="717" ht="14.25" customHeight="1"/>
-    <row r="718" ht="14.25" customHeight="1"/>
-    <row r="719" ht="14.25" customHeight="1"/>
-    <row r="720" ht="14.25" customHeight="1"/>
-    <row r="721" ht="14.25" customHeight="1"/>
-    <row r="722" ht="14.25" customHeight="1"/>
-    <row r="723" ht="14.25" customHeight="1"/>
-    <row r="724" ht="14.25" customHeight="1"/>
-    <row r="725" ht="14.25" customHeight="1"/>
-    <row r="726" ht="14.25" customHeight="1"/>
-    <row r="727" ht="14.25" customHeight="1"/>
-    <row r="728" ht="14.25" customHeight="1"/>
-    <row r="729" ht="14.25" customHeight="1"/>
-    <row r="730" ht="14.25" customHeight="1"/>
-    <row r="731" ht="14.25" customHeight="1"/>
-    <row r="732" ht="14.25" customHeight="1"/>
-    <row r="733" ht="14.25" customHeight="1"/>
-    <row r="734" ht="14.25" customHeight="1"/>
-    <row r="735" ht="14.25" customHeight="1"/>
-    <row r="736" ht="14.25" customHeight="1"/>
-    <row r="737" ht="14.25" customHeight="1"/>
-    <row r="738" ht="14.25" customHeight="1"/>
-    <row r="739" ht="14.25" customHeight="1"/>
-    <row r="740" ht="14.25" customHeight="1"/>
-    <row r="741" ht="14.25" customHeight="1"/>
-    <row r="742" ht="14.25" customHeight="1"/>
-    <row r="743" ht="14.25" customHeight="1"/>
-    <row r="744" ht="14.25" customHeight="1"/>
-    <row r="745" ht="14.25" customHeight="1"/>
-    <row r="746" ht="14.25" customHeight="1"/>
-    <row r="747" ht="14.25" customHeight="1"/>
-    <row r="748" ht="14.25" customHeight="1"/>
-    <row r="749" ht="14.25" customHeight="1"/>
-    <row r="750" ht="14.25" customHeight="1"/>
-    <row r="751" ht="14.25" customHeight="1"/>
-    <row r="752" ht="14.25" customHeight="1"/>
-    <row r="753" ht="14.25" customHeight="1"/>
-    <row r="754" ht="14.25" customHeight="1"/>
-    <row r="755" ht="14.25" customHeight="1"/>
-    <row r="756" ht="14.25" customHeight="1"/>
-    <row r="757" ht="14.25" customHeight="1"/>
-    <row r="758" ht="14.25" customHeight="1"/>
-    <row r="759" ht="14.25" customHeight="1"/>
-    <row r="760" ht="14.25" customHeight="1"/>
-    <row r="761" ht="14.25" customHeight="1"/>
-    <row r="762" ht="14.25" customHeight="1"/>
-    <row r="763" ht="14.25" customHeight="1"/>
-    <row r="764" ht="14.25" customHeight="1"/>
-    <row r="765" ht="14.25" customHeight="1"/>
-    <row r="766" ht="14.25" customHeight="1"/>
-    <row r="767" ht="14.25" customHeight="1"/>
-    <row r="768" ht="14.25" customHeight="1"/>
-    <row r="769" ht="14.25" customHeight="1"/>
-    <row r="770" ht="14.25" customHeight="1"/>
-    <row r="771" ht="14.25" customHeight="1"/>
-    <row r="772" ht="14.25" customHeight="1"/>
-    <row r="773" ht="14.25" customHeight="1"/>
-    <row r="774" ht="14.25" customHeight="1"/>
-    <row r="775" ht="14.25" customHeight="1"/>
-    <row r="776" ht="14.25" customHeight="1"/>
-    <row r="777" ht="14.25" customHeight="1"/>
-    <row r="778" ht="14.25" customHeight="1"/>
-    <row r="779" ht="14.25" customHeight="1"/>
-    <row r="780" ht="14.25" customHeight="1"/>
-    <row r="781" ht="14.25" customHeight="1"/>
-    <row r="782" ht="14.25" customHeight="1"/>
-    <row r="783" ht="14.25" customHeight="1"/>
-    <row r="784" ht="14.25" customHeight="1"/>
-    <row r="785" ht="14.25" customHeight="1"/>
-    <row r="786" ht="14.25" customHeight="1"/>
-    <row r="787" ht="14.25" customHeight="1"/>
-    <row r="788" ht="14.25" customHeight="1"/>
-    <row r="789" ht="14.25" customHeight="1"/>
-    <row r="790" ht="14.25" customHeight="1"/>
-    <row r="791" ht="14.25" customHeight="1"/>
-    <row r="792" ht="14.25" customHeight="1"/>
-    <row r="793" ht="14.25" customHeight="1"/>
-    <row r="794" ht="14.25" customHeight="1"/>
-    <row r="795" ht="14.25" customHeight="1"/>
-    <row r="796" ht="14.25" customHeight="1"/>
-    <row r="797" ht="14.25" customHeight="1"/>
-    <row r="798" ht="14.25" customHeight="1"/>
-    <row r="799" ht="14.25" customHeight="1"/>
-    <row r="800" ht="14.25" customHeight="1"/>
-    <row r="801" ht="14.25" customHeight="1"/>
-    <row r="802" ht="14.25" customHeight="1"/>
-    <row r="803" ht="14.25" customHeight="1"/>
-    <row r="804" ht="14.25" customHeight="1"/>
-    <row r="805" ht="14.25" customHeight="1"/>
-    <row r="806" ht="14.25" customHeight="1"/>
-    <row r="807" ht="14.25" customHeight="1"/>
-    <row r="808" ht="14.25" customHeight="1"/>
-    <row r="809" ht="14.25" customHeight="1"/>
-    <row r="810" ht="14.25" customHeight="1"/>
-    <row r="811" ht="14.25" customHeight="1"/>
-    <row r="812" ht="14.25" customHeight="1"/>
-    <row r="813" ht="14.25" customHeight="1"/>
-    <row r="814" ht="14.25" customHeight="1"/>
-    <row r="815" ht="14.25" customHeight="1"/>
-    <row r="816" ht="14.25" customHeight="1"/>
-    <row r="817" ht="14.25" customHeight="1"/>
-    <row r="818" ht="14.25" customHeight="1"/>
-    <row r="819" ht="14.25" customHeight="1"/>
-    <row r="820" ht="14.25" customHeight="1"/>
-    <row r="821" ht="14.25" customHeight="1"/>
-    <row r="822" ht="14.25" customHeight="1"/>
-    <row r="823" ht="14.25" customHeight="1"/>
-    <row r="824" ht="14.25" customHeight="1"/>
-    <row r="825" ht="14.25" customHeight="1"/>
-    <row r="826" ht="14.25" customHeight="1"/>
-    <row r="827" ht="14.25" customHeight="1"/>
-    <row r="828" ht="14.25" customHeight="1"/>
-    <row r="829" ht="14.25" customHeight="1"/>
-    <row r="830" ht="14.25" customHeight="1"/>
-    <row r="831" ht="14.25" customHeight="1"/>
-    <row r="832" ht="14.25" customHeight="1"/>
-    <row r="833" ht="14.25" customHeight="1"/>
-    <row r="834" ht="14.25" customHeight="1"/>
-    <row r="835" ht="14.25" customHeight="1"/>
-    <row r="836" ht="14.25" customHeight="1"/>
-    <row r="837" ht="14.25" customHeight="1"/>
-    <row r="838" ht="14.25" customHeight="1"/>
-    <row r="839" ht="14.25" customHeight="1"/>
-    <row r="840" ht="14.25" customHeight="1"/>
-    <row r="841" ht="14.25" customHeight="1"/>
-    <row r="842" ht="14.25" customHeight="1"/>
-    <row r="843" ht="14.25" customHeight="1"/>
-    <row r="844" ht="14.25" customHeight="1"/>
-    <row r="845" ht="14.25" customHeight="1"/>
-    <row r="846" ht="14.25" customHeight="1"/>
-    <row r="847" ht="14.25" customHeight="1"/>
-    <row r="848" ht="14.25" customHeight="1"/>
-    <row r="849" ht="14.25" customHeight="1"/>
-    <row r="850" ht="14.25" customHeight="1"/>
-    <row r="851" ht="14.25" customHeight="1"/>
-    <row r="852" ht="14.25" customHeight="1"/>
-    <row r="853" ht="14.25" customHeight="1"/>
-    <row r="854" ht="14.25" customHeight="1"/>
-    <row r="855" ht="14.25" customHeight="1"/>
-    <row r="856" ht="14.25" customHeight="1"/>
-    <row r="857" ht="14.25" customHeight="1"/>
-    <row r="858" ht="14.25" customHeight="1"/>
-    <row r="859" ht="14.25" customHeight="1"/>
-    <row r="860" ht="14.25" customHeight="1"/>
-    <row r="861" ht="14.25" customHeight="1"/>
-    <row r="862" ht="14.25" customHeight="1"/>
-    <row r="863" ht="14.25" customHeight="1"/>
-    <row r="864" ht="14.25" customHeight="1"/>
-    <row r="865" ht="14.25" customHeight="1"/>
-    <row r="866" ht="14.25" customHeight="1"/>
-    <row r="867" ht="14.25" customHeight="1"/>
-    <row r="868" ht="14.25" customHeight="1"/>
-    <row r="869" ht="14.25" customHeight="1"/>
-    <row r="870" ht="14.25" customHeight="1"/>
-    <row r="871" ht="14.25" customHeight="1"/>
-    <row r="872" ht="14.25" customHeight="1"/>
-    <row r="873" ht="14.25" customHeight="1"/>
-    <row r="874" ht="14.25" customHeight="1"/>
-    <row r="875" ht="14.25" customHeight="1"/>
-    <row r="876" ht="14.25" customHeight="1"/>
-    <row r="877" ht="14.25" customHeight="1"/>
-    <row r="878" ht="14.25" customHeight="1"/>
-    <row r="879" ht="14.25" customHeight="1"/>
-    <row r="880" ht="14.25" customHeight="1"/>
-    <row r="881" ht="14.25" customHeight="1"/>
-    <row r="882" ht="14.25" customHeight="1"/>
-    <row r="883" ht="14.25" customHeight="1"/>
-    <row r="884" ht="14.25" customHeight="1"/>
-    <row r="885" ht="14.25" customHeight="1"/>
-    <row r="886" ht="14.25" customHeight="1"/>
-    <row r="887" ht="14.25" customHeight="1"/>
-    <row r="888" ht="14.25" customHeight="1"/>
-    <row r="889" ht="14.25" customHeight="1"/>
-    <row r="890" ht="14.25" customHeight="1"/>
-    <row r="891" ht="14.25" customHeight="1"/>
-    <row r="892" ht="14.25" customHeight="1"/>
-    <row r="893" ht="14.25" customHeight="1"/>
-    <row r="894" ht="14.25" customHeight="1"/>
-    <row r="895" ht="14.25" customHeight="1"/>
-    <row r="896" ht="14.25" customHeight="1"/>
-    <row r="897" ht="14.25" customHeight="1"/>
-    <row r="898" ht="14.25" customHeight="1"/>
-    <row r="899" ht="14.25" customHeight="1"/>
-    <row r="900" ht="14.25" customHeight="1"/>
-    <row r="901" ht="14.25" customHeight="1"/>
-    <row r="902" ht="14.25" customHeight="1"/>
-    <row r="903" ht="14.25" customHeight="1"/>
-    <row r="904" ht="14.25" customHeight="1"/>
-    <row r="905" ht="14.25" customHeight="1"/>
-    <row r="906" ht="14.25" customHeight="1"/>
-    <row r="907" ht="14.25" customHeight="1"/>
-    <row r="908" ht="14.25" customHeight="1"/>
-    <row r="909" ht="14.25" customHeight="1"/>
-    <row r="910" ht="14.25" customHeight="1"/>
-    <row r="911" ht="14.25" customHeight="1"/>
-    <row r="912" ht="14.25" customHeight="1"/>
-    <row r="913" ht="14.25" customHeight="1"/>
-    <row r="914" ht="14.25" customHeight="1"/>
-    <row r="915" ht="14.25" customHeight="1"/>
-    <row r="916" ht="14.25" customHeight="1"/>
-    <row r="917" ht="14.25" customHeight="1"/>
-    <row r="918" ht="14.25" customHeight="1"/>
-    <row r="919" ht="14.25" customHeight="1"/>
-    <row r="920" ht="14.25" customHeight="1"/>
-    <row r="921" ht="14.25" customHeight="1"/>
-    <row r="922" ht="14.25" customHeight="1"/>
-    <row r="923" ht="14.25" customHeight="1"/>
-    <row r="924" ht="14.25" customHeight="1"/>
-    <row r="925" ht="14.25" customHeight="1"/>
-    <row r="926" ht="14.25" customHeight="1"/>
-    <row r="927" ht="14.25" customHeight="1"/>
-    <row r="928" ht="14.25" customHeight="1"/>
-    <row r="929" ht="14.25" customHeight="1"/>
-    <row r="930" ht="14.25" customHeight="1"/>
-    <row r="931" ht="14.25" customHeight="1"/>
-    <row r="932" ht="14.25" customHeight="1"/>
-    <row r="933" ht="14.25" customHeight="1"/>
-    <row r="934" ht="14.25" customHeight="1"/>
-    <row r="935" ht="14.25" customHeight="1"/>
-    <row r="936" ht="14.25" customHeight="1"/>
-    <row r="937" ht="14.25" customHeight="1"/>
-    <row r="938" ht="14.25" customHeight="1"/>
-    <row r="939" ht="14.25" customHeight="1"/>
-    <row r="940" ht="14.25" customHeight="1"/>
-    <row r="941" ht="14.25" customHeight="1"/>
-    <row r="942" ht="14.25" customHeight="1"/>
-    <row r="943" ht="14.25" customHeight="1"/>
-    <row r="944" ht="14.25" customHeight="1"/>
-    <row r="945" ht="14.25" customHeight="1"/>
-    <row r="946" ht="14.25" customHeight="1"/>
-    <row r="947" ht="14.25" customHeight="1"/>
-    <row r="948" ht="14.25" customHeight="1"/>
-    <row r="949" ht="14.25" customHeight="1"/>
-    <row r="950" ht="14.25" customHeight="1"/>
-    <row r="951" ht="14.25" customHeight="1"/>
-    <row r="952" ht="14.25" customHeight="1"/>
-    <row r="953" ht="14.25" customHeight="1"/>
-    <row r="954" ht="14.25" customHeight="1"/>
-    <row r="955" ht="14.25" customHeight="1"/>
-    <row r="956" ht="14.25" customHeight="1"/>
-    <row r="957" ht="14.25" customHeight="1"/>
-    <row r="958" ht="14.25" customHeight="1"/>
-    <row r="959" ht="14.25" customHeight="1"/>
-    <row r="960" ht="14.25" customHeight="1"/>
-    <row r="961" ht="14.25" customHeight="1"/>
-    <row r="962" ht="14.25" customHeight="1"/>
-    <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
-    <row r="973" ht="14.25" customHeight="1"/>
-    <row r="974" ht="14.25" customHeight="1"/>
-    <row r="975" ht="14.25" customHeight="1"/>
-    <row r="976" ht="14.25" customHeight="1"/>
-    <row r="977" ht="14.25" customHeight="1"/>
-    <row r="978" ht="14.25" customHeight="1"/>
-    <row r="979" ht="14.25" customHeight="1"/>
-    <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="3" ht="14.25" customHeight="true"/>
+    <row r="4" ht="14.25" customHeight="true"/>
+    <row r="5" ht="14.25" customHeight="true"/>
+    <row r="6" ht="14.25" customHeight="true"/>
+    <row r="7" ht="14.25" customHeight="true"/>
+    <row r="8" ht="14.25" customHeight="true"/>
+    <row r="9" ht="14.25" customHeight="true"/>
+    <row r="10" ht="14.25" customHeight="true"/>
+    <row r="11" ht="14.25" customHeight="true"/>
+    <row r="12" ht="14.25" customHeight="true"/>
+    <row r="13" ht="14.25" customHeight="true"/>
+    <row r="14" ht="14.25" customHeight="true"/>
+    <row r="15" ht="14.25" customHeight="true"/>
+    <row r="16" ht="14.25" customHeight="true"/>
+    <row r="17" ht="14.25" customHeight="true"/>
+    <row r="18" ht="14.25" customHeight="true"/>
+    <row r="19" ht="14.25" customHeight="true"/>
+    <row r="20" ht="14.25" customHeight="true"/>
+    <row r="21" ht="14.25" customHeight="true"/>
+    <row r="22" ht="14.25" customHeight="true"/>
+    <row r="23" ht="14.25" customHeight="true"/>
+    <row r="24" ht="14.25" customHeight="true"/>
+    <row r="25" ht="14.25" customHeight="true"/>
+    <row r="26" ht="14.25" customHeight="true"/>
+    <row r="27" ht="14.25" customHeight="true"/>
+    <row r="28" ht="14.25" customHeight="true"/>
+    <row r="29" ht="14.25" customHeight="true"/>
+    <row r="30" ht="14.25" customHeight="true"/>
+    <row r="31" ht="14.25" customHeight="true"/>
+    <row r="32" ht="14.25" customHeight="true"/>
+    <row r="33" ht="14.25" customHeight="true"/>
+    <row r="34" ht="14.25" customHeight="true"/>
+    <row r="35" ht="14.25" customHeight="true"/>
+    <row r="36" ht="14.25" customHeight="true"/>
+    <row r="37" ht="14.25" customHeight="true"/>
+    <row r="38" ht="14.25" customHeight="true"/>
+    <row r="39" ht="14.25" customHeight="true"/>
+    <row r="40" ht="14.25" customHeight="true"/>
+    <row r="41" ht="14.25" customHeight="true"/>
+    <row r="42" ht="14.25" customHeight="true"/>
+    <row r="43" ht="14.25" customHeight="true"/>
+    <row r="44" ht="14.25" customHeight="true"/>
+    <row r="45" ht="14.25" customHeight="true"/>
+    <row r="46" ht="14.25" customHeight="true"/>
+    <row r="47" ht="14.25" customHeight="true"/>
+    <row r="48" ht="14.25" customHeight="true"/>
+    <row r="49" ht="14.25" customHeight="true"/>
+    <row r="50" ht="14.25" customHeight="true"/>
+    <row r="51" ht="14.25" customHeight="true"/>
+    <row r="52" ht="14.25" customHeight="true"/>
+    <row r="53" ht="14.25" customHeight="true"/>
+    <row r="54" ht="14.25" customHeight="true"/>
+    <row r="55" ht="14.25" customHeight="true"/>
+    <row r="56" ht="14.25" customHeight="true"/>
+    <row r="57" ht="14.25" customHeight="true"/>
+    <row r="58" ht="14.25" customHeight="true"/>
+    <row r="59" ht="14.25" customHeight="true"/>
+    <row r="60" ht="14.25" customHeight="true"/>
+    <row r="61" ht="14.25" customHeight="true"/>
+    <row r="62" ht="14.25" customHeight="true"/>
+    <row r="63" ht="14.25" customHeight="true"/>
+    <row r="64" ht="14.25" customHeight="true"/>
+    <row r="65" ht="14.25" customHeight="true"/>
+    <row r="66" ht="14.25" customHeight="true"/>
+    <row r="67" ht="14.25" customHeight="true"/>
+    <row r="68" ht="14.25" customHeight="true"/>
+    <row r="69" ht="14.25" customHeight="true"/>
+    <row r="70" ht="14.25" customHeight="true"/>
+    <row r="71" ht="14.25" customHeight="true"/>
+    <row r="72" ht="14.25" customHeight="true"/>
+    <row r="73" ht="14.25" customHeight="true"/>
+    <row r="74" ht="14.25" customHeight="true"/>
+    <row r="75" ht="14.25" customHeight="true"/>
+    <row r="76" ht="14.25" customHeight="true"/>
+    <row r="77" ht="14.25" customHeight="true"/>
+    <row r="78" ht="14.25" customHeight="true"/>
+    <row r="79" ht="14.25" customHeight="true"/>
+    <row r="80" ht="14.25" customHeight="true"/>
+    <row r="81" ht="14.25" customHeight="true"/>
+    <row r="82" ht="14.25" customHeight="true"/>
+    <row r="83" ht="14.25" customHeight="true"/>
+    <row r="84" ht="14.25" customHeight="true"/>
+    <row r="85" ht="14.25" customHeight="true"/>
+    <row r="86" ht="14.25" customHeight="true"/>
+    <row r="87" ht="14.25" customHeight="true"/>
+    <row r="88" ht="14.25" customHeight="true"/>
+    <row r="89" ht="14.25" customHeight="true"/>
+    <row r="90" ht="14.25" customHeight="true"/>
+    <row r="91" ht="14.25" customHeight="true"/>
+    <row r="92" ht="14.25" customHeight="true"/>
+    <row r="93" ht="14.25" customHeight="true"/>
+    <row r="94" ht="14.25" customHeight="true"/>
+    <row r="95" ht="14.25" customHeight="true"/>
+    <row r="96" ht="14.25" customHeight="true"/>
+    <row r="97" ht="14.25" customHeight="true"/>
+    <row r="98" ht="14.25" customHeight="true"/>
+    <row r="99" ht="14.25" customHeight="true"/>
+    <row r="100" ht="14.25" customHeight="true"/>
+    <row r="101" ht="14.25" customHeight="true"/>
+    <row r="102" ht="14.25" customHeight="true"/>
+    <row r="103" ht="14.25" customHeight="true"/>
+    <row r="104" ht="14.25" customHeight="true"/>
+    <row r="105" ht="14.25" customHeight="true"/>
+    <row r="106" ht="14.25" customHeight="true"/>
+    <row r="107" ht="14.25" customHeight="true"/>
+    <row r="108" ht="14.25" customHeight="true"/>
+    <row r="109" ht="14.25" customHeight="true"/>
+    <row r="110" ht="14.25" customHeight="true"/>
+    <row r="111" ht="14.25" customHeight="true"/>
+    <row r="112" ht="14.25" customHeight="true"/>
+    <row r="113" ht="14.25" customHeight="true"/>
+    <row r="114" ht="14.25" customHeight="true"/>
+    <row r="115" ht="14.25" customHeight="true"/>
+    <row r="116" ht="14.25" customHeight="true"/>
+    <row r="117" ht="14.25" customHeight="true"/>
+    <row r="118" ht="14.25" customHeight="true"/>
+    <row r="119" ht="14.25" customHeight="true"/>
+    <row r="120" ht="14.25" customHeight="true"/>
+    <row r="121" ht="14.25" customHeight="true"/>
+    <row r="122" ht="14.25" customHeight="true"/>
+    <row r="123" ht="14.25" customHeight="true"/>
+    <row r="124" ht="14.25" customHeight="true"/>
+    <row r="125" ht="14.25" customHeight="true"/>
+    <row r="126" ht="14.25" customHeight="true"/>
+    <row r="127" ht="14.25" customHeight="true"/>
+    <row r="128" ht="14.25" customHeight="true"/>
+    <row r="129" ht="14.25" customHeight="true"/>
+    <row r="130" ht="14.25" customHeight="true"/>
+    <row r="131" ht="14.25" customHeight="true"/>
+    <row r="132" ht="14.25" customHeight="true"/>
+    <row r="133" ht="14.25" customHeight="true"/>
+    <row r="134" ht="14.25" customHeight="true"/>
+    <row r="135" ht="14.25" customHeight="true"/>
+    <row r="136" ht="14.25" customHeight="true"/>
+    <row r="137" ht="14.25" customHeight="true"/>
+    <row r="138" ht="14.25" customHeight="true"/>
+    <row r="139" ht="14.25" customHeight="true"/>
+    <row r="140" ht="14.25" customHeight="true"/>
+    <row r="141" ht="14.25" customHeight="true"/>
+    <row r="142" ht="14.25" customHeight="true"/>
+    <row r="143" ht="14.25" customHeight="true"/>
+    <row r="144" ht="14.25" customHeight="true"/>
+    <row r="145" ht="14.25" customHeight="true"/>
+    <row r="146" ht="14.25" customHeight="true"/>
+    <row r="147" ht="14.25" customHeight="true"/>
+    <row r="148" ht="14.25" customHeight="true"/>
+    <row r="149" ht="14.25" customHeight="true"/>
+    <row r="150" ht="14.25" customHeight="true"/>
+    <row r="151" ht="14.25" customHeight="true"/>
+    <row r="152" ht="14.25" customHeight="true"/>
+    <row r="153" ht="14.25" customHeight="true"/>
+    <row r="154" ht="14.25" customHeight="true"/>
+    <row r="155" ht="14.25" customHeight="true"/>
+    <row r="156" ht="14.25" customHeight="true"/>
+    <row r="157" ht="14.25" customHeight="true"/>
+    <row r="158" ht="14.25" customHeight="true"/>
+    <row r="159" ht="14.25" customHeight="true"/>
+    <row r="160" ht="14.25" customHeight="true"/>
+    <row r="161" ht="14.25" customHeight="true"/>
+    <row r="162" ht="14.25" customHeight="true"/>
+    <row r="163" ht="14.25" customHeight="true"/>
+    <row r="164" ht="14.25" customHeight="true"/>
+    <row r="165" ht="14.25" customHeight="true"/>
+    <row r="166" ht="14.25" customHeight="true"/>
+    <row r="167" ht="14.25" customHeight="true"/>
+    <row r="168" ht="14.25" customHeight="true"/>
+    <row r="169" ht="14.25" customHeight="true"/>
+    <row r="170" ht="14.25" customHeight="true"/>
+    <row r="171" ht="14.25" customHeight="true"/>
+    <row r="172" ht="14.25" customHeight="true"/>
+    <row r="173" ht="14.25" customHeight="true"/>
+    <row r="174" ht="14.25" customHeight="true"/>
+    <row r="175" ht="14.25" customHeight="true"/>
+    <row r="176" ht="14.25" customHeight="true"/>
+    <row r="177" ht="14.25" customHeight="true"/>
+    <row r="178" ht="14.25" customHeight="true"/>
+    <row r="179" ht="14.25" customHeight="true"/>
+    <row r="180" ht="14.25" customHeight="true"/>
+    <row r="181" ht="14.25" customHeight="true"/>
+    <row r="182" ht="14.25" customHeight="true"/>
+    <row r="183" ht="14.25" customHeight="true"/>
+    <row r="184" ht="14.25" customHeight="true"/>
+    <row r="185" ht="14.25" customHeight="true"/>
+    <row r="186" ht="14.25" customHeight="true"/>
+    <row r="187" ht="14.25" customHeight="true"/>
+    <row r="188" ht="14.25" customHeight="true"/>
+    <row r="189" ht="14.25" customHeight="true"/>
+    <row r="190" ht="14.25" customHeight="true"/>
+    <row r="191" ht="14.25" customHeight="true"/>
+    <row r="192" ht="14.25" customHeight="true"/>
+    <row r="193" ht="14.25" customHeight="true"/>
+    <row r="194" ht="14.25" customHeight="true"/>
+    <row r="195" ht="14.25" customHeight="true"/>
+    <row r="196" ht="14.25" customHeight="true"/>
+    <row r="197" ht="14.25" customHeight="true"/>
+    <row r="198" ht="14.25" customHeight="true"/>
+    <row r="199" ht="14.25" customHeight="true"/>
+    <row r="200" ht="14.25" customHeight="true"/>
+    <row r="201" ht="14.25" customHeight="true"/>
+    <row r="202" ht="14.25" customHeight="true"/>
+    <row r="203" ht="14.25" customHeight="true"/>
+    <row r="204" ht="14.25" customHeight="true"/>
+    <row r="205" ht="14.25" customHeight="true"/>
+    <row r="206" ht="14.25" customHeight="true"/>
+    <row r="207" ht="14.25" customHeight="true"/>
+    <row r="208" ht="14.25" customHeight="true"/>
+    <row r="209" ht="14.25" customHeight="true"/>
+    <row r="210" ht="14.25" customHeight="true"/>
+    <row r="211" ht="14.25" customHeight="true"/>
+    <row r="212" ht="14.25" customHeight="true"/>
+    <row r="213" ht="14.25" customHeight="true"/>
+    <row r="214" ht="14.25" customHeight="true"/>
+    <row r="215" ht="14.25" customHeight="true"/>
+    <row r="216" ht="14.25" customHeight="true"/>
+    <row r="217" ht="14.25" customHeight="true"/>
+    <row r="218" ht="14.25" customHeight="true"/>
+    <row r="219" ht="14.25" customHeight="true"/>
+    <row r="220" ht="14.25" customHeight="true"/>
+    <row r="221" ht="14.25" customHeight="true"/>
+    <row r="222" ht="14.25" customHeight="true"/>
+    <row r="223" ht="14.25" customHeight="true"/>
+    <row r="224" ht="14.25" customHeight="true"/>
+    <row r="225" ht="14.25" customHeight="true"/>
+    <row r="226" ht="14.25" customHeight="true"/>
+    <row r="227" ht="14.25" customHeight="true"/>
+    <row r="228" ht="14.25" customHeight="true"/>
+    <row r="229" ht="14.25" customHeight="true"/>
+    <row r="230" ht="14.25" customHeight="true"/>
+    <row r="231" ht="14.25" customHeight="true"/>
+    <row r="232" ht="14.25" customHeight="true"/>
+    <row r="233" ht="14.25" customHeight="true"/>
+    <row r="234" ht="14.25" customHeight="true"/>
+    <row r="235" ht="14.25" customHeight="true"/>
+    <row r="236" ht="14.25" customHeight="true"/>
+    <row r="237" ht="14.25" customHeight="true"/>
+    <row r="238" ht="14.25" customHeight="true"/>
+    <row r="239" ht="14.25" customHeight="true"/>
+    <row r="240" ht="14.25" customHeight="true"/>
+    <row r="241" ht="14.25" customHeight="true"/>
+    <row r="242" ht="14.25" customHeight="true"/>
+    <row r="243" ht="14.25" customHeight="true"/>
+    <row r="244" ht="14.25" customHeight="true"/>
+    <row r="245" ht="14.25" customHeight="true"/>
+    <row r="246" ht="14.25" customHeight="true"/>
+    <row r="247" ht="14.25" customHeight="true"/>
+    <row r="248" ht="14.25" customHeight="true"/>
+    <row r="249" ht="14.25" customHeight="true"/>
+    <row r="250" ht="14.25" customHeight="true"/>
+    <row r="251" ht="14.25" customHeight="true"/>
+    <row r="252" ht="14.25" customHeight="true"/>
+    <row r="253" ht="14.25" customHeight="true"/>
+    <row r="254" ht="14.25" customHeight="true"/>
+    <row r="255" ht="14.25" customHeight="true"/>
+    <row r="256" ht="14.25" customHeight="true"/>
+    <row r="257" ht="14.25" customHeight="true"/>
+    <row r="258" ht="14.25" customHeight="true"/>
+    <row r="259" ht="14.25" customHeight="true"/>
+    <row r="260" ht="14.25" customHeight="true"/>
+    <row r="261" ht="14.25" customHeight="true"/>
+    <row r="262" ht="14.25" customHeight="true"/>
+    <row r="263" ht="14.25" customHeight="true"/>
+    <row r="264" ht="14.25" customHeight="true"/>
+    <row r="265" ht="14.25" customHeight="true"/>
+    <row r="266" ht="14.25" customHeight="true"/>
+    <row r="267" ht="14.25" customHeight="true"/>
+    <row r="268" ht="14.25" customHeight="true"/>
+    <row r="269" ht="14.25" customHeight="true"/>
+    <row r="270" ht="14.25" customHeight="true"/>
+    <row r="271" ht="14.25" customHeight="true"/>
+    <row r="272" ht="14.25" customHeight="true"/>
+    <row r="273" ht="14.25" customHeight="true"/>
+    <row r="274" ht="14.25" customHeight="true"/>
+    <row r="275" ht="14.25" customHeight="true"/>
+    <row r="276" ht="14.25" customHeight="true"/>
+    <row r="277" ht="14.25" customHeight="true"/>
+    <row r="278" ht="14.25" customHeight="true"/>
+    <row r="279" ht="14.25" customHeight="true"/>
+    <row r="280" ht="14.25" customHeight="true"/>
+    <row r="281" ht="14.25" customHeight="true"/>
+    <row r="282" ht="14.25" customHeight="true"/>
+    <row r="283" ht="14.25" customHeight="true"/>
+    <row r="284" ht="14.25" customHeight="true"/>
+    <row r="285" ht="14.25" customHeight="true"/>
+    <row r="286" ht="14.25" customHeight="true"/>
+    <row r="287" ht="14.25" customHeight="true"/>
+    <row r="288" ht="14.25" customHeight="true"/>
+    <row r="289" ht="14.25" customHeight="true"/>
+    <row r="290" ht="14.25" customHeight="true"/>
+    <row r="291" ht="14.25" customHeight="true"/>
+    <row r="292" ht="14.25" customHeight="true"/>
+    <row r="293" ht="14.25" customHeight="true"/>
+    <row r="294" ht="14.25" customHeight="true"/>
+    <row r="295" ht="14.25" customHeight="true"/>
+    <row r="296" ht="14.25" customHeight="true"/>
+    <row r="297" ht="14.25" customHeight="true"/>
+    <row r="298" ht="14.25" customHeight="true"/>
+    <row r="299" ht="14.25" customHeight="true"/>
+    <row r="300" ht="14.25" customHeight="true"/>
+    <row r="301" ht="14.25" customHeight="true"/>
+    <row r="302" ht="14.25" customHeight="true"/>
+    <row r="303" ht="14.25" customHeight="true"/>
+    <row r="304" ht="14.25" customHeight="true"/>
+    <row r="305" ht="14.25" customHeight="true"/>
+    <row r="306" ht="14.25" customHeight="true"/>
+    <row r="307" ht="14.25" customHeight="true"/>
+    <row r="308" ht="14.25" customHeight="true"/>
+    <row r="309" ht="14.25" customHeight="true"/>
+    <row r="310" ht="14.25" customHeight="true"/>
+    <row r="311" ht="14.25" customHeight="true"/>
+    <row r="312" ht="14.25" customHeight="true"/>
+    <row r="313" ht="14.25" customHeight="true"/>
+    <row r="314" ht="14.25" customHeight="true"/>
+    <row r="315" ht="14.25" customHeight="true"/>
+    <row r="316" ht="14.25" customHeight="true"/>
+    <row r="317" ht="14.25" customHeight="true"/>
+    <row r="318" ht="14.25" customHeight="true"/>
+    <row r="319" ht="14.25" customHeight="true"/>
+    <row r="320" ht="14.25" customHeight="true"/>
+    <row r="321" ht="14.25" customHeight="true"/>
+    <row r="322" ht="14.25" customHeight="true"/>
+    <row r="323" ht="14.25" customHeight="true"/>
+    <row r="324" ht="14.25" customHeight="true"/>
+    <row r="325" ht="14.25" customHeight="true"/>
+    <row r="326" ht="14.25" customHeight="true"/>
+    <row r="327" ht="14.25" customHeight="true"/>
+    <row r="328" ht="14.25" customHeight="true"/>
+    <row r="329" ht="14.25" customHeight="true"/>
+    <row r="330" ht="14.25" customHeight="true"/>
+    <row r="331" ht="14.25" customHeight="true"/>
+    <row r="332" ht="14.25" customHeight="true"/>
+    <row r="333" ht="14.25" customHeight="true"/>
+    <row r="334" ht="14.25" customHeight="true"/>
+    <row r="335" ht="14.25" customHeight="true"/>
+    <row r="336" ht="14.25" customHeight="true"/>
+    <row r="337" ht="14.25" customHeight="true"/>
+    <row r="338" ht="14.25" customHeight="true"/>
+    <row r="339" ht="14.25" customHeight="true"/>
+    <row r="340" ht="14.25" customHeight="true"/>
+    <row r="341" ht="14.25" customHeight="true"/>
+    <row r="342" ht="14.25" customHeight="true"/>
+    <row r="343" ht="14.25" customHeight="true"/>
+    <row r="344" ht="14.25" customHeight="true"/>
+    <row r="345" ht="14.25" customHeight="true"/>
+    <row r="346" ht="14.25" customHeight="true"/>
+    <row r="347" ht="14.25" customHeight="true"/>
+    <row r="348" ht="14.25" customHeight="true"/>
+    <row r="349" ht="14.25" customHeight="true"/>
+    <row r="350" ht="14.25" customHeight="true"/>
+    <row r="351" ht="14.25" customHeight="true"/>
+    <row r="352" ht="14.25" customHeight="true"/>
+    <row r="353" ht="14.25" customHeight="true"/>
+    <row r="354" ht="14.25" customHeight="true"/>
+    <row r="355" ht="14.25" customHeight="true"/>
+    <row r="356" ht="14.25" customHeight="true"/>
+    <row r="357" ht="14.25" customHeight="true"/>
+    <row r="358" ht="14.25" customHeight="true"/>
+    <row r="359" ht="14.25" customHeight="true"/>
+    <row r="360" ht="14.25" customHeight="true"/>
+    <row r="361" ht="14.25" customHeight="true"/>
+    <row r="362" ht="14.25" customHeight="true"/>
+    <row r="363" ht="14.25" customHeight="true"/>
+    <row r="364" ht="14.25" customHeight="true"/>
+    <row r="365" ht="14.25" customHeight="true"/>
+    <row r="366" ht="14.25" customHeight="true"/>
+    <row r="367" ht="14.25" customHeight="true"/>
+    <row r="368" ht="14.25" customHeight="true"/>
+    <row r="369" ht="14.25" customHeight="true"/>
+    <row r="370" ht="14.25" customHeight="true"/>
+    <row r="371" ht="14.25" customHeight="true"/>
+    <row r="372" ht="14.25" customHeight="true"/>
+    <row r="373" ht="14.25" customHeight="true"/>
+    <row r="374" ht="14.25" customHeight="true"/>
+    <row r="375" ht="14.25" customHeight="true"/>
+    <row r="376" ht="14.25" customHeight="true"/>
+    <row r="377" ht="14.25" customHeight="true"/>
+    <row r="378" ht="14.25" customHeight="true"/>
+    <row r="379" ht="14.25" customHeight="true"/>
+    <row r="380" ht="14.25" customHeight="true"/>
+    <row r="381" ht="14.25" customHeight="true"/>
+    <row r="382" ht="14.25" customHeight="true"/>
+    <row r="383" ht="14.25" customHeight="true"/>
+    <row r="384" ht="14.25" customHeight="true"/>
+    <row r="385" ht="14.25" customHeight="true"/>
+    <row r="386" ht="14.25" customHeight="true"/>
+    <row r="387" ht="14.25" customHeight="true"/>
+    <row r="388" ht="14.25" customHeight="true"/>
+    <row r="389" ht="14.25" customHeight="true"/>
+    <row r="390" ht="14.25" customHeight="true"/>
+    <row r="391" ht="14.25" customHeight="true"/>
+    <row r="392" ht="14.25" customHeight="true"/>
+    <row r="393" ht="14.25" customHeight="true"/>
+    <row r="394" ht="14.25" customHeight="true"/>
+    <row r="395" ht="14.25" customHeight="true"/>
+    <row r="396" ht="14.25" customHeight="true"/>
+    <row r="397" ht="14.25" customHeight="true"/>
+    <row r="398" ht="14.25" customHeight="true"/>
+    <row r="399" ht="14.25" customHeight="true"/>
+    <row r="400" ht="14.25" customHeight="true"/>
+    <row r="401" ht="14.25" customHeight="true"/>
+    <row r="402" ht="14.25" customHeight="true"/>
+    <row r="403" ht="14.25" customHeight="true"/>
+    <row r="404" ht="14.25" customHeight="true"/>
+    <row r="405" ht="14.25" customHeight="true"/>
+    <row r="406" ht="14.25" customHeight="true"/>
+    <row r="407" ht="14.25" customHeight="true"/>
+    <row r="408" ht="14.25" customHeight="true"/>
+    <row r="409" ht="14.25" customHeight="true"/>
+    <row r="410" ht="14.25" customHeight="true"/>
+    <row r="411" ht="14.25" customHeight="true"/>
+    <row r="412" ht="14.25" customHeight="true"/>
+    <row r="413" ht="14.25" customHeight="true"/>
+    <row r="414" ht="14.25" customHeight="true"/>
+    <row r="415" ht="14.25" customHeight="true"/>
+    <row r="416" ht="14.25" customHeight="true"/>
+    <row r="417" ht="14.25" customHeight="true"/>
+    <row r="418" ht="14.25" customHeight="true"/>
+    <row r="419" ht="14.25" customHeight="true"/>
+    <row r="420" ht="14.25" customHeight="true"/>
+    <row r="421" ht="14.25" customHeight="true"/>
+    <row r="422" ht="14.25" customHeight="true"/>
+    <row r="423" ht="14.25" customHeight="true"/>
+    <row r="424" ht="14.25" customHeight="true"/>
+    <row r="425" ht="14.25" customHeight="true"/>
+    <row r="426" ht="14.25" customHeight="true"/>
+    <row r="427" ht="14.25" customHeight="true"/>
+    <row r="428" ht="14.25" customHeight="true"/>
+    <row r="429" ht="14.25" customHeight="true"/>
+    <row r="430" ht="14.25" customHeight="true"/>
+    <row r="431" ht="14.25" customHeight="true"/>
+    <row r="432" ht="14.25" customHeight="true"/>
+    <row r="433" ht="14.25" customHeight="true"/>
+    <row r="434" ht="14.25" customHeight="true"/>
+    <row r="435" ht="14.25" customHeight="true"/>
+    <row r="436" ht="14.25" customHeight="true"/>
+    <row r="437" ht="14.25" customHeight="true"/>
+    <row r="438" ht="14.25" customHeight="true"/>
+    <row r="439" ht="14.25" customHeight="true"/>
+    <row r="440" ht="14.25" customHeight="true"/>
+    <row r="441" ht="14.25" customHeight="true"/>
+    <row r="442" ht="14.25" customHeight="true"/>
+    <row r="443" ht="14.25" customHeight="true"/>
+    <row r="444" ht="14.25" customHeight="true"/>
+    <row r="445" ht="14.25" customHeight="true"/>
+    <row r="446" ht="14.25" customHeight="true"/>
+    <row r="447" ht="14.25" customHeight="true"/>
+    <row r="448" ht="14.25" customHeight="true"/>
+    <row r="449" ht="14.25" customHeight="true"/>
+    <row r="450" ht="14.25" customHeight="true"/>
+    <row r="451" ht="14.25" customHeight="true"/>
+    <row r="452" ht="14.25" customHeight="true"/>
+    <row r="453" ht="14.25" customHeight="true"/>
+    <row r="454" ht="14.25" customHeight="true"/>
+    <row r="455" ht="14.25" customHeight="true"/>
+    <row r="456" ht="14.25" customHeight="true"/>
+    <row r="457" ht="14.25" customHeight="true"/>
+    <row r="458" ht="14.25" customHeight="true"/>
+    <row r="459" ht="14.25" customHeight="true"/>
+    <row r="460" ht="14.25" customHeight="true"/>
+    <row r="461" ht="14.25" customHeight="true"/>
+    <row r="462" ht="14.25" customHeight="true"/>
+    <row r="463" ht="14.25" customHeight="true"/>
+    <row r="464" ht="14.25" customHeight="true"/>
+    <row r="465" ht="14.25" customHeight="true"/>
+    <row r="466" ht="14.25" customHeight="true"/>
+    <row r="467" ht="14.25" customHeight="true"/>
+    <row r="468" ht="14.25" customHeight="true"/>
+    <row r="469" ht="14.25" customHeight="true"/>
+    <row r="470" ht="14.25" customHeight="true"/>
+    <row r="471" ht="14.25" customHeight="true"/>
+    <row r="472" ht="14.25" customHeight="true"/>
+    <row r="473" ht="14.25" customHeight="true"/>
+    <row r="474" ht="14.25" customHeight="true"/>
+    <row r="475" ht="14.25" customHeight="true"/>
+    <row r="476" ht="14.25" customHeight="true"/>
+    <row r="477" ht="14.25" customHeight="true"/>
+    <row r="478" ht="14.25" customHeight="true"/>
+    <row r="479" ht="14.25" customHeight="true"/>
+    <row r="480" ht="14.25" customHeight="true"/>
+    <row r="481" ht="14.25" customHeight="true"/>
+    <row r="482" ht="14.25" customHeight="true"/>
+    <row r="483" ht="14.25" customHeight="true"/>
+    <row r="484" ht="14.25" customHeight="true"/>
+    <row r="485" ht="14.25" customHeight="true"/>
+    <row r="486" ht="14.25" customHeight="true"/>
+    <row r="487" ht="14.25" customHeight="true"/>
+    <row r="488" ht="14.25" customHeight="true"/>
+    <row r="489" ht="14.25" customHeight="true"/>
+    <row r="490" ht="14.25" customHeight="true"/>
+    <row r="491" ht="14.25" customHeight="true"/>
+    <row r="492" ht="14.25" customHeight="true"/>
+    <row r="493" ht="14.25" customHeight="true"/>
+    <row r="494" ht="14.25" customHeight="true"/>
+    <row r="495" ht="14.25" customHeight="true"/>
+    <row r="496" ht="14.25" customHeight="true"/>
+    <row r="497" ht="14.25" customHeight="true"/>
+    <row r="498" ht="14.25" customHeight="true"/>
+    <row r="499" ht="14.25" customHeight="true"/>
+    <row r="500" ht="14.25" customHeight="true"/>
+    <row r="501" ht="14.25" customHeight="true"/>
+    <row r="502" ht="14.25" customHeight="true"/>
+    <row r="503" ht="14.25" customHeight="true"/>
+    <row r="504" ht="14.25" customHeight="true"/>
+    <row r="505" ht="14.25" customHeight="true"/>
+    <row r="506" ht="14.25" customHeight="true"/>
+    <row r="507" ht="14.25" customHeight="true"/>
+    <row r="508" ht="14.25" customHeight="true"/>
+    <row r="509" ht="14.25" customHeight="true"/>
+    <row r="510" ht="14.25" customHeight="true"/>
+    <row r="511" ht="14.25" customHeight="true"/>
+    <row r="512" ht="14.25" customHeight="true"/>
+    <row r="513" ht="14.25" customHeight="true"/>
+    <row r="514" ht="14.25" customHeight="true"/>
+    <row r="515" ht="14.25" customHeight="true"/>
+    <row r="516" ht="14.25" customHeight="true"/>
+    <row r="517" ht="14.25" customHeight="true"/>
+    <row r="518" ht="14.25" customHeight="true"/>
+    <row r="519" ht="14.25" customHeight="true"/>
+    <row r="520" ht="14.25" customHeight="true"/>
+    <row r="521" ht="14.25" customHeight="true"/>
+    <row r="522" ht="14.25" customHeight="true"/>
+    <row r="523" ht="14.25" customHeight="true"/>
+    <row r="524" ht="14.25" customHeight="true"/>
+    <row r="525" ht="14.25" customHeight="true"/>
+    <row r="526" ht="14.25" customHeight="true"/>
+    <row r="527" ht="14.25" customHeight="true"/>
+    <row r="528" ht="14.25" customHeight="true"/>
+    <row r="529" ht="14.25" customHeight="true"/>
+    <row r="530" ht="14.25" customHeight="true"/>
+    <row r="531" ht="14.25" customHeight="true"/>
+    <row r="532" ht="14.25" customHeight="true"/>
+    <row r="533" ht="14.25" customHeight="true"/>
+    <row r="534" ht="14.25" customHeight="true"/>
+    <row r="535" ht="14.25" customHeight="true"/>
+    <row r="536" ht="14.25" customHeight="true"/>
+    <row r="537" ht="14.25" customHeight="true"/>
+    <row r="538" ht="14.25" customHeight="true"/>
+    <row r="539" ht="14.25" customHeight="true"/>
+    <row r="540" ht="14.25" customHeight="true"/>
+    <row r="541" ht="14.25" customHeight="true"/>
+    <row r="542" ht="14.25" customHeight="true"/>
+    <row r="543" ht="14.25" customHeight="true"/>
+    <row r="544" ht="14.25" customHeight="true"/>
+    <row r="545" ht="14.25" customHeight="true"/>
+    <row r="546" ht="14.25" customHeight="true"/>
+    <row r="547" ht="14.25" customHeight="true"/>
+    <row r="548" ht="14.25" customHeight="true"/>
+    <row r="549" ht="14.25" customHeight="true"/>
+    <row r="550" ht="14.25" customHeight="true"/>
+    <row r="551" ht="14.25" customHeight="true"/>
+    <row r="552" ht="14.25" customHeight="true"/>
+    <row r="553" ht="14.25" customHeight="true"/>
+    <row r="554" ht="14.25" customHeight="true"/>
+    <row r="555" ht="14.25" customHeight="true"/>
+    <row r="556" ht="14.25" customHeight="true"/>
+    <row r="557" ht="14.25" customHeight="true"/>
+    <row r="558" ht="14.25" customHeight="true"/>
+    <row r="559" ht="14.25" customHeight="true"/>
+    <row r="560" ht="14.25" customHeight="true"/>
+    <row r="561" ht="14.25" customHeight="true"/>
+    <row r="562" ht="14.25" customHeight="true"/>
+    <row r="563" ht="14.25" customHeight="true"/>
+    <row r="564" ht="14.25" customHeight="true"/>
+    <row r="565" ht="14.25" customHeight="true"/>
+    <row r="566" ht="14.25" customHeight="true"/>
+    <row r="567" ht="14.25" customHeight="true"/>
+    <row r="568" ht="14.25" customHeight="true"/>
+    <row r="569" ht="14.25" customHeight="true"/>
+    <row r="570" ht="14.25" customHeight="true"/>
+    <row r="571" ht="14.25" customHeight="true"/>
+    <row r="572" ht="14.25" customHeight="true"/>
+    <row r="573" ht="14.25" customHeight="true"/>
+    <row r="574" ht="14.25" customHeight="true"/>
+    <row r="575" ht="14.25" customHeight="true"/>
+    <row r="576" ht="14.25" customHeight="true"/>
+    <row r="577" ht="14.25" customHeight="true"/>
+    <row r="578" ht="14.25" customHeight="true"/>
+    <row r="579" ht="14.25" customHeight="true"/>
+    <row r="580" ht="14.25" customHeight="true"/>
+    <row r="581" ht="14.25" customHeight="true"/>
+    <row r="582" ht="14.25" customHeight="true"/>
+    <row r="583" ht="14.25" customHeight="true"/>
+    <row r="584" ht="14.25" customHeight="true"/>
+    <row r="585" ht="14.25" customHeight="true"/>
+    <row r="586" ht="14.25" customHeight="true"/>
+    <row r="587" ht="14.25" customHeight="true"/>
+    <row r="588" ht="14.25" customHeight="true"/>
+    <row r="589" ht="14.25" customHeight="true"/>
+    <row r="590" ht="14.25" customHeight="true"/>
+    <row r="591" ht="14.25" customHeight="true"/>
+    <row r="592" ht="14.25" customHeight="true"/>
+    <row r="593" ht="14.25" customHeight="true"/>
+    <row r="594" ht="14.25" customHeight="true"/>
+    <row r="595" ht="14.25" customHeight="true"/>
+    <row r="596" ht="14.25" customHeight="true"/>
+    <row r="597" ht="14.25" customHeight="true"/>
+    <row r="598" ht="14.25" customHeight="true"/>
+    <row r="599" ht="14.25" customHeight="true"/>
+    <row r="600" ht="14.25" customHeight="true"/>
+    <row r="601" ht="14.25" customHeight="true"/>
+    <row r="602" ht="14.25" customHeight="true"/>
+    <row r="603" ht="14.25" customHeight="true"/>
+    <row r="604" ht="14.25" customHeight="true"/>
+    <row r="605" ht="14.25" customHeight="true"/>
+    <row r="606" ht="14.25" customHeight="true"/>
+    <row r="607" ht="14.25" customHeight="true"/>
+    <row r="608" ht="14.25" customHeight="true"/>
+    <row r="609" ht="14.25" customHeight="true"/>
+    <row r="610" ht="14.25" customHeight="true"/>
+    <row r="611" ht="14.25" customHeight="true"/>
+    <row r="612" ht="14.25" customHeight="true"/>
+    <row r="613" ht="14.25" customHeight="true"/>
+    <row r="614" ht="14.25" customHeight="true"/>
+    <row r="615" ht="14.25" customHeight="true"/>
+    <row r="616" ht="14.25" customHeight="true"/>
+    <row r="617" ht="14.25" customHeight="true"/>
+    <row r="618" ht="14.25" customHeight="true"/>
+    <row r="619" ht="14.25" customHeight="true"/>
+    <row r="620" ht="14.25" customHeight="true"/>
+    <row r="621" ht="14.25" customHeight="true"/>
+    <row r="622" ht="14.25" customHeight="true"/>
+    <row r="623" ht="14.25" customHeight="true"/>
+    <row r="624" ht="14.25" customHeight="true"/>
+    <row r="625" ht="14.25" customHeight="true"/>
+    <row r="626" ht="14.25" customHeight="true"/>
+    <row r="627" ht="14.25" customHeight="true"/>
+    <row r="628" ht="14.25" customHeight="true"/>
+    <row r="629" ht="14.25" customHeight="true"/>
+    <row r="630" ht="14.25" customHeight="true"/>
+    <row r="631" ht="14.25" customHeight="true"/>
+    <row r="632" ht="14.25" customHeight="true"/>
+    <row r="633" ht="14.25" customHeight="true"/>
+    <row r="634" ht="14.25" customHeight="true"/>
+    <row r="635" ht="14.25" customHeight="true"/>
+    <row r="636" ht="14.25" customHeight="true"/>
+    <row r="637" ht="14.25" customHeight="true"/>
+    <row r="638" ht="14.25" customHeight="true"/>
+    <row r="639" ht="14.25" customHeight="true"/>
+    <row r="640" ht="14.25" customHeight="true"/>
+    <row r="641" ht="14.25" customHeight="true"/>
+    <row r="642" ht="14.25" customHeight="true"/>
+    <row r="643" ht="14.25" customHeight="true"/>
+    <row r="644" ht="14.25" customHeight="true"/>
+    <row r="645" ht="14.25" customHeight="true"/>
+    <row r="646" ht="14.25" customHeight="true"/>
+    <row r="647" ht="14.25" customHeight="true"/>
+    <row r="648" ht="14.25" customHeight="true"/>
+    <row r="649" ht="14.25" customHeight="true"/>
+    <row r="650" ht="14.25" customHeight="true"/>
+    <row r="651" ht="14.25" customHeight="true"/>
+    <row r="652" ht="14.25" customHeight="true"/>
+    <row r="653" ht="14.25" customHeight="true"/>
+    <row r="654" ht="14.25" customHeight="true"/>
+    <row r="655" ht="14.25" customHeight="true"/>
+    <row r="656" ht="14.25" customHeight="true"/>
+    <row r="657" ht="14.25" customHeight="true"/>
+    <row r="658" ht="14.25" customHeight="true"/>
+    <row r="659" ht="14.25" customHeight="true"/>
+    <row r="660" ht="14.25" customHeight="true"/>
+    <row r="661" ht="14.25" customHeight="true"/>
+    <row r="662" ht="14.25" customHeight="true"/>
+    <row r="663" ht="14.25" customHeight="true"/>
+    <row r="664" ht="14.25" customHeight="true"/>
+    <row r="665" ht="14.25" customHeight="true"/>
+    <row r="666" ht="14.25" customHeight="true"/>
+    <row r="667" ht="14.25" customHeight="true"/>
+    <row r="668" ht="14.25" customHeight="true"/>
+    <row r="669" ht="14.25" customHeight="true"/>
+    <row r="670" ht="14.25" customHeight="true"/>
+    <row r="671" ht="14.25" customHeight="true"/>
+    <row r="672" ht="14.25" customHeight="true"/>
+    <row r="673" ht="14.25" customHeight="true"/>
+    <row r="674" ht="14.25" customHeight="true"/>
+    <row r="675" ht="14.25" customHeight="true"/>
+    <row r="676" ht="14.25" customHeight="true"/>
+    <row r="677" ht="14.25" customHeight="true"/>
+    <row r="678" ht="14.25" customHeight="true"/>
+    <row r="679" ht="14.25" customHeight="true"/>
+    <row r="680" ht="14.25" customHeight="true"/>
+    <row r="681" ht="14.25" customHeight="true"/>
+    <row r="682" ht="14.25" customHeight="true"/>
+    <row r="683" ht="14.25" customHeight="true"/>
+    <row r="684" ht="14.25" customHeight="true"/>
+    <row r="685" ht="14.25" customHeight="true"/>
+    <row r="686" ht="14.25" customHeight="true"/>
+    <row r="687" ht="14.25" customHeight="true"/>
+    <row r="688" ht="14.25" customHeight="true"/>
+    <row r="689" ht="14.25" customHeight="true"/>
+    <row r="690" ht="14.25" customHeight="true"/>
+    <row r="691" ht="14.25" customHeight="true"/>
+    <row r="692" ht="14.25" customHeight="true"/>
+    <row r="693" ht="14.25" customHeight="true"/>
+    <row r="694" ht="14.25" customHeight="true"/>
+    <row r="695" ht="14.25" customHeight="true"/>
+    <row r="696" ht="14.25" customHeight="true"/>
+    <row r="697" ht="14.25" customHeight="true"/>
+    <row r="698" ht="14.25" customHeight="true"/>
+    <row r="699" ht="14.25" customHeight="true"/>
+    <row r="700" ht="14.25" customHeight="true"/>
+    <row r="701" ht="14.25" customHeight="true"/>
+    <row r="702" ht="14.25" customHeight="true"/>
+    <row r="703" ht="14.25" customHeight="true"/>
+    <row r="704" ht="14.25" customHeight="true"/>
+    <row r="705" ht="14.25" customHeight="true"/>
+    <row r="706" ht="14.25" customHeight="true"/>
+    <row r="707" ht="14.25" customHeight="true"/>
+    <row r="708" ht="14.25" customHeight="true"/>
+    <row r="709" ht="14.25" customHeight="true"/>
+    <row r="710" ht="14.25" customHeight="true"/>
+    <row r="711" ht="14.25" customHeight="true"/>
+    <row r="712" ht="14.25" customHeight="true"/>
+    <row r="713" ht="14.25" customHeight="true"/>
+    <row r="714" ht="14.25" customHeight="true"/>
+    <row r="715" ht="14.25" customHeight="true"/>
+    <row r="716" ht="14.25" customHeight="true"/>
+    <row r="717" ht="14.25" customHeight="true"/>
+    <row r="718" ht="14.25" customHeight="true"/>
+    <row r="719" ht="14.25" customHeight="true"/>
+    <row r="720" ht="14.25" customHeight="true"/>
+    <row r="721" ht="14.25" customHeight="true"/>
+    <row r="722" ht="14.25" customHeight="true"/>
+    <row r="723" ht="14.25" customHeight="true"/>
+    <row r="724" ht="14.25" customHeight="true"/>
+    <row r="725" ht="14.25" customHeight="true"/>
+    <row r="726" ht="14.25" customHeight="true"/>
+    <row r="727" ht="14.25" customHeight="true"/>
+    <row r="728" ht="14.25" customHeight="true"/>
+    <row r="729" ht="14.25" customHeight="true"/>
+    <row r="730" ht="14.25" customHeight="true"/>
+    <row r="731" ht="14.25" customHeight="true"/>
+    <row r="732" ht="14.25" customHeight="true"/>
+    <row r="733" ht="14.25" customHeight="true"/>
+    <row r="734" ht="14.25" customHeight="true"/>
+    <row r="735" ht="14.25" customHeight="true"/>
+    <row r="736" ht="14.25" customHeight="true"/>
+    <row r="737" ht="14.25" customHeight="true"/>
+    <row r="738" ht="14.25" customHeight="true"/>
+    <row r="739" ht="14.25" customHeight="true"/>
+    <row r="740" ht="14.25" customHeight="true"/>
+    <row r="741" ht="14.25" customHeight="true"/>
+    <row r="742" ht="14.25" customHeight="true"/>
+    <row r="743" ht="14.25" customHeight="true"/>
+    <row r="744" ht="14.25" customHeight="true"/>
+    <row r="745" ht="14.25" customHeight="true"/>
+    <row r="746" ht="14.25" customHeight="true"/>
+    <row r="747" ht="14.25" customHeight="true"/>
+    <row r="748" ht="14.25" customHeight="true"/>
+    <row r="749" ht="14.25" customHeight="true"/>
+    <row r="750" ht="14.25" customHeight="true"/>
+    <row r="751" ht="14.25" customHeight="true"/>
+    <row r="752" ht="14.25" customHeight="true"/>
+    <row r="753" ht="14.25" customHeight="true"/>
+    <row r="754" ht="14.25" customHeight="true"/>
+    <row r="755" ht="14.25" customHeight="true"/>
+    <row r="756" ht="14.25" customHeight="true"/>
+    <row r="757" ht="14.25" customHeight="true"/>
+    <row r="758" ht="14.25" customHeight="true"/>
+    <row r="759" ht="14.25" customHeight="true"/>
+    <row r="760" ht="14.25" customHeight="true"/>
+    <row r="761" ht="14.25" customHeight="true"/>
+    <row r="762" ht="14.25" customHeight="true"/>
+    <row r="763" ht="14.25" customHeight="true"/>
+    <row r="764" ht="14.25" customHeight="true"/>
+    <row r="765" ht="14.25" customHeight="true"/>
+    <row r="766" ht="14.25" customHeight="true"/>
+    <row r="767" ht="14.25" customHeight="true"/>
+    <row r="768" ht="14.25" customHeight="true"/>
+    <row r="769" ht="14.25" customHeight="true"/>
+    <row r="770" ht="14.25" customHeight="true"/>
+    <row r="771" ht="14.25" customHeight="true"/>
+    <row r="772" ht="14.25" customHeight="true"/>
+    <row r="773" ht="14.25" customHeight="true"/>
+    <row r="774" ht="14.25" customHeight="true"/>
+    <row r="775" ht="14.25" customHeight="true"/>
+    <row r="776" ht="14.25" customHeight="true"/>
+    <row r="777" ht="14.25" customHeight="true"/>
+    <row r="778" ht="14.25" customHeight="true"/>
+    <row r="779" ht="14.25" customHeight="true"/>
+    <row r="780" ht="14.25" customHeight="true"/>
+    <row r="781" ht="14.25" customHeight="true"/>
+    <row r="782" ht="14.25" customHeight="true"/>
+    <row r="783" ht="14.25" customHeight="true"/>
+    <row r="784" ht="14.25" customHeight="true"/>
+    <row r="785" ht="14.25" customHeight="true"/>
+    <row r="786" ht="14.25" customHeight="true"/>
+    <row r="787" ht="14.25" customHeight="true"/>
+    <row r="788" ht="14.25" customHeight="true"/>
+    <row r="789" ht="14.25" customHeight="true"/>
+    <row r="790" ht="14.25" customHeight="true"/>
+    <row r="791" ht="14.25" customHeight="true"/>
+    <row r="792" ht="14.25" customHeight="true"/>
+    <row r="793" ht="14.25" customHeight="true"/>
+    <row r="794" ht="14.25" customHeight="true"/>
+    <row r="795" ht="14.25" customHeight="true"/>
+    <row r="796" ht="14.25" customHeight="true"/>
+    <row r="797" ht="14.25" customHeight="true"/>
+    <row r="798" ht="14.25" customHeight="true"/>
+    <row r="799" ht="14.25" customHeight="true"/>
+    <row r="800" ht="14.25" customHeight="true"/>
+    <row r="801" ht="14.25" customHeight="true"/>
+    <row r="802" ht="14.25" customHeight="true"/>
+    <row r="803" ht="14.25" customHeight="true"/>
+    <row r="804" ht="14.25" customHeight="true"/>
+    <row r="805" ht="14.25" customHeight="true"/>
+    <row r="806" ht="14.25" customHeight="true"/>
+    <row r="807" ht="14.25" customHeight="true"/>
+    <row r="808" ht="14.25" customHeight="true"/>
+    <row r="809" ht="14.25" customHeight="true"/>
+    <row r="810" ht="14.25" customHeight="true"/>
+    <row r="811" ht="14.25" customHeight="true"/>
+    <row r="812" ht="14.25" customHeight="true"/>
+    <row r="813" ht="14.25" customHeight="true"/>
+    <row r="814" ht="14.25" customHeight="true"/>
+    <row r="815" ht="14.25" customHeight="true"/>
+    <row r="816" ht="14.25" customHeight="true"/>
+    <row r="817" ht="14.25" customHeight="true"/>
+    <row r="818" ht="14.25" customHeight="true"/>
+    <row r="819" ht="14.25" customHeight="true"/>
+    <row r="820" ht="14.25" customHeight="true"/>
+    <row r="821" ht="14.25" customHeight="true"/>
+    <row r="822" ht="14.25" customHeight="true"/>
+    <row r="823" ht="14.25" customHeight="true"/>
+    <row r="824" ht="14.25" customHeight="true"/>
+    <row r="825" ht="14.25" customHeight="true"/>
+    <row r="826" ht="14.25" customHeight="true"/>
+    <row r="827" ht="14.25" customHeight="true"/>
+    <row r="828" ht="14.25" customHeight="true"/>
+    <row r="829" ht="14.25" customHeight="true"/>
+    <row r="830" ht="14.25" customHeight="true"/>
+    <row r="831" ht="14.25" customHeight="true"/>
+    <row r="832" ht="14.25" customHeight="true"/>
+    <row r="833" ht="14.25" customHeight="true"/>
+    <row r="834" ht="14.25" customHeight="true"/>
+    <row r="835" ht="14.25" customHeight="true"/>
+    <row r="836" ht="14.25" customHeight="true"/>
+    <row r="837" ht="14.25" customHeight="true"/>
+    <row r="838" ht="14.25" customHeight="true"/>
+    <row r="839" ht="14.25" customHeight="true"/>
+    <row r="840" ht="14.25" customHeight="true"/>
+    <row r="841" ht="14.25" customHeight="true"/>
+    <row r="842" ht="14.25" customHeight="true"/>
+    <row r="843" ht="14.25" customHeight="true"/>
+    <row r="844" ht="14.25" customHeight="true"/>
+    <row r="845" ht="14.25" customHeight="true"/>
+    <row r="846" ht="14.25" customHeight="true"/>
+    <row r="847" ht="14.25" customHeight="true"/>
+    <row r="848" ht="14.25" customHeight="true"/>
+    <row r="849" ht="14.25" customHeight="true"/>
+    <row r="850" ht="14.25" customHeight="true"/>
+    <row r="851" ht="14.25" customHeight="true"/>
+    <row r="852" ht="14.25" customHeight="true"/>
+    <row r="853" ht="14.25" customHeight="true"/>
+    <row r="854" ht="14.25" customHeight="true"/>
+    <row r="855" ht="14.25" customHeight="true"/>
+    <row r="856" ht="14.25" customHeight="true"/>
+    <row r="857" ht="14.25" customHeight="true"/>
+    <row r="858" ht="14.25" customHeight="true"/>
+    <row r="859" ht="14.25" customHeight="true"/>
+    <row r="860" ht="14.25" customHeight="true"/>
+    <row r="861" ht="14.25" customHeight="true"/>
+    <row r="862" ht="14.25" customHeight="true"/>
+    <row r="863" ht="14.25" customHeight="true"/>
+    <row r="864" ht="14.25" customHeight="true"/>
+    <row r="865" ht="14.25" customHeight="true"/>
+    <row r="866" ht="14.25" customHeight="true"/>
+    <row r="867" ht="14.25" customHeight="true"/>
+    <row r="868" ht="14.25" customHeight="true"/>
+    <row r="869" ht="14.25" customHeight="true"/>
+    <row r="870" ht="14.25" customHeight="true"/>
+    <row r="871" ht="14.25" customHeight="true"/>
+    <row r="872" ht="14.25" customHeight="true"/>
+    <row r="873" ht="14.25" customHeight="true"/>
+    <row r="874" ht="14.25" customHeight="true"/>
+    <row r="875" ht="14.25" customHeight="true"/>
+    <row r="876" ht="14.25" customHeight="true"/>
+    <row r="877" ht="14.25" customHeight="true"/>
+    <row r="878" ht="14.25" customHeight="true"/>
+    <row r="879" ht="14.25" customHeight="true"/>
+    <row r="880" ht="14.25" customHeight="true"/>
+    <row r="881" ht="14.25" customHeight="true"/>
+    <row r="882" ht="14.25" customHeight="true"/>
+    <row r="883" ht="14.25" customHeight="true"/>
+    <row r="884" ht="14.25" customHeight="true"/>
+    <row r="885" ht="14.25" customHeight="true"/>
+    <row r="886" ht="14.25" customHeight="true"/>
+    <row r="887" ht="14.25" customHeight="true"/>
+    <row r="888" ht="14.25" customHeight="true"/>
+    <row r="889" ht="14.25" customHeight="true"/>
+    <row r="890" ht="14.25" customHeight="true"/>
+    <row r="891" ht="14.25" customHeight="true"/>
+    <row r="892" ht="14.25" customHeight="true"/>
+    <row r="893" ht="14.25" customHeight="true"/>
+    <row r="894" ht="14.25" customHeight="true"/>
+    <row r="895" ht="14.25" customHeight="true"/>
+    <row r="896" ht="14.25" customHeight="true"/>
+    <row r="897" ht="14.25" customHeight="true"/>
+    <row r="898" ht="14.25" customHeight="true"/>
+    <row r="899" ht="14.25" customHeight="true"/>
+    <row r="900" ht="14.25" customHeight="true"/>
+    <row r="901" ht="14.25" customHeight="true"/>
+    <row r="902" ht="14.25" customHeight="true"/>
+    <row r="903" ht="14.25" customHeight="true"/>
+    <row r="904" ht="14.25" customHeight="true"/>
+    <row r="905" ht="14.25" customHeight="true"/>
+    <row r="906" ht="14.25" customHeight="true"/>
+    <row r="907" ht="14.25" customHeight="true"/>
+    <row r="908" ht="14.25" customHeight="true"/>
+    <row r="909" ht="14.25" customHeight="true"/>
+    <row r="910" ht="14.25" customHeight="true"/>
+    <row r="911" ht="14.25" customHeight="true"/>
+    <row r="912" ht="14.25" customHeight="true"/>
+    <row r="913" ht="14.25" customHeight="true"/>
+    <row r="914" ht="14.25" customHeight="true"/>
+    <row r="915" ht="14.25" customHeight="true"/>
+    <row r="916" ht="14.25" customHeight="true"/>
+    <row r="917" ht="14.25" customHeight="true"/>
+    <row r="918" ht="14.25" customHeight="true"/>
+    <row r="919" ht="14.25" customHeight="true"/>
+    <row r="920" ht="14.25" customHeight="true"/>
+    <row r="921" ht="14.25" customHeight="true"/>
+    <row r="922" ht="14.25" customHeight="true"/>
+    <row r="923" ht="14.25" customHeight="true"/>
+    <row r="924" ht="14.25" customHeight="true"/>
+    <row r="925" ht="14.25" customHeight="true"/>
+    <row r="926" ht="14.25" customHeight="true"/>
+    <row r="927" ht="14.25" customHeight="true"/>
+    <row r="928" ht="14.25" customHeight="true"/>
+    <row r="929" ht="14.25" customHeight="true"/>
+    <row r="930" ht="14.25" customHeight="true"/>
+    <row r="931" ht="14.25" customHeight="true"/>
+    <row r="932" ht="14.25" customHeight="true"/>
+    <row r="933" ht="14.25" customHeight="true"/>
+    <row r="934" ht="14.25" customHeight="true"/>
+    <row r="935" ht="14.25" customHeight="true"/>
+    <row r="936" ht="14.25" customHeight="true"/>
+    <row r="937" ht="14.25" customHeight="true"/>
+    <row r="938" ht="14.25" customHeight="true"/>
+    <row r="939" ht="14.25" customHeight="true"/>
+    <row r="940" ht="14.25" customHeight="true"/>
+    <row r="941" ht="14.25" customHeight="true"/>
+    <row r="942" ht="14.25" customHeight="true"/>
+    <row r="943" ht="14.25" customHeight="true"/>
+    <row r="944" ht="14.25" customHeight="true"/>
+    <row r="945" ht="14.25" customHeight="true"/>
+    <row r="946" ht="14.25" customHeight="true"/>
+    <row r="947" ht="14.25" customHeight="true"/>
+    <row r="948" ht="14.25" customHeight="true"/>
+    <row r="949" ht="14.25" customHeight="true"/>
+    <row r="950" ht="14.25" customHeight="true"/>
+    <row r="951" ht="14.25" customHeight="true"/>
+    <row r="952" ht="14.25" customHeight="true"/>
+    <row r="953" ht="14.25" customHeight="true"/>
+    <row r="954" ht="14.25" customHeight="true"/>
+    <row r="955" ht="14.25" customHeight="true"/>
+    <row r="956" ht="14.25" customHeight="true"/>
+    <row r="957" ht="14.25" customHeight="true"/>
+    <row r="958" ht="14.25" customHeight="true"/>
+    <row r="959" ht="14.25" customHeight="true"/>
+    <row r="960" ht="14.25" customHeight="true"/>
+    <row r="961" ht="14.25" customHeight="true"/>
+    <row r="962" ht="14.25" customHeight="true"/>
+    <row r="963" ht="14.25" customHeight="true"/>
+    <row r="964" ht="14.25" customHeight="true"/>
+    <row r="965" ht="14.25" customHeight="true"/>
+    <row r="966" ht="14.25" customHeight="true"/>
+    <row r="967" ht="14.25" customHeight="true"/>
+    <row r="968" ht="14.25" customHeight="true"/>
+    <row r="969" ht="14.25" customHeight="true"/>
+    <row r="970" ht="14.25" customHeight="true"/>
+    <row r="971" ht="14.25" customHeight="true"/>
+    <row r="972" ht="14.25" customHeight="true"/>
+    <row r="973" ht="14.25" customHeight="true"/>
+    <row r="974" ht="14.25" customHeight="true"/>
+    <row r="975" ht="14.25" customHeight="true"/>
+    <row r="976" ht="14.25" customHeight="true"/>
+    <row r="977" ht="14.25" customHeight="true"/>
+    <row r="978" ht="14.25" customHeight="true"/>
+    <row r="979" ht="14.25" customHeight="true"/>
+    <row r="980" ht="14.25" customHeight="true"/>
+    <row r="981" ht="14.25" customHeight="true"/>
+    <row r="982" ht="14.25" customHeight="true"/>
+    <row r="983" ht="14.25" customHeight="true"/>
+    <row r="984" ht="14.25" customHeight="true"/>
+    <row r="985" ht="14.25" customHeight="true"/>
+    <row r="986" ht="14.25" customHeight="true"/>
+    <row r="987" ht="14.25" customHeight="true"/>
+    <row r="988" ht="14.25" customHeight="true"/>
+    <row r="989" ht="14.25" customHeight="true"/>
+    <row r="990" ht="14.25" customHeight="true"/>
+    <row r="991" ht="14.25" customHeight="true"/>
+    <row r="992" ht="14.25" customHeight="true"/>
+    <row r="993" ht="14.25" customHeight="true"/>
+    <row r="994" ht="14.25" customHeight="true"/>
+    <row r="995" ht="14.25" customHeight="true"/>
+    <row r="996" ht="14.25" customHeight="true"/>
+    <row r="997" ht="14.25" customHeight="true"/>
+    <row r="998" ht="14.25" customHeight="true"/>
+    <row r="999" ht="14.25" customHeight="true"/>
+    <row r="1000" ht="14.25" customHeight="true"/>
   </sheetData>
   <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: (user) update deleteUser response to return success message and filter out deleted users in GetUsers query
</commit_message>
<xml_diff>
--- a/db/seeds/excel/seeds.xlsx
+++ b/db/seeds/excel/seeds.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="279">
   <si>
     <t>ID</t>
   </si>
@@ -70,153 +70,231 @@
     <t>Akses Penuh terhadap aplikasi</t>
   </si>
   <si>
+    <t>01JQ2GQBNQJ16HR0F7XY1MFC48</t>
+  </si>
+  <si>
     <t>student_read</t>
   </si>
   <si>
     <t>Melihat list santri</t>
   </si>
   <si>
+    <t>01JQ2GQBRM60EXZTBN5C91VVDM</t>
+  </si>
+  <si>
     <t>student_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus santri</t>
   </si>
   <si>
+    <t>01JQ2GQBVSDM4FD7CYE54MQGBD</t>
+  </si>
+  <si>
     <t>student_manager_read</t>
   </si>
   <si>
     <t>Melihat list MS</t>
   </si>
   <si>
+    <t>01JQ2GQBXCEMQFZ5YGX7K49GB7</t>
+  </si>
+  <si>
     <t>student_manager_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus MS</t>
   </si>
   <si>
+    <t>01JQ2GQBYV8GDR2EGWFJ7TB28A</t>
+  </si>
+  <si>
     <t>academic_manager_read</t>
   </si>
   <si>
     <t>Melihat list MA</t>
   </si>
   <si>
+    <t>01JQ2GQC0JNSJ1S1BXS2XTKGCY</t>
+  </si>
+  <si>
     <t>academic_manager_write</t>
   </si>
   <si>
+    <t>01JQ2GQC1Z145KEPCWGDV26RR0</t>
+  </si>
+  <si>
     <t>mpa_read</t>
   </si>
   <si>
     <t>Melihat list MPA</t>
   </si>
   <si>
+    <t>01JQ2GQC4P62JKEJQP2636NYWC</t>
+  </si>
+  <si>
     <t>mpa_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus MPA</t>
   </si>
   <si>
+    <t>01JQ2GQC6ARCMA5ANEKS0NYV9A</t>
+  </si>
+  <si>
     <t>mentor_read</t>
   </si>
   <si>
     <t>Melihat list pengajar</t>
   </si>
   <si>
+    <t>01JQ2GQC7PKPWMEBG3T4PGWMM3</t>
+  </si>
+  <si>
     <t>mentor_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus pengaja</t>
   </si>
   <si>
+    <t>01JQ2GQCBS5P7YE2JN714RDHES</t>
+  </si>
+  <si>
     <t>program_read</t>
   </si>
   <si>
     <t>Melihat list program</t>
   </si>
   <si>
+    <t>01JQ2GQCD9BQWZZXZN2JGGW6AV</t>
+  </si>
+  <si>
     <t>program_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus program</t>
   </si>
   <si>
+    <t>01JQ2GQCEN6D7AZEHTT2SF23GJ</t>
+  </si>
+  <si>
     <t>template_read</t>
   </si>
   <si>
     <t>Melihat list template CFO 1</t>
   </si>
   <si>
+    <t>01JQ2GQCG7Z81E4V2ZX8EVYP5E</t>
+  </si>
+  <si>
     <t>template_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus template CFO 1</t>
   </si>
   <si>
+    <t>01JQ2GQCJ840QN1NQMX7XMGFN3</t>
+  </si>
+  <si>
     <t>report_cfo1_read</t>
   </si>
   <si>
     <t>Melihat list laporan CFO 1</t>
   </si>
   <si>
+    <t>01JQ2GQCMBAYHE44ZREF673XTX</t>
+  </si>
+  <si>
     <t>report_cfo1_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus CFO 1</t>
   </si>
   <si>
+    <t>01JQ2GQCNR4125SZ6YMT81AYN5</t>
+  </si>
+  <si>
     <t>report_cfo2_academic_finance_read</t>
   </si>
   <si>
     <t>Melihat list data keuangan akademik di CFO 2</t>
   </si>
   <si>
+    <t>01JQ2GQCV4QWRZX68XWPH9TPJZ</t>
+  </si>
+  <si>
     <t>report_cfo2_academic_finance_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus data keuangan akademik di CFO 2</t>
   </si>
   <si>
+    <t>01JQ2GQCWGY3ZRVCWA15N5P19T</t>
+  </si>
+  <si>
     <t>report_cfo2_mentor_fee_read</t>
   </si>
   <si>
     <t>Melihat list gaji mentor di CFO 2</t>
   </si>
   <si>
+    <t>01JQ2GQCXZRXSJ6E695GHD58KF</t>
+  </si>
+  <si>
     <t>report_cfo2_mentor_fee_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus data keuangan mentor di CFO 2</t>
   </si>
   <si>
+    <t>01JQ2GQCZGWVA531J7KF14XAGD</t>
+  </si>
+  <si>
     <t>report_fee_recapitulation_read</t>
   </si>
   <si>
     <t>Melihat list laporan rekap gaji</t>
   </si>
   <si>
+    <t>01JQ2GQD1T59NR49TDNGW8V49B</t>
+  </si>
+  <si>
     <t>report_fee_recapitulation_write</t>
   </si>
   <si>
     <t>Mengubah rekap gaji</t>
   </si>
   <si>
+    <t>01JQ2GQD37B07JDVV8GNNYEQ9Z</t>
+  </si>
+  <si>
     <t>user_management_read</t>
   </si>
   <si>
     <t>Melihat list user</t>
   </si>
   <si>
+    <t>01JQ2GQD4MXZYMP0TCMWE9E856</t>
+  </si>
+  <si>
     <t>user_management_write</t>
   </si>
   <si>
     <t>Membuat, Mengubah, dan menghapus user</t>
   </si>
   <si>
+    <t>01JQ2GQD80RX286JMYD2AY0MVV</t>
+  </si>
+  <si>
     <t>role_management_read</t>
   </si>
   <si>
     <t>Melihat list role</t>
   </si>
   <si>
+    <t>01JQ2GQDD3K0GKJMZ8STS209ZP</t>
+  </si>
+  <si>
     <t>role_management_write</t>
   </si>
   <si>
@@ -772,82 +850,10 @@
     <t>admin#admin</t>
   </si>
   <si>
-    <t>01JQ2GQBNQJ16HR0F7XY1MFC48</t>
-  </si>
-  <si>
-    <t>01JQ2GQBRM60EXZTBN5C91VVDM</t>
-  </si>
-  <si>
-    <t>01JQ2GQBVSDM4FD7CYE54MQGBD</t>
-  </si>
-  <si>
-    <t>01JQ2GQBXCEMQFZ5YGX7K49GB7</t>
-  </si>
-  <si>
-    <t>01JQ2GQBYV8GDR2EGWFJ7TB28A</t>
-  </si>
-  <si>
-    <t>01JQ2GQC0JNSJ1S1BXS2XTKGCY</t>
-  </si>
-  <si>
-    <t>01JQ2GQC1Z145KEPCWGDV26RR0</t>
-  </si>
-  <si>
-    <t>01JQ2GQC4P62JKEJQP2636NYWC</t>
-  </si>
-  <si>
-    <t>01JQ2GQC6ARCMA5ANEKS0NYV9A</t>
-  </si>
-  <si>
-    <t>01JQ2GQC7PKPWMEBG3T4PGWMM3</t>
-  </si>
-  <si>
-    <t>01JQ2GQCBS5P7YE2JN714RDHES</t>
-  </si>
-  <si>
-    <t>01JQ2GQCD9BQWZZXZN2JGGW6AV</t>
-  </si>
-  <si>
-    <t>01JQ2GQCEN6D7AZEHTT2SF23GJ</t>
-  </si>
-  <si>
-    <t>01JQ2GQCG7Z81E4V2ZX8EVYP5E</t>
-  </si>
-  <si>
-    <t>01JQ2GQCJ840QN1NQMX7XMGFN3</t>
-  </si>
-  <si>
-    <t>01JQ2GQCMBAYHE44ZREF673XTX</t>
-  </si>
-  <si>
-    <t>01JQ2GQCNR4125SZ6YMT81AYN5</t>
-  </si>
-  <si>
-    <t>01JQ2GQCV4QWRZX68XWPH9TPJZ</t>
-  </si>
-  <si>
-    <t>01JQ2GQCWGY3ZRVCWA15N5P19T</t>
-  </si>
-  <si>
-    <t>01JQ2GQCXZRXSJ6E695GHD58KF</t>
-  </si>
-  <si>
-    <t>01JQ2GQCZGWVA531J7KF14XAGD</t>
-  </si>
-  <si>
-    <t>01JQ2GQD1T59NR49TDNGW8V49B</t>
-  </si>
-  <si>
-    <t>01JQ2GQD37B07JDVV8GNNYEQ9Z</t>
-  </si>
-  <si>
-    <t>01JQ2GQD4MXZYMP0TCMWE9E856</t>
-  </si>
-  <si>
-    <t>01JQ2GQD80RX286JMYD2AY0MVV</t>
-  </si>
-  <si>
-    <t>01JQ2GQDD3K0GKJMZ8STS209ZP</t>
+    <t>01JQQGC9CW1MZA38F7KB07NZFA</t>
+  </si>
+  <si>
+    <t>01JQQGC9EQXM78NZH09RXNVHHJ</t>
   </si>
   <si>
     <t>01JH58TXMWEW5EMHQ2GES2TF77</t>
@@ -857,7 +863,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -876,7 +882,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -925,39 +945,48 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyAlignment="true"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2289,450 +2318,450 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>166</v>
+        <v>192</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>167</v>
+        <v>193</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>129</v>
+        <v>155</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>168</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>170</v>
+        <v>195</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>196</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>174</v>
+        <v>199</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>200</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>175</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>177</v>
+        <v>202</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>203</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>178</v>
+        <v>199</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>204</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>179</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>181</v>
+        <v>206</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>207</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>182</v>
+        <v>199</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>208</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>183</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>185</v>
+        <v>210</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>211</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>186</v>
+        <v>199</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>212</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>187</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>189</v>
+        <v>214</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>215</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>190</v>
+        <v>199</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>216</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>191</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>193</v>
+        <v>218</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>219</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>194</v>
+        <v>199</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>220</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>195</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B8" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>171</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>198</v>
+        <v>199</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>224</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>199</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>201</v>
+        <v>226</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>227</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>202</v>
+        <v>199</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>228</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>203</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>205</v>
+        <v>230</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>231</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>207</v>
+        <v>232</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>233</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>208</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>210</v>
+        <v>235</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>236</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>212</v>
+        <v>232</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>238</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>213</v>
+        <v>239</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>214</v>
+        <v>240</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>215</v>
+        <v>241</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>216</v>
+        <v>242</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>217</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>218</v>
+        <v>244</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>219</v>
+        <v>245</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>220</v>
+        <v>246</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>221</v>
+        <v>247</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>222</v>
+        <v>248</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>223</v>
+        <v>249</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>225</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>226</v>
+        <v>252</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>227</v>
+        <v>253</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>228</v>
+        <v>254</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>229</v>
+        <v>255</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>230</v>
+        <v>256</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>231</v>
+        <v>257</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>232</v>
+        <v>258</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>233</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>234</v>
+        <v>260</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>235</v>
+        <v>261</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>236</v>
+        <v>262</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>237</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>238</v>
+        <v>264</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>239</v>
+        <v>265</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>240</v>
+        <v>266</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>241</v>
+        <v>267</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>242</v>
+        <v>268</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>243</v>
+        <v>269</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>244</v>
+        <v>270</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>245</v>
+        <v>271</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>246</v>
+        <v>272</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>247</v>
+        <v>273</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F20" s="13" t="s">
-        <v>248</v>
+      <c r="F20" s="18" t="s">
+        <v>274</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>249</v>
+        <v>275</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1"/>
@@ -3733,7 +3762,7 @@
   </sheetPr>
   <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="true"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="25.14"/>
+    <col customWidth="true" max="1" min="1" width="28.71"/>
     <col customWidth="true" max="2" min="2" width="38"/>
     <col customWidth="true" max="3" min="3" width="73.86"/>
     <col customWidth="true" max="26" min="4" width="8.71"/>
@@ -3751,7 +3780,7 @@
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="true">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -3762,301 +3791,321 @@
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="true">
-      <c r="A3" t="s">
-        <v>250</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>17</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="true">
-      <c r="A4" t="s">
-        <v>251</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>19</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="true">
-      <c r="A5" t="s">
-        <v>252</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>21</v>
+      <c r="A5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="true">
-      <c r="A6" t="s">
-        <v>253</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>23</v>
+      <c r="A6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="true">
-      <c r="A7" t="s">
-        <v>254</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>25</v>
+      <c r="A7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="true">
-      <c r="A8" t="s">
-        <v>255</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>23</v>
+      <c r="A8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="true">
-      <c r="A9" t="s">
-        <v>256</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>28</v>
+      <c r="A9" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="true">
-      <c r="A10" t="s">
-        <v>257</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>30</v>
+      <c r="A10" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="true">
-      <c r="A11" t="s">
-        <v>258</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>32</v>
+      <c r="A11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="true">
-      <c r="A12" t="s">
-        <v>259</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>34</v>
+      <c r="A12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="true">
-      <c r="A13" t="s">
-        <v>260</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>36</v>
+      <c r="A13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="true">
-      <c r="A14" t="s">
-        <v>261</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>38</v>
+      <c r="A14" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="true">
-      <c r="A15" t="s">
-        <v>262</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>40</v>
+      <c r="A15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="true">
-      <c r="A16" t="s">
-        <v>263</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>42</v>
+      <c r="A16" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="true">
-      <c r="A17" t="s">
-        <v>264</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>44</v>
+      <c r="A17" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="true">
-      <c r="A18" t="s">
-        <v>265</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>46</v>
+      <c r="A18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="true">
-      <c r="A19" t="s">
-        <v>266</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>48</v>
+      <c r="A19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="true">
-      <c r="A20" t="s">
-        <v>267</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>50</v>
+      <c r="A20" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="true">
-      <c r="A21" t="s">
-        <v>268</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>52</v>
+      <c r="A21" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="true">
-      <c r="A22" t="s">
-        <v>269</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>54</v>
+      <c r="A22" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="true">
-      <c r="A23" t="s">
-        <v>270</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>56</v>
+      <c r="A23" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="true">
-      <c r="A24" t="s">
-        <v>271</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>58</v>
+      <c r="A24" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="25" ht="14.25" customHeight="true">
-      <c r="A25" t="s">
-        <v>272</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>60</v>
+      <c r="A25" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="true">
-      <c r="A26" t="s">
-        <v>273</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>62</v>
+      <c r="A26" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="true">
-      <c r="A27" t="s">
-        <v>274</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>64</v>
+      <c r="A27" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="true">
-      <c r="A28" t="s">
-        <v>275</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>66</v>
+      <c r="A28" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="true">
-      <c r="A29" t="s">
+      <c r="A29" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" ht="14.25" customHeight="true">
+      <c r="A30" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" ht="14.25" customHeight="true">
+      <c r="A31" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="B31" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="30" ht="14.25" customHeight="true"/>
-    <row r="31" ht="14.25" customHeight="true"/>
     <row r="32" ht="14.25" customHeight="true"/>
     <row r="33" ht="14.25" customHeight="true"/>
     <row r="34" ht="14.25" customHeight="true"/>
@@ -5062,507 +5111,507 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>74</v>
+        <v>97</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="D2" s="7">
+        <v>101</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="12">
         <v>720000.0</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F2" s="7">
+        <v>104</v>
+      </c>
+      <c r="F2" s="12">
         <v>100000.0</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="12">
         <v>485000.0</v>
       </c>
-      <c r="H2" s="8">
+      <c r="H2" s="13">
         <v>34000.0</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="14">
         <v>445000.0</v>
       </c>
-      <c r="J2" s="10">
+      <c r="J2" s="15">
         <v>1.0</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="D3" s="7">
+        <v>105</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="12">
         <v>1070000.0</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F3" s="7">
+        <v>104</v>
+      </c>
+      <c r="F3" s="12">
         <v>200000.0</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="12">
         <v>725000.0</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="13">
         <v>49500.0</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="14">
         <v>645000.0</v>
       </c>
-      <c r="J3" s="10">
+      <c r="J3" s="15">
         <v>2.0</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="D4" s="7">
+        <v>108</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="12">
         <v>1420000.0</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F4" s="7">
+        <v>104</v>
+      </c>
+      <c r="F4" s="12">
         <v>300000.0</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="12">
         <v>965000.0</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="13">
         <v>65000.0</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="14">
         <v>845000.0</v>
       </c>
-      <c r="J4" s="10">
+      <c r="J4" s="15">
         <v>3.0</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="D5" s="7">
+        <v>111</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" s="12">
         <v>675000.0</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F5" s="7">
+        <v>114</v>
+      </c>
+      <c r="F5" s="12">
         <v>100000.0</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="12">
         <v>440000.0</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="13">
         <v>17000.0</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="14">
         <v>400000.0</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="15">
         <v>1.0</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="D6" s="7">
+        <v>115</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="12">
         <v>475000.0</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F6" s="7">
+        <v>114</v>
+      </c>
+      <c r="F6" s="12">
         <v>100000.0</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="12">
         <v>240000.0</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="13">
         <v>8500.0</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="14">
         <v>200000.0</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="15">
         <v>1.0</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D7" s="7">
+        <v>118</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D7" s="12">
         <v>595000.0</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F7" s="7">
+        <v>121</v>
+      </c>
+      <c r="F7" s="12">
         <v>100000.0</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="12">
         <v>360000.0</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="13">
         <v>35500.0</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="14">
         <v>320000.0</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="15">
         <v>1.0</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="D8" s="7">
+        <v>122</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" s="12">
         <v>885000.0</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F8" s="7">
+        <v>121</v>
+      </c>
+      <c r="F8" s="12">
         <v>200000.0</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="12">
         <v>540000.0</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="13">
         <v>51000.0</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="14">
         <v>460000.0</v>
       </c>
-      <c r="J8" s="10">
+      <c r="J8" s="15">
         <v>2.0</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="D9" s="7">
+        <v>125</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="12">
         <v>1170000.0</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F9" s="7">
+        <v>121</v>
+      </c>
+      <c r="F9" s="12">
         <v>300000.0</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="12">
         <v>715000.0</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="13">
         <v>66000.0</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="14">
         <v>595000.0</v>
       </c>
-      <c r="J9" s="10">
+      <c r="J9" s="15">
         <v>3.0</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="D10" s="7">
+        <v>128</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="D10" s="12">
         <v>450000.0</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F10" s="7">
+        <v>121</v>
+      </c>
+      <c r="F10" s="12">
         <v>100000.0</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="12">
         <v>215000.0</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="13">
         <v>17500.0</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="14">
         <v>175000.0</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="15">
         <v>1.0</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="D11" s="7">
+        <v>131</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="D11" s="12">
         <v>720000.0</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F11" s="7">
+        <v>134</v>
+      </c>
+      <c r="F11" s="12">
         <v>100000.0</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="12">
         <v>485000.0</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="13">
         <v>49000.0</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="14">
         <v>445000.0</v>
       </c>
-      <c r="J11" s="10">
+      <c r="J11" s="15">
         <v>1.0</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="D12" s="7">
+        <v>135</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="D12" s="12">
         <v>970000.0</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F12" s="7">
+        <v>134</v>
+      </c>
+      <c r="F12" s="12">
         <v>200000.0</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="12">
         <v>625000.0</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="13">
         <v>60500.0</v>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="14">
         <v>545000.0</v>
       </c>
-      <c r="J12" s="10">
+      <c r="J12" s="15">
         <v>2.0</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="D13" s="7">
+        <v>138</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="D13" s="12">
         <v>1220000.0</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F13" s="7">
+        <v>134</v>
+      </c>
+      <c r="F13" s="12">
         <v>300000.0</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="12">
         <v>765000.0</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="13">
         <v>71500.0</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="14">
         <v>645000.0</v>
       </c>
-      <c r="J13" s="10">
+      <c r="J13" s="15">
         <v>3.0</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="D14" s="7">
+        <v>141</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="D14" s="12">
         <v>600000.0</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F14" s="7">
+        <v>134</v>
+      </c>
+      <c r="F14" s="12">
         <v>100000.0</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="12">
         <v>365000.0</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="13">
         <v>36000.0</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="14">
         <v>325000.0</v>
       </c>
-      <c r="J14" s="10">
+      <c r="J14" s="15">
         <v>1.0</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="D15" s="7">
+        <v>144</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D15" s="12">
         <v>550000.0</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="F15" s="7">
+        <v>147</v>
+      </c>
+      <c r="F15" s="12">
         <v>100000.0</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="12">
         <v>315000.0</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="13">
         <v>18000.0</v>
       </c>
-      <c r="I15" s="9">
+      <c r="I15" s="14">
         <v>275000.0</v>
       </c>
-      <c r="J15" s="10">
+      <c r="J15" s="15">
         <v>1.0</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="D16" s="7">
+        <v>148</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D16" s="12">
         <v>620000.0</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="F16" s="7">
+        <v>147</v>
+      </c>
+      <c r="F16" s="12">
         <v>100000.0</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="12">
         <v>385000.0</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="13">
         <v>23000.0</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="14">
         <v>345000.0</v>
       </c>
-      <c r="J16" s="10">
+      <c r="J16" s="15">
         <v>1.0</v>
       </c>
     </row>
@@ -6581,18 +6630,18 @@
       <c r="D1" s="1"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="B2" s="10" t="s">
-        <v>125</v>
+      <c r="B2" s="15" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="B3" s="10" t="s">
-        <v>126</v>
+      <c r="B3" s="15" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="B4" s="10" t="s">
-        <v>127</v>
+      <c r="B4" s="15" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -7615,50 +7664,50 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>128</v>
+      <c r="B1" s="10" t="s">
+        <v>154</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>129</v>
+        <v>155</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>130</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>132</v>
+        <v>157</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>158</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>133</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>135</v>
+        <v>160</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>161</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>136</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>138</v>
+        <v>163</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>164</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>139</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -8684,34 +8733,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>129</v>
+        <v>155</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>130</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>140</v>
+        <v>166</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>141</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>142</v>
+        <v>168</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>143</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>144</v>
+        <v>170</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>145</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -9735,49 +9784,49 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>146</v>
+        <v>172</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>129</v>
+        <v>155</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>130</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>147</v>
+        <v>173</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>140</v>
+        <v>166</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>148</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>149</v>
+        <v>175</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>142</v>
+        <v>168</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>150</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>151</v>
+        <v>177</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>144</v>
+        <v>170</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>152</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -10801,7 +10850,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>153</v>
+        <v>179</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -10811,35 +10860,35 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>155</v>
+        <v>181</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>156</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>157</v>
+        <v>183</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>158</v>
+        <v>184</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>159</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>160</v>
+        <v>186</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>161</v>
+        <v>187</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>162</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1"/>
@@ -11868,10 +11917,10 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>164</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
chore: update seeds.xlsx with new data
</commit_message>
<xml_diff>
--- a/db/seeds/excel/seeds.xlsx
+++ b/db/seeds/excel/seeds.xlsx
@@ -1273,14 +1273,14 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="true"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="29.71"/>
-    <col customWidth="1" min="2" max="2" width="13.86"/>
-    <col customWidth="1" min="3" max="26" width="8.71"/>
+    <col customWidth="true" max="1" min="1" width="29.71"/>
+    <col customWidth="true" max="2" min="2" width="13.86"/>
+    <col customWidth="true" max="26" min="3" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
+    <row r="1" ht="14.25" customHeight="true">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1">
+    <row r="2" ht="14.25" customHeight="true">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1">
+    <row r="3" ht="14.25" customHeight="true">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1">
+    <row r="4" ht="14.25" customHeight="true">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="14.25" customHeight="1">
+    <row r="5" ht="14.25" customHeight="true">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -1320,7 +1320,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" ht="14.25" customHeight="1">
+    <row r="6" ht="14.25" customHeight="true">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -1328,1003 +1328,1003 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="14.25" customHeight="1"/>
-    <row r="8" ht="14.25" customHeight="1"/>
-    <row r="9" ht="14.25" customHeight="1"/>
-    <row r="10" ht="14.25" customHeight="1"/>
-    <row r="11" ht="14.25" customHeight="1"/>
-    <row r="12" ht="14.25" customHeight="1"/>
-    <row r="13" ht="14.25" customHeight="1"/>
-    <row r="14" ht="14.25" customHeight="1"/>
-    <row r="15" ht="14.25" customHeight="1"/>
-    <row r="16" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
-    <row r="65" ht="14.25" customHeight="1"/>
-    <row r="66" ht="14.25" customHeight="1"/>
-    <row r="67" ht="14.25" customHeight="1"/>
-    <row r="68" ht="14.25" customHeight="1"/>
-    <row r="69" ht="14.25" customHeight="1"/>
-    <row r="70" ht="14.25" customHeight="1"/>
-    <row r="71" ht="14.25" customHeight="1"/>
-    <row r="72" ht="14.25" customHeight="1"/>
-    <row r="73" ht="14.25" customHeight="1"/>
-    <row r="74" ht="14.25" customHeight="1"/>
-    <row r="75" ht="14.25" customHeight="1"/>
-    <row r="76" ht="14.25" customHeight="1"/>
-    <row r="77" ht="14.25" customHeight="1"/>
-    <row r="78" ht="14.25" customHeight="1"/>
-    <row r="79" ht="14.25" customHeight="1"/>
-    <row r="80" ht="14.25" customHeight="1"/>
-    <row r="81" ht="14.25" customHeight="1"/>
-    <row r="82" ht="14.25" customHeight="1"/>
-    <row r="83" ht="14.25" customHeight="1"/>
-    <row r="84" ht="14.25" customHeight="1"/>
-    <row r="85" ht="14.25" customHeight="1"/>
-    <row r="86" ht="14.25" customHeight="1"/>
-    <row r="87" ht="14.25" customHeight="1"/>
-    <row r="88" ht="14.25" customHeight="1"/>
-    <row r="89" ht="14.25" customHeight="1"/>
-    <row r="90" ht="14.25" customHeight="1"/>
-    <row r="91" ht="14.25" customHeight="1"/>
-    <row r="92" ht="14.25" customHeight="1"/>
-    <row r="93" ht="14.25" customHeight="1"/>
-    <row r="94" ht="14.25" customHeight="1"/>
-    <row r="95" ht="14.25" customHeight="1"/>
-    <row r="96" ht="14.25" customHeight="1"/>
-    <row r="97" ht="14.25" customHeight="1"/>
-    <row r="98" ht="14.25" customHeight="1"/>
-    <row r="99" ht="14.25" customHeight="1"/>
-    <row r="100" ht="14.25" customHeight="1"/>
-    <row r="101" ht="14.25" customHeight="1"/>
-    <row r="102" ht="14.25" customHeight="1"/>
-    <row r="103" ht="14.25" customHeight="1"/>
-    <row r="104" ht="14.25" customHeight="1"/>
-    <row r="105" ht="14.25" customHeight="1"/>
-    <row r="106" ht="14.25" customHeight="1"/>
-    <row r="107" ht="14.25" customHeight="1"/>
-    <row r="108" ht="14.25" customHeight="1"/>
-    <row r="109" ht="14.25" customHeight="1"/>
-    <row r="110" ht="14.25" customHeight="1"/>
-    <row r="111" ht="14.25" customHeight="1"/>
-    <row r="112" ht="14.25" customHeight="1"/>
-    <row r="113" ht="14.25" customHeight="1"/>
-    <row r="114" ht="14.25" customHeight="1"/>
-    <row r="115" ht="14.25" customHeight="1"/>
-    <row r="116" ht="14.25" customHeight="1"/>
-    <row r="117" ht="14.25" customHeight="1"/>
-    <row r="118" ht="14.25" customHeight="1"/>
-    <row r="119" ht="14.25" customHeight="1"/>
-    <row r="120" ht="14.25" customHeight="1"/>
-    <row r="121" ht="14.25" customHeight="1"/>
-    <row r="122" ht="14.25" customHeight="1"/>
-    <row r="123" ht="14.25" customHeight="1"/>
-    <row r="124" ht="14.25" customHeight="1"/>
-    <row r="125" ht="14.25" customHeight="1"/>
-    <row r="126" ht="14.25" customHeight="1"/>
-    <row r="127" ht="14.25" customHeight="1"/>
-    <row r="128" ht="14.25" customHeight="1"/>
-    <row r="129" ht="14.25" customHeight="1"/>
-    <row r="130" ht="14.25" customHeight="1"/>
-    <row r="131" ht="14.25" customHeight="1"/>
-    <row r="132" ht="14.25" customHeight="1"/>
-    <row r="133" ht="14.25" customHeight="1"/>
-    <row r="134" ht="14.25" customHeight="1"/>
-    <row r="135" ht="14.25" customHeight="1"/>
-    <row r="136" ht="14.25" customHeight="1"/>
-    <row r="137" ht="14.25" customHeight="1"/>
-    <row r="138" ht="14.25" customHeight="1"/>
-    <row r="139" ht="14.25" customHeight="1"/>
-    <row r="140" ht="14.25" customHeight="1"/>
-    <row r="141" ht="14.25" customHeight="1"/>
-    <row r="142" ht="14.25" customHeight="1"/>
-    <row r="143" ht="14.25" customHeight="1"/>
-    <row r="144" ht="14.25" customHeight="1"/>
-    <row r="145" ht="14.25" customHeight="1"/>
-    <row r="146" ht="14.25" customHeight="1"/>
-    <row r="147" ht="14.25" customHeight="1"/>
-    <row r="148" ht="14.25" customHeight="1"/>
-    <row r="149" ht="14.25" customHeight="1"/>
-    <row r="150" ht="14.25" customHeight="1"/>
-    <row r="151" ht="14.25" customHeight="1"/>
-    <row r="152" ht="14.25" customHeight="1"/>
-    <row r="153" ht="14.25" customHeight="1"/>
-    <row r="154" ht="14.25" customHeight="1"/>
-    <row r="155" ht="14.25" customHeight="1"/>
-    <row r="156" ht="14.25" customHeight="1"/>
-    <row r="157" ht="14.25" customHeight="1"/>
-    <row r="158" ht="14.25" customHeight="1"/>
-    <row r="159" ht="14.25" customHeight="1"/>
-    <row r="160" ht="14.25" customHeight="1"/>
-    <row r="161" ht="14.25" customHeight="1"/>
-    <row r="162" ht="14.25" customHeight="1"/>
-    <row r="163" ht="14.25" customHeight="1"/>
-    <row r="164" ht="14.25" customHeight="1"/>
-    <row r="165" ht="14.25" customHeight="1"/>
-    <row r="166" ht="14.25" customHeight="1"/>
-    <row r="167" ht="14.25" customHeight="1"/>
-    <row r="168" ht="14.25" customHeight="1"/>
-    <row r="169" ht="14.25" customHeight="1"/>
-    <row r="170" ht="14.25" customHeight="1"/>
-    <row r="171" ht="14.25" customHeight="1"/>
-    <row r="172" ht="14.25" customHeight="1"/>
-    <row r="173" ht="14.25" customHeight="1"/>
-    <row r="174" ht="14.25" customHeight="1"/>
-    <row r="175" ht="14.25" customHeight="1"/>
-    <row r="176" ht="14.25" customHeight="1"/>
-    <row r="177" ht="14.25" customHeight="1"/>
-    <row r="178" ht="14.25" customHeight="1"/>
-    <row r="179" ht="14.25" customHeight="1"/>
-    <row r="180" ht="14.25" customHeight="1"/>
-    <row r="181" ht="14.25" customHeight="1"/>
-    <row r="182" ht="14.25" customHeight="1"/>
-    <row r="183" ht="14.25" customHeight="1"/>
-    <row r="184" ht="14.25" customHeight="1"/>
-    <row r="185" ht="14.25" customHeight="1"/>
-    <row r="186" ht="14.25" customHeight="1"/>
-    <row r="187" ht="14.25" customHeight="1"/>
-    <row r="188" ht="14.25" customHeight="1"/>
-    <row r="189" ht="14.25" customHeight="1"/>
-    <row r="190" ht="14.25" customHeight="1"/>
-    <row r="191" ht="14.25" customHeight="1"/>
-    <row r="192" ht="14.25" customHeight="1"/>
-    <row r="193" ht="14.25" customHeight="1"/>
-    <row r="194" ht="14.25" customHeight="1"/>
-    <row r="195" ht="14.25" customHeight="1"/>
-    <row r="196" ht="14.25" customHeight="1"/>
-    <row r="197" ht="14.25" customHeight="1"/>
-    <row r="198" ht="14.25" customHeight="1"/>
-    <row r="199" ht="14.25" customHeight="1"/>
-    <row r="200" ht="14.25" customHeight="1"/>
-    <row r="201" ht="14.25" customHeight="1"/>
-    <row r="202" ht="14.25" customHeight="1"/>
-    <row r="203" ht="14.25" customHeight="1"/>
-    <row r="204" ht="14.25" customHeight="1"/>
-    <row r="205" ht="14.25" customHeight="1"/>
-    <row r="206" ht="14.25" customHeight="1"/>
-    <row r="207" ht="14.25" customHeight="1"/>
-    <row r="208" ht="14.25" customHeight="1"/>
-    <row r="209" ht="14.25" customHeight="1"/>
-    <row r="210" ht="14.25" customHeight="1"/>
-    <row r="211" ht="14.25" customHeight="1"/>
-    <row r="212" ht="14.25" customHeight="1"/>
-    <row r="213" ht="14.25" customHeight="1"/>
-    <row r="214" ht="14.25" customHeight="1"/>
-    <row r="215" ht="14.25" customHeight="1"/>
-    <row r="216" ht="14.25" customHeight="1"/>
-    <row r="217" ht="14.25" customHeight="1"/>
-    <row r="218" ht="14.25" customHeight="1"/>
-    <row r="219" ht="14.25" customHeight="1"/>
-    <row r="220" ht="14.25" customHeight="1"/>
-    <row r="221" ht="14.25" customHeight="1"/>
-    <row r="222" ht="14.25" customHeight="1"/>
-    <row r="223" ht="14.25" customHeight="1"/>
-    <row r="224" ht="14.25" customHeight="1"/>
-    <row r="225" ht="14.25" customHeight="1"/>
-    <row r="226" ht="14.25" customHeight="1"/>
-    <row r="227" ht="14.25" customHeight="1"/>
-    <row r="228" ht="14.25" customHeight="1"/>
-    <row r="229" ht="14.25" customHeight="1"/>
-    <row r="230" ht="14.25" customHeight="1"/>
-    <row r="231" ht="14.25" customHeight="1"/>
-    <row r="232" ht="14.25" customHeight="1"/>
-    <row r="233" ht="14.25" customHeight="1"/>
-    <row r="234" ht="14.25" customHeight="1"/>
-    <row r="235" ht="14.25" customHeight="1"/>
-    <row r="236" ht="14.25" customHeight="1"/>
-    <row r="237" ht="14.25" customHeight="1"/>
-    <row r="238" ht="14.25" customHeight="1"/>
-    <row r="239" ht="14.25" customHeight="1"/>
-    <row r="240" ht="14.25" customHeight="1"/>
-    <row r="241" ht="14.25" customHeight="1"/>
-    <row r="242" ht="14.25" customHeight="1"/>
-    <row r="243" ht="14.25" customHeight="1"/>
-    <row r="244" ht="14.25" customHeight="1"/>
-    <row r="245" ht="14.25" customHeight="1"/>
-    <row r="246" ht="14.25" customHeight="1"/>
-    <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
-    <row r="249" ht="14.25" customHeight="1"/>
-    <row r="250" ht="14.25" customHeight="1"/>
-    <row r="251" ht="14.25" customHeight="1"/>
-    <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1"/>
-    <row r="254" ht="14.25" customHeight="1"/>
-    <row r="255" ht="14.25" customHeight="1"/>
-    <row r="256" ht="14.25" customHeight="1"/>
-    <row r="257" ht="14.25" customHeight="1"/>
-    <row r="258" ht="14.25" customHeight="1"/>
-    <row r="259" ht="14.25" customHeight="1"/>
-    <row r="260" ht="14.25" customHeight="1"/>
-    <row r="261" ht="14.25" customHeight="1"/>
-    <row r="262" ht="14.25" customHeight="1"/>
-    <row r="263" ht="14.25" customHeight="1"/>
-    <row r="264" ht="14.25" customHeight="1"/>
-    <row r="265" ht="14.25" customHeight="1"/>
-    <row r="266" ht="14.25" customHeight="1"/>
-    <row r="267" ht="14.25" customHeight="1"/>
-    <row r="268" ht="14.25" customHeight="1"/>
-    <row r="269" ht="14.25" customHeight="1"/>
-    <row r="270" ht="14.25" customHeight="1"/>
-    <row r="271" ht="14.25" customHeight="1"/>
-    <row r="272" ht="14.25" customHeight="1"/>
-    <row r="273" ht="14.25" customHeight="1"/>
-    <row r="274" ht="14.25" customHeight="1"/>
-    <row r="275" ht="14.25" customHeight="1"/>
-    <row r="276" ht="14.25" customHeight="1"/>
-    <row r="277" ht="14.25" customHeight="1"/>
-    <row r="278" ht="14.25" customHeight="1"/>
-    <row r="279" ht="14.25" customHeight="1"/>
-    <row r="280" ht="14.25" customHeight="1"/>
-    <row r="281" ht="14.25" customHeight="1"/>
-    <row r="282" ht="14.25" customHeight="1"/>
-    <row r="283" ht="14.25" customHeight="1"/>
-    <row r="284" ht="14.25" customHeight="1"/>
-    <row r="285" ht="14.25" customHeight="1"/>
-    <row r="286" ht="14.25" customHeight="1"/>
-    <row r="287" ht="14.25" customHeight="1"/>
-    <row r="288" ht="14.25" customHeight="1"/>
-    <row r="289" ht="14.25" customHeight="1"/>
-    <row r="290" ht="14.25" customHeight="1"/>
-    <row r="291" ht="14.25" customHeight="1"/>
-    <row r="292" ht="14.25" customHeight="1"/>
-    <row r="293" ht="14.25" customHeight="1"/>
-    <row r="294" ht="14.25" customHeight="1"/>
-    <row r="295" ht="14.25" customHeight="1"/>
-    <row r="296" ht="14.25" customHeight="1"/>
-    <row r="297" ht="14.25" customHeight="1"/>
-    <row r="298" ht="14.25" customHeight="1"/>
-    <row r="299" ht="14.25" customHeight="1"/>
-    <row r="300" ht="14.25" customHeight="1"/>
-    <row r="301" ht="14.25" customHeight="1"/>
-    <row r="302" ht="14.25" customHeight="1"/>
-    <row r="303" ht="14.25" customHeight="1"/>
-    <row r="304" ht="14.25" customHeight="1"/>
-    <row r="305" ht="14.25" customHeight="1"/>
-    <row r="306" ht="14.25" customHeight="1"/>
-    <row r="307" ht="14.25" customHeight="1"/>
-    <row r="308" ht="14.25" customHeight="1"/>
-    <row r="309" ht="14.25" customHeight="1"/>
-    <row r="310" ht="14.25" customHeight="1"/>
-    <row r="311" ht="14.25" customHeight="1"/>
-    <row r="312" ht="14.25" customHeight="1"/>
-    <row r="313" ht="14.25" customHeight="1"/>
-    <row r="314" ht="14.25" customHeight="1"/>
-    <row r="315" ht="14.25" customHeight="1"/>
-    <row r="316" ht="14.25" customHeight="1"/>
-    <row r="317" ht="14.25" customHeight="1"/>
-    <row r="318" ht="14.25" customHeight="1"/>
-    <row r="319" ht="14.25" customHeight="1"/>
-    <row r="320" ht="14.25" customHeight="1"/>
-    <row r="321" ht="14.25" customHeight="1"/>
-    <row r="322" ht="14.25" customHeight="1"/>
-    <row r="323" ht="14.25" customHeight="1"/>
-    <row r="324" ht="14.25" customHeight="1"/>
-    <row r="325" ht="14.25" customHeight="1"/>
-    <row r="326" ht="14.25" customHeight="1"/>
-    <row r="327" ht="14.25" customHeight="1"/>
-    <row r="328" ht="14.25" customHeight="1"/>
-    <row r="329" ht="14.25" customHeight="1"/>
-    <row r="330" ht="14.25" customHeight="1"/>
-    <row r="331" ht="14.25" customHeight="1"/>
-    <row r="332" ht="14.25" customHeight="1"/>
-    <row r="333" ht="14.25" customHeight="1"/>
-    <row r="334" ht="14.25" customHeight="1"/>
-    <row r="335" ht="14.25" customHeight="1"/>
-    <row r="336" ht="14.25" customHeight="1"/>
-    <row r="337" ht="14.25" customHeight="1"/>
-    <row r="338" ht="14.25" customHeight="1"/>
-    <row r="339" ht="14.25" customHeight="1"/>
-    <row r="340" ht="14.25" customHeight="1"/>
-    <row r="341" ht="14.25" customHeight="1"/>
-    <row r="342" ht="14.25" customHeight="1"/>
-    <row r="343" ht="14.25" customHeight="1"/>
-    <row r="344" ht="14.25" customHeight="1"/>
-    <row r="345" ht="14.25" customHeight="1"/>
-    <row r="346" ht="14.25" customHeight="1"/>
-    <row r="347" ht="14.25" customHeight="1"/>
-    <row r="348" ht="14.25" customHeight="1"/>
-    <row r="349" ht="14.25" customHeight="1"/>
-    <row r="350" ht="14.25" customHeight="1"/>
-    <row r="351" ht="14.25" customHeight="1"/>
-    <row r="352" ht="14.25" customHeight="1"/>
-    <row r="353" ht="14.25" customHeight="1"/>
-    <row r="354" ht="14.25" customHeight="1"/>
-    <row r="355" ht="14.25" customHeight="1"/>
-    <row r="356" ht="14.25" customHeight="1"/>
-    <row r="357" ht="14.25" customHeight="1"/>
-    <row r="358" ht="14.25" customHeight="1"/>
-    <row r="359" ht="14.25" customHeight="1"/>
-    <row r="360" ht="14.25" customHeight="1"/>
-    <row r="361" ht="14.25" customHeight="1"/>
-    <row r="362" ht="14.25" customHeight="1"/>
-    <row r="363" ht="14.25" customHeight="1"/>
-    <row r="364" ht="14.25" customHeight="1"/>
-    <row r="365" ht="14.25" customHeight="1"/>
-    <row r="366" ht="14.25" customHeight="1"/>
-    <row r="367" ht="14.25" customHeight="1"/>
-    <row r="368" ht="14.25" customHeight="1"/>
-    <row r="369" ht="14.25" customHeight="1"/>
-    <row r="370" ht="14.25" customHeight="1"/>
-    <row r="371" ht="14.25" customHeight="1"/>
-    <row r="372" ht="14.25" customHeight="1"/>
-    <row r="373" ht="14.25" customHeight="1"/>
-    <row r="374" ht="14.25" customHeight="1"/>
-    <row r="375" ht="14.25" customHeight="1"/>
-    <row r="376" ht="14.25" customHeight="1"/>
-    <row r="377" ht="14.25" customHeight="1"/>
-    <row r="378" ht="14.25" customHeight="1"/>
-    <row r="379" ht="14.25" customHeight="1"/>
-    <row r="380" ht="14.25" customHeight="1"/>
-    <row r="381" ht="14.25" customHeight="1"/>
-    <row r="382" ht="14.25" customHeight="1"/>
-    <row r="383" ht="14.25" customHeight="1"/>
-    <row r="384" ht="14.25" customHeight="1"/>
-    <row r="385" ht="14.25" customHeight="1"/>
-    <row r="386" ht="14.25" customHeight="1"/>
-    <row r="387" ht="14.25" customHeight="1"/>
-    <row r="388" ht="14.25" customHeight="1"/>
-    <row r="389" ht="14.25" customHeight="1"/>
-    <row r="390" ht="14.25" customHeight="1"/>
-    <row r="391" ht="14.25" customHeight="1"/>
-    <row r="392" ht="14.25" customHeight="1"/>
-    <row r="393" ht="14.25" customHeight="1"/>
-    <row r="394" ht="14.25" customHeight="1"/>
-    <row r="395" ht="14.25" customHeight="1"/>
-    <row r="396" ht="14.25" customHeight="1"/>
-    <row r="397" ht="14.25" customHeight="1"/>
-    <row r="398" ht="14.25" customHeight="1"/>
-    <row r="399" ht="14.25" customHeight="1"/>
-    <row r="400" ht="14.25" customHeight="1"/>
-    <row r="401" ht="14.25" customHeight="1"/>
-    <row r="402" ht="14.25" customHeight="1"/>
-    <row r="403" ht="14.25" customHeight="1"/>
-    <row r="404" ht="14.25" customHeight="1"/>
-    <row r="405" ht="14.25" customHeight="1"/>
-    <row r="406" ht="14.25" customHeight="1"/>
-    <row r="407" ht="14.25" customHeight="1"/>
-    <row r="408" ht="14.25" customHeight="1"/>
-    <row r="409" ht="14.25" customHeight="1"/>
-    <row r="410" ht="14.25" customHeight="1"/>
-    <row r="411" ht="14.25" customHeight="1"/>
-    <row r="412" ht="14.25" customHeight="1"/>
-    <row r="413" ht="14.25" customHeight="1"/>
-    <row r="414" ht="14.25" customHeight="1"/>
-    <row r="415" ht="14.25" customHeight="1"/>
-    <row r="416" ht="14.25" customHeight="1"/>
-    <row r="417" ht="14.25" customHeight="1"/>
-    <row r="418" ht="14.25" customHeight="1"/>
-    <row r="419" ht="14.25" customHeight="1"/>
-    <row r="420" ht="14.25" customHeight="1"/>
-    <row r="421" ht="14.25" customHeight="1"/>
-    <row r="422" ht="14.25" customHeight="1"/>
-    <row r="423" ht="14.25" customHeight="1"/>
-    <row r="424" ht="14.25" customHeight="1"/>
-    <row r="425" ht="14.25" customHeight="1"/>
-    <row r="426" ht="14.25" customHeight="1"/>
-    <row r="427" ht="14.25" customHeight="1"/>
-    <row r="428" ht="14.25" customHeight="1"/>
-    <row r="429" ht="14.25" customHeight="1"/>
-    <row r="430" ht="14.25" customHeight="1"/>
-    <row r="431" ht="14.25" customHeight="1"/>
-    <row r="432" ht="14.25" customHeight="1"/>
-    <row r="433" ht="14.25" customHeight="1"/>
-    <row r="434" ht="14.25" customHeight="1"/>
-    <row r="435" ht="14.25" customHeight="1"/>
-    <row r="436" ht="14.25" customHeight="1"/>
-    <row r="437" ht="14.25" customHeight="1"/>
-    <row r="438" ht="14.25" customHeight="1"/>
-    <row r="439" ht="14.25" customHeight="1"/>
-    <row r="440" ht="14.25" customHeight="1"/>
-    <row r="441" ht="14.25" customHeight="1"/>
-    <row r="442" ht="14.25" customHeight="1"/>
-    <row r="443" ht="14.25" customHeight="1"/>
-    <row r="444" ht="14.25" customHeight="1"/>
-    <row r="445" ht="14.25" customHeight="1"/>
-    <row r="446" ht="14.25" customHeight="1"/>
-    <row r="447" ht="14.25" customHeight="1"/>
-    <row r="448" ht="14.25" customHeight="1"/>
-    <row r="449" ht="14.25" customHeight="1"/>
-    <row r="450" ht="14.25" customHeight="1"/>
-    <row r="451" ht="14.25" customHeight="1"/>
-    <row r="452" ht="14.25" customHeight="1"/>
-    <row r="453" ht="14.25" customHeight="1"/>
-    <row r="454" ht="14.25" customHeight="1"/>
-    <row r="455" ht="14.25" customHeight="1"/>
-    <row r="456" ht="14.25" customHeight="1"/>
-    <row r="457" ht="14.25" customHeight="1"/>
-    <row r="458" ht="14.25" customHeight="1"/>
-    <row r="459" ht="14.25" customHeight="1"/>
-    <row r="460" ht="14.25" customHeight="1"/>
-    <row r="461" ht="14.25" customHeight="1"/>
-    <row r="462" ht="14.25" customHeight="1"/>
-    <row r="463" ht="14.25" customHeight="1"/>
-    <row r="464" ht="14.25" customHeight="1"/>
-    <row r="465" ht="14.25" customHeight="1"/>
-    <row r="466" ht="14.25" customHeight="1"/>
-    <row r="467" ht="14.25" customHeight="1"/>
-    <row r="468" ht="14.25" customHeight="1"/>
-    <row r="469" ht="14.25" customHeight="1"/>
-    <row r="470" ht="14.25" customHeight="1"/>
-    <row r="471" ht="14.25" customHeight="1"/>
-    <row r="472" ht="14.25" customHeight="1"/>
-    <row r="473" ht="14.25" customHeight="1"/>
-    <row r="474" ht="14.25" customHeight="1"/>
-    <row r="475" ht="14.25" customHeight="1"/>
-    <row r="476" ht="14.25" customHeight="1"/>
-    <row r="477" ht="14.25" customHeight="1"/>
-    <row r="478" ht="14.25" customHeight="1"/>
-    <row r="479" ht="14.25" customHeight="1"/>
-    <row r="480" ht="14.25" customHeight="1"/>
-    <row r="481" ht="14.25" customHeight="1"/>
-    <row r="482" ht="14.25" customHeight="1"/>
-    <row r="483" ht="14.25" customHeight="1"/>
-    <row r="484" ht="14.25" customHeight="1"/>
-    <row r="485" ht="14.25" customHeight="1"/>
-    <row r="486" ht="14.25" customHeight="1"/>
-    <row r="487" ht="14.25" customHeight="1"/>
-    <row r="488" ht="14.25" customHeight="1"/>
-    <row r="489" ht="14.25" customHeight="1"/>
-    <row r="490" ht="14.25" customHeight="1"/>
-    <row r="491" ht="14.25" customHeight="1"/>
-    <row r="492" ht="14.25" customHeight="1"/>
-    <row r="493" ht="14.25" customHeight="1"/>
-    <row r="494" ht="14.25" customHeight="1"/>
-    <row r="495" ht="14.25" customHeight="1"/>
-    <row r="496" ht="14.25" customHeight="1"/>
-    <row r="497" ht="14.25" customHeight="1"/>
-    <row r="498" ht="14.25" customHeight="1"/>
-    <row r="499" ht="14.25" customHeight="1"/>
-    <row r="500" ht="14.25" customHeight="1"/>
-    <row r="501" ht="14.25" customHeight="1"/>
-    <row r="502" ht="14.25" customHeight="1"/>
-    <row r="503" ht="14.25" customHeight="1"/>
-    <row r="504" ht="14.25" customHeight="1"/>
-    <row r="505" ht="14.25" customHeight="1"/>
-    <row r="506" ht="14.25" customHeight="1"/>
-    <row r="507" ht="14.25" customHeight="1"/>
-    <row r="508" ht="14.25" customHeight="1"/>
-    <row r="509" ht="14.25" customHeight="1"/>
-    <row r="510" ht="14.25" customHeight="1"/>
-    <row r="511" ht="14.25" customHeight="1"/>
-    <row r="512" ht="14.25" customHeight="1"/>
-    <row r="513" ht="14.25" customHeight="1"/>
-    <row r="514" ht="14.25" customHeight="1"/>
-    <row r="515" ht="14.25" customHeight="1"/>
-    <row r="516" ht="14.25" customHeight="1"/>
-    <row r="517" ht="14.25" customHeight="1"/>
-    <row r="518" ht="14.25" customHeight="1"/>
-    <row r="519" ht="14.25" customHeight="1"/>
-    <row r="520" ht="14.25" customHeight="1"/>
-    <row r="521" ht="14.25" customHeight="1"/>
-    <row r="522" ht="14.25" customHeight="1"/>
-    <row r="523" ht="14.25" customHeight="1"/>
-    <row r="524" ht="14.25" customHeight="1"/>
-    <row r="525" ht="14.25" customHeight="1"/>
-    <row r="526" ht="14.25" customHeight="1"/>
-    <row r="527" ht="14.25" customHeight="1"/>
-    <row r="528" ht="14.25" customHeight="1"/>
-    <row r="529" ht="14.25" customHeight="1"/>
-    <row r="530" ht="14.25" customHeight="1"/>
-    <row r="531" ht="14.25" customHeight="1"/>
-    <row r="532" ht="14.25" customHeight="1"/>
-    <row r="533" ht="14.25" customHeight="1"/>
-    <row r="534" ht="14.25" customHeight="1"/>
-    <row r="535" ht="14.25" customHeight="1"/>
-    <row r="536" ht="14.25" customHeight="1"/>
-    <row r="537" ht="14.25" customHeight="1"/>
-    <row r="538" ht="14.25" customHeight="1"/>
-    <row r="539" ht="14.25" customHeight="1"/>
-    <row r="540" ht="14.25" customHeight="1"/>
-    <row r="541" ht="14.25" customHeight="1"/>
-    <row r="542" ht="14.25" customHeight="1"/>
-    <row r="543" ht="14.25" customHeight="1"/>
-    <row r="544" ht="14.25" customHeight="1"/>
-    <row r="545" ht="14.25" customHeight="1"/>
-    <row r="546" ht="14.25" customHeight="1"/>
-    <row r="547" ht="14.25" customHeight="1"/>
-    <row r="548" ht="14.25" customHeight="1"/>
-    <row r="549" ht="14.25" customHeight="1"/>
-    <row r="550" ht="14.25" customHeight="1"/>
-    <row r="551" ht="14.25" customHeight="1"/>
-    <row r="552" ht="14.25" customHeight="1"/>
-    <row r="553" ht="14.25" customHeight="1"/>
-    <row r="554" ht="14.25" customHeight="1"/>
-    <row r="555" ht="14.25" customHeight="1"/>
-    <row r="556" ht="14.25" customHeight="1"/>
-    <row r="557" ht="14.25" customHeight="1"/>
-    <row r="558" ht="14.25" customHeight="1"/>
-    <row r="559" ht="14.25" customHeight="1"/>
-    <row r="560" ht="14.25" customHeight="1"/>
-    <row r="561" ht="14.25" customHeight="1"/>
-    <row r="562" ht="14.25" customHeight="1"/>
-    <row r="563" ht="14.25" customHeight="1"/>
-    <row r="564" ht="14.25" customHeight="1"/>
-    <row r="565" ht="14.25" customHeight="1"/>
-    <row r="566" ht="14.25" customHeight="1"/>
-    <row r="567" ht="14.25" customHeight="1"/>
-    <row r="568" ht="14.25" customHeight="1"/>
-    <row r="569" ht="14.25" customHeight="1"/>
-    <row r="570" ht="14.25" customHeight="1"/>
-    <row r="571" ht="14.25" customHeight="1"/>
-    <row r="572" ht="14.25" customHeight="1"/>
-    <row r="573" ht="14.25" customHeight="1"/>
-    <row r="574" ht="14.25" customHeight="1"/>
-    <row r="575" ht="14.25" customHeight="1"/>
-    <row r="576" ht="14.25" customHeight="1"/>
-    <row r="577" ht="14.25" customHeight="1"/>
-    <row r="578" ht="14.25" customHeight="1"/>
-    <row r="579" ht="14.25" customHeight="1"/>
-    <row r="580" ht="14.25" customHeight="1"/>
-    <row r="581" ht="14.25" customHeight="1"/>
-    <row r="582" ht="14.25" customHeight="1"/>
-    <row r="583" ht="14.25" customHeight="1"/>
-    <row r="584" ht="14.25" customHeight="1"/>
-    <row r="585" ht="14.25" customHeight="1"/>
-    <row r="586" ht="14.25" customHeight="1"/>
-    <row r="587" ht="14.25" customHeight="1"/>
-    <row r="588" ht="14.25" customHeight="1"/>
-    <row r="589" ht="14.25" customHeight="1"/>
-    <row r="590" ht="14.25" customHeight="1"/>
-    <row r="591" ht="14.25" customHeight="1"/>
-    <row r="592" ht="14.25" customHeight="1"/>
-    <row r="593" ht="14.25" customHeight="1"/>
-    <row r="594" ht="14.25" customHeight="1"/>
-    <row r="595" ht="14.25" customHeight="1"/>
-    <row r="596" ht="14.25" customHeight="1"/>
-    <row r="597" ht="14.25" customHeight="1"/>
-    <row r="598" ht="14.25" customHeight="1"/>
-    <row r="599" ht="14.25" customHeight="1"/>
-    <row r="600" ht="14.25" customHeight="1"/>
-    <row r="601" ht="14.25" customHeight="1"/>
-    <row r="602" ht="14.25" customHeight="1"/>
-    <row r="603" ht="14.25" customHeight="1"/>
-    <row r="604" ht="14.25" customHeight="1"/>
-    <row r="605" ht="14.25" customHeight="1"/>
-    <row r="606" ht="14.25" customHeight="1"/>
-    <row r="607" ht="14.25" customHeight="1"/>
-    <row r="608" ht="14.25" customHeight="1"/>
-    <row r="609" ht="14.25" customHeight="1"/>
-    <row r="610" ht="14.25" customHeight="1"/>
-    <row r="611" ht="14.25" customHeight="1"/>
-    <row r="612" ht="14.25" customHeight="1"/>
-    <row r="613" ht="14.25" customHeight="1"/>
-    <row r="614" ht="14.25" customHeight="1"/>
-    <row r="615" ht="14.25" customHeight="1"/>
-    <row r="616" ht="14.25" customHeight="1"/>
-    <row r="617" ht="14.25" customHeight="1"/>
-    <row r="618" ht="14.25" customHeight="1"/>
-    <row r="619" ht="14.25" customHeight="1"/>
-    <row r="620" ht="14.25" customHeight="1"/>
-    <row r="621" ht="14.25" customHeight="1"/>
-    <row r="622" ht="14.25" customHeight="1"/>
-    <row r="623" ht="14.25" customHeight="1"/>
-    <row r="624" ht="14.25" customHeight="1"/>
-    <row r="625" ht="14.25" customHeight="1"/>
-    <row r="626" ht="14.25" customHeight="1"/>
-    <row r="627" ht="14.25" customHeight="1"/>
-    <row r="628" ht="14.25" customHeight="1"/>
-    <row r="629" ht="14.25" customHeight="1"/>
-    <row r="630" ht="14.25" customHeight="1"/>
-    <row r="631" ht="14.25" customHeight="1"/>
-    <row r="632" ht="14.25" customHeight="1"/>
-    <row r="633" ht="14.25" customHeight="1"/>
-    <row r="634" ht="14.25" customHeight="1"/>
-    <row r="635" ht="14.25" customHeight="1"/>
-    <row r="636" ht="14.25" customHeight="1"/>
-    <row r="637" ht="14.25" customHeight="1"/>
-    <row r="638" ht="14.25" customHeight="1"/>
-    <row r="639" ht="14.25" customHeight="1"/>
-    <row r="640" ht="14.25" customHeight="1"/>
-    <row r="641" ht="14.25" customHeight="1"/>
-    <row r="642" ht="14.25" customHeight="1"/>
-    <row r="643" ht="14.25" customHeight="1"/>
-    <row r="644" ht="14.25" customHeight="1"/>
-    <row r="645" ht="14.25" customHeight="1"/>
-    <row r="646" ht="14.25" customHeight="1"/>
-    <row r="647" ht="14.25" customHeight="1"/>
-    <row r="648" ht="14.25" customHeight="1"/>
-    <row r="649" ht="14.25" customHeight="1"/>
-    <row r="650" ht="14.25" customHeight="1"/>
-    <row r="651" ht="14.25" customHeight="1"/>
-    <row r="652" ht="14.25" customHeight="1"/>
-    <row r="653" ht="14.25" customHeight="1"/>
-    <row r="654" ht="14.25" customHeight="1"/>
-    <row r="655" ht="14.25" customHeight="1"/>
-    <row r="656" ht="14.25" customHeight="1"/>
-    <row r="657" ht="14.25" customHeight="1"/>
-    <row r="658" ht="14.25" customHeight="1"/>
-    <row r="659" ht="14.25" customHeight="1"/>
-    <row r="660" ht="14.25" customHeight="1"/>
-    <row r="661" ht="14.25" customHeight="1"/>
-    <row r="662" ht="14.25" customHeight="1"/>
-    <row r="663" ht="14.25" customHeight="1"/>
-    <row r="664" ht="14.25" customHeight="1"/>
-    <row r="665" ht="14.25" customHeight="1"/>
-    <row r="666" ht="14.25" customHeight="1"/>
-    <row r="667" ht="14.25" customHeight="1"/>
-    <row r="668" ht="14.25" customHeight="1"/>
-    <row r="669" ht="14.25" customHeight="1"/>
-    <row r="670" ht="14.25" customHeight="1"/>
-    <row r="671" ht="14.25" customHeight="1"/>
-    <row r="672" ht="14.25" customHeight="1"/>
-    <row r="673" ht="14.25" customHeight="1"/>
-    <row r="674" ht="14.25" customHeight="1"/>
-    <row r="675" ht="14.25" customHeight="1"/>
-    <row r="676" ht="14.25" customHeight="1"/>
-    <row r="677" ht="14.25" customHeight="1"/>
-    <row r="678" ht="14.25" customHeight="1"/>
-    <row r="679" ht="14.25" customHeight="1"/>
-    <row r="680" ht="14.25" customHeight="1"/>
-    <row r="681" ht="14.25" customHeight="1"/>
-    <row r="682" ht="14.25" customHeight="1"/>
-    <row r="683" ht="14.25" customHeight="1"/>
-    <row r="684" ht="14.25" customHeight="1"/>
-    <row r="685" ht="14.25" customHeight="1"/>
-    <row r="686" ht="14.25" customHeight="1"/>
-    <row r="687" ht="14.25" customHeight="1"/>
-    <row r="688" ht="14.25" customHeight="1"/>
-    <row r="689" ht="14.25" customHeight="1"/>
-    <row r="690" ht="14.25" customHeight="1"/>
-    <row r="691" ht="14.25" customHeight="1"/>
-    <row r="692" ht="14.25" customHeight="1"/>
-    <row r="693" ht="14.25" customHeight="1"/>
-    <row r="694" ht="14.25" customHeight="1"/>
-    <row r="695" ht="14.25" customHeight="1"/>
-    <row r="696" ht="14.25" customHeight="1"/>
-    <row r="697" ht="14.25" customHeight="1"/>
-    <row r="698" ht="14.25" customHeight="1"/>
-    <row r="699" ht="14.25" customHeight="1"/>
-    <row r="700" ht="14.25" customHeight="1"/>
-    <row r="701" ht="14.25" customHeight="1"/>
-    <row r="702" ht="14.25" customHeight="1"/>
-    <row r="703" ht="14.25" customHeight="1"/>
-    <row r="704" ht="14.25" customHeight="1"/>
-    <row r="705" ht="14.25" customHeight="1"/>
-    <row r="706" ht="14.25" customHeight="1"/>
-    <row r="707" ht="14.25" customHeight="1"/>
-    <row r="708" ht="14.25" customHeight="1"/>
-    <row r="709" ht="14.25" customHeight="1"/>
-    <row r="710" ht="14.25" customHeight="1"/>
-    <row r="711" ht="14.25" customHeight="1"/>
-    <row r="712" ht="14.25" customHeight="1"/>
-    <row r="713" ht="14.25" customHeight="1"/>
-    <row r="714" ht="14.25" customHeight="1"/>
-    <row r="715" ht="14.25" customHeight="1"/>
-    <row r="716" ht="14.25" customHeight="1"/>
-    <row r="717" ht="14.25" customHeight="1"/>
-    <row r="718" ht="14.25" customHeight="1"/>
-    <row r="719" ht="14.25" customHeight="1"/>
-    <row r="720" ht="14.25" customHeight="1"/>
-    <row r="721" ht="14.25" customHeight="1"/>
-    <row r="722" ht="14.25" customHeight="1"/>
-    <row r="723" ht="14.25" customHeight="1"/>
-    <row r="724" ht="14.25" customHeight="1"/>
-    <row r="725" ht="14.25" customHeight="1"/>
-    <row r="726" ht="14.25" customHeight="1"/>
-    <row r="727" ht="14.25" customHeight="1"/>
-    <row r="728" ht="14.25" customHeight="1"/>
-    <row r="729" ht="14.25" customHeight="1"/>
-    <row r="730" ht="14.25" customHeight="1"/>
-    <row r="731" ht="14.25" customHeight="1"/>
-    <row r="732" ht="14.25" customHeight="1"/>
-    <row r="733" ht="14.25" customHeight="1"/>
-    <row r="734" ht="14.25" customHeight="1"/>
-    <row r="735" ht="14.25" customHeight="1"/>
-    <row r="736" ht="14.25" customHeight="1"/>
-    <row r="737" ht="14.25" customHeight="1"/>
-    <row r="738" ht="14.25" customHeight="1"/>
-    <row r="739" ht="14.25" customHeight="1"/>
-    <row r="740" ht="14.25" customHeight="1"/>
-    <row r="741" ht="14.25" customHeight="1"/>
-    <row r="742" ht="14.25" customHeight="1"/>
-    <row r="743" ht="14.25" customHeight="1"/>
-    <row r="744" ht="14.25" customHeight="1"/>
-    <row r="745" ht="14.25" customHeight="1"/>
-    <row r="746" ht="14.25" customHeight="1"/>
-    <row r="747" ht="14.25" customHeight="1"/>
-    <row r="748" ht="14.25" customHeight="1"/>
-    <row r="749" ht="14.25" customHeight="1"/>
-    <row r="750" ht="14.25" customHeight="1"/>
-    <row r="751" ht="14.25" customHeight="1"/>
-    <row r="752" ht="14.25" customHeight="1"/>
-    <row r="753" ht="14.25" customHeight="1"/>
-    <row r="754" ht="14.25" customHeight="1"/>
-    <row r="755" ht="14.25" customHeight="1"/>
-    <row r="756" ht="14.25" customHeight="1"/>
-    <row r="757" ht="14.25" customHeight="1"/>
-    <row r="758" ht="14.25" customHeight="1"/>
-    <row r="759" ht="14.25" customHeight="1"/>
-    <row r="760" ht="14.25" customHeight="1"/>
-    <row r="761" ht="14.25" customHeight="1"/>
-    <row r="762" ht="14.25" customHeight="1"/>
-    <row r="763" ht="14.25" customHeight="1"/>
-    <row r="764" ht="14.25" customHeight="1"/>
-    <row r="765" ht="14.25" customHeight="1"/>
-    <row r="766" ht="14.25" customHeight="1"/>
-    <row r="767" ht="14.25" customHeight="1"/>
-    <row r="768" ht="14.25" customHeight="1"/>
-    <row r="769" ht="14.25" customHeight="1"/>
-    <row r="770" ht="14.25" customHeight="1"/>
-    <row r="771" ht="14.25" customHeight="1"/>
-    <row r="772" ht="14.25" customHeight="1"/>
-    <row r="773" ht="14.25" customHeight="1"/>
-    <row r="774" ht="14.25" customHeight="1"/>
-    <row r="775" ht="14.25" customHeight="1"/>
-    <row r="776" ht="14.25" customHeight="1"/>
-    <row r="777" ht="14.25" customHeight="1"/>
-    <row r="778" ht="14.25" customHeight="1"/>
-    <row r="779" ht="14.25" customHeight="1"/>
-    <row r="780" ht="14.25" customHeight="1"/>
-    <row r="781" ht="14.25" customHeight="1"/>
-    <row r="782" ht="14.25" customHeight="1"/>
-    <row r="783" ht="14.25" customHeight="1"/>
-    <row r="784" ht="14.25" customHeight="1"/>
-    <row r="785" ht="14.25" customHeight="1"/>
-    <row r="786" ht="14.25" customHeight="1"/>
-    <row r="787" ht="14.25" customHeight="1"/>
-    <row r="788" ht="14.25" customHeight="1"/>
-    <row r="789" ht="14.25" customHeight="1"/>
-    <row r="790" ht="14.25" customHeight="1"/>
-    <row r="791" ht="14.25" customHeight="1"/>
-    <row r="792" ht="14.25" customHeight="1"/>
-    <row r="793" ht="14.25" customHeight="1"/>
-    <row r="794" ht="14.25" customHeight="1"/>
-    <row r="795" ht="14.25" customHeight="1"/>
-    <row r="796" ht="14.25" customHeight="1"/>
-    <row r="797" ht="14.25" customHeight="1"/>
-    <row r="798" ht="14.25" customHeight="1"/>
-    <row r="799" ht="14.25" customHeight="1"/>
-    <row r="800" ht="14.25" customHeight="1"/>
-    <row r="801" ht="14.25" customHeight="1"/>
-    <row r="802" ht="14.25" customHeight="1"/>
-    <row r="803" ht="14.25" customHeight="1"/>
-    <row r="804" ht="14.25" customHeight="1"/>
-    <row r="805" ht="14.25" customHeight="1"/>
-    <row r="806" ht="14.25" customHeight="1"/>
-    <row r="807" ht="14.25" customHeight="1"/>
-    <row r="808" ht="14.25" customHeight="1"/>
-    <row r="809" ht="14.25" customHeight="1"/>
-    <row r="810" ht="14.25" customHeight="1"/>
-    <row r="811" ht="14.25" customHeight="1"/>
-    <row r="812" ht="14.25" customHeight="1"/>
-    <row r="813" ht="14.25" customHeight="1"/>
-    <row r="814" ht="14.25" customHeight="1"/>
-    <row r="815" ht="14.25" customHeight="1"/>
-    <row r="816" ht="14.25" customHeight="1"/>
-    <row r="817" ht="14.25" customHeight="1"/>
-    <row r="818" ht="14.25" customHeight="1"/>
-    <row r="819" ht="14.25" customHeight="1"/>
-    <row r="820" ht="14.25" customHeight="1"/>
-    <row r="821" ht="14.25" customHeight="1"/>
-    <row r="822" ht="14.25" customHeight="1"/>
-    <row r="823" ht="14.25" customHeight="1"/>
-    <row r="824" ht="14.25" customHeight="1"/>
-    <row r="825" ht="14.25" customHeight="1"/>
-    <row r="826" ht="14.25" customHeight="1"/>
-    <row r="827" ht="14.25" customHeight="1"/>
-    <row r="828" ht="14.25" customHeight="1"/>
-    <row r="829" ht="14.25" customHeight="1"/>
-    <row r="830" ht="14.25" customHeight="1"/>
-    <row r="831" ht="14.25" customHeight="1"/>
-    <row r="832" ht="14.25" customHeight="1"/>
-    <row r="833" ht="14.25" customHeight="1"/>
-    <row r="834" ht="14.25" customHeight="1"/>
-    <row r="835" ht="14.25" customHeight="1"/>
-    <row r="836" ht="14.25" customHeight="1"/>
-    <row r="837" ht="14.25" customHeight="1"/>
-    <row r="838" ht="14.25" customHeight="1"/>
-    <row r="839" ht="14.25" customHeight="1"/>
-    <row r="840" ht="14.25" customHeight="1"/>
-    <row r="841" ht="14.25" customHeight="1"/>
-    <row r="842" ht="14.25" customHeight="1"/>
-    <row r="843" ht="14.25" customHeight="1"/>
-    <row r="844" ht="14.25" customHeight="1"/>
-    <row r="845" ht="14.25" customHeight="1"/>
-    <row r="846" ht="14.25" customHeight="1"/>
-    <row r="847" ht="14.25" customHeight="1"/>
-    <row r="848" ht="14.25" customHeight="1"/>
-    <row r="849" ht="14.25" customHeight="1"/>
-    <row r="850" ht="14.25" customHeight="1"/>
-    <row r="851" ht="14.25" customHeight="1"/>
-    <row r="852" ht="14.25" customHeight="1"/>
-    <row r="853" ht="14.25" customHeight="1"/>
-    <row r="854" ht="14.25" customHeight="1"/>
-    <row r="855" ht="14.25" customHeight="1"/>
-    <row r="856" ht="14.25" customHeight="1"/>
-    <row r="857" ht="14.25" customHeight="1"/>
-    <row r="858" ht="14.25" customHeight="1"/>
-    <row r="859" ht="14.25" customHeight="1"/>
-    <row r="860" ht="14.25" customHeight="1"/>
-    <row r="861" ht="14.25" customHeight="1"/>
-    <row r="862" ht="14.25" customHeight="1"/>
-    <row r="863" ht="14.25" customHeight="1"/>
-    <row r="864" ht="14.25" customHeight="1"/>
-    <row r="865" ht="14.25" customHeight="1"/>
-    <row r="866" ht="14.25" customHeight="1"/>
-    <row r="867" ht="14.25" customHeight="1"/>
-    <row r="868" ht="14.25" customHeight="1"/>
-    <row r="869" ht="14.25" customHeight="1"/>
-    <row r="870" ht="14.25" customHeight="1"/>
-    <row r="871" ht="14.25" customHeight="1"/>
-    <row r="872" ht="14.25" customHeight="1"/>
-    <row r="873" ht="14.25" customHeight="1"/>
-    <row r="874" ht="14.25" customHeight="1"/>
-    <row r="875" ht="14.25" customHeight="1"/>
-    <row r="876" ht="14.25" customHeight="1"/>
-    <row r="877" ht="14.25" customHeight="1"/>
-    <row r="878" ht="14.25" customHeight="1"/>
-    <row r="879" ht="14.25" customHeight="1"/>
-    <row r="880" ht="14.25" customHeight="1"/>
-    <row r="881" ht="14.25" customHeight="1"/>
-    <row r="882" ht="14.25" customHeight="1"/>
-    <row r="883" ht="14.25" customHeight="1"/>
-    <row r="884" ht="14.25" customHeight="1"/>
-    <row r="885" ht="14.25" customHeight="1"/>
-    <row r="886" ht="14.25" customHeight="1"/>
-    <row r="887" ht="14.25" customHeight="1"/>
-    <row r="888" ht="14.25" customHeight="1"/>
-    <row r="889" ht="14.25" customHeight="1"/>
-    <row r="890" ht="14.25" customHeight="1"/>
-    <row r="891" ht="14.25" customHeight="1"/>
-    <row r="892" ht="14.25" customHeight="1"/>
-    <row r="893" ht="14.25" customHeight="1"/>
-    <row r="894" ht="14.25" customHeight="1"/>
-    <row r="895" ht="14.25" customHeight="1"/>
-    <row r="896" ht="14.25" customHeight="1"/>
-    <row r="897" ht="14.25" customHeight="1"/>
-    <row r="898" ht="14.25" customHeight="1"/>
-    <row r="899" ht="14.25" customHeight="1"/>
-    <row r="900" ht="14.25" customHeight="1"/>
-    <row r="901" ht="14.25" customHeight="1"/>
-    <row r="902" ht="14.25" customHeight="1"/>
-    <row r="903" ht="14.25" customHeight="1"/>
-    <row r="904" ht="14.25" customHeight="1"/>
-    <row r="905" ht="14.25" customHeight="1"/>
-    <row r="906" ht="14.25" customHeight="1"/>
-    <row r="907" ht="14.25" customHeight="1"/>
-    <row r="908" ht="14.25" customHeight="1"/>
-    <row r="909" ht="14.25" customHeight="1"/>
-    <row r="910" ht="14.25" customHeight="1"/>
-    <row r="911" ht="14.25" customHeight="1"/>
-    <row r="912" ht="14.25" customHeight="1"/>
-    <row r="913" ht="14.25" customHeight="1"/>
-    <row r="914" ht="14.25" customHeight="1"/>
-    <row r="915" ht="14.25" customHeight="1"/>
-    <row r="916" ht="14.25" customHeight="1"/>
-    <row r="917" ht="14.25" customHeight="1"/>
-    <row r="918" ht="14.25" customHeight="1"/>
-    <row r="919" ht="14.25" customHeight="1"/>
-    <row r="920" ht="14.25" customHeight="1"/>
-    <row r="921" ht="14.25" customHeight="1"/>
-    <row r="922" ht="14.25" customHeight="1"/>
-    <row r="923" ht="14.25" customHeight="1"/>
-    <row r="924" ht="14.25" customHeight="1"/>
-    <row r="925" ht="14.25" customHeight="1"/>
-    <row r="926" ht="14.25" customHeight="1"/>
-    <row r="927" ht="14.25" customHeight="1"/>
-    <row r="928" ht="14.25" customHeight="1"/>
-    <row r="929" ht="14.25" customHeight="1"/>
-    <row r="930" ht="14.25" customHeight="1"/>
-    <row r="931" ht="14.25" customHeight="1"/>
-    <row r="932" ht="14.25" customHeight="1"/>
-    <row r="933" ht="14.25" customHeight="1"/>
-    <row r="934" ht="14.25" customHeight="1"/>
-    <row r="935" ht="14.25" customHeight="1"/>
-    <row r="936" ht="14.25" customHeight="1"/>
-    <row r="937" ht="14.25" customHeight="1"/>
-    <row r="938" ht="14.25" customHeight="1"/>
-    <row r="939" ht="14.25" customHeight="1"/>
-    <row r="940" ht="14.25" customHeight="1"/>
-    <row r="941" ht="14.25" customHeight="1"/>
-    <row r="942" ht="14.25" customHeight="1"/>
-    <row r="943" ht="14.25" customHeight="1"/>
-    <row r="944" ht="14.25" customHeight="1"/>
-    <row r="945" ht="14.25" customHeight="1"/>
-    <row r="946" ht="14.25" customHeight="1"/>
-    <row r="947" ht="14.25" customHeight="1"/>
-    <row r="948" ht="14.25" customHeight="1"/>
-    <row r="949" ht="14.25" customHeight="1"/>
-    <row r="950" ht="14.25" customHeight="1"/>
-    <row r="951" ht="14.25" customHeight="1"/>
-    <row r="952" ht="14.25" customHeight="1"/>
-    <row r="953" ht="14.25" customHeight="1"/>
-    <row r="954" ht="14.25" customHeight="1"/>
-    <row r="955" ht="14.25" customHeight="1"/>
-    <row r="956" ht="14.25" customHeight="1"/>
-    <row r="957" ht="14.25" customHeight="1"/>
-    <row r="958" ht="14.25" customHeight="1"/>
-    <row r="959" ht="14.25" customHeight="1"/>
-    <row r="960" ht="14.25" customHeight="1"/>
-    <row r="961" ht="14.25" customHeight="1"/>
-    <row r="962" ht="14.25" customHeight="1"/>
-    <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
-    <row r="973" ht="14.25" customHeight="1"/>
-    <row r="974" ht="14.25" customHeight="1"/>
-    <row r="975" ht="14.25" customHeight="1"/>
-    <row r="976" ht="14.25" customHeight="1"/>
-    <row r="977" ht="14.25" customHeight="1"/>
-    <row r="978" ht="14.25" customHeight="1"/>
-    <row r="979" ht="14.25" customHeight="1"/>
-    <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="7" ht="14.25" customHeight="true"/>
+    <row r="8" ht="14.25" customHeight="true"/>
+    <row r="9" ht="14.25" customHeight="true"/>
+    <row r="10" ht="14.25" customHeight="true"/>
+    <row r="11" ht="14.25" customHeight="true"/>
+    <row r="12" ht="14.25" customHeight="true"/>
+    <row r="13" ht="14.25" customHeight="true"/>
+    <row r="14" ht="14.25" customHeight="true"/>
+    <row r="15" ht="14.25" customHeight="true"/>
+    <row r="16" ht="14.25" customHeight="true"/>
+    <row r="17" ht="14.25" customHeight="true"/>
+    <row r="18" ht="14.25" customHeight="true"/>
+    <row r="19" ht="14.25" customHeight="true"/>
+    <row r="20" ht="14.25" customHeight="true"/>
+    <row r="21" ht="14.25" customHeight="true"/>
+    <row r="22" ht="14.25" customHeight="true"/>
+    <row r="23" ht="14.25" customHeight="true"/>
+    <row r="24" ht="14.25" customHeight="true"/>
+    <row r="25" ht="14.25" customHeight="true"/>
+    <row r="26" ht="14.25" customHeight="true"/>
+    <row r="27" ht="14.25" customHeight="true"/>
+    <row r="28" ht="14.25" customHeight="true"/>
+    <row r="29" ht="14.25" customHeight="true"/>
+    <row r="30" ht="14.25" customHeight="true"/>
+    <row r="31" ht="14.25" customHeight="true"/>
+    <row r="32" ht="14.25" customHeight="true"/>
+    <row r="33" ht="14.25" customHeight="true"/>
+    <row r="34" ht="14.25" customHeight="true"/>
+    <row r="35" ht="14.25" customHeight="true"/>
+    <row r="36" ht="14.25" customHeight="true"/>
+    <row r="37" ht="14.25" customHeight="true"/>
+    <row r="38" ht="14.25" customHeight="true"/>
+    <row r="39" ht="14.25" customHeight="true"/>
+    <row r="40" ht="14.25" customHeight="true"/>
+    <row r="41" ht="14.25" customHeight="true"/>
+    <row r="42" ht="14.25" customHeight="true"/>
+    <row r="43" ht="14.25" customHeight="true"/>
+    <row r="44" ht="14.25" customHeight="true"/>
+    <row r="45" ht="14.25" customHeight="true"/>
+    <row r="46" ht="14.25" customHeight="true"/>
+    <row r="47" ht="14.25" customHeight="true"/>
+    <row r="48" ht="14.25" customHeight="true"/>
+    <row r="49" ht="14.25" customHeight="true"/>
+    <row r="50" ht="14.25" customHeight="true"/>
+    <row r="51" ht="14.25" customHeight="true"/>
+    <row r="52" ht="14.25" customHeight="true"/>
+    <row r="53" ht="14.25" customHeight="true"/>
+    <row r="54" ht="14.25" customHeight="true"/>
+    <row r="55" ht="14.25" customHeight="true"/>
+    <row r="56" ht="14.25" customHeight="true"/>
+    <row r="57" ht="14.25" customHeight="true"/>
+    <row r="58" ht="14.25" customHeight="true"/>
+    <row r="59" ht="14.25" customHeight="true"/>
+    <row r="60" ht="14.25" customHeight="true"/>
+    <row r="61" ht="14.25" customHeight="true"/>
+    <row r="62" ht="14.25" customHeight="true"/>
+    <row r="63" ht="14.25" customHeight="true"/>
+    <row r="64" ht="14.25" customHeight="true"/>
+    <row r="65" ht="14.25" customHeight="true"/>
+    <row r="66" ht="14.25" customHeight="true"/>
+    <row r="67" ht="14.25" customHeight="true"/>
+    <row r="68" ht="14.25" customHeight="true"/>
+    <row r="69" ht="14.25" customHeight="true"/>
+    <row r="70" ht="14.25" customHeight="true"/>
+    <row r="71" ht="14.25" customHeight="true"/>
+    <row r="72" ht="14.25" customHeight="true"/>
+    <row r="73" ht="14.25" customHeight="true"/>
+    <row r="74" ht="14.25" customHeight="true"/>
+    <row r="75" ht="14.25" customHeight="true"/>
+    <row r="76" ht="14.25" customHeight="true"/>
+    <row r="77" ht="14.25" customHeight="true"/>
+    <row r="78" ht="14.25" customHeight="true"/>
+    <row r="79" ht="14.25" customHeight="true"/>
+    <row r="80" ht="14.25" customHeight="true"/>
+    <row r="81" ht="14.25" customHeight="true"/>
+    <row r="82" ht="14.25" customHeight="true"/>
+    <row r="83" ht="14.25" customHeight="true"/>
+    <row r="84" ht="14.25" customHeight="true"/>
+    <row r="85" ht="14.25" customHeight="true"/>
+    <row r="86" ht="14.25" customHeight="true"/>
+    <row r="87" ht="14.25" customHeight="true"/>
+    <row r="88" ht="14.25" customHeight="true"/>
+    <row r="89" ht="14.25" customHeight="true"/>
+    <row r="90" ht="14.25" customHeight="true"/>
+    <row r="91" ht="14.25" customHeight="true"/>
+    <row r="92" ht="14.25" customHeight="true"/>
+    <row r="93" ht="14.25" customHeight="true"/>
+    <row r="94" ht="14.25" customHeight="true"/>
+    <row r="95" ht="14.25" customHeight="true"/>
+    <row r="96" ht="14.25" customHeight="true"/>
+    <row r="97" ht="14.25" customHeight="true"/>
+    <row r="98" ht="14.25" customHeight="true"/>
+    <row r="99" ht="14.25" customHeight="true"/>
+    <row r="100" ht="14.25" customHeight="true"/>
+    <row r="101" ht="14.25" customHeight="true"/>
+    <row r="102" ht="14.25" customHeight="true"/>
+    <row r="103" ht="14.25" customHeight="true"/>
+    <row r="104" ht="14.25" customHeight="true"/>
+    <row r="105" ht="14.25" customHeight="true"/>
+    <row r="106" ht="14.25" customHeight="true"/>
+    <row r="107" ht="14.25" customHeight="true"/>
+    <row r="108" ht="14.25" customHeight="true"/>
+    <row r="109" ht="14.25" customHeight="true"/>
+    <row r="110" ht="14.25" customHeight="true"/>
+    <row r="111" ht="14.25" customHeight="true"/>
+    <row r="112" ht="14.25" customHeight="true"/>
+    <row r="113" ht="14.25" customHeight="true"/>
+    <row r="114" ht="14.25" customHeight="true"/>
+    <row r="115" ht="14.25" customHeight="true"/>
+    <row r="116" ht="14.25" customHeight="true"/>
+    <row r="117" ht="14.25" customHeight="true"/>
+    <row r="118" ht="14.25" customHeight="true"/>
+    <row r="119" ht="14.25" customHeight="true"/>
+    <row r="120" ht="14.25" customHeight="true"/>
+    <row r="121" ht="14.25" customHeight="true"/>
+    <row r="122" ht="14.25" customHeight="true"/>
+    <row r="123" ht="14.25" customHeight="true"/>
+    <row r="124" ht="14.25" customHeight="true"/>
+    <row r="125" ht="14.25" customHeight="true"/>
+    <row r="126" ht="14.25" customHeight="true"/>
+    <row r="127" ht="14.25" customHeight="true"/>
+    <row r="128" ht="14.25" customHeight="true"/>
+    <row r="129" ht="14.25" customHeight="true"/>
+    <row r="130" ht="14.25" customHeight="true"/>
+    <row r="131" ht="14.25" customHeight="true"/>
+    <row r="132" ht="14.25" customHeight="true"/>
+    <row r="133" ht="14.25" customHeight="true"/>
+    <row r="134" ht="14.25" customHeight="true"/>
+    <row r="135" ht="14.25" customHeight="true"/>
+    <row r="136" ht="14.25" customHeight="true"/>
+    <row r="137" ht="14.25" customHeight="true"/>
+    <row r="138" ht="14.25" customHeight="true"/>
+    <row r="139" ht="14.25" customHeight="true"/>
+    <row r="140" ht="14.25" customHeight="true"/>
+    <row r="141" ht="14.25" customHeight="true"/>
+    <row r="142" ht="14.25" customHeight="true"/>
+    <row r="143" ht="14.25" customHeight="true"/>
+    <row r="144" ht="14.25" customHeight="true"/>
+    <row r="145" ht="14.25" customHeight="true"/>
+    <row r="146" ht="14.25" customHeight="true"/>
+    <row r="147" ht="14.25" customHeight="true"/>
+    <row r="148" ht="14.25" customHeight="true"/>
+    <row r="149" ht="14.25" customHeight="true"/>
+    <row r="150" ht="14.25" customHeight="true"/>
+    <row r="151" ht="14.25" customHeight="true"/>
+    <row r="152" ht="14.25" customHeight="true"/>
+    <row r="153" ht="14.25" customHeight="true"/>
+    <row r="154" ht="14.25" customHeight="true"/>
+    <row r="155" ht="14.25" customHeight="true"/>
+    <row r="156" ht="14.25" customHeight="true"/>
+    <row r="157" ht="14.25" customHeight="true"/>
+    <row r="158" ht="14.25" customHeight="true"/>
+    <row r="159" ht="14.25" customHeight="true"/>
+    <row r="160" ht="14.25" customHeight="true"/>
+    <row r="161" ht="14.25" customHeight="true"/>
+    <row r="162" ht="14.25" customHeight="true"/>
+    <row r="163" ht="14.25" customHeight="true"/>
+    <row r="164" ht="14.25" customHeight="true"/>
+    <row r="165" ht="14.25" customHeight="true"/>
+    <row r="166" ht="14.25" customHeight="true"/>
+    <row r="167" ht="14.25" customHeight="true"/>
+    <row r="168" ht="14.25" customHeight="true"/>
+    <row r="169" ht="14.25" customHeight="true"/>
+    <row r="170" ht="14.25" customHeight="true"/>
+    <row r="171" ht="14.25" customHeight="true"/>
+    <row r="172" ht="14.25" customHeight="true"/>
+    <row r="173" ht="14.25" customHeight="true"/>
+    <row r="174" ht="14.25" customHeight="true"/>
+    <row r="175" ht="14.25" customHeight="true"/>
+    <row r="176" ht="14.25" customHeight="true"/>
+    <row r="177" ht="14.25" customHeight="true"/>
+    <row r="178" ht="14.25" customHeight="true"/>
+    <row r="179" ht="14.25" customHeight="true"/>
+    <row r="180" ht="14.25" customHeight="true"/>
+    <row r="181" ht="14.25" customHeight="true"/>
+    <row r="182" ht="14.25" customHeight="true"/>
+    <row r="183" ht="14.25" customHeight="true"/>
+    <row r="184" ht="14.25" customHeight="true"/>
+    <row r="185" ht="14.25" customHeight="true"/>
+    <row r="186" ht="14.25" customHeight="true"/>
+    <row r="187" ht="14.25" customHeight="true"/>
+    <row r="188" ht="14.25" customHeight="true"/>
+    <row r="189" ht="14.25" customHeight="true"/>
+    <row r="190" ht="14.25" customHeight="true"/>
+    <row r="191" ht="14.25" customHeight="true"/>
+    <row r="192" ht="14.25" customHeight="true"/>
+    <row r="193" ht="14.25" customHeight="true"/>
+    <row r="194" ht="14.25" customHeight="true"/>
+    <row r="195" ht="14.25" customHeight="true"/>
+    <row r="196" ht="14.25" customHeight="true"/>
+    <row r="197" ht="14.25" customHeight="true"/>
+    <row r="198" ht="14.25" customHeight="true"/>
+    <row r="199" ht="14.25" customHeight="true"/>
+    <row r="200" ht="14.25" customHeight="true"/>
+    <row r="201" ht="14.25" customHeight="true"/>
+    <row r="202" ht="14.25" customHeight="true"/>
+    <row r="203" ht="14.25" customHeight="true"/>
+    <row r="204" ht="14.25" customHeight="true"/>
+    <row r="205" ht="14.25" customHeight="true"/>
+    <row r="206" ht="14.25" customHeight="true"/>
+    <row r="207" ht="14.25" customHeight="true"/>
+    <row r="208" ht="14.25" customHeight="true"/>
+    <row r="209" ht="14.25" customHeight="true"/>
+    <row r="210" ht="14.25" customHeight="true"/>
+    <row r="211" ht="14.25" customHeight="true"/>
+    <row r="212" ht="14.25" customHeight="true"/>
+    <row r="213" ht="14.25" customHeight="true"/>
+    <row r="214" ht="14.25" customHeight="true"/>
+    <row r="215" ht="14.25" customHeight="true"/>
+    <row r="216" ht="14.25" customHeight="true"/>
+    <row r="217" ht="14.25" customHeight="true"/>
+    <row r="218" ht="14.25" customHeight="true"/>
+    <row r="219" ht="14.25" customHeight="true"/>
+    <row r="220" ht="14.25" customHeight="true"/>
+    <row r="221" ht="14.25" customHeight="true"/>
+    <row r="222" ht="14.25" customHeight="true"/>
+    <row r="223" ht="14.25" customHeight="true"/>
+    <row r="224" ht="14.25" customHeight="true"/>
+    <row r="225" ht="14.25" customHeight="true"/>
+    <row r="226" ht="14.25" customHeight="true"/>
+    <row r="227" ht="14.25" customHeight="true"/>
+    <row r="228" ht="14.25" customHeight="true"/>
+    <row r="229" ht="14.25" customHeight="true"/>
+    <row r="230" ht="14.25" customHeight="true"/>
+    <row r="231" ht="14.25" customHeight="true"/>
+    <row r="232" ht="14.25" customHeight="true"/>
+    <row r="233" ht="14.25" customHeight="true"/>
+    <row r="234" ht="14.25" customHeight="true"/>
+    <row r="235" ht="14.25" customHeight="true"/>
+    <row r="236" ht="14.25" customHeight="true"/>
+    <row r="237" ht="14.25" customHeight="true"/>
+    <row r="238" ht="14.25" customHeight="true"/>
+    <row r="239" ht="14.25" customHeight="true"/>
+    <row r="240" ht="14.25" customHeight="true"/>
+    <row r="241" ht="14.25" customHeight="true"/>
+    <row r="242" ht="14.25" customHeight="true"/>
+    <row r="243" ht="14.25" customHeight="true"/>
+    <row r="244" ht="14.25" customHeight="true"/>
+    <row r="245" ht="14.25" customHeight="true"/>
+    <row r="246" ht="14.25" customHeight="true"/>
+    <row r="247" ht="14.25" customHeight="true"/>
+    <row r="248" ht="14.25" customHeight="true"/>
+    <row r="249" ht="14.25" customHeight="true"/>
+    <row r="250" ht="14.25" customHeight="true"/>
+    <row r="251" ht="14.25" customHeight="true"/>
+    <row r="252" ht="14.25" customHeight="true"/>
+    <row r="253" ht="14.25" customHeight="true"/>
+    <row r="254" ht="14.25" customHeight="true"/>
+    <row r="255" ht="14.25" customHeight="true"/>
+    <row r="256" ht="14.25" customHeight="true"/>
+    <row r="257" ht="14.25" customHeight="true"/>
+    <row r="258" ht="14.25" customHeight="true"/>
+    <row r="259" ht="14.25" customHeight="true"/>
+    <row r="260" ht="14.25" customHeight="true"/>
+    <row r="261" ht="14.25" customHeight="true"/>
+    <row r="262" ht="14.25" customHeight="true"/>
+    <row r="263" ht="14.25" customHeight="true"/>
+    <row r="264" ht="14.25" customHeight="true"/>
+    <row r="265" ht="14.25" customHeight="true"/>
+    <row r="266" ht="14.25" customHeight="true"/>
+    <row r="267" ht="14.25" customHeight="true"/>
+    <row r="268" ht="14.25" customHeight="true"/>
+    <row r="269" ht="14.25" customHeight="true"/>
+    <row r="270" ht="14.25" customHeight="true"/>
+    <row r="271" ht="14.25" customHeight="true"/>
+    <row r="272" ht="14.25" customHeight="true"/>
+    <row r="273" ht="14.25" customHeight="true"/>
+    <row r="274" ht="14.25" customHeight="true"/>
+    <row r="275" ht="14.25" customHeight="true"/>
+    <row r="276" ht="14.25" customHeight="true"/>
+    <row r="277" ht="14.25" customHeight="true"/>
+    <row r="278" ht="14.25" customHeight="true"/>
+    <row r="279" ht="14.25" customHeight="true"/>
+    <row r="280" ht="14.25" customHeight="true"/>
+    <row r="281" ht="14.25" customHeight="true"/>
+    <row r="282" ht="14.25" customHeight="true"/>
+    <row r="283" ht="14.25" customHeight="true"/>
+    <row r="284" ht="14.25" customHeight="true"/>
+    <row r="285" ht="14.25" customHeight="true"/>
+    <row r="286" ht="14.25" customHeight="true"/>
+    <row r="287" ht="14.25" customHeight="true"/>
+    <row r="288" ht="14.25" customHeight="true"/>
+    <row r="289" ht="14.25" customHeight="true"/>
+    <row r="290" ht="14.25" customHeight="true"/>
+    <row r="291" ht="14.25" customHeight="true"/>
+    <row r="292" ht="14.25" customHeight="true"/>
+    <row r="293" ht="14.25" customHeight="true"/>
+    <row r="294" ht="14.25" customHeight="true"/>
+    <row r="295" ht="14.25" customHeight="true"/>
+    <row r="296" ht="14.25" customHeight="true"/>
+    <row r="297" ht="14.25" customHeight="true"/>
+    <row r="298" ht="14.25" customHeight="true"/>
+    <row r="299" ht="14.25" customHeight="true"/>
+    <row r="300" ht="14.25" customHeight="true"/>
+    <row r="301" ht="14.25" customHeight="true"/>
+    <row r="302" ht="14.25" customHeight="true"/>
+    <row r="303" ht="14.25" customHeight="true"/>
+    <row r="304" ht="14.25" customHeight="true"/>
+    <row r="305" ht="14.25" customHeight="true"/>
+    <row r="306" ht="14.25" customHeight="true"/>
+    <row r="307" ht="14.25" customHeight="true"/>
+    <row r="308" ht="14.25" customHeight="true"/>
+    <row r="309" ht="14.25" customHeight="true"/>
+    <row r="310" ht="14.25" customHeight="true"/>
+    <row r="311" ht="14.25" customHeight="true"/>
+    <row r="312" ht="14.25" customHeight="true"/>
+    <row r="313" ht="14.25" customHeight="true"/>
+    <row r="314" ht="14.25" customHeight="true"/>
+    <row r="315" ht="14.25" customHeight="true"/>
+    <row r="316" ht="14.25" customHeight="true"/>
+    <row r="317" ht="14.25" customHeight="true"/>
+    <row r="318" ht="14.25" customHeight="true"/>
+    <row r="319" ht="14.25" customHeight="true"/>
+    <row r="320" ht="14.25" customHeight="true"/>
+    <row r="321" ht="14.25" customHeight="true"/>
+    <row r="322" ht="14.25" customHeight="true"/>
+    <row r="323" ht="14.25" customHeight="true"/>
+    <row r="324" ht="14.25" customHeight="true"/>
+    <row r="325" ht="14.25" customHeight="true"/>
+    <row r="326" ht="14.25" customHeight="true"/>
+    <row r="327" ht="14.25" customHeight="true"/>
+    <row r="328" ht="14.25" customHeight="true"/>
+    <row r="329" ht="14.25" customHeight="true"/>
+    <row r="330" ht="14.25" customHeight="true"/>
+    <row r="331" ht="14.25" customHeight="true"/>
+    <row r="332" ht="14.25" customHeight="true"/>
+    <row r="333" ht="14.25" customHeight="true"/>
+    <row r="334" ht="14.25" customHeight="true"/>
+    <row r="335" ht="14.25" customHeight="true"/>
+    <row r="336" ht="14.25" customHeight="true"/>
+    <row r="337" ht="14.25" customHeight="true"/>
+    <row r="338" ht="14.25" customHeight="true"/>
+    <row r="339" ht="14.25" customHeight="true"/>
+    <row r="340" ht="14.25" customHeight="true"/>
+    <row r="341" ht="14.25" customHeight="true"/>
+    <row r="342" ht="14.25" customHeight="true"/>
+    <row r="343" ht="14.25" customHeight="true"/>
+    <row r="344" ht="14.25" customHeight="true"/>
+    <row r="345" ht="14.25" customHeight="true"/>
+    <row r="346" ht="14.25" customHeight="true"/>
+    <row r="347" ht="14.25" customHeight="true"/>
+    <row r="348" ht="14.25" customHeight="true"/>
+    <row r="349" ht="14.25" customHeight="true"/>
+    <row r="350" ht="14.25" customHeight="true"/>
+    <row r="351" ht="14.25" customHeight="true"/>
+    <row r="352" ht="14.25" customHeight="true"/>
+    <row r="353" ht="14.25" customHeight="true"/>
+    <row r="354" ht="14.25" customHeight="true"/>
+    <row r="355" ht="14.25" customHeight="true"/>
+    <row r="356" ht="14.25" customHeight="true"/>
+    <row r="357" ht="14.25" customHeight="true"/>
+    <row r="358" ht="14.25" customHeight="true"/>
+    <row r="359" ht="14.25" customHeight="true"/>
+    <row r="360" ht="14.25" customHeight="true"/>
+    <row r="361" ht="14.25" customHeight="true"/>
+    <row r="362" ht="14.25" customHeight="true"/>
+    <row r="363" ht="14.25" customHeight="true"/>
+    <row r="364" ht="14.25" customHeight="true"/>
+    <row r="365" ht="14.25" customHeight="true"/>
+    <row r="366" ht="14.25" customHeight="true"/>
+    <row r="367" ht="14.25" customHeight="true"/>
+    <row r="368" ht="14.25" customHeight="true"/>
+    <row r="369" ht="14.25" customHeight="true"/>
+    <row r="370" ht="14.25" customHeight="true"/>
+    <row r="371" ht="14.25" customHeight="true"/>
+    <row r="372" ht="14.25" customHeight="true"/>
+    <row r="373" ht="14.25" customHeight="true"/>
+    <row r="374" ht="14.25" customHeight="true"/>
+    <row r="375" ht="14.25" customHeight="true"/>
+    <row r="376" ht="14.25" customHeight="true"/>
+    <row r="377" ht="14.25" customHeight="true"/>
+    <row r="378" ht="14.25" customHeight="true"/>
+    <row r="379" ht="14.25" customHeight="true"/>
+    <row r="380" ht="14.25" customHeight="true"/>
+    <row r="381" ht="14.25" customHeight="true"/>
+    <row r="382" ht="14.25" customHeight="true"/>
+    <row r="383" ht="14.25" customHeight="true"/>
+    <row r="384" ht="14.25" customHeight="true"/>
+    <row r="385" ht="14.25" customHeight="true"/>
+    <row r="386" ht="14.25" customHeight="true"/>
+    <row r="387" ht="14.25" customHeight="true"/>
+    <row r="388" ht="14.25" customHeight="true"/>
+    <row r="389" ht="14.25" customHeight="true"/>
+    <row r="390" ht="14.25" customHeight="true"/>
+    <row r="391" ht="14.25" customHeight="true"/>
+    <row r="392" ht="14.25" customHeight="true"/>
+    <row r="393" ht="14.25" customHeight="true"/>
+    <row r="394" ht="14.25" customHeight="true"/>
+    <row r="395" ht="14.25" customHeight="true"/>
+    <row r="396" ht="14.25" customHeight="true"/>
+    <row r="397" ht="14.25" customHeight="true"/>
+    <row r="398" ht="14.25" customHeight="true"/>
+    <row r="399" ht="14.25" customHeight="true"/>
+    <row r="400" ht="14.25" customHeight="true"/>
+    <row r="401" ht="14.25" customHeight="true"/>
+    <row r="402" ht="14.25" customHeight="true"/>
+    <row r="403" ht="14.25" customHeight="true"/>
+    <row r="404" ht="14.25" customHeight="true"/>
+    <row r="405" ht="14.25" customHeight="true"/>
+    <row r="406" ht="14.25" customHeight="true"/>
+    <row r="407" ht="14.25" customHeight="true"/>
+    <row r="408" ht="14.25" customHeight="true"/>
+    <row r="409" ht="14.25" customHeight="true"/>
+    <row r="410" ht="14.25" customHeight="true"/>
+    <row r="411" ht="14.25" customHeight="true"/>
+    <row r="412" ht="14.25" customHeight="true"/>
+    <row r="413" ht="14.25" customHeight="true"/>
+    <row r="414" ht="14.25" customHeight="true"/>
+    <row r="415" ht="14.25" customHeight="true"/>
+    <row r="416" ht="14.25" customHeight="true"/>
+    <row r="417" ht="14.25" customHeight="true"/>
+    <row r="418" ht="14.25" customHeight="true"/>
+    <row r="419" ht="14.25" customHeight="true"/>
+    <row r="420" ht="14.25" customHeight="true"/>
+    <row r="421" ht="14.25" customHeight="true"/>
+    <row r="422" ht="14.25" customHeight="true"/>
+    <row r="423" ht="14.25" customHeight="true"/>
+    <row r="424" ht="14.25" customHeight="true"/>
+    <row r="425" ht="14.25" customHeight="true"/>
+    <row r="426" ht="14.25" customHeight="true"/>
+    <row r="427" ht="14.25" customHeight="true"/>
+    <row r="428" ht="14.25" customHeight="true"/>
+    <row r="429" ht="14.25" customHeight="true"/>
+    <row r="430" ht="14.25" customHeight="true"/>
+    <row r="431" ht="14.25" customHeight="true"/>
+    <row r="432" ht="14.25" customHeight="true"/>
+    <row r="433" ht="14.25" customHeight="true"/>
+    <row r="434" ht="14.25" customHeight="true"/>
+    <row r="435" ht="14.25" customHeight="true"/>
+    <row r="436" ht="14.25" customHeight="true"/>
+    <row r="437" ht="14.25" customHeight="true"/>
+    <row r="438" ht="14.25" customHeight="true"/>
+    <row r="439" ht="14.25" customHeight="true"/>
+    <row r="440" ht="14.25" customHeight="true"/>
+    <row r="441" ht="14.25" customHeight="true"/>
+    <row r="442" ht="14.25" customHeight="true"/>
+    <row r="443" ht="14.25" customHeight="true"/>
+    <row r="444" ht="14.25" customHeight="true"/>
+    <row r="445" ht="14.25" customHeight="true"/>
+    <row r="446" ht="14.25" customHeight="true"/>
+    <row r="447" ht="14.25" customHeight="true"/>
+    <row r="448" ht="14.25" customHeight="true"/>
+    <row r="449" ht="14.25" customHeight="true"/>
+    <row r="450" ht="14.25" customHeight="true"/>
+    <row r="451" ht="14.25" customHeight="true"/>
+    <row r="452" ht="14.25" customHeight="true"/>
+    <row r="453" ht="14.25" customHeight="true"/>
+    <row r="454" ht="14.25" customHeight="true"/>
+    <row r="455" ht="14.25" customHeight="true"/>
+    <row r="456" ht="14.25" customHeight="true"/>
+    <row r="457" ht="14.25" customHeight="true"/>
+    <row r="458" ht="14.25" customHeight="true"/>
+    <row r="459" ht="14.25" customHeight="true"/>
+    <row r="460" ht="14.25" customHeight="true"/>
+    <row r="461" ht="14.25" customHeight="true"/>
+    <row r="462" ht="14.25" customHeight="true"/>
+    <row r="463" ht="14.25" customHeight="true"/>
+    <row r="464" ht="14.25" customHeight="true"/>
+    <row r="465" ht="14.25" customHeight="true"/>
+    <row r="466" ht="14.25" customHeight="true"/>
+    <row r="467" ht="14.25" customHeight="true"/>
+    <row r="468" ht="14.25" customHeight="true"/>
+    <row r="469" ht="14.25" customHeight="true"/>
+    <row r="470" ht="14.25" customHeight="true"/>
+    <row r="471" ht="14.25" customHeight="true"/>
+    <row r="472" ht="14.25" customHeight="true"/>
+    <row r="473" ht="14.25" customHeight="true"/>
+    <row r="474" ht="14.25" customHeight="true"/>
+    <row r="475" ht="14.25" customHeight="true"/>
+    <row r="476" ht="14.25" customHeight="true"/>
+    <row r="477" ht="14.25" customHeight="true"/>
+    <row r="478" ht="14.25" customHeight="true"/>
+    <row r="479" ht="14.25" customHeight="true"/>
+    <row r="480" ht="14.25" customHeight="true"/>
+    <row r="481" ht="14.25" customHeight="true"/>
+    <row r="482" ht="14.25" customHeight="true"/>
+    <row r="483" ht="14.25" customHeight="true"/>
+    <row r="484" ht="14.25" customHeight="true"/>
+    <row r="485" ht="14.25" customHeight="true"/>
+    <row r="486" ht="14.25" customHeight="true"/>
+    <row r="487" ht="14.25" customHeight="true"/>
+    <row r="488" ht="14.25" customHeight="true"/>
+    <row r="489" ht="14.25" customHeight="true"/>
+    <row r="490" ht="14.25" customHeight="true"/>
+    <row r="491" ht="14.25" customHeight="true"/>
+    <row r="492" ht="14.25" customHeight="true"/>
+    <row r="493" ht="14.25" customHeight="true"/>
+    <row r="494" ht="14.25" customHeight="true"/>
+    <row r="495" ht="14.25" customHeight="true"/>
+    <row r="496" ht="14.25" customHeight="true"/>
+    <row r="497" ht="14.25" customHeight="true"/>
+    <row r="498" ht="14.25" customHeight="true"/>
+    <row r="499" ht="14.25" customHeight="true"/>
+    <row r="500" ht="14.25" customHeight="true"/>
+    <row r="501" ht="14.25" customHeight="true"/>
+    <row r="502" ht="14.25" customHeight="true"/>
+    <row r="503" ht="14.25" customHeight="true"/>
+    <row r="504" ht="14.25" customHeight="true"/>
+    <row r="505" ht="14.25" customHeight="true"/>
+    <row r="506" ht="14.25" customHeight="true"/>
+    <row r="507" ht="14.25" customHeight="true"/>
+    <row r="508" ht="14.25" customHeight="true"/>
+    <row r="509" ht="14.25" customHeight="true"/>
+    <row r="510" ht="14.25" customHeight="true"/>
+    <row r="511" ht="14.25" customHeight="true"/>
+    <row r="512" ht="14.25" customHeight="true"/>
+    <row r="513" ht="14.25" customHeight="true"/>
+    <row r="514" ht="14.25" customHeight="true"/>
+    <row r="515" ht="14.25" customHeight="true"/>
+    <row r="516" ht="14.25" customHeight="true"/>
+    <row r="517" ht="14.25" customHeight="true"/>
+    <row r="518" ht="14.25" customHeight="true"/>
+    <row r="519" ht="14.25" customHeight="true"/>
+    <row r="520" ht="14.25" customHeight="true"/>
+    <row r="521" ht="14.25" customHeight="true"/>
+    <row r="522" ht="14.25" customHeight="true"/>
+    <row r="523" ht="14.25" customHeight="true"/>
+    <row r="524" ht="14.25" customHeight="true"/>
+    <row r="525" ht="14.25" customHeight="true"/>
+    <row r="526" ht="14.25" customHeight="true"/>
+    <row r="527" ht="14.25" customHeight="true"/>
+    <row r="528" ht="14.25" customHeight="true"/>
+    <row r="529" ht="14.25" customHeight="true"/>
+    <row r="530" ht="14.25" customHeight="true"/>
+    <row r="531" ht="14.25" customHeight="true"/>
+    <row r="532" ht="14.25" customHeight="true"/>
+    <row r="533" ht="14.25" customHeight="true"/>
+    <row r="534" ht="14.25" customHeight="true"/>
+    <row r="535" ht="14.25" customHeight="true"/>
+    <row r="536" ht="14.25" customHeight="true"/>
+    <row r="537" ht="14.25" customHeight="true"/>
+    <row r="538" ht="14.25" customHeight="true"/>
+    <row r="539" ht="14.25" customHeight="true"/>
+    <row r="540" ht="14.25" customHeight="true"/>
+    <row r="541" ht="14.25" customHeight="true"/>
+    <row r="542" ht="14.25" customHeight="true"/>
+    <row r="543" ht="14.25" customHeight="true"/>
+    <row r="544" ht="14.25" customHeight="true"/>
+    <row r="545" ht="14.25" customHeight="true"/>
+    <row r="546" ht="14.25" customHeight="true"/>
+    <row r="547" ht="14.25" customHeight="true"/>
+    <row r="548" ht="14.25" customHeight="true"/>
+    <row r="549" ht="14.25" customHeight="true"/>
+    <row r="550" ht="14.25" customHeight="true"/>
+    <row r="551" ht="14.25" customHeight="true"/>
+    <row r="552" ht="14.25" customHeight="true"/>
+    <row r="553" ht="14.25" customHeight="true"/>
+    <row r="554" ht="14.25" customHeight="true"/>
+    <row r="555" ht="14.25" customHeight="true"/>
+    <row r="556" ht="14.25" customHeight="true"/>
+    <row r="557" ht="14.25" customHeight="true"/>
+    <row r="558" ht="14.25" customHeight="true"/>
+    <row r="559" ht="14.25" customHeight="true"/>
+    <row r="560" ht="14.25" customHeight="true"/>
+    <row r="561" ht="14.25" customHeight="true"/>
+    <row r="562" ht="14.25" customHeight="true"/>
+    <row r="563" ht="14.25" customHeight="true"/>
+    <row r="564" ht="14.25" customHeight="true"/>
+    <row r="565" ht="14.25" customHeight="true"/>
+    <row r="566" ht="14.25" customHeight="true"/>
+    <row r="567" ht="14.25" customHeight="true"/>
+    <row r="568" ht="14.25" customHeight="true"/>
+    <row r="569" ht="14.25" customHeight="true"/>
+    <row r="570" ht="14.25" customHeight="true"/>
+    <row r="571" ht="14.25" customHeight="true"/>
+    <row r="572" ht="14.25" customHeight="true"/>
+    <row r="573" ht="14.25" customHeight="true"/>
+    <row r="574" ht="14.25" customHeight="true"/>
+    <row r="575" ht="14.25" customHeight="true"/>
+    <row r="576" ht="14.25" customHeight="true"/>
+    <row r="577" ht="14.25" customHeight="true"/>
+    <row r="578" ht="14.25" customHeight="true"/>
+    <row r="579" ht="14.25" customHeight="true"/>
+    <row r="580" ht="14.25" customHeight="true"/>
+    <row r="581" ht="14.25" customHeight="true"/>
+    <row r="582" ht="14.25" customHeight="true"/>
+    <row r="583" ht="14.25" customHeight="true"/>
+    <row r="584" ht="14.25" customHeight="true"/>
+    <row r="585" ht="14.25" customHeight="true"/>
+    <row r="586" ht="14.25" customHeight="true"/>
+    <row r="587" ht="14.25" customHeight="true"/>
+    <row r="588" ht="14.25" customHeight="true"/>
+    <row r="589" ht="14.25" customHeight="true"/>
+    <row r="590" ht="14.25" customHeight="true"/>
+    <row r="591" ht="14.25" customHeight="true"/>
+    <row r="592" ht="14.25" customHeight="true"/>
+    <row r="593" ht="14.25" customHeight="true"/>
+    <row r="594" ht="14.25" customHeight="true"/>
+    <row r="595" ht="14.25" customHeight="true"/>
+    <row r="596" ht="14.25" customHeight="true"/>
+    <row r="597" ht="14.25" customHeight="true"/>
+    <row r="598" ht="14.25" customHeight="true"/>
+    <row r="599" ht="14.25" customHeight="true"/>
+    <row r="600" ht="14.25" customHeight="true"/>
+    <row r="601" ht="14.25" customHeight="true"/>
+    <row r="602" ht="14.25" customHeight="true"/>
+    <row r="603" ht="14.25" customHeight="true"/>
+    <row r="604" ht="14.25" customHeight="true"/>
+    <row r="605" ht="14.25" customHeight="true"/>
+    <row r="606" ht="14.25" customHeight="true"/>
+    <row r="607" ht="14.25" customHeight="true"/>
+    <row r="608" ht="14.25" customHeight="true"/>
+    <row r="609" ht="14.25" customHeight="true"/>
+    <row r="610" ht="14.25" customHeight="true"/>
+    <row r="611" ht="14.25" customHeight="true"/>
+    <row r="612" ht="14.25" customHeight="true"/>
+    <row r="613" ht="14.25" customHeight="true"/>
+    <row r="614" ht="14.25" customHeight="true"/>
+    <row r="615" ht="14.25" customHeight="true"/>
+    <row r="616" ht="14.25" customHeight="true"/>
+    <row r="617" ht="14.25" customHeight="true"/>
+    <row r="618" ht="14.25" customHeight="true"/>
+    <row r="619" ht="14.25" customHeight="true"/>
+    <row r="620" ht="14.25" customHeight="true"/>
+    <row r="621" ht="14.25" customHeight="true"/>
+    <row r="622" ht="14.25" customHeight="true"/>
+    <row r="623" ht="14.25" customHeight="true"/>
+    <row r="624" ht="14.25" customHeight="true"/>
+    <row r="625" ht="14.25" customHeight="true"/>
+    <row r="626" ht="14.25" customHeight="true"/>
+    <row r="627" ht="14.25" customHeight="true"/>
+    <row r="628" ht="14.25" customHeight="true"/>
+    <row r="629" ht="14.25" customHeight="true"/>
+    <row r="630" ht="14.25" customHeight="true"/>
+    <row r="631" ht="14.25" customHeight="true"/>
+    <row r="632" ht="14.25" customHeight="true"/>
+    <row r="633" ht="14.25" customHeight="true"/>
+    <row r="634" ht="14.25" customHeight="true"/>
+    <row r="635" ht="14.25" customHeight="true"/>
+    <row r="636" ht="14.25" customHeight="true"/>
+    <row r="637" ht="14.25" customHeight="true"/>
+    <row r="638" ht="14.25" customHeight="true"/>
+    <row r="639" ht="14.25" customHeight="true"/>
+    <row r="640" ht="14.25" customHeight="true"/>
+    <row r="641" ht="14.25" customHeight="true"/>
+    <row r="642" ht="14.25" customHeight="true"/>
+    <row r="643" ht="14.25" customHeight="true"/>
+    <row r="644" ht="14.25" customHeight="true"/>
+    <row r="645" ht="14.25" customHeight="true"/>
+    <row r="646" ht="14.25" customHeight="true"/>
+    <row r="647" ht="14.25" customHeight="true"/>
+    <row r="648" ht="14.25" customHeight="true"/>
+    <row r="649" ht="14.25" customHeight="true"/>
+    <row r="650" ht="14.25" customHeight="true"/>
+    <row r="651" ht="14.25" customHeight="true"/>
+    <row r="652" ht="14.25" customHeight="true"/>
+    <row r="653" ht="14.25" customHeight="true"/>
+    <row r="654" ht="14.25" customHeight="true"/>
+    <row r="655" ht="14.25" customHeight="true"/>
+    <row r="656" ht="14.25" customHeight="true"/>
+    <row r="657" ht="14.25" customHeight="true"/>
+    <row r="658" ht="14.25" customHeight="true"/>
+    <row r="659" ht="14.25" customHeight="true"/>
+    <row r="660" ht="14.25" customHeight="true"/>
+    <row r="661" ht="14.25" customHeight="true"/>
+    <row r="662" ht="14.25" customHeight="true"/>
+    <row r="663" ht="14.25" customHeight="true"/>
+    <row r="664" ht="14.25" customHeight="true"/>
+    <row r="665" ht="14.25" customHeight="true"/>
+    <row r="666" ht="14.25" customHeight="true"/>
+    <row r="667" ht="14.25" customHeight="true"/>
+    <row r="668" ht="14.25" customHeight="true"/>
+    <row r="669" ht="14.25" customHeight="true"/>
+    <row r="670" ht="14.25" customHeight="true"/>
+    <row r="671" ht="14.25" customHeight="true"/>
+    <row r="672" ht="14.25" customHeight="true"/>
+    <row r="673" ht="14.25" customHeight="true"/>
+    <row r="674" ht="14.25" customHeight="true"/>
+    <row r="675" ht="14.25" customHeight="true"/>
+    <row r="676" ht="14.25" customHeight="true"/>
+    <row r="677" ht="14.25" customHeight="true"/>
+    <row r="678" ht="14.25" customHeight="true"/>
+    <row r="679" ht="14.25" customHeight="true"/>
+    <row r="680" ht="14.25" customHeight="true"/>
+    <row r="681" ht="14.25" customHeight="true"/>
+    <row r="682" ht="14.25" customHeight="true"/>
+    <row r="683" ht="14.25" customHeight="true"/>
+    <row r="684" ht="14.25" customHeight="true"/>
+    <row r="685" ht="14.25" customHeight="true"/>
+    <row r="686" ht="14.25" customHeight="true"/>
+    <row r="687" ht="14.25" customHeight="true"/>
+    <row r="688" ht="14.25" customHeight="true"/>
+    <row r="689" ht="14.25" customHeight="true"/>
+    <row r="690" ht="14.25" customHeight="true"/>
+    <row r="691" ht="14.25" customHeight="true"/>
+    <row r="692" ht="14.25" customHeight="true"/>
+    <row r="693" ht="14.25" customHeight="true"/>
+    <row r="694" ht="14.25" customHeight="true"/>
+    <row r="695" ht="14.25" customHeight="true"/>
+    <row r="696" ht="14.25" customHeight="true"/>
+    <row r="697" ht="14.25" customHeight="true"/>
+    <row r="698" ht="14.25" customHeight="true"/>
+    <row r="699" ht="14.25" customHeight="true"/>
+    <row r="700" ht="14.25" customHeight="true"/>
+    <row r="701" ht="14.25" customHeight="true"/>
+    <row r="702" ht="14.25" customHeight="true"/>
+    <row r="703" ht="14.25" customHeight="true"/>
+    <row r="704" ht="14.25" customHeight="true"/>
+    <row r="705" ht="14.25" customHeight="true"/>
+    <row r="706" ht="14.25" customHeight="true"/>
+    <row r="707" ht="14.25" customHeight="true"/>
+    <row r="708" ht="14.25" customHeight="true"/>
+    <row r="709" ht="14.25" customHeight="true"/>
+    <row r="710" ht="14.25" customHeight="true"/>
+    <row r="711" ht="14.25" customHeight="true"/>
+    <row r="712" ht="14.25" customHeight="true"/>
+    <row r="713" ht="14.25" customHeight="true"/>
+    <row r="714" ht="14.25" customHeight="true"/>
+    <row r="715" ht="14.25" customHeight="true"/>
+    <row r="716" ht="14.25" customHeight="true"/>
+    <row r="717" ht="14.25" customHeight="true"/>
+    <row r="718" ht="14.25" customHeight="true"/>
+    <row r="719" ht="14.25" customHeight="true"/>
+    <row r="720" ht="14.25" customHeight="true"/>
+    <row r="721" ht="14.25" customHeight="true"/>
+    <row r="722" ht="14.25" customHeight="true"/>
+    <row r="723" ht="14.25" customHeight="true"/>
+    <row r="724" ht="14.25" customHeight="true"/>
+    <row r="725" ht="14.25" customHeight="true"/>
+    <row r="726" ht="14.25" customHeight="true"/>
+    <row r="727" ht="14.25" customHeight="true"/>
+    <row r="728" ht="14.25" customHeight="true"/>
+    <row r="729" ht="14.25" customHeight="true"/>
+    <row r="730" ht="14.25" customHeight="true"/>
+    <row r="731" ht="14.25" customHeight="true"/>
+    <row r="732" ht="14.25" customHeight="true"/>
+    <row r="733" ht="14.25" customHeight="true"/>
+    <row r="734" ht="14.25" customHeight="true"/>
+    <row r="735" ht="14.25" customHeight="true"/>
+    <row r="736" ht="14.25" customHeight="true"/>
+    <row r="737" ht="14.25" customHeight="true"/>
+    <row r="738" ht="14.25" customHeight="true"/>
+    <row r="739" ht="14.25" customHeight="true"/>
+    <row r="740" ht="14.25" customHeight="true"/>
+    <row r="741" ht="14.25" customHeight="true"/>
+    <row r="742" ht="14.25" customHeight="true"/>
+    <row r="743" ht="14.25" customHeight="true"/>
+    <row r="744" ht="14.25" customHeight="true"/>
+    <row r="745" ht="14.25" customHeight="true"/>
+    <row r="746" ht="14.25" customHeight="true"/>
+    <row r="747" ht="14.25" customHeight="true"/>
+    <row r="748" ht="14.25" customHeight="true"/>
+    <row r="749" ht="14.25" customHeight="true"/>
+    <row r="750" ht="14.25" customHeight="true"/>
+    <row r="751" ht="14.25" customHeight="true"/>
+    <row r="752" ht="14.25" customHeight="true"/>
+    <row r="753" ht="14.25" customHeight="true"/>
+    <row r="754" ht="14.25" customHeight="true"/>
+    <row r="755" ht="14.25" customHeight="true"/>
+    <row r="756" ht="14.25" customHeight="true"/>
+    <row r="757" ht="14.25" customHeight="true"/>
+    <row r="758" ht="14.25" customHeight="true"/>
+    <row r="759" ht="14.25" customHeight="true"/>
+    <row r="760" ht="14.25" customHeight="true"/>
+    <row r="761" ht="14.25" customHeight="true"/>
+    <row r="762" ht="14.25" customHeight="true"/>
+    <row r="763" ht="14.25" customHeight="true"/>
+    <row r="764" ht="14.25" customHeight="true"/>
+    <row r="765" ht="14.25" customHeight="true"/>
+    <row r="766" ht="14.25" customHeight="true"/>
+    <row r="767" ht="14.25" customHeight="true"/>
+    <row r="768" ht="14.25" customHeight="true"/>
+    <row r="769" ht="14.25" customHeight="true"/>
+    <row r="770" ht="14.25" customHeight="true"/>
+    <row r="771" ht="14.25" customHeight="true"/>
+    <row r="772" ht="14.25" customHeight="true"/>
+    <row r="773" ht="14.25" customHeight="true"/>
+    <row r="774" ht="14.25" customHeight="true"/>
+    <row r="775" ht="14.25" customHeight="true"/>
+    <row r="776" ht="14.25" customHeight="true"/>
+    <row r="777" ht="14.25" customHeight="true"/>
+    <row r="778" ht="14.25" customHeight="true"/>
+    <row r="779" ht="14.25" customHeight="true"/>
+    <row r="780" ht="14.25" customHeight="true"/>
+    <row r="781" ht="14.25" customHeight="true"/>
+    <row r="782" ht="14.25" customHeight="true"/>
+    <row r="783" ht="14.25" customHeight="true"/>
+    <row r="784" ht="14.25" customHeight="true"/>
+    <row r="785" ht="14.25" customHeight="true"/>
+    <row r="786" ht="14.25" customHeight="true"/>
+    <row r="787" ht="14.25" customHeight="true"/>
+    <row r="788" ht="14.25" customHeight="true"/>
+    <row r="789" ht="14.25" customHeight="true"/>
+    <row r="790" ht="14.25" customHeight="true"/>
+    <row r="791" ht="14.25" customHeight="true"/>
+    <row r="792" ht="14.25" customHeight="true"/>
+    <row r="793" ht="14.25" customHeight="true"/>
+    <row r="794" ht="14.25" customHeight="true"/>
+    <row r="795" ht="14.25" customHeight="true"/>
+    <row r="796" ht="14.25" customHeight="true"/>
+    <row r="797" ht="14.25" customHeight="true"/>
+    <row r="798" ht="14.25" customHeight="true"/>
+    <row r="799" ht="14.25" customHeight="true"/>
+    <row r="800" ht="14.25" customHeight="true"/>
+    <row r="801" ht="14.25" customHeight="true"/>
+    <row r="802" ht="14.25" customHeight="true"/>
+    <row r="803" ht="14.25" customHeight="true"/>
+    <row r="804" ht="14.25" customHeight="true"/>
+    <row r="805" ht="14.25" customHeight="true"/>
+    <row r="806" ht="14.25" customHeight="true"/>
+    <row r="807" ht="14.25" customHeight="true"/>
+    <row r="808" ht="14.25" customHeight="true"/>
+    <row r="809" ht="14.25" customHeight="true"/>
+    <row r="810" ht="14.25" customHeight="true"/>
+    <row r="811" ht="14.25" customHeight="true"/>
+    <row r="812" ht="14.25" customHeight="true"/>
+    <row r="813" ht="14.25" customHeight="true"/>
+    <row r="814" ht="14.25" customHeight="true"/>
+    <row r="815" ht="14.25" customHeight="true"/>
+    <row r="816" ht="14.25" customHeight="true"/>
+    <row r="817" ht="14.25" customHeight="true"/>
+    <row r="818" ht="14.25" customHeight="true"/>
+    <row r="819" ht="14.25" customHeight="true"/>
+    <row r="820" ht="14.25" customHeight="true"/>
+    <row r="821" ht="14.25" customHeight="true"/>
+    <row r="822" ht="14.25" customHeight="true"/>
+    <row r="823" ht="14.25" customHeight="true"/>
+    <row r="824" ht="14.25" customHeight="true"/>
+    <row r="825" ht="14.25" customHeight="true"/>
+    <row r="826" ht="14.25" customHeight="true"/>
+    <row r="827" ht="14.25" customHeight="true"/>
+    <row r="828" ht="14.25" customHeight="true"/>
+    <row r="829" ht="14.25" customHeight="true"/>
+    <row r="830" ht="14.25" customHeight="true"/>
+    <row r="831" ht="14.25" customHeight="true"/>
+    <row r="832" ht="14.25" customHeight="true"/>
+    <row r="833" ht="14.25" customHeight="true"/>
+    <row r="834" ht="14.25" customHeight="true"/>
+    <row r="835" ht="14.25" customHeight="true"/>
+    <row r="836" ht="14.25" customHeight="true"/>
+    <row r="837" ht="14.25" customHeight="true"/>
+    <row r="838" ht="14.25" customHeight="true"/>
+    <row r="839" ht="14.25" customHeight="true"/>
+    <row r="840" ht="14.25" customHeight="true"/>
+    <row r="841" ht="14.25" customHeight="true"/>
+    <row r="842" ht="14.25" customHeight="true"/>
+    <row r="843" ht="14.25" customHeight="true"/>
+    <row r="844" ht="14.25" customHeight="true"/>
+    <row r="845" ht="14.25" customHeight="true"/>
+    <row r="846" ht="14.25" customHeight="true"/>
+    <row r="847" ht="14.25" customHeight="true"/>
+    <row r="848" ht="14.25" customHeight="true"/>
+    <row r="849" ht="14.25" customHeight="true"/>
+    <row r="850" ht="14.25" customHeight="true"/>
+    <row r="851" ht="14.25" customHeight="true"/>
+    <row r="852" ht="14.25" customHeight="true"/>
+    <row r="853" ht="14.25" customHeight="true"/>
+    <row r="854" ht="14.25" customHeight="true"/>
+    <row r="855" ht="14.25" customHeight="true"/>
+    <row r="856" ht="14.25" customHeight="true"/>
+    <row r="857" ht="14.25" customHeight="true"/>
+    <row r="858" ht="14.25" customHeight="true"/>
+    <row r="859" ht="14.25" customHeight="true"/>
+    <row r="860" ht="14.25" customHeight="true"/>
+    <row r="861" ht="14.25" customHeight="true"/>
+    <row r="862" ht="14.25" customHeight="true"/>
+    <row r="863" ht="14.25" customHeight="true"/>
+    <row r="864" ht="14.25" customHeight="true"/>
+    <row r="865" ht="14.25" customHeight="true"/>
+    <row r="866" ht="14.25" customHeight="true"/>
+    <row r="867" ht="14.25" customHeight="true"/>
+    <row r="868" ht="14.25" customHeight="true"/>
+    <row r="869" ht="14.25" customHeight="true"/>
+    <row r="870" ht="14.25" customHeight="true"/>
+    <row r="871" ht="14.25" customHeight="true"/>
+    <row r="872" ht="14.25" customHeight="true"/>
+    <row r="873" ht="14.25" customHeight="true"/>
+    <row r="874" ht="14.25" customHeight="true"/>
+    <row r="875" ht="14.25" customHeight="true"/>
+    <row r="876" ht="14.25" customHeight="true"/>
+    <row r="877" ht="14.25" customHeight="true"/>
+    <row r="878" ht="14.25" customHeight="true"/>
+    <row r="879" ht="14.25" customHeight="true"/>
+    <row r="880" ht="14.25" customHeight="true"/>
+    <row r="881" ht="14.25" customHeight="true"/>
+    <row r="882" ht="14.25" customHeight="true"/>
+    <row r="883" ht="14.25" customHeight="true"/>
+    <row r="884" ht="14.25" customHeight="true"/>
+    <row r="885" ht="14.25" customHeight="true"/>
+    <row r="886" ht="14.25" customHeight="true"/>
+    <row r="887" ht="14.25" customHeight="true"/>
+    <row r="888" ht="14.25" customHeight="true"/>
+    <row r="889" ht="14.25" customHeight="true"/>
+    <row r="890" ht="14.25" customHeight="true"/>
+    <row r="891" ht="14.25" customHeight="true"/>
+    <row r="892" ht="14.25" customHeight="true"/>
+    <row r="893" ht="14.25" customHeight="true"/>
+    <row r="894" ht="14.25" customHeight="true"/>
+    <row r="895" ht="14.25" customHeight="true"/>
+    <row r="896" ht="14.25" customHeight="true"/>
+    <row r="897" ht="14.25" customHeight="true"/>
+    <row r="898" ht="14.25" customHeight="true"/>
+    <row r="899" ht="14.25" customHeight="true"/>
+    <row r="900" ht="14.25" customHeight="true"/>
+    <row r="901" ht="14.25" customHeight="true"/>
+    <row r="902" ht="14.25" customHeight="true"/>
+    <row r="903" ht="14.25" customHeight="true"/>
+    <row r="904" ht="14.25" customHeight="true"/>
+    <row r="905" ht="14.25" customHeight="true"/>
+    <row r="906" ht="14.25" customHeight="true"/>
+    <row r="907" ht="14.25" customHeight="true"/>
+    <row r="908" ht="14.25" customHeight="true"/>
+    <row r="909" ht="14.25" customHeight="true"/>
+    <row r="910" ht="14.25" customHeight="true"/>
+    <row r="911" ht="14.25" customHeight="true"/>
+    <row r="912" ht="14.25" customHeight="true"/>
+    <row r="913" ht="14.25" customHeight="true"/>
+    <row r="914" ht="14.25" customHeight="true"/>
+    <row r="915" ht="14.25" customHeight="true"/>
+    <row r="916" ht="14.25" customHeight="true"/>
+    <row r="917" ht="14.25" customHeight="true"/>
+    <row r="918" ht="14.25" customHeight="true"/>
+    <row r="919" ht="14.25" customHeight="true"/>
+    <row r="920" ht="14.25" customHeight="true"/>
+    <row r="921" ht="14.25" customHeight="true"/>
+    <row r="922" ht="14.25" customHeight="true"/>
+    <row r="923" ht="14.25" customHeight="true"/>
+    <row r="924" ht="14.25" customHeight="true"/>
+    <row r="925" ht="14.25" customHeight="true"/>
+    <row r="926" ht="14.25" customHeight="true"/>
+    <row r="927" ht="14.25" customHeight="true"/>
+    <row r="928" ht="14.25" customHeight="true"/>
+    <row r="929" ht="14.25" customHeight="true"/>
+    <row r="930" ht="14.25" customHeight="true"/>
+    <row r="931" ht="14.25" customHeight="true"/>
+    <row r="932" ht="14.25" customHeight="true"/>
+    <row r="933" ht="14.25" customHeight="true"/>
+    <row r="934" ht="14.25" customHeight="true"/>
+    <row r="935" ht="14.25" customHeight="true"/>
+    <row r="936" ht="14.25" customHeight="true"/>
+    <row r="937" ht="14.25" customHeight="true"/>
+    <row r="938" ht="14.25" customHeight="true"/>
+    <row r="939" ht="14.25" customHeight="true"/>
+    <row r="940" ht="14.25" customHeight="true"/>
+    <row r="941" ht="14.25" customHeight="true"/>
+    <row r="942" ht="14.25" customHeight="true"/>
+    <row r="943" ht="14.25" customHeight="true"/>
+    <row r="944" ht="14.25" customHeight="true"/>
+    <row r="945" ht="14.25" customHeight="true"/>
+    <row r="946" ht="14.25" customHeight="true"/>
+    <row r="947" ht="14.25" customHeight="true"/>
+    <row r="948" ht="14.25" customHeight="true"/>
+    <row r="949" ht="14.25" customHeight="true"/>
+    <row r="950" ht="14.25" customHeight="true"/>
+    <row r="951" ht="14.25" customHeight="true"/>
+    <row r="952" ht="14.25" customHeight="true"/>
+    <row r="953" ht="14.25" customHeight="true"/>
+    <row r="954" ht="14.25" customHeight="true"/>
+    <row r="955" ht="14.25" customHeight="true"/>
+    <row r="956" ht="14.25" customHeight="true"/>
+    <row r="957" ht="14.25" customHeight="true"/>
+    <row r="958" ht="14.25" customHeight="true"/>
+    <row r="959" ht="14.25" customHeight="true"/>
+    <row r="960" ht="14.25" customHeight="true"/>
+    <row r="961" ht="14.25" customHeight="true"/>
+    <row r="962" ht="14.25" customHeight="true"/>
+    <row r="963" ht="14.25" customHeight="true"/>
+    <row r="964" ht="14.25" customHeight="true"/>
+    <row r="965" ht="14.25" customHeight="true"/>
+    <row r="966" ht="14.25" customHeight="true"/>
+    <row r="967" ht="14.25" customHeight="true"/>
+    <row r="968" ht="14.25" customHeight="true"/>
+    <row r="969" ht="14.25" customHeight="true"/>
+    <row r="970" ht="14.25" customHeight="true"/>
+    <row r="971" ht="14.25" customHeight="true"/>
+    <row r="972" ht="14.25" customHeight="true"/>
+    <row r="973" ht="14.25" customHeight="true"/>
+    <row r="974" ht="14.25" customHeight="true"/>
+    <row r="975" ht="14.25" customHeight="true"/>
+    <row r="976" ht="14.25" customHeight="true"/>
+    <row r="977" ht="14.25" customHeight="true"/>
+    <row r="978" ht="14.25" customHeight="true"/>
+    <row r="979" ht="14.25" customHeight="true"/>
+    <row r="980" ht="14.25" customHeight="true"/>
+    <row r="981" ht="14.25" customHeight="true"/>
+    <row r="982" ht="14.25" customHeight="true"/>
+    <row r="983" ht="14.25" customHeight="true"/>
+    <row r="984" ht="14.25" customHeight="true"/>
+    <row r="985" ht="14.25" customHeight="true"/>
+    <row r="986" ht="14.25" customHeight="true"/>
+    <row r="987" ht="14.25" customHeight="true"/>
+    <row r="988" ht="14.25" customHeight="true"/>
+    <row r="989" ht="14.25" customHeight="true"/>
+    <row r="990" ht="14.25" customHeight="true"/>
+    <row r="991" ht="14.25" customHeight="true"/>
+    <row r="992" ht="14.25" customHeight="true"/>
+    <row r="993" ht="14.25" customHeight="true"/>
+    <row r="994" ht="14.25" customHeight="true"/>
+    <row r="995" ht="14.25" customHeight="true"/>
+    <row r="996" ht="14.25" customHeight="true"/>
+    <row r="997" ht="14.25" customHeight="true"/>
+    <row r="998" ht="14.25" customHeight="true"/>
+    <row r="999" ht="14.25" customHeight="true"/>
+    <row r="1000" ht="14.25" customHeight="true"/>
   </sheetData>
   <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add yearly exported registrations functionality with Excel export
</commit_message>
<xml_diff>
--- a/db/seeds/excel/seeds.xlsx
+++ b/db/seeds/excel/seeds.xlsx
@@ -5158,22 +5158,22 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="true"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="30.29"/>
-    <col customWidth="1" min="2" max="2" width="15.71"/>
-    <col customWidth="1" min="3" max="3" width="25.14"/>
-    <col customWidth="1" min="4" max="4" width="8.71"/>
-    <col customWidth="1" min="5" max="5" width="10.0"/>
-    <col customWidth="1" min="6" max="6" width="24.43"/>
-    <col customWidth="1" min="7" max="7" width="23.86"/>
-    <col customWidth="1" min="8" max="8" width="18.0"/>
-    <col customWidth="1" min="9" max="9" width="20.86"/>
-    <col customWidth="1" min="10" max="10" width="21.0"/>
-    <col customWidth="1" min="11" max="26" width="8.71"/>
+    <col customWidth="true" max="1" min="1" width="30.29"/>
+    <col customWidth="true" max="2" min="2" width="15.71"/>
+    <col customWidth="true" max="3" min="3" width="25.14"/>
+    <col customWidth="true" max="4" min="4" width="8.71"/>
+    <col customWidth="true" max="5" min="5" width="10"/>
+    <col customWidth="true" max="6" min="6" width="24.43"/>
+    <col customWidth="true" max="7" min="7" width="23.86"/>
+    <col customWidth="true" max="8" min="8" width="18"/>
+    <col customWidth="true" max="9" min="9" width="20.86"/>
+    <col customWidth="true" max="10" min="10" width="21"/>
+    <col customWidth="true" max="26" min="11" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
+    <row r="1" ht="14.25" customHeight="true">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5205,7 +5205,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1">
+    <row r="2" ht="14.25" customHeight="true">
       <c r="A2" s="2" t="s">
         <v>114</v>
       </c>
@@ -5237,7 +5237,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1">
+    <row r="3" ht="14.25" customHeight="true">
       <c r="A3" s="2" t="s">
         <v>118</v>
       </c>
@@ -5269,7 +5269,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1">
+    <row r="4" ht="14.25" customHeight="true">
       <c r="A4" s="2" t="s">
         <v>121</v>
       </c>
@@ -5301,7 +5301,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="5" ht="14.25" customHeight="1">
+    <row r="5" ht="14.25" customHeight="true">
       <c r="A5" s="2" t="s">
         <v>124</v>
       </c>
@@ -5333,7 +5333,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="6" ht="14.25" customHeight="1">
+    <row r="6" ht="14.25" customHeight="true">
       <c r="A6" s="2" t="s">
         <v>128</v>
       </c>
@@ -5365,7 +5365,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="7" ht="14.25" customHeight="1">
+    <row r="7" ht="14.25" customHeight="true">
       <c r="A7" s="2" t="s">
         <v>131</v>
       </c>
@@ -5397,7 +5397,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="8" ht="14.25" customHeight="1">
+    <row r="8" ht="14.25" customHeight="true">
       <c r="A8" s="2" t="s">
         <v>135</v>
       </c>
@@ -5429,7 +5429,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="9" ht="14.25" customHeight="1">
+    <row r="9" ht="14.25" customHeight="true">
       <c r="A9" s="2" t="s">
         <v>138</v>
       </c>
@@ -5461,7 +5461,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="10" ht="14.25" customHeight="1">
+    <row r="10" ht="14.25" customHeight="true">
       <c r="A10" s="2" t="s">
         <v>141</v>
       </c>
@@ -5493,7 +5493,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="11" ht="14.25" customHeight="1">
+    <row r="11" ht="14.25" customHeight="true">
       <c r="A11" s="2" t="s">
         <v>144</v>
       </c>
@@ -5525,7 +5525,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="12" ht="14.25" customHeight="1">
+    <row r="12" ht="14.25" customHeight="true">
       <c r="A12" s="2" t="s">
         <v>148</v>
       </c>
@@ -5557,7 +5557,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="13" ht="14.25" customHeight="1">
+    <row r="13" ht="14.25" customHeight="true">
       <c r="A13" s="2" t="s">
         <v>151</v>
       </c>
@@ -5589,7 +5589,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="14" ht="14.25" customHeight="1">
+    <row r="14" ht="14.25" customHeight="true">
       <c r="A14" s="2" t="s">
         <v>154</v>
       </c>
@@ -5621,7 +5621,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="15" ht="14.25" customHeight="1">
+    <row r="15" ht="14.25" customHeight="true">
       <c r="A15" s="2" t="s">
         <v>157</v>
       </c>
@@ -5653,7 +5653,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="16" ht="14.25" customHeight="1">
+    <row r="16" ht="14.25" customHeight="true">
       <c r="A16" s="2" t="s">
         <v>161</v>
       </c>
@@ -5685,993 +5685,993 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
-    <row r="65" ht="14.25" customHeight="1"/>
-    <row r="66" ht="14.25" customHeight="1"/>
-    <row r="67" ht="14.25" customHeight="1"/>
-    <row r="68" ht="14.25" customHeight="1"/>
-    <row r="69" ht="14.25" customHeight="1"/>
-    <row r="70" ht="14.25" customHeight="1"/>
-    <row r="71" ht="14.25" customHeight="1"/>
-    <row r="72" ht="14.25" customHeight="1"/>
-    <row r="73" ht="14.25" customHeight="1"/>
-    <row r="74" ht="14.25" customHeight="1"/>
-    <row r="75" ht="14.25" customHeight="1"/>
-    <row r="76" ht="14.25" customHeight="1"/>
-    <row r="77" ht="14.25" customHeight="1"/>
-    <row r="78" ht="14.25" customHeight="1"/>
-    <row r="79" ht="14.25" customHeight="1"/>
-    <row r="80" ht="14.25" customHeight="1"/>
-    <row r="81" ht="14.25" customHeight="1"/>
-    <row r="82" ht="14.25" customHeight="1"/>
-    <row r="83" ht="14.25" customHeight="1"/>
-    <row r="84" ht="14.25" customHeight="1"/>
-    <row r="85" ht="14.25" customHeight="1"/>
-    <row r="86" ht="14.25" customHeight="1"/>
-    <row r="87" ht="14.25" customHeight="1"/>
-    <row r="88" ht="14.25" customHeight="1"/>
-    <row r="89" ht="14.25" customHeight="1"/>
-    <row r="90" ht="14.25" customHeight="1"/>
-    <row r="91" ht="14.25" customHeight="1"/>
-    <row r="92" ht="14.25" customHeight="1"/>
-    <row r="93" ht="14.25" customHeight="1"/>
-    <row r="94" ht="14.25" customHeight="1"/>
-    <row r="95" ht="14.25" customHeight="1"/>
-    <row r="96" ht="14.25" customHeight="1"/>
-    <row r="97" ht="14.25" customHeight="1"/>
-    <row r="98" ht="14.25" customHeight="1"/>
-    <row r="99" ht="14.25" customHeight="1"/>
-    <row r="100" ht="14.25" customHeight="1"/>
-    <row r="101" ht="14.25" customHeight="1"/>
-    <row r="102" ht="14.25" customHeight="1"/>
-    <row r="103" ht="14.25" customHeight="1"/>
-    <row r="104" ht="14.25" customHeight="1"/>
-    <row r="105" ht="14.25" customHeight="1"/>
-    <row r="106" ht="14.25" customHeight="1"/>
-    <row r="107" ht="14.25" customHeight="1"/>
-    <row r="108" ht="14.25" customHeight="1"/>
-    <row r="109" ht="14.25" customHeight="1"/>
-    <row r="110" ht="14.25" customHeight="1"/>
-    <row r="111" ht="14.25" customHeight="1"/>
-    <row r="112" ht="14.25" customHeight="1"/>
-    <row r="113" ht="14.25" customHeight="1"/>
-    <row r="114" ht="14.25" customHeight="1"/>
-    <row r="115" ht="14.25" customHeight="1"/>
-    <row r="116" ht="14.25" customHeight="1"/>
-    <row r="117" ht="14.25" customHeight="1"/>
-    <row r="118" ht="14.25" customHeight="1"/>
-    <row r="119" ht="14.25" customHeight="1"/>
-    <row r="120" ht="14.25" customHeight="1"/>
-    <row r="121" ht="14.25" customHeight="1"/>
-    <row r="122" ht="14.25" customHeight="1"/>
-    <row r="123" ht="14.25" customHeight="1"/>
-    <row r="124" ht="14.25" customHeight="1"/>
-    <row r="125" ht="14.25" customHeight="1"/>
-    <row r="126" ht="14.25" customHeight="1"/>
-    <row r="127" ht="14.25" customHeight="1"/>
-    <row r="128" ht="14.25" customHeight="1"/>
-    <row r="129" ht="14.25" customHeight="1"/>
-    <row r="130" ht="14.25" customHeight="1"/>
-    <row r="131" ht="14.25" customHeight="1"/>
-    <row r="132" ht="14.25" customHeight="1"/>
-    <row r="133" ht="14.25" customHeight="1"/>
-    <row r="134" ht="14.25" customHeight="1"/>
-    <row r="135" ht="14.25" customHeight="1"/>
-    <row r="136" ht="14.25" customHeight="1"/>
-    <row r="137" ht="14.25" customHeight="1"/>
-    <row r="138" ht="14.25" customHeight="1"/>
-    <row r="139" ht="14.25" customHeight="1"/>
-    <row r="140" ht="14.25" customHeight="1"/>
-    <row r="141" ht="14.25" customHeight="1"/>
-    <row r="142" ht="14.25" customHeight="1"/>
-    <row r="143" ht="14.25" customHeight="1"/>
-    <row r="144" ht="14.25" customHeight="1"/>
-    <row r="145" ht="14.25" customHeight="1"/>
-    <row r="146" ht="14.25" customHeight="1"/>
-    <row r="147" ht="14.25" customHeight="1"/>
-    <row r="148" ht="14.25" customHeight="1"/>
-    <row r="149" ht="14.25" customHeight="1"/>
-    <row r="150" ht="14.25" customHeight="1"/>
-    <row r="151" ht="14.25" customHeight="1"/>
-    <row r="152" ht="14.25" customHeight="1"/>
-    <row r="153" ht="14.25" customHeight="1"/>
-    <row r="154" ht="14.25" customHeight="1"/>
-    <row r="155" ht="14.25" customHeight="1"/>
-    <row r="156" ht="14.25" customHeight="1"/>
-    <row r="157" ht="14.25" customHeight="1"/>
-    <row r="158" ht="14.25" customHeight="1"/>
-    <row r="159" ht="14.25" customHeight="1"/>
-    <row r="160" ht="14.25" customHeight="1"/>
-    <row r="161" ht="14.25" customHeight="1"/>
-    <row r="162" ht="14.25" customHeight="1"/>
-    <row r="163" ht="14.25" customHeight="1"/>
-    <row r="164" ht="14.25" customHeight="1"/>
-    <row r="165" ht="14.25" customHeight="1"/>
-    <row r="166" ht="14.25" customHeight="1"/>
-    <row r="167" ht="14.25" customHeight="1"/>
-    <row r="168" ht="14.25" customHeight="1"/>
-    <row r="169" ht="14.25" customHeight="1"/>
-    <row r="170" ht="14.25" customHeight="1"/>
-    <row r="171" ht="14.25" customHeight="1"/>
-    <row r="172" ht="14.25" customHeight="1"/>
-    <row r="173" ht="14.25" customHeight="1"/>
-    <row r="174" ht="14.25" customHeight="1"/>
-    <row r="175" ht="14.25" customHeight="1"/>
-    <row r="176" ht="14.25" customHeight="1"/>
-    <row r="177" ht="14.25" customHeight="1"/>
-    <row r="178" ht="14.25" customHeight="1"/>
-    <row r="179" ht="14.25" customHeight="1"/>
-    <row r="180" ht="14.25" customHeight="1"/>
-    <row r="181" ht="14.25" customHeight="1"/>
-    <row r="182" ht="14.25" customHeight="1"/>
-    <row r="183" ht="14.25" customHeight="1"/>
-    <row r="184" ht="14.25" customHeight="1"/>
-    <row r="185" ht="14.25" customHeight="1"/>
-    <row r="186" ht="14.25" customHeight="1"/>
-    <row r="187" ht="14.25" customHeight="1"/>
-    <row r="188" ht="14.25" customHeight="1"/>
-    <row r="189" ht="14.25" customHeight="1"/>
-    <row r="190" ht="14.25" customHeight="1"/>
-    <row r="191" ht="14.25" customHeight="1"/>
-    <row r="192" ht="14.25" customHeight="1"/>
-    <row r="193" ht="14.25" customHeight="1"/>
-    <row r="194" ht="14.25" customHeight="1"/>
-    <row r="195" ht="14.25" customHeight="1"/>
-    <row r="196" ht="14.25" customHeight="1"/>
-    <row r="197" ht="14.25" customHeight="1"/>
-    <row r="198" ht="14.25" customHeight="1"/>
-    <row r="199" ht="14.25" customHeight="1"/>
-    <row r="200" ht="14.25" customHeight="1"/>
-    <row r="201" ht="14.25" customHeight="1"/>
-    <row r="202" ht="14.25" customHeight="1"/>
-    <row r="203" ht="14.25" customHeight="1"/>
-    <row r="204" ht="14.25" customHeight="1"/>
-    <row r="205" ht="14.25" customHeight="1"/>
-    <row r="206" ht="14.25" customHeight="1"/>
-    <row r="207" ht="14.25" customHeight="1"/>
-    <row r="208" ht="14.25" customHeight="1"/>
-    <row r="209" ht="14.25" customHeight="1"/>
-    <row r="210" ht="14.25" customHeight="1"/>
-    <row r="211" ht="14.25" customHeight="1"/>
-    <row r="212" ht="14.25" customHeight="1"/>
-    <row r="213" ht="14.25" customHeight="1"/>
-    <row r="214" ht="14.25" customHeight="1"/>
-    <row r="215" ht="14.25" customHeight="1"/>
-    <row r="216" ht="14.25" customHeight="1"/>
-    <row r="217" ht="14.25" customHeight="1"/>
-    <row r="218" ht="14.25" customHeight="1"/>
-    <row r="219" ht="14.25" customHeight="1"/>
-    <row r="220" ht="14.25" customHeight="1"/>
-    <row r="221" ht="14.25" customHeight="1"/>
-    <row r="222" ht="14.25" customHeight="1"/>
-    <row r="223" ht="14.25" customHeight="1"/>
-    <row r="224" ht="14.25" customHeight="1"/>
-    <row r="225" ht="14.25" customHeight="1"/>
-    <row r="226" ht="14.25" customHeight="1"/>
-    <row r="227" ht="14.25" customHeight="1"/>
-    <row r="228" ht="14.25" customHeight="1"/>
-    <row r="229" ht="14.25" customHeight="1"/>
-    <row r="230" ht="14.25" customHeight="1"/>
-    <row r="231" ht="14.25" customHeight="1"/>
-    <row r="232" ht="14.25" customHeight="1"/>
-    <row r="233" ht="14.25" customHeight="1"/>
-    <row r="234" ht="14.25" customHeight="1"/>
-    <row r="235" ht="14.25" customHeight="1"/>
-    <row r="236" ht="14.25" customHeight="1"/>
-    <row r="237" ht="14.25" customHeight="1"/>
-    <row r="238" ht="14.25" customHeight="1"/>
-    <row r="239" ht="14.25" customHeight="1"/>
-    <row r="240" ht="14.25" customHeight="1"/>
-    <row r="241" ht="14.25" customHeight="1"/>
-    <row r="242" ht="14.25" customHeight="1"/>
-    <row r="243" ht="14.25" customHeight="1"/>
-    <row r="244" ht="14.25" customHeight="1"/>
-    <row r="245" ht="14.25" customHeight="1"/>
-    <row r="246" ht="14.25" customHeight="1"/>
-    <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
-    <row r="249" ht="14.25" customHeight="1"/>
-    <row r="250" ht="14.25" customHeight="1"/>
-    <row r="251" ht="14.25" customHeight="1"/>
-    <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1"/>
-    <row r="254" ht="14.25" customHeight="1"/>
-    <row r="255" ht="14.25" customHeight="1"/>
-    <row r="256" ht="14.25" customHeight="1"/>
-    <row r="257" ht="14.25" customHeight="1"/>
-    <row r="258" ht="14.25" customHeight="1"/>
-    <row r="259" ht="14.25" customHeight="1"/>
-    <row r="260" ht="14.25" customHeight="1"/>
-    <row r="261" ht="14.25" customHeight="1"/>
-    <row r="262" ht="14.25" customHeight="1"/>
-    <row r="263" ht="14.25" customHeight="1"/>
-    <row r="264" ht="14.25" customHeight="1"/>
-    <row r="265" ht="14.25" customHeight="1"/>
-    <row r="266" ht="14.25" customHeight="1"/>
-    <row r="267" ht="14.25" customHeight="1"/>
-    <row r="268" ht="14.25" customHeight="1"/>
-    <row r="269" ht="14.25" customHeight="1"/>
-    <row r="270" ht="14.25" customHeight="1"/>
-    <row r="271" ht="14.25" customHeight="1"/>
-    <row r="272" ht="14.25" customHeight="1"/>
-    <row r="273" ht="14.25" customHeight="1"/>
-    <row r="274" ht="14.25" customHeight="1"/>
-    <row r="275" ht="14.25" customHeight="1"/>
-    <row r="276" ht="14.25" customHeight="1"/>
-    <row r="277" ht="14.25" customHeight="1"/>
-    <row r="278" ht="14.25" customHeight="1"/>
-    <row r="279" ht="14.25" customHeight="1"/>
-    <row r="280" ht="14.25" customHeight="1"/>
-    <row r="281" ht="14.25" customHeight="1"/>
-    <row r="282" ht="14.25" customHeight="1"/>
-    <row r="283" ht="14.25" customHeight="1"/>
-    <row r="284" ht="14.25" customHeight="1"/>
-    <row r="285" ht="14.25" customHeight="1"/>
-    <row r="286" ht="14.25" customHeight="1"/>
-    <row r="287" ht="14.25" customHeight="1"/>
-    <row r="288" ht="14.25" customHeight="1"/>
-    <row r="289" ht="14.25" customHeight="1"/>
-    <row r="290" ht="14.25" customHeight="1"/>
-    <row r="291" ht="14.25" customHeight="1"/>
-    <row r="292" ht="14.25" customHeight="1"/>
-    <row r="293" ht="14.25" customHeight="1"/>
-    <row r="294" ht="14.25" customHeight="1"/>
-    <row r="295" ht="14.25" customHeight="1"/>
-    <row r="296" ht="14.25" customHeight="1"/>
-    <row r="297" ht="14.25" customHeight="1"/>
-    <row r="298" ht="14.25" customHeight="1"/>
-    <row r="299" ht="14.25" customHeight="1"/>
-    <row r="300" ht="14.25" customHeight="1"/>
-    <row r="301" ht="14.25" customHeight="1"/>
-    <row r="302" ht="14.25" customHeight="1"/>
-    <row r="303" ht="14.25" customHeight="1"/>
-    <row r="304" ht="14.25" customHeight="1"/>
-    <row r="305" ht="14.25" customHeight="1"/>
-    <row r="306" ht="14.25" customHeight="1"/>
-    <row r="307" ht="14.25" customHeight="1"/>
-    <row r="308" ht="14.25" customHeight="1"/>
-    <row r="309" ht="14.25" customHeight="1"/>
-    <row r="310" ht="14.25" customHeight="1"/>
-    <row r="311" ht="14.25" customHeight="1"/>
-    <row r="312" ht="14.25" customHeight="1"/>
-    <row r="313" ht="14.25" customHeight="1"/>
-    <row r="314" ht="14.25" customHeight="1"/>
-    <row r="315" ht="14.25" customHeight="1"/>
-    <row r="316" ht="14.25" customHeight="1"/>
-    <row r="317" ht="14.25" customHeight="1"/>
-    <row r="318" ht="14.25" customHeight="1"/>
-    <row r="319" ht="14.25" customHeight="1"/>
-    <row r="320" ht="14.25" customHeight="1"/>
-    <row r="321" ht="14.25" customHeight="1"/>
-    <row r="322" ht="14.25" customHeight="1"/>
-    <row r="323" ht="14.25" customHeight="1"/>
-    <row r="324" ht="14.25" customHeight="1"/>
-    <row r="325" ht="14.25" customHeight="1"/>
-    <row r="326" ht="14.25" customHeight="1"/>
-    <row r="327" ht="14.25" customHeight="1"/>
-    <row r="328" ht="14.25" customHeight="1"/>
-    <row r="329" ht="14.25" customHeight="1"/>
-    <row r="330" ht="14.25" customHeight="1"/>
-    <row r="331" ht="14.25" customHeight="1"/>
-    <row r="332" ht="14.25" customHeight="1"/>
-    <row r="333" ht="14.25" customHeight="1"/>
-    <row r="334" ht="14.25" customHeight="1"/>
-    <row r="335" ht="14.25" customHeight="1"/>
-    <row r="336" ht="14.25" customHeight="1"/>
-    <row r="337" ht="14.25" customHeight="1"/>
-    <row r="338" ht="14.25" customHeight="1"/>
-    <row r="339" ht="14.25" customHeight="1"/>
-    <row r="340" ht="14.25" customHeight="1"/>
-    <row r="341" ht="14.25" customHeight="1"/>
-    <row r="342" ht="14.25" customHeight="1"/>
-    <row r="343" ht="14.25" customHeight="1"/>
-    <row r="344" ht="14.25" customHeight="1"/>
-    <row r="345" ht="14.25" customHeight="1"/>
-    <row r="346" ht="14.25" customHeight="1"/>
-    <row r="347" ht="14.25" customHeight="1"/>
-    <row r="348" ht="14.25" customHeight="1"/>
-    <row r="349" ht="14.25" customHeight="1"/>
-    <row r="350" ht="14.25" customHeight="1"/>
-    <row r="351" ht="14.25" customHeight="1"/>
-    <row r="352" ht="14.25" customHeight="1"/>
-    <row r="353" ht="14.25" customHeight="1"/>
-    <row r="354" ht="14.25" customHeight="1"/>
-    <row r="355" ht="14.25" customHeight="1"/>
-    <row r="356" ht="14.25" customHeight="1"/>
-    <row r="357" ht="14.25" customHeight="1"/>
-    <row r="358" ht="14.25" customHeight="1"/>
-    <row r="359" ht="14.25" customHeight="1"/>
-    <row r="360" ht="14.25" customHeight="1"/>
-    <row r="361" ht="14.25" customHeight="1"/>
-    <row r="362" ht="14.25" customHeight="1"/>
-    <row r="363" ht="14.25" customHeight="1"/>
-    <row r="364" ht="14.25" customHeight="1"/>
-    <row r="365" ht="14.25" customHeight="1"/>
-    <row r="366" ht="14.25" customHeight="1"/>
-    <row r="367" ht="14.25" customHeight="1"/>
-    <row r="368" ht="14.25" customHeight="1"/>
-    <row r="369" ht="14.25" customHeight="1"/>
-    <row r="370" ht="14.25" customHeight="1"/>
-    <row r="371" ht="14.25" customHeight="1"/>
-    <row r="372" ht="14.25" customHeight="1"/>
-    <row r="373" ht="14.25" customHeight="1"/>
-    <row r="374" ht="14.25" customHeight="1"/>
-    <row r="375" ht="14.25" customHeight="1"/>
-    <row r="376" ht="14.25" customHeight="1"/>
-    <row r="377" ht="14.25" customHeight="1"/>
-    <row r="378" ht="14.25" customHeight="1"/>
-    <row r="379" ht="14.25" customHeight="1"/>
-    <row r="380" ht="14.25" customHeight="1"/>
-    <row r="381" ht="14.25" customHeight="1"/>
-    <row r="382" ht="14.25" customHeight="1"/>
-    <row r="383" ht="14.25" customHeight="1"/>
-    <row r="384" ht="14.25" customHeight="1"/>
-    <row r="385" ht="14.25" customHeight="1"/>
-    <row r="386" ht="14.25" customHeight="1"/>
-    <row r="387" ht="14.25" customHeight="1"/>
-    <row r="388" ht="14.25" customHeight="1"/>
-    <row r="389" ht="14.25" customHeight="1"/>
-    <row r="390" ht="14.25" customHeight="1"/>
-    <row r="391" ht="14.25" customHeight="1"/>
-    <row r="392" ht="14.25" customHeight="1"/>
-    <row r="393" ht="14.25" customHeight="1"/>
-    <row r="394" ht="14.25" customHeight="1"/>
-    <row r="395" ht="14.25" customHeight="1"/>
-    <row r="396" ht="14.25" customHeight="1"/>
-    <row r="397" ht="14.25" customHeight="1"/>
-    <row r="398" ht="14.25" customHeight="1"/>
-    <row r="399" ht="14.25" customHeight="1"/>
-    <row r="400" ht="14.25" customHeight="1"/>
-    <row r="401" ht="14.25" customHeight="1"/>
-    <row r="402" ht="14.25" customHeight="1"/>
-    <row r="403" ht="14.25" customHeight="1"/>
-    <row r="404" ht="14.25" customHeight="1"/>
-    <row r="405" ht="14.25" customHeight="1"/>
-    <row r="406" ht="14.25" customHeight="1"/>
-    <row r="407" ht="14.25" customHeight="1"/>
-    <row r="408" ht="14.25" customHeight="1"/>
-    <row r="409" ht="14.25" customHeight="1"/>
-    <row r="410" ht="14.25" customHeight="1"/>
-    <row r="411" ht="14.25" customHeight="1"/>
-    <row r="412" ht="14.25" customHeight="1"/>
-    <row r="413" ht="14.25" customHeight="1"/>
-    <row r="414" ht="14.25" customHeight="1"/>
-    <row r="415" ht="14.25" customHeight="1"/>
-    <row r="416" ht="14.25" customHeight="1"/>
-    <row r="417" ht="14.25" customHeight="1"/>
-    <row r="418" ht="14.25" customHeight="1"/>
-    <row r="419" ht="14.25" customHeight="1"/>
-    <row r="420" ht="14.25" customHeight="1"/>
-    <row r="421" ht="14.25" customHeight="1"/>
-    <row r="422" ht="14.25" customHeight="1"/>
-    <row r="423" ht="14.25" customHeight="1"/>
-    <row r="424" ht="14.25" customHeight="1"/>
-    <row r="425" ht="14.25" customHeight="1"/>
-    <row r="426" ht="14.25" customHeight="1"/>
-    <row r="427" ht="14.25" customHeight="1"/>
-    <row r="428" ht="14.25" customHeight="1"/>
-    <row r="429" ht="14.25" customHeight="1"/>
-    <row r="430" ht="14.25" customHeight="1"/>
-    <row r="431" ht="14.25" customHeight="1"/>
-    <row r="432" ht="14.25" customHeight="1"/>
-    <row r="433" ht="14.25" customHeight="1"/>
-    <row r="434" ht="14.25" customHeight="1"/>
-    <row r="435" ht="14.25" customHeight="1"/>
-    <row r="436" ht="14.25" customHeight="1"/>
-    <row r="437" ht="14.25" customHeight="1"/>
-    <row r="438" ht="14.25" customHeight="1"/>
-    <row r="439" ht="14.25" customHeight="1"/>
-    <row r="440" ht="14.25" customHeight="1"/>
-    <row r="441" ht="14.25" customHeight="1"/>
-    <row r="442" ht="14.25" customHeight="1"/>
-    <row r="443" ht="14.25" customHeight="1"/>
-    <row r="444" ht="14.25" customHeight="1"/>
-    <row r="445" ht="14.25" customHeight="1"/>
-    <row r="446" ht="14.25" customHeight="1"/>
-    <row r="447" ht="14.25" customHeight="1"/>
-    <row r="448" ht="14.25" customHeight="1"/>
-    <row r="449" ht="14.25" customHeight="1"/>
-    <row r="450" ht="14.25" customHeight="1"/>
-    <row r="451" ht="14.25" customHeight="1"/>
-    <row r="452" ht="14.25" customHeight="1"/>
-    <row r="453" ht="14.25" customHeight="1"/>
-    <row r="454" ht="14.25" customHeight="1"/>
-    <row r="455" ht="14.25" customHeight="1"/>
-    <row r="456" ht="14.25" customHeight="1"/>
-    <row r="457" ht="14.25" customHeight="1"/>
-    <row r="458" ht="14.25" customHeight="1"/>
-    <row r="459" ht="14.25" customHeight="1"/>
-    <row r="460" ht="14.25" customHeight="1"/>
-    <row r="461" ht="14.25" customHeight="1"/>
-    <row r="462" ht="14.25" customHeight="1"/>
-    <row r="463" ht="14.25" customHeight="1"/>
-    <row r="464" ht="14.25" customHeight="1"/>
-    <row r="465" ht="14.25" customHeight="1"/>
-    <row r="466" ht="14.25" customHeight="1"/>
-    <row r="467" ht="14.25" customHeight="1"/>
-    <row r="468" ht="14.25" customHeight="1"/>
-    <row r="469" ht="14.25" customHeight="1"/>
-    <row r="470" ht="14.25" customHeight="1"/>
-    <row r="471" ht="14.25" customHeight="1"/>
-    <row r="472" ht="14.25" customHeight="1"/>
-    <row r="473" ht="14.25" customHeight="1"/>
-    <row r="474" ht="14.25" customHeight="1"/>
-    <row r="475" ht="14.25" customHeight="1"/>
-    <row r="476" ht="14.25" customHeight="1"/>
-    <row r="477" ht="14.25" customHeight="1"/>
-    <row r="478" ht="14.25" customHeight="1"/>
-    <row r="479" ht="14.25" customHeight="1"/>
-    <row r="480" ht="14.25" customHeight="1"/>
-    <row r="481" ht="14.25" customHeight="1"/>
-    <row r="482" ht="14.25" customHeight="1"/>
-    <row r="483" ht="14.25" customHeight="1"/>
-    <row r="484" ht="14.25" customHeight="1"/>
-    <row r="485" ht="14.25" customHeight="1"/>
-    <row r="486" ht="14.25" customHeight="1"/>
-    <row r="487" ht="14.25" customHeight="1"/>
-    <row r="488" ht="14.25" customHeight="1"/>
-    <row r="489" ht="14.25" customHeight="1"/>
-    <row r="490" ht="14.25" customHeight="1"/>
-    <row r="491" ht="14.25" customHeight="1"/>
-    <row r="492" ht="14.25" customHeight="1"/>
-    <row r="493" ht="14.25" customHeight="1"/>
-    <row r="494" ht="14.25" customHeight="1"/>
-    <row r="495" ht="14.25" customHeight="1"/>
-    <row r="496" ht="14.25" customHeight="1"/>
-    <row r="497" ht="14.25" customHeight="1"/>
-    <row r="498" ht="14.25" customHeight="1"/>
-    <row r="499" ht="14.25" customHeight="1"/>
-    <row r="500" ht="14.25" customHeight="1"/>
-    <row r="501" ht="14.25" customHeight="1"/>
-    <row r="502" ht="14.25" customHeight="1"/>
-    <row r="503" ht="14.25" customHeight="1"/>
-    <row r="504" ht="14.25" customHeight="1"/>
-    <row r="505" ht="14.25" customHeight="1"/>
-    <row r="506" ht="14.25" customHeight="1"/>
-    <row r="507" ht="14.25" customHeight="1"/>
-    <row r="508" ht="14.25" customHeight="1"/>
-    <row r="509" ht="14.25" customHeight="1"/>
-    <row r="510" ht="14.25" customHeight="1"/>
-    <row r="511" ht="14.25" customHeight="1"/>
-    <row r="512" ht="14.25" customHeight="1"/>
-    <row r="513" ht="14.25" customHeight="1"/>
-    <row r="514" ht="14.25" customHeight="1"/>
-    <row r="515" ht="14.25" customHeight="1"/>
-    <row r="516" ht="14.25" customHeight="1"/>
-    <row r="517" ht="14.25" customHeight="1"/>
-    <row r="518" ht="14.25" customHeight="1"/>
-    <row r="519" ht="14.25" customHeight="1"/>
-    <row r="520" ht="14.25" customHeight="1"/>
-    <row r="521" ht="14.25" customHeight="1"/>
-    <row r="522" ht="14.25" customHeight="1"/>
-    <row r="523" ht="14.25" customHeight="1"/>
-    <row r="524" ht="14.25" customHeight="1"/>
-    <row r="525" ht="14.25" customHeight="1"/>
-    <row r="526" ht="14.25" customHeight="1"/>
-    <row r="527" ht="14.25" customHeight="1"/>
-    <row r="528" ht="14.25" customHeight="1"/>
-    <row r="529" ht="14.25" customHeight="1"/>
-    <row r="530" ht="14.25" customHeight="1"/>
-    <row r="531" ht="14.25" customHeight="1"/>
-    <row r="532" ht="14.25" customHeight="1"/>
-    <row r="533" ht="14.25" customHeight="1"/>
-    <row r="534" ht="14.25" customHeight="1"/>
-    <row r="535" ht="14.25" customHeight="1"/>
-    <row r="536" ht="14.25" customHeight="1"/>
-    <row r="537" ht="14.25" customHeight="1"/>
-    <row r="538" ht="14.25" customHeight="1"/>
-    <row r="539" ht="14.25" customHeight="1"/>
-    <row r="540" ht="14.25" customHeight="1"/>
-    <row r="541" ht="14.25" customHeight="1"/>
-    <row r="542" ht="14.25" customHeight="1"/>
-    <row r="543" ht="14.25" customHeight="1"/>
-    <row r="544" ht="14.25" customHeight="1"/>
-    <row r="545" ht="14.25" customHeight="1"/>
-    <row r="546" ht="14.25" customHeight="1"/>
-    <row r="547" ht="14.25" customHeight="1"/>
-    <row r="548" ht="14.25" customHeight="1"/>
-    <row r="549" ht="14.25" customHeight="1"/>
-    <row r="550" ht="14.25" customHeight="1"/>
-    <row r="551" ht="14.25" customHeight="1"/>
-    <row r="552" ht="14.25" customHeight="1"/>
-    <row r="553" ht="14.25" customHeight="1"/>
-    <row r="554" ht="14.25" customHeight="1"/>
-    <row r="555" ht="14.25" customHeight="1"/>
-    <row r="556" ht="14.25" customHeight="1"/>
-    <row r="557" ht="14.25" customHeight="1"/>
-    <row r="558" ht="14.25" customHeight="1"/>
-    <row r="559" ht="14.25" customHeight="1"/>
-    <row r="560" ht="14.25" customHeight="1"/>
-    <row r="561" ht="14.25" customHeight="1"/>
-    <row r="562" ht="14.25" customHeight="1"/>
-    <row r="563" ht="14.25" customHeight="1"/>
-    <row r="564" ht="14.25" customHeight="1"/>
-    <row r="565" ht="14.25" customHeight="1"/>
-    <row r="566" ht="14.25" customHeight="1"/>
-    <row r="567" ht="14.25" customHeight="1"/>
-    <row r="568" ht="14.25" customHeight="1"/>
-    <row r="569" ht="14.25" customHeight="1"/>
-    <row r="570" ht="14.25" customHeight="1"/>
-    <row r="571" ht="14.25" customHeight="1"/>
-    <row r="572" ht="14.25" customHeight="1"/>
-    <row r="573" ht="14.25" customHeight="1"/>
-    <row r="574" ht="14.25" customHeight="1"/>
-    <row r="575" ht="14.25" customHeight="1"/>
-    <row r="576" ht="14.25" customHeight="1"/>
-    <row r="577" ht="14.25" customHeight="1"/>
-    <row r="578" ht="14.25" customHeight="1"/>
-    <row r="579" ht="14.25" customHeight="1"/>
-    <row r="580" ht="14.25" customHeight="1"/>
-    <row r="581" ht="14.25" customHeight="1"/>
-    <row r="582" ht="14.25" customHeight="1"/>
-    <row r="583" ht="14.25" customHeight="1"/>
-    <row r="584" ht="14.25" customHeight="1"/>
-    <row r="585" ht="14.25" customHeight="1"/>
-    <row r="586" ht="14.25" customHeight="1"/>
-    <row r="587" ht="14.25" customHeight="1"/>
-    <row r="588" ht="14.25" customHeight="1"/>
-    <row r="589" ht="14.25" customHeight="1"/>
-    <row r="590" ht="14.25" customHeight="1"/>
-    <row r="591" ht="14.25" customHeight="1"/>
-    <row r="592" ht="14.25" customHeight="1"/>
-    <row r="593" ht="14.25" customHeight="1"/>
-    <row r="594" ht="14.25" customHeight="1"/>
-    <row r="595" ht="14.25" customHeight="1"/>
-    <row r="596" ht="14.25" customHeight="1"/>
-    <row r="597" ht="14.25" customHeight="1"/>
-    <row r="598" ht="14.25" customHeight="1"/>
-    <row r="599" ht="14.25" customHeight="1"/>
-    <row r="600" ht="14.25" customHeight="1"/>
-    <row r="601" ht="14.25" customHeight="1"/>
-    <row r="602" ht="14.25" customHeight="1"/>
-    <row r="603" ht="14.25" customHeight="1"/>
-    <row r="604" ht="14.25" customHeight="1"/>
-    <row r="605" ht="14.25" customHeight="1"/>
-    <row r="606" ht="14.25" customHeight="1"/>
-    <row r="607" ht="14.25" customHeight="1"/>
-    <row r="608" ht="14.25" customHeight="1"/>
-    <row r="609" ht="14.25" customHeight="1"/>
-    <row r="610" ht="14.25" customHeight="1"/>
-    <row r="611" ht="14.25" customHeight="1"/>
-    <row r="612" ht="14.25" customHeight="1"/>
-    <row r="613" ht="14.25" customHeight="1"/>
-    <row r="614" ht="14.25" customHeight="1"/>
-    <row r="615" ht="14.25" customHeight="1"/>
-    <row r="616" ht="14.25" customHeight="1"/>
-    <row r="617" ht="14.25" customHeight="1"/>
-    <row r="618" ht="14.25" customHeight="1"/>
-    <row r="619" ht="14.25" customHeight="1"/>
-    <row r="620" ht="14.25" customHeight="1"/>
-    <row r="621" ht="14.25" customHeight="1"/>
-    <row r="622" ht="14.25" customHeight="1"/>
-    <row r="623" ht="14.25" customHeight="1"/>
-    <row r="624" ht="14.25" customHeight="1"/>
-    <row r="625" ht="14.25" customHeight="1"/>
-    <row r="626" ht="14.25" customHeight="1"/>
-    <row r="627" ht="14.25" customHeight="1"/>
-    <row r="628" ht="14.25" customHeight="1"/>
-    <row r="629" ht="14.25" customHeight="1"/>
-    <row r="630" ht="14.25" customHeight="1"/>
-    <row r="631" ht="14.25" customHeight="1"/>
-    <row r="632" ht="14.25" customHeight="1"/>
-    <row r="633" ht="14.25" customHeight="1"/>
-    <row r="634" ht="14.25" customHeight="1"/>
-    <row r="635" ht="14.25" customHeight="1"/>
-    <row r="636" ht="14.25" customHeight="1"/>
-    <row r="637" ht="14.25" customHeight="1"/>
-    <row r="638" ht="14.25" customHeight="1"/>
-    <row r="639" ht="14.25" customHeight="1"/>
-    <row r="640" ht="14.25" customHeight="1"/>
-    <row r="641" ht="14.25" customHeight="1"/>
-    <row r="642" ht="14.25" customHeight="1"/>
-    <row r="643" ht="14.25" customHeight="1"/>
-    <row r="644" ht="14.25" customHeight="1"/>
-    <row r="645" ht="14.25" customHeight="1"/>
-    <row r="646" ht="14.25" customHeight="1"/>
-    <row r="647" ht="14.25" customHeight="1"/>
-    <row r="648" ht="14.25" customHeight="1"/>
-    <row r="649" ht="14.25" customHeight="1"/>
-    <row r="650" ht="14.25" customHeight="1"/>
-    <row r="651" ht="14.25" customHeight="1"/>
-    <row r="652" ht="14.25" customHeight="1"/>
-    <row r="653" ht="14.25" customHeight="1"/>
-    <row r="654" ht="14.25" customHeight="1"/>
-    <row r="655" ht="14.25" customHeight="1"/>
-    <row r="656" ht="14.25" customHeight="1"/>
-    <row r="657" ht="14.25" customHeight="1"/>
-    <row r="658" ht="14.25" customHeight="1"/>
-    <row r="659" ht="14.25" customHeight="1"/>
-    <row r="660" ht="14.25" customHeight="1"/>
-    <row r="661" ht="14.25" customHeight="1"/>
-    <row r="662" ht="14.25" customHeight="1"/>
-    <row r="663" ht="14.25" customHeight="1"/>
-    <row r="664" ht="14.25" customHeight="1"/>
-    <row r="665" ht="14.25" customHeight="1"/>
-    <row r="666" ht="14.25" customHeight="1"/>
-    <row r="667" ht="14.25" customHeight="1"/>
-    <row r="668" ht="14.25" customHeight="1"/>
-    <row r="669" ht="14.25" customHeight="1"/>
-    <row r="670" ht="14.25" customHeight="1"/>
-    <row r="671" ht="14.25" customHeight="1"/>
-    <row r="672" ht="14.25" customHeight="1"/>
-    <row r="673" ht="14.25" customHeight="1"/>
-    <row r="674" ht="14.25" customHeight="1"/>
-    <row r="675" ht="14.25" customHeight="1"/>
-    <row r="676" ht="14.25" customHeight="1"/>
-    <row r="677" ht="14.25" customHeight="1"/>
-    <row r="678" ht="14.25" customHeight="1"/>
-    <row r="679" ht="14.25" customHeight="1"/>
-    <row r="680" ht="14.25" customHeight="1"/>
-    <row r="681" ht="14.25" customHeight="1"/>
-    <row r="682" ht="14.25" customHeight="1"/>
-    <row r="683" ht="14.25" customHeight="1"/>
-    <row r="684" ht="14.25" customHeight="1"/>
-    <row r="685" ht="14.25" customHeight="1"/>
-    <row r="686" ht="14.25" customHeight="1"/>
-    <row r="687" ht="14.25" customHeight="1"/>
-    <row r="688" ht="14.25" customHeight="1"/>
-    <row r="689" ht="14.25" customHeight="1"/>
-    <row r="690" ht="14.25" customHeight="1"/>
-    <row r="691" ht="14.25" customHeight="1"/>
-    <row r="692" ht="14.25" customHeight="1"/>
-    <row r="693" ht="14.25" customHeight="1"/>
-    <row r="694" ht="14.25" customHeight="1"/>
-    <row r="695" ht="14.25" customHeight="1"/>
-    <row r="696" ht="14.25" customHeight="1"/>
-    <row r="697" ht="14.25" customHeight="1"/>
-    <row r="698" ht="14.25" customHeight="1"/>
-    <row r="699" ht="14.25" customHeight="1"/>
-    <row r="700" ht="14.25" customHeight="1"/>
-    <row r="701" ht="14.25" customHeight="1"/>
-    <row r="702" ht="14.25" customHeight="1"/>
-    <row r="703" ht="14.25" customHeight="1"/>
-    <row r="704" ht="14.25" customHeight="1"/>
-    <row r="705" ht="14.25" customHeight="1"/>
-    <row r="706" ht="14.25" customHeight="1"/>
-    <row r="707" ht="14.25" customHeight="1"/>
-    <row r="708" ht="14.25" customHeight="1"/>
-    <row r="709" ht="14.25" customHeight="1"/>
-    <row r="710" ht="14.25" customHeight="1"/>
-    <row r="711" ht="14.25" customHeight="1"/>
-    <row r="712" ht="14.25" customHeight="1"/>
-    <row r="713" ht="14.25" customHeight="1"/>
-    <row r="714" ht="14.25" customHeight="1"/>
-    <row r="715" ht="14.25" customHeight="1"/>
-    <row r="716" ht="14.25" customHeight="1"/>
-    <row r="717" ht="14.25" customHeight="1"/>
-    <row r="718" ht="14.25" customHeight="1"/>
-    <row r="719" ht="14.25" customHeight="1"/>
-    <row r="720" ht="14.25" customHeight="1"/>
-    <row r="721" ht="14.25" customHeight="1"/>
-    <row r="722" ht="14.25" customHeight="1"/>
-    <row r="723" ht="14.25" customHeight="1"/>
-    <row r="724" ht="14.25" customHeight="1"/>
-    <row r="725" ht="14.25" customHeight="1"/>
-    <row r="726" ht="14.25" customHeight="1"/>
-    <row r="727" ht="14.25" customHeight="1"/>
-    <row r="728" ht="14.25" customHeight="1"/>
-    <row r="729" ht="14.25" customHeight="1"/>
-    <row r="730" ht="14.25" customHeight="1"/>
-    <row r="731" ht="14.25" customHeight="1"/>
-    <row r="732" ht="14.25" customHeight="1"/>
-    <row r="733" ht="14.25" customHeight="1"/>
-    <row r="734" ht="14.25" customHeight="1"/>
-    <row r="735" ht="14.25" customHeight="1"/>
-    <row r="736" ht="14.25" customHeight="1"/>
-    <row r="737" ht="14.25" customHeight="1"/>
-    <row r="738" ht="14.25" customHeight="1"/>
-    <row r="739" ht="14.25" customHeight="1"/>
-    <row r="740" ht="14.25" customHeight="1"/>
-    <row r="741" ht="14.25" customHeight="1"/>
-    <row r="742" ht="14.25" customHeight="1"/>
-    <row r="743" ht="14.25" customHeight="1"/>
-    <row r="744" ht="14.25" customHeight="1"/>
-    <row r="745" ht="14.25" customHeight="1"/>
-    <row r="746" ht="14.25" customHeight="1"/>
-    <row r="747" ht="14.25" customHeight="1"/>
-    <row r="748" ht="14.25" customHeight="1"/>
-    <row r="749" ht="14.25" customHeight="1"/>
-    <row r="750" ht="14.25" customHeight="1"/>
-    <row r="751" ht="14.25" customHeight="1"/>
-    <row r="752" ht="14.25" customHeight="1"/>
-    <row r="753" ht="14.25" customHeight="1"/>
-    <row r="754" ht="14.25" customHeight="1"/>
-    <row r="755" ht="14.25" customHeight="1"/>
-    <row r="756" ht="14.25" customHeight="1"/>
-    <row r="757" ht="14.25" customHeight="1"/>
-    <row r="758" ht="14.25" customHeight="1"/>
-    <row r="759" ht="14.25" customHeight="1"/>
-    <row r="760" ht="14.25" customHeight="1"/>
-    <row r="761" ht="14.25" customHeight="1"/>
-    <row r="762" ht="14.25" customHeight="1"/>
-    <row r="763" ht="14.25" customHeight="1"/>
-    <row r="764" ht="14.25" customHeight="1"/>
-    <row r="765" ht="14.25" customHeight="1"/>
-    <row r="766" ht="14.25" customHeight="1"/>
-    <row r="767" ht="14.25" customHeight="1"/>
-    <row r="768" ht="14.25" customHeight="1"/>
-    <row r="769" ht="14.25" customHeight="1"/>
-    <row r="770" ht="14.25" customHeight="1"/>
-    <row r="771" ht="14.25" customHeight="1"/>
-    <row r="772" ht="14.25" customHeight="1"/>
-    <row r="773" ht="14.25" customHeight="1"/>
-    <row r="774" ht="14.25" customHeight="1"/>
-    <row r="775" ht="14.25" customHeight="1"/>
-    <row r="776" ht="14.25" customHeight="1"/>
-    <row r="777" ht="14.25" customHeight="1"/>
-    <row r="778" ht="14.25" customHeight="1"/>
-    <row r="779" ht="14.25" customHeight="1"/>
-    <row r="780" ht="14.25" customHeight="1"/>
-    <row r="781" ht="14.25" customHeight="1"/>
-    <row r="782" ht="14.25" customHeight="1"/>
-    <row r="783" ht="14.25" customHeight="1"/>
-    <row r="784" ht="14.25" customHeight="1"/>
-    <row r="785" ht="14.25" customHeight="1"/>
-    <row r="786" ht="14.25" customHeight="1"/>
-    <row r="787" ht="14.25" customHeight="1"/>
-    <row r="788" ht="14.25" customHeight="1"/>
-    <row r="789" ht="14.25" customHeight="1"/>
-    <row r="790" ht="14.25" customHeight="1"/>
-    <row r="791" ht="14.25" customHeight="1"/>
-    <row r="792" ht="14.25" customHeight="1"/>
-    <row r="793" ht="14.25" customHeight="1"/>
-    <row r="794" ht="14.25" customHeight="1"/>
-    <row r="795" ht="14.25" customHeight="1"/>
-    <row r="796" ht="14.25" customHeight="1"/>
-    <row r="797" ht="14.25" customHeight="1"/>
-    <row r="798" ht="14.25" customHeight="1"/>
-    <row r="799" ht="14.25" customHeight="1"/>
-    <row r="800" ht="14.25" customHeight="1"/>
-    <row r="801" ht="14.25" customHeight="1"/>
-    <row r="802" ht="14.25" customHeight="1"/>
-    <row r="803" ht="14.25" customHeight="1"/>
-    <row r="804" ht="14.25" customHeight="1"/>
-    <row r="805" ht="14.25" customHeight="1"/>
-    <row r="806" ht="14.25" customHeight="1"/>
-    <row r="807" ht="14.25" customHeight="1"/>
-    <row r="808" ht="14.25" customHeight="1"/>
-    <row r="809" ht="14.25" customHeight="1"/>
-    <row r="810" ht="14.25" customHeight="1"/>
-    <row r="811" ht="14.25" customHeight="1"/>
-    <row r="812" ht="14.25" customHeight="1"/>
-    <row r="813" ht="14.25" customHeight="1"/>
-    <row r="814" ht="14.25" customHeight="1"/>
-    <row r="815" ht="14.25" customHeight="1"/>
-    <row r="816" ht="14.25" customHeight="1"/>
-    <row r="817" ht="14.25" customHeight="1"/>
-    <row r="818" ht="14.25" customHeight="1"/>
-    <row r="819" ht="14.25" customHeight="1"/>
-    <row r="820" ht="14.25" customHeight="1"/>
-    <row r="821" ht="14.25" customHeight="1"/>
-    <row r="822" ht="14.25" customHeight="1"/>
-    <row r="823" ht="14.25" customHeight="1"/>
-    <row r="824" ht="14.25" customHeight="1"/>
-    <row r="825" ht="14.25" customHeight="1"/>
-    <row r="826" ht="14.25" customHeight="1"/>
-    <row r="827" ht="14.25" customHeight="1"/>
-    <row r="828" ht="14.25" customHeight="1"/>
-    <row r="829" ht="14.25" customHeight="1"/>
-    <row r="830" ht="14.25" customHeight="1"/>
-    <row r="831" ht="14.25" customHeight="1"/>
-    <row r="832" ht="14.25" customHeight="1"/>
-    <row r="833" ht="14.25" customHeight="1"/>
-    <row r="834" ht="14.25" customHeight="1"/>
-    <row r="835" ht="14.25" customHeight="1"/>
-    <row r="836" ht="14.25" customHeight="1"/>
-    <row r="837" ht="14.25" customHeight="1"/>
-    <row r="838" ht="14.25" customHeight="1"/>
-    <row r="839" ht="14.25" customHeight="1"/>
-    <row r="840" ht="14.25" customHeight="1"/>
-    <row r="841" ht="14.25" customHeight="1"/>
-    <row r="842" ht="14.25" customHeight="1"/>
-    <row r="843" ht="14.25" customHeight="1"/>
-    <row r="844" ht="14.25" customHeight="1"/>
-    <row r="845" ht="14.25" customHeight="1"/>
-    <row r="846" ht="14.25" customHeight="1"/>
-    <row r="847" ht="14.25" customHeight="1"/>
-    <row r="848" ht="14.25" customHeight="1"/>
-    <row r="849" ht="14.25" customHeight="1"/>
-    <row r="850" ht="14.25" customHeight="1"/>
-    <row r="851" ht="14.25" customHeight="1"/>
-    <row r="852" ht="14.25" customHeight="1"/>
-    <row r="853" ht="14.25" customHeight="1"/>
-    <row r="854" ht="14.25" customHeight="1"/>
-    <row r="855" ht="14.25" customHeight="1"/>
-    <row r="856" ht="14.25" customHeight="1"/>
-    <row r="857" ht="14.25" customHeight="1"/>
-    <row r="858" ht="14.25" customHeight="1"/>
-    <row r="859" ht="14.25" customHeight="1"/>
-    <row r="860" ht="14.25" customHeight="1"/>
-    <row r="861" ht="14.25" customHeight="1"/>
-    <row r="862" ht="14.25" customHeight="1"/>
-    <row r="863" ht="14.25" customHeight="1"/>
-    <row r="864" ht="14.25" customHeight="1"/>
-    <row r="865" ht="14.25" customHeight="1"/>
-    <row r="866" ht="14.25" customHeight="1"/>
-    <row r="867" ht="14.25" customHeight="1"/>
-    <row r="868" ht="14.25" customHeight="1"/>
-    <row r="869" ht="14.25" customHeight="1"/>
-    <row r="870" ht="14.25" customHeight="1"/>
-    <row r="871" ht="14.25" customHeight="1"/>
-    <row r="872" ht="14.25" customHeight="1"/>
-    <row r="873" ht="14.25" customHeight="1"/>
-    <row r="874" ht="14.25" customHeight="1"/>
-    <row r="875" ht="14.25" customHeight="1"/>
-    <row r="876" ht="14.25" customHeight="1"/>
-    <row r="877" ht="14.25" customHeight="1"/>
-    <row r="878" ht="14.25" customHeight="1"/>
-    <row r="879" ht="14.25" customHeight="1"/>
-    <row r="880" ht="14.25" customHeight="1"/>
-    <row r="881" ht="14.25" customHeight="1"/>
-    <row r="882" ht="14.25" customHeight="1"/>
-    <row r="883" ht="14.25" customHeight="1"/>
-    <row r="884" ht="14.25" customHeight="1"/>
-    <row r="885" ht="14.25" customHeight="1"/>
-    <row r="886" ht="14.25" customHeight="1"/>
-    <row r="887" ht="14.25" customHeight="1"/>
-    <row r="888" ht="14.25" customHeight="1"/>
-    <row r="889" ht="14.25" customHeight="1"/>
-    <row r="890" ht="14.25" customHeight="1"/>
-    <row r="891" ht="14.25" customHeight="1"/>
-    <row r="892" ht="14.25" customHeight="1"/>
-    <row r="893" ht="14.25" customHeight="1"/>
-    <row r="894" ht="14.25" customHeight="1"/>
-    <row r="895" ht="14.25" customHeight="1"/>
-    <row r="896" ht="14.25" customHeight="1"/>
-    <row r="897" ht="14.25" customHeight="1"/>
-    <row r="898" ht="14.25" customHeight="1"/>
-    <row r="899" ht="14.25" customHeight="1"/>
-    <row r="900" ht="14.25" customHeight="1"/>
-    <row r="901" ht="14.25" customHeight="1"/>
-    <row r="902" ht="14.25" customHeight="1"/>
-    <row r="903" ht="14.25" customHeight="1"/>
-    <row r="904" ht="14.25" customHeight="1"/>
-    <row r="905" ht="14.25" customHeight="1"/>
-    <row r="906" ht="14.25" customHeight="1"/>
-    <row r="907" ht="14.25" customHeight="1"/>
-    <row r="908" ht="14.25" customHeight="1"/>
-    <row r="909" ht="14.25" customHeight="1"/>
-    <row r="910" ht="14.25" customHeight="1"/>
-    <row r="911" ht="14.25" customHeight="1"/>
-    <row r="912" ht="14.25" customHeight="1"/>
-    <row r="913" ht="14.25" customHeight="1"/>
-    <row r="914" ht="14.25" customHeight="1"/>
-    <row r="915" ht="14.25" customHeight="1"/>
-    <row r="916" ht="14.25" customHeight="1"/>
-    <row r="917" ht="14.25" customHeight="1"/>
-    <row r="918" ht="14.25" customHeight="1"/>
-    <row r="919" ht="14.25" customHeight="1"/>
-    <row r="920" ht="14.25" customHeight="1"/>
-    <row r="921" ht="14.25" customHeight="1"/>
-    <row r="922" ht="14.25" customHeight="1"/>
-    <row r="923" ht="14.25" customHeight="1"/>
-    <row r="924" ht="14.25" customHeight="1"/>
-    <row r="925" ht="14.25" customHeight="1"/>
-    <row r="926" ht="14.25" customHeight="1"/>
-    <row r="927" ht="14.25" customHeight="1"/>
-    <row r="928" ht="14.25" customHeight="1"/>
-    <row r="929" ht="14.25" customHeight="1"/>
-    <row r="930" ht="14.25" customHeight="1"/>
-    <row r="931" ht="14.25" customHeight="1"/>
-    <row r="932" ht="14.25" customHeight="1"/>
-    <row r="933" ht="14.25" customHeight="1"/>
-    <row r="934" ht="14.25" customHeight="1"/>
-    <row r="935" ht="14.25" customHeight="1"/>
-    <row r="936" ht="14.25" customHeight="1"/>
-    <row r="937" ht="14.25" customHeight="1"/>
-    <row r="938" ht="14.25" customHeight="1"/>
-    <row r="939" ht="14.25" customHeight="1"/>
-    <row r="940" ht="14.25" customHeight="1"/>
-    <row r="941" ht="14.25" customHeight="1"/>
-    <row r="942" ht="14.25" customHeight="1"/>
-    <row r="943" ht="14.25" customHeight="1"/>
-    <row r="944" ht="14.25" customHeight="1"/>
-    <row r="945" ht="14.25" customHeight="1"/>
-    <row r="946" ht="14.25" customHeight="1"/>
-    <row r="947" ht="14.25" customHeight="1"/>
-    <row r="948" ht="14.25" customHeight="1"/>
-    <row r="949" ht="14.25" customHeight="1"/>
-    <row r="950" ht="14.25" customHeight="1"/>
-    <row r="951" ht="14.25" customHeight="1"/>
-    <row r="952" ht="14.25" customHeight="1"/>
-    <row r="953" ht="14.25" customHeight="1"/>
-    <row r="954" ht="14.25" customHeight="1"/>
-    <row r="955" ht="14.25" customHeight="1"/>
-    <row r="956" ht="14.25" customHeight="1"/>
-    <row r="957" ht="14.25" customHeight="1"/>
-    <row r="958" ht="14.25" customHeight="1"/>
-    <row r="959" ht="14.25" customHeight="1"/>
-    <row r="960" ht="14.25" customHeight="1"/>
-    <row r="961" ht="14.25" customHeight="1"/>
-    <row r="962" ht="14.25" customHeight="1"/>
-    <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
-    <row r="973" ht="14.25" customHeight="1"/>
-    <row r="974" ht="14.25" customHeight="1"/>
-    <row r="975" ht="14.25" customHeight="1"/>
-    <row r="976" ht="14.25" customHeight="1"/>
-    <row r="977" ht="14.25" customHeight="1"/>
-    <row r="978" ht="14.25" customHeight="1"/>
-    <row r="979" ht="14.25" customHeight="1"/>
-    <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="17" ht="14.25" customHeight="true"/>
+    <row r="18" ht="14.25" customHeight="true"/>
+    <row r="19" ht="14.25" customHeight="true"/>
+    <row r="20" ht="14.25" customHeight="true"/>
+    <row r="21" ht="14.25" customHeight="true"/>
+    <row r="22" ht="14.25" customHeight="true"/>
+    <row r="23" ht="14.25" customHeight="true"/>
+    <row r="24" ht="14.25" customHeight="true"/>
+    <row r="25" ht="14.25" customHeight="true"/>
+    <row r="26" ht="14.25" customHeight="true"/>
+    <row r="27" ht="14.25" customHeight="true"/>
+    <row r="28" ht="14.25" customHeight="true"/>
+    <row r="29" ht="14.25" customHeight="true"/>
+    <row r="30" ht="14.25" customHeight="true"/>
+    <row r="31" ht="14.25" customHeight="true"/>
+    <row r="32" ht="14.25" customHeight="true"/>
+    <row r="33" ht="14.25" customHeight="true"/>
+    <row r="34" ht="14.25" customHeight="true"/>
+    <row r="35" ht="14.25" customHeight="true"/>
+    <row r="36" ht="14.25" customHeight="true"/>
+    <row r="37" ht="14.25" customHeight="true"/>
+    <row r="38" ht="14.25" customHeight="true"/>
+    <row r="39" ht="14.25" customHeight="true"/>
+    <row r="40" ht="14.25" customHeight="true"/>
+    <row r="41" ht="14.25" customHeight="true"/>
+    <row r="42" ht="14.25" customHeight="true"/>
+    <row r="43" ht="14.25" customHeight="true"/>
+    <row r="44" ht="14.25" customHeight="true"/>
+    <row r="45" ht="14.25" customHeight="true"/>
+    <row r="46" ht="14.25" customHeight="true"/>
+    <row r="47" ht="14.25" customHeight="true"/>
+    <row r="48" ht="14.25" customHeight="true"/>
+    <row r="49" ht="14.25" customHeight="true"/>
+    <row r="50" ht="14.25" customHeight="true"/>
+    <row r="51" ht="14.25" customHeight="true"/>
+    <row r="52" ht="14.25" customHeight="true"/>
+    <row r="53" ht="14.25" customHeight="true"/>
+    <row r="54" ht="14.25" customHeight="true"/>
+    <row r="55" ht="14.25" customHeight="true"/>
+    <row r="56" ht="14.25" customHeight="true"/>
+    <row r="57" ht="14.25" customHeight="true"/>
+    <row r="58" ht="14.25" customHeight="true"/>
+    <row r="59" ht="14.25" customHeight="true"/>
+    <row r="60" ht="14.25" customHeight="true"/>
+    <row r="61" ht="14.25" customHeight="true"/>
+    <row r="62" ht="14.25" customHeight="true"/>
+    <row r="63" ht="14.25" customHeight="true"/>
+    <row r="64" ht="14.25" customHeight="true"/>
+    <row r="65" ht="14.25" customHeight="true"/>
+    <row r="66" ht="14.25" customHeight="true"/>
+    <row r="67" ht="14.25" customHeight="true"/>
+    <row r="68" ht="14.25" customHeight="true"/>
+    <row r="69" ht="14.25" customHeight="true"/>
+    <row r="70" ht="14.25" customHeight="true"/>
+    <row r="71" ht="14.25" customHeight="true"/>
+    <row r="72" ht="14.25" customHeight="true"/>
+    <row r="73" ht="14.25" customHeight="true"/>
+    <row r="74" ht="14.25" customHeight="true"/>
+    <row r="75" ht="14.25" customHeight="true"/>
+    <row r="76" ht="14.25" customHeight="true"/>
+    <row r="77" ht="14.25" customHeight="true"/>
+    <row r="78" ht="14.25" customHeight="true"/>
+    <row r="79" ht="14.25" customHeight="true"/>
+    <row r="80" ht="14.25" customHeight="true"/>
+    <row r="81" ht="14.25" customHeight="true"/>
+    <row r="82" ht="14.25" customHeight="true"/>
+    <row r="83" ht="14.25" customHeight="true"/>
+    <row r="84" ht="14.25" customHeight="true"/>
+    <row r="85" ht="14.25" customHeight="true"/>
+    <row r="86" ht="14.25" customHeight="true"/>
+    <row r="87" ht="14.25" customHeight="true"/>
+    <row r="88" ht="14.25" customHeight="true"/>
+    <row r="89" ht="14.25" customHeight="true"/>
+    <row r="90" ht="14.25" customHeight="true"/>
+    <row r="91" ht="14.25" customHeight="true"/>
+    <row r="92" ht="14.25" customHeight="true"/>
+    <row r="93" ht="14.25" customHeight="true"/>
+    <row r="94" ht="14.25" customHeight="true"/>
+    <row r="95" ht="14.25" customHeight="true"/>
+    <row r="96" ht="14.25" customHeight="true"/>
+    <row r="97" ht="14.25" customHeight="true"/>
+    <row r="98" ht="14.25" customHeight="true"/>
+    <row r="99" ht="14.25" customHeight="true"/>
+    <row r="100" ht="14.25" customHeight="true"/>
+    <row r="101" ht="14.25" customHeight="true"/>
+    <row r="102" ht="14.25" customHeight="true"/>
+    <row r="103" ht="14.25" customHeight="true"/>
+    <row r="104" ht="14.25" customHeight="true"/>
+    <row r="105" ht="14.25" customHeight="true"/>
+    <row r="106" ht="14.25" customHeight="true"/>
+    <row r="107" ht="14.25" customHeight="true"/>
+    <row r="108" ht="14.25" customHeight="true"/>
+    <row r="109" ht="14.25" customHeight="true"/>
+    <row r="110" ht="14.25" customHeight="true"/>
+    <row r="111" ht="14.25" customHeight="true"/>
+    <row r="112" ht="14.25" customHeight="true"/>
+    <row r="113" ht="14.25" customHeight="true"/>
+    <row r="114" ht="14.25" customHeight="true"/>
+    <row r="115" ht="14.25" customHeight="true"/>
+    <row r="116" ht="14.25" customHeight="true"/>
+    <row r="117" ht="14.25" customHeight="true"/>
+    <row r="118" ht="14.25" customHeight="true"/>
+    <row r="119" ht="14.25" customHeight="true"/>
+    <row r="120" ht="14.25" customHeight="true"/>
+    <row r="121" ht="14.25" customHeight="true"/>
+    <row r="122" ht="14.25" customHeight="true"/>
+    <row r="123" ht="14.25" customHeight="true"/>
+    <row r="124" ht="14.25" customHeight="true"/>
+    <row r="125" ht="14.25" customHeight="true"/>
+    <row r="126" ht="14.25" customHeight="true"/>
+    <row r="127" ht="14.25" customHeight="true"/>
+    <row r="128" ht="14.25" customHeight="true"/>
+    <row r="129" ht="14.25" customHeight="true"/>
+    <row r="130" ht="14.25" customHeight="true"/>
+    <row r="131" ht="14.25" customHeight="true"/>
+    <row r="132" ht="14.25" customHeight="true"/>
+    <row r="133" ht="14.25" customHeight="true"/>
+    <row r="134" ht="14.25" customHeight="true"/>
+    <row r="135" ht="14.25" customHeight="true"/>
+    <row r="136" ht="14.25" customHeight="true"/>
+    <row r="137" ht="14.25" customHeight="true"/>
+    <row r="138" ht="14.25" customHeight="true"/>
+    <row r="139" ht="14.25" customHeight="true"/>
+    <row r="140" ht="14.25" customHeight="true"/>
+    <row r="141" ht="14.25" customHeight="true"/>
+    <row r="142" ht="14.25" customHeight="true"/>
+    <row r="143" ht="14.25" customHeight="true"/>
+    <row r="144" ht="14.25" customHeight="true"/>
+    <row r="145" ht="14.25" customHeight="true"/>
+    <row r="146" ht="14.25" customHeight="true"/>
+    <row r="147" ht="14.25" customHeight="true"/>
+    <row r="148" ht="14.25" customHeight="true"/>
+    <row r="149" ht="14.25" customHeight="true"/>
+    <row r="150" ht="14.25" customHeight="true"/>
+    <row r="151" ht="14.25" customHeight="true"/>
+    <row r="152" ht="14.25" customHeight="true"/>
+    <row r="153" ht="14.25" customHeight="true"/>
+    <row r="154" ht="14.25" customHeight="true"/>
+    <row r="155" ht="14.25" customHeight="true"/>
+    <row r="156" ht="14.25" customHeight="true"/>
+    <row r="157" ht="14.25" customHeight="true"/>
+    <row r="158" ht="14.25" customHeight="true"/>
+    <row r="159" ht="14.25" customHeight="true"/>
+    <row r="160" ht="14.25" customHeight="true"/>
+    <row r="161" ht="14.25" customHeight="true"/>
+    <row r="162" ht="14.25" customHeight="true"/>
+    <row r="163" ht="14.25" customHeight="true"/>
+    <row r="164" ht="14.25" customHeight="true"/>
+    <row r="165" ht="14.25" customHeight="true"/>
+    <row r="166" ht="14.25" customHeight="true"/>
+    <row r="167" ht="14.25" customHeight="true"/>
+    <row r="168" ht="14.25" customHeight="true"/>
+    <row r="169" ht="14.25" customHeight="true"/>
+    <row r="170" ht="14.25" customHeight="true"/>
+    <row r="171" ht="14.25" customHeight="true"/>
+    <row r="172" ht="14.25" customHeight="true"/>
+    <row r="173" ht="14.25" customHeight="true"/>
+    <row r="174" ht="14.25" customHeight="true"/>
+    <row r="175" ht="14.25" customHeight="true"/>
+    <row r="176" ht="14.25" customHeight="true"/>
+    <row r="177" ht="14.25" customHeight="true"/>
+    <row r="178" ht="14.25" customHeight="true"/>
+    <row r="179" ht="14.25" customHeight="true"/>
+    <row r="180" ht="14.25" customHeight="true"/>
+    <row r="181" ht="14.25" customHeight="true"/>
+    <row r="182" ht="14.25" customHeight="true"/>
+    <row r="183" ht="14.25" customHeight="true"/>
+    <row r="184" ht="14.25" customHeight="true"/>
+    <row r="185" ht="14.25" customHeight="true"/>
+    <row r="186" ht="14.25" customHeight="true"/>
+    <row r="187" ht="14.25" customHeight="true"/>
+    <row r="188" ht="14.25" customHeight="true"/>
+    <row r="189" ht="14.25" customHeight="true"/>
+    <row r="190" ht="14.25" customHeight="true"/>
+    <row r="191" ht="14.25" customHeight="true"/>
+    <row r="192" ht="14.25" customHeight="true"/>
+    <row r="193" ht="14.25" customHeight="true"/>
+    <row r="194" ht="14.25" customHeight="true"/>
+    <row r="195" ht="14.25" customHeight="true"/>
+    <row r="196" ht="14.25" customHeight="true"/>
+    <row r="197" ht="14.25" customHeight="true"/>
+    <row r="198" ht="14.25" customHeight="true"/>
+    <row r="199" ht="14.25" customHeight="true"/>
+    <row r="200" ht="14.25" customHeight="true"/>
+    <row r="201" ht="14.25" customHeight="true"/>
+    <row r="202" ht="14.25" customHeight="true"/>
+    <row r="203" ht="14.25" customHeight="true"/>
+    <row r="204" ht="14.25" customHeight="true"/>
+    <row r="205" ht="14.25" customHeight="true"/>
+    <row r="206" ht="14.25" customHeight="true"/>
+    <row r="207" ht="14.25" customHeight="true"/>
+    <row r="208" ht="14.25" customHeight="true"/>
+    <row r="209" ht="14.25" customHeight="true"/>
+    <row r="210" ht="14.25" customHeight="true"/>
+    <row r="211" ht="14.25" customHeight="true"/>
+    <row r="212" ht="14.25" customHeight="true"/>
+    <row r="213" ht="14.25" customHeight="true"/>
+    <row r="214" ht="14.25" customHeight="true"/>
+    <row r="215" ht="14.25" customHeight="true"/>
+    <row r="216" ht="14.25" customHeight="true"/>
+    <row r="217" ht="14.25" customHeight="true"/>
+    <row r="218" ht="14.25" customHeight="true"/>
+    <row r="219" ht="14.25" customHeight="true"/>
+    <row r="220" ht="14.25" customHeight="true"/>
+    <row r="221" ht="14.25" customHeight="true"/>
+    <row r="222" ht="14.25" customHeight="true"/>
+    <row r="223" ht="14.25" customHeight="true"/>
+    <row r="224" ht="14.25" customHeight="true"/>
+    <row r="225" ht="14.25" customHeight="true"/>
+    <row r="226" ht="14.25" customHeight="true"/>
+    <row r="227" ht="14.25" customHeight="true"/>
+    <row r="228" ht="14.25" customHeight="true"/>
+    <row r="229" ht="14.25" customHeight="true"/>
+    <row r="230" ht="14.25" customHeight="true"/>
+    <row r="231" ht="14.25" customHeight="true"/>
+    <row r="232" ht="14.25" customHeight="true"/>
+    <row r="233" ht="14.25" customHeight="true"/>
+    <row r="234" ht="14.25" customHeight="true"/>
+    <row r="235" ht="14.25" customHeight="true"/>
+    <row r="236" ht="14.25" customHeight="true"/>
+    <row r="237" ht="14.25" customHeight="true"/>
+    <row r="238" ht="14.25" customHeight="true"/>
+    <row r="239" ht="14.25" customHeight="true"/>
+    <row r="240" ht="14.25" customHeight="true"/>
+    <row r="241" ht="14.25" customHeight="true"/>
+    <row r="242" ht="14.25" customHeight="true"/>
+    <row r="243" ht="14.25" customHeight="true"/>
+    <row r="244" ht="14.25" customHeight="true"/>
+    <row r="245" ht="14.25" customHeight="true"/>
+    <row r="246" ht="14.25" customHeight="true"/>
+    <row r="247" ht="14.25" customHeight="true"/>
+    <row r="248" ht="14.25" customHeight="true"/>
+    <row r="249" ht="14.25" customHeight="true"/>
+    <row r="250" ht="14.25" customHeight="true"/>
+    <row r="251" ht="14.25" customHeight="true"/>
+    <row r="252" ht="14.25" customHeight="true"/>
+    <row r="253" ht="14.25" customHeight="true"/>
+    <row r="254" ht="14.25" customHeight="true"/>
+    <row r="255" ht="14.25" customHeight="true"/>
+    <row r="256" ht="14.25" customHeight="true"/>
+    <row r="257" ht="14.25" customHeight="true"/>
+    <row r="258" ht="14.25" customHeight="true"/>
+    <row r="259" ht="14.25" customHeight="true"/>
+    <row r="260" ht="14.25" customHeight="true"/>
+    <row r="261" ht="14.25" customHeight="true"/>
+    <row r="262" ht="14.25" customHeight="true"/>
+    <row r="263" ht="14.25" customHeight="true"/>
+    <row r="264" ht="14.25" customHeight="true"/>
+    <row r="265" ht="14.25" customHeight="true"/>
+    <row r="266" ht="14.25" customHeight="true"/>
+    <row r="267" ht="14.25" customHeight="true"/>
+    <row r="268" ht="14.25" customHeight="true"/>
+    <row r="269" ht="14.25" customHeight="true"/>
+    <row r="270" ht="14.25" customHeight="true"/>
+    <row r="271" ht="14.25" customHeight="true"/>
+    <row r="272" ht="14.25" customHeight="true"/>
+    <row r="273" ht="14.25" customHeight="true"/>
+    <row r="274" ht="14.25" customHeight="true"/>
+    <row r="275" ht="14.25" customHeight="true"/>
+    <row r="276" ht="14.25" customHeight="true"/>
+    <row r="277" ht="14.25" customHeight="true"/>
+    <row r="278" ht="14.25" customHeight="true"/>
+    <row r="279" ht="14.25" customHeight="true"/>
+    <row r="280" ht="14.25" customHeight="true"/>
+    <row r="281" ht="14.25" customHeight="true"/>
+    <row r="282" ht="14.25" customHeight="true"/>
+    <row r="283" ht="14.25" customHeight="true"/>
+    <row r="284" ht="14.25" customHeight="true"/>
+    <row r="285" ht="14.25" customHeight="true"/>
+    <row r="286" ht="14.25" customHeight="true"/>
+    <row r="287" ht="14.25" customHeight="true"/>
+    <row r="288" ht="14.25" customHeight="true"/>
+    <row r="289" ht="14.25" customHeight="true"/>
+    <row r="290" ht="14.25" customHeight="true"/>
+    <row r="291" ht="14.25" customHeight="true"/>
+    <row r="292" ht="14.25" customHeight="true"/>
+    <row r="293" ht="14.25" customHeight="true"/>
+    <row r="294" ht="14.25" customHeight="true"/>
+    <row r="295" ht="14.25" customHeight="true"/>
+    <row r="296" ht="14.25" customHeight="true"/>
+    <row r="297" ht="14.25" customHeight="true"/>
+    <row r="298" ht="14.25" customHeight="true"/>
+    <row r="299" ht="14.25" customHeight="true"/>
+    <row r="300" ht="14.25" customHeight="true"/>
+    <row r="301" ht="14.25" customHeight="true"/>
+    <row r="302" ht="14.25" customHeight="true"/>
+    <row r="303" ht="14.25" customHeight="true"/>
+    <row r="304" ht="14.25" customHeight="true"/>
+    <row r="305" ht="14.25" customHeight="true"/>
+    <row r="306" ht="14.25" customHeight="true"/>
+    <row r="307" ht="14.25" customHeight="true"/>
+    <row r="308" ht="14.25" customHeight="true"/>
+    <row r="309" ht="14.25" customHeight="true"/>
+    <row r="310" ht="14.25" customHeight="true"/>
+    <row r="311" ht="14.25" customHeight="true"/>
+    <row r="312" ht="14.25" customHeight="true"/>
+    <row r="313" ht="14.25" customHeight="true"/>
+    <row r="314" ht="14.25" customHeight="true"/>
+    <row r="315" ht="14.25" customHeight="true"/>
+    <row r="316" ht="14.25" customHeight="true"/>
+    <row r="317" ht="14.25" customHeight="true"/>
+    <row r="318" ht="14.25" customHeight="true"/>
+    <row r="319" ht="14.25" customHeight="true"/>
+    <row r="320" ht="14.25" customHeight="true"/>
+    <row r="321" ht="14.25" customHeight="true"/>
+    <row r="322" ht="14.25" customHeight="true"/>
+    <row r="323" ht="14.25" customHeight="true"/>
+    <row r="324" ht="14.25" customHeight="true"/>
+    <row r="325" ht="14.25" customHeight="true"/>
+    <row r="326" ht="14.25" customHeight="true"/>
+    <row r="327" ht="14.25" customHeight="true"/>
+    <row r="328" ht="14.25" customHeight="true"/>
+    <row r="329" ht="14.25" customHeight="true"/>
+    <row r="330" ht="14.25" customHeight="true"/>
+    <row r="331" ht="14.25" customHeight="true"/>
+    <row r="332" ht="14.25" customHeight="true"/>
+    <row r="333" ht="14.25" customHeight="true"/>
+    <row r="334" ht="14.25" customHeight="true"/>
+    <row r="335" ht="14.25" customHeight="true"/>
+    <row r="336" ht="14.25" customHeight="true"/>
+    <row r="337" ht="14.25" customHeight="true"/>
+    <row r="338" ht="14.25" customHeight="true"/>
+    <row r="339" ht="14.25" customHeight="true"/>
+    <row r="340" ht="14.25" customHeight="true"/>
+    <row r="341" ht="14.25" customHeight="true"/>
+    <row r="342" ht="14.25" customHeight="true"/>
+    <row r="343" ht="14.25" customHeight="true"/>
+    <row r="344" ht="14.25" customHeight="true"/>
+    <row r="345" ht="14.25" customHeight="true"/>
+    <row r="346" ht="14.25" customHeight="true"/>
+    <row r="347" ht="14.25" customHeight="true"/>
+    <row r="348" ht="14.25" customHeight="true"/>
+    <row r="349" ht="14.25" customHeight="true"/>
+    <row r="350" ht="14.25" customHeight="true"/>
+    <row r="351" ht="14.25" customHeight="true"/>
+    <row r="352" ht="14.25" customHeight="true"/>
+    <row r="353" ht="14.25" customHeight="true"/>
+    <row r="354" ht="14.25" customHeight="true"/>
+    <row r="355" ht="14.25" customHeight="true"/>
+    <row r="356" ht="14.25" customHeight="true"/>
+    <row r="357" ht="14.25" customHeight="true"/>
+    <row r="358" ht="14.25" customHeight="true"/>
+    <row r="359" ht="14.25" customHeight="true"/>
+    <row r="360" ht="14.25" customHeight="true"/>
+    <row r="361" ht="14.25" customHeight="true"/>
+    <row r="362" ht="14.25" customHeight="true"/>
+    <row r="363" ht="14.25" customHeight="true"/>
+    <row r="364" ht="14.25" customHeight="true"/>
+    <row r="365" ht="14.25" customHeight="true"/>
+    <row r="366" ht="14.25" customHeight="true"/>
+    <row r="367" ht="14.25" customHeight="true"/>
+    <row r="368" ht="14.25" customHeight="true"/>
+    <row r="369" ht="14.25" customHeight="true"/>
+    <row r="370" ht="14.25" customHeight="true"/>
+    <row r="371" ht="14.25" customHeight="true"/>
+    <row r="372" ht="14.25" customHeight="true"/>
+    <row r="373" ht="14.25" customHeight="true"/>
+    <row r="374" ht="14.25" customHeight="true"/>
+    <row r="375" ht="14.25" customHeight="true"/>
+    <row r="376" ht="14.25" customHeight="true"/>
+    <row r="377" ht="14.25" customHeight="true"/>
+    <row r="378" ht="14.25" customHeight="true"/>
+    <row r="379" ht="14.25" customHeight="true"/>
+    <row r="380" ht="14.25" customHeight="true"/>
+    <row r="381" ht="14.25" customHeight="true"/>
+    <row r="382" ht="14.25" customHeight="true"/>
+    <row r="383" ht="14.25" customHeight="true"/>
+    <row r="384" ht="14.25" customHeight="true"/>
+    <row r="385" ht="14.25" customHeight="true"/>
+    <row r="386" ht="14.25" customHeight="true"/>
+    <row r="387" ht="14.25" customHeight="true"/>
+    <row r="388" ht="14.25" customHeight="true"/>
+    <row r="389" ht="14.25" customHeight="true"/>
+    <row r="390" ht="14.25" customHeight="true"/>
+    <row r="391" ht="14.25" customHeight="true"/>
+    <row r="392" ht="14.25" customHeight="true"/>
+    <row r="393" ht="14.25" customHeight="true"/>
+    <row r="394" ht="14.25" customHeight="true"/>
+    <row r="395" ht="14.25" customHeight="true"/>
+    <row r="396" ht="14.25" customHeight="true"/>
+    <row r="397" ht="14.25" customHeight="true"/>
+    <row r="398" ht="14.25" customHeight="true"/>
+    <row r="399" ht="14.25" customHeight="true"/>
+    <row r="400" ht="14.25" customHeight="true"/>
+    <row r="401" ht="14.25" customHeight="true"/>
+    <row r="402" ht="14.25" customHeight="true"/>
+    <row r="403" ht="14.25" customHeight="true"/>
+    <row r="404" ht="14.25" customHeight="true"/>
+    <row r="405" ht="14.25" customHeight="true"/>
+    <row r="406" ht="14.25" customHeight="true"/>
+    <row r="407" ht="14.25" customHeight="true"/>
+    <row r="408" ht="14.25" customHeight="true"/>
+    <row r="409" ht="14.25" customHeight="true"/>
+    <row r="410" ht="14.25" customHeight="true"/>
+    <row r="411" ht="14.25" customHeight="true"/>
+    <row r="412" ht="14.25" customHeight="true"/>
+    <row r="413" ht="14.25" customHeight="true"/>
+    <row r="414" ht="14.25" customHeight="true"/>
+    <row r="415" ht="14.25" customHeight="true"/>
+    <row r="416" ht="14.25" customHeight="true"/>
+    <row r="417" ht="14.25" customHeight="true"/>
+    <row r="418" ht="14.25" customHeight="true"/>
+    <row r="419" ht="14.25" customHeight="true"/>
+    <row r="420" ht="14.25" customHeight="true"/>
+    <row r="421" ht="14.25" customHeight="true"/>
+    <row r="422" ht="14.25" customHeight="true"/>
+    <row r="423" ht="14.25" customHeight="true"/>
+    <row r="424" ht="14.25" customHeight="true"/>
+    <row r="425" ht="14.25" customHeight="true"/>
+    <row r="426" ht="14.25" customHeight="true"/>
+    <row r="427" ht="14.25" customHeight="true"/>
+    <row r="428" ht="14.25" customHeight="true"/>
+    <row r="429" ht="14.25" customHeight="true"/>
+    <row r="430" ht="14.25" customHeight="true"/>
+    <row r="431" ht="14.25" customHeight="true"/>
+    <row r="432" ht="14.25" customHeight="true"/>
+    <row r="433" ht="14.25" customHeight="true"/>
+    <row r="434" ht="14.25" customHeight="true"/>
+    <row r="435" ht="14.25" customHeight="true"/>
+    <row r="436" ht="14.25" customHeight="true"/>
+    <row r="437" ht="14.25" customHeight="true"/>
+    <row r="438" ht="14.25" customHeight="true"/>
+    <row r="439" ht="14.25" customHeight="true"/>
+    <row r="440" ht="14.25" customHeight="true"/>
+    <row r="441" ht="14.25" customHeight="true"/>
+    <row r="442" ht="14.25" customHeight="true"/>
+    <row r="443" ht="14.25" customHeight="true"/>
+    <row r="444" ht="14.25" customHeight="true"/>
+    <row r="445" ht="14.25" customHeight="true"/>
+    <row r="446" ht="14.25" customHeight="true"/>
+    <row r="447" ht="14.25" customHeight="true"/>
+    <row r="448" ht="14.25" customHeight="true"/>
+    <row r="449" ht="14.25" customHeight="true"/>
+    <row r="450" ht="14.25" customHeight="true"/>
+    <row r="451" ht="14.25" customHeight="true"/>
+    <row r="452" ht="14.25" customHeight="true"/>
+    <row r="453" ht="14.25" customHeight="true"/>
+    <row r="454" ht="14.25" customHeight="true"/>
+    <row r="455" ht="14.25" customHeight="true"/>
+    <row r="456" ht="14.25" customHeight="true"/>
+    <row r="457" ht="14.25" customHeight="true"/>
+    <row r="458" ht="14.25" customHeight="true"/>
+    <row r="459" ht="14.25" customHeight="true"/>
+    <row r="460" ht="14.25" customHeight="true"/>
+    <row r="461" ht="14.25" customHeight="true"/>
+    <row r="462" ht="14.25" customHeight="true"/>
+    <row r="463" ht="14.25" customHeight="true"/>
+    <row r="464" ht="14.25" customHeight="true"/>
+    <row r="465" ht="14.25" customHeight="true"/>
+    <row r="466" ht="14.25" customHeight="true"/>
+    <row r="467" ht="14.25" customHeight="true"/>
+    <row r="468" ht="14.25" customHeight="true"/>
+    <row r="469" ht="14.25" customHeight="true"/>
+    <row r="470" ht="14.25" customHeight="true"/>
+    <row r="471" ht="14.25" customHeight="true"/>
+    <row r="472" ht="14.25" customHeight="true"/>
+    <row r="473" ht="14.25" customHeight="true"/>
+    <row r="474" ht="14.25" customHeight="true"/>
+    <row r="475" ht="14.25" customHeight="true"/>
+    <row r="476" ht="14.25" customHeight="true"/>
+    <row r="477" ht="14.25" customHeight="true"/>
+    <row r="478" ht="14.25" customHeight="true"/>
+    <row r="479" ht="14.25" customHeight="true"/>
+    <row r="480" ht="14.25" customHeight="true"/>
+    <row r="481" ht="14.25" customHeight="true"/>
+    <row r="482" ht="14.25" customHeight="true"/>
+    <row r="483" ht="14.25" customHeight="true"/>
+    <row r="484" ht="14.25" customHeight="true"/>
+    <row r="485" ht="14.25" customHeight="true"/>
+    <row r="486" ht="14.25" customHeight="true"/>
+    <row r="487" ht="14.25" customHeight="true"/>
+    <row r="488" ht="14.25" customHeight="true"/>
+    <row r="489" ht="14.25" customHeight="true"/>
+    <row r="490" ht="14.25" customHeight="true"/>
+    <row r="491" ht="14.25" customHeight="true"/>
+    <row r="492" ht="14.25" customHeight="true"/>
+    <row r="493" ht="14.25" customHeight="true"/>
+    <row r="494" ht="14.25" customHeight="true"/>
+    <row r="495" ht="14.25" customHeight="true"/>
+    <row r="496" ht="14.25" customHeight="true"/>
+    <row r="497" ht="14.25" customHeight="true"/>
+    <row r="498" ht="14.25" customHeight="true"/>
+    <row r="499" ht="14.25" customHeight="true"/>
+    <row r="500" ht="14.25" customHeight="true"/>
+    <row r="501" ht="14.25" customHeight="true"/>
+    <row r="502" ht="14.25" customHeight="true"/>
+    <row r="503" ht="14.25" customHeight="true"/>
+    <row r="504" ht="14.25" customHeight="true"/>
+    <row r="505" ht="14.25" customHeight="true"/>
+    <row r="506" ht="14.25" customHeight="true"/>
+    <row r="507" ht="14.25" customHeight="true"/>
+    <row r="508" ht="14.25" customHeight="true"/>
+    <row r="509" ht="14.25" customHeight="true"/>
+    <row r="510" ht="14.25" customHeight="true"/>
+    <row r="511" ht="14.25" customHeight="true"/>
+    <row r="512" ht="14.25" customHeight="true"/>
+    <row r="513" ht="14.25" customHeight="true"/>
+    <row r="514" ht="14.25" customHeight="true"/>
+    <row r="515" ht="14.25" customHeight="true"/>
+    <row r="516" ht="14.25" customHeight="true"/>
+    <row r="517" ht="14.25" customHeight="true"/>
+    <row r="518" ht="14.25" customHeight="true"/>
+    <row r="519" ht="14.25" customHeight="true"/>
+    <row r="520" ht="14.25" customHeight="true"/>
+    <row r="521" ht="14.25" customHeight="true"/>
+    <row r="522" ht="14.25" customHeight="true"/>
+    <row r="523" ht="14.25" customHeight="true"/>
+    <row r="524" ht="14.25" customHeight="true"/>
+    <row r="525" ht="14.25" customHeight="true"/>
+    <row r="526" ht="14.25" customHeight="true"/>
+    <row r="527" ht="14.25" customHeight="true"/>
+    <row r="528" ht="14.25" customHeight="true"/>
+    <row r="529" ht="14.25" customHeight="true"/>
+    <row r="530" ht="14.25" customHeight="true"/>
+    <row r="531" ht="14.25" customHeight="true"/>
+    <row r="532" ht="14.25" customHeight="true"/>
+    <row r="533" ht="14.25" customHeight="true"/>
+    <row r="534" ht="14.25" customHeight="true"/>
+    <row r="535" ht="14.25" customHeight="true"/>
+    <row r="536" ht="14.25" customHeight="true"/>
+    <row r="537" ht="14.25" customHeight="true"/>
+    <row r="538" ht="14.25" customHeight="true"/>
+    <row r="539" ht="14.25" customHeight="true"/>
+    <row r="540" ht="14.25" customHeight="true"/>
+    <row r="541" ht="14.25" customHeight="true"/>
+    <row r="542" ht="14.25" customHeight="true"/>
+    <row r="543" ht="14.25" customHeight="true"/>
+    <row r="544" ht="14.25" customHeight="true"/>
+    <row r="545" ht="14.25" customHeight="true"/>
+    <row r="546" ht="14.25" customHeight="true"/>
+    <row r="547" ht="14.25" customHeight="true"/>
+    <row r="548" ht="14.25" customHeight="true"/>
+    <row r="549" ht="14.25" customHeight="true"/>
+    <row r="550" ht="14.25" customHeight="true"/>
+    <row r="551" ht="14.25" customHeight="true"/>
+    <row r="552" ht="14.25" customHeight="true"/>
+    <row r="553" ht="14.25" customHeight="true"/>
+    <row r="554" ht="14.25" customHeight="true"/>
+    <row r="555" ht="14.25" customHeight="true"/>
+    <row r="556" ht="14.25" customHeight="true"/>
+    <row r="557" ht="14.25" customHeight="true"/>
+    <row r="558" ht="14.25" customHeight="true"/>
+    <row r="559" ht="14.25" customHeight="true"/>
+    <row r="560" ht="14.25" customHeight="true"/>
+    <row r="561" ht="14.25" customHeight="true"/>
+    <row r="562" ht="14.25" customHeight="true"/>
+    <row r="563" ht="14.25" customHeight="true"/>
+    <row r="564" ht="14.25" customHeight="true"/>
+    <row r="565" ht="14.25" customHeight="true"/>
+    <row r="566" ht="14.25" customHeight="true"/>
+    <row r="567" ht="14.25" customHeight="true"/>
+    <row r="568" ht="14.25" customHeight="true"/>
+    <row r="569" ht="14.25" customHeight="true"/>
+    <row r="570" ht="14.25" customHeight="true"/>
+    <row r="571" ht="14.25" customHeight="true"/>
+    <row r="572" ht="14.25" customHeight="true"/>
+    <row r="573" ht="14.25" customHeight="true"/>
+    <row r="574" ht="14.25" customHeight="true"/>
+    <row r="575" ht="14.25" customHeight="true"/>
+    <row r="576" ht="14.25" customHeight="true"/>
+    <row r="577" ht="14.25" customHeight="true"/>
+    <row r="578" ht="14.25" customHeight="true"/>
+    <row r="579" ht="14.25" customHeight="true"/>
+    <row r="580" ht="14.25" customHeight="true"/>
+    <row r="581" ht="14.25" customHeight="true"/>
+    <row r="582" ht="14.25" customHeight="true"/>
+    <row r="583" ht="14.25" customHeight="true"/>
+    <row r="584" ht="14.25" customHeight="true"/>
+    <row r="585" ht="14.25" customHeight="true"/>
+    <row r="586" ht="14.25" customHeight="true"/>
+    <row r="587" ht="14.25" customHeight="true"/>
+    <row r="588" ht="14.25" customHeight="true"/>
+    <row r="589" ht="14.25" customHeight="true"/>
+    <row r="590" ht="14.25" customHeight="true"/>
+    <row r="591" ht="14.25" customHeight="true"/>
+    <row r="592" ht="14.25" customHeight="true"/>
+    <row r="593" ht="14.25" customHeight="true"/>
+    <row r="594" ht="14.25" customHeight="true"/>
+    <row r="595" ht="14.25" customHeight="true"/>
+    <row r="596" ht="14.25" customHeight="true"/>
+    <row r="597" ht="14.25" customHeight="true"/>
+    <row r="598" ht="14.25" customHeight="true"/>
+    <row r="599" ht="14.25" customHeight="true"/>
+    <row r="600" ht="14.25" customHeight="true"/>
+    <row r="601" ht="14.25" customHeight="true"/>
+    <row r="602" ht="14.25" customHeight="true"/>
+    <row r="603" ht="14.25" customHeight="true"/>
+    <row r="604" ht="14.25" customHeight="true"/>
+    <row r="605" ht="14.25" customHeight="true"/>
+    <row r="606" ht="14.25" customHeight="true"/>
+    <row r="607" ht="14.25" customHeight="true"/>
+    <row r="608" ht="14.25" customHeight="true"/>
+    <row r="609" ht="14.25" customHeight="true"/>
+    <row r="610" ht="14.25" customHeight="true"/>
+    <row r="611" ht="14.25" customHeight="true"/>
+    <row r="612" ht="14.25" customHeight="true"/>
+    <row r="613" ht="14.25" customHeight="true"/>
+    <row r="614" ht="14.25" customHeight="true"/>
+    <row r="615" ht="14.25" customHeight="true"/>
+    <row r="616" ht="14.25" customHeight="true"/>
+    <row r="617" ht="14.25" customHeight="true"/>
+    <row r="618" ht="14.25" customHeight="true"/>
+    <row r="619" ht="14.25" customHeight="true"/>
+    <row r="620" ht="14.25" customHeight="true"/>
+    <row r="621" ht="14.25" customHeight="true"/>
+    <row r="622" ht="14.25" customHeight="true"/>
+    <row r="623" ht="14.25" customHeight="true"/>
+    <row r="624" ht="14.25" customHeight="true"/>
+    <row r="625" ht="14.25" customHeight="true"/>
+    <row r="626" ht="14.25" customHeight="true"/>
+    <row r="627" ht="14.25" customHeight="true"/>
+    <row r="628" ht="14.25" customHeight="true"/>
+    <row r="629" ht="14.25" customHeight="true"/>
+    <row r="630" ht="14.25" customHeight="true"/>
+    <row r="631" ht="14.25" customHeight="true"/>
+    <row r="632" ht="14.25" customHeight="true"/>
+    <row r="633" ht="14.25" customHeight="true"/>
+    <row r="634" ht="14.25" customHeight="true"/>
+    <row r="635" ht="14.25" customHeight="true"/>
+    <row r="636" ht="14.25" customHeight="true"/>
+    <row r="637" ht="14.25" customHeight="true"/>
+    <row r="638" ht="14.25" customHeight="true"/>
+    <row r="639" ht="14.25" customHeight="true"/>
+    <row r="640" ht="14.25" customHeight="true"/>
+    <row r="641" ht="14.25" customHeight="true"/>
+    <row r="642" ht="14.25" customHeight="true"/>
+    <row r="643" ht="14.25" customHeight="true"/>
+    <row r="644" ht="14.25" customHeight="true"/>
+    <row r="645" ht="14.25" customHeight="true"/>
+    <row r="646" ht="14.25" customHeight="true"/>
+    <row r="647" ht="14.25" customHeight="true"/>
+    <row r="648" ht="14.25" customHeight="true"/>
+    <row r="649" ht="14.25" customHeight="true"/>
+    <row r="650" ht="14.25" customHeight="true"/>
+    <row r="651" ht="14.25" customHeight="true"/>
+    <row r="652" ht="14.25" customHeight="true"/>
+    <row r="653" ht="14.25" customHeight="true"/>
+    <row r="654" ht="14.25" customHeight="true"/>
+    <row r="655" ht="14.25" customHeight="true"/>
+    <row r="656" ht="14.25" customHeight="true"/>
+    <row r="657" ht="14.25" customHeight="true"/>
+    <row r="658" ht="14.25" customHeight="true"/>
+    <row r="659" ht="14.25" customHeight="true"/>
+    <row r="660" ht="14.25" customHeight="true"/>
+    <row r="661" ht="14.25" customHeight="true"/>
+    <row r="662" ht="14.25" customHeight="true"/>
+    <row r="663" ht="14.25" customHeight="true"/>
+    <row r="664" ht="14.25" customHeight="true"/>
+    <row r="665" ht="14.25" customHeight="true"/>
+    <row r="666" ht="14.25" customHeight="true"/>
+    <row r="667" ht="14.25" customHeight="true"/>
+    <row r="668" ht="14.25" customHeight="true"/>
+    <row r="669" ht="14.25" customHeight="true"/>
+    <row r="670" ht="14.25" customHeight="true"/>
+    <row r="671" ht="14.25" customHeight="true"/>
+    <row r="672" ht="14.25" customHeight="true"/>
+    <row r="673" ht="14.25" customHeight="true"/>
+    <row r="674" ht="14.25" customHeight="true"/>
+    <row r="675" ht="14.25" customHeight="true"/>
+    <row r="676" ht="14.25" customHeight="true"/>
+    <row r="677" ht="14.25" customHeight="true"/>
+    <row r="678" ht="14.25" customHeight="true"/>
+    <row r="679" ht="14.25" customHeight="true"/>
+    <row r="680" ht="14.25" customHeight="true"/>
+    <row r="681" ht="14.25" customHeight="true"/>
+    <row r="682" ht="14.25" customHeight="true"/>
+    <row r="683" ht="14.25" customHeight="true"/>
+    <row r="684" ht="14.25" customHeight="true"/>
+    <row r="685" ht="14.25" customHeight="true"/>
+    <row r="686" ht="14.25" customHeight="true"/>
+    <row r="687" ht="14.25" customHeight="true"/>
+    <row r="688" ht="14.25" customHeight="true"/>
+    <row r="689" ht="14.25" customHeight="true"/>
+    <row r="690" ht="14.25" customHeight="true"/>
+    <row r="691" ht="14.25" customHeight="true"/>
+    <row r="692" ht="14.25" customHeight="true"/>
+    <row r="693" ht="14.25" customHeight="true"/>
+    <row r="694" ht="14.25" customHeight="true"/>
+    <row r="695" ht="14.25" customHeight="true"/>
+    <row r="696" ht="14.25" customHeight="true"/>
+    <row r="697" ht="14.25" customHeight="true"/>
+    <row r="698" ht="14.25" customHeight="true"/>
+    <row r="699" ht="14.25" customHeight="true"/>
+    <row r="700" ht="14.25" customHeight="true"/>
+    <row r="701" ht="14.25" customHeight="true"/>
+    <row r="702" ht="14.25" customHeight="true"/>
+    <row r="703" ht="14.25" customHeight="true"/>
+    <row r="704" ht="14.25" customHeight="true"/>
+    <row r="705" ht="14.25" customHeight="true"/>
+    <row r="706" ht="14.25" customHeight="true"/>
+    <row r="707" ht="14.25" customHeight="true"/>
+    <row r="708" ht="14.25" customHeight="true"/>
+    <row r="709" ht="14.25" customHeight="true"/>
+    <row r="710" ht="14.25" customHeight="true"/>
+    <row r="711" ht="14.25" customHeight="true"/>
+    <row r="712" ht="14.25" customHeight="true"/>
+    <row r="713" ht="14.25" customHeight="true"/>
+    <row r="714" ht="14.25" customHeight="true"/>
+    <row r="715" ht="14.25" customHeight="true"/>
+    <row r="716" ht="14.25" customHeight="true"/>
+    <row r="717" ht="14.25" customHeight="true"/>
+    <row r="718" ht="14.25" customHeight="true"/>
+    <row r="719" ht="14.25" customHeight="true"/>
+    <row r="720" ht="14.25" customHeight="true"/>
+    <row r="721" ht="14.25" customHeight="true"/>
+    <row r="722" ht="14.25" customHeight="true"/>
+    <row r="723" ht="14.25" customHeight="true"/>
+    <row r="724" ht="14.25" customHeight="true"/>
+    <row r="725" ht="14.25" customHeight="true"/>
+    <row r="726" ht="14.25" customHeight="true"/>
+    <row r="727" ht="14.25" customHeight="true"/>
+    <row r="728" ht="14.25" customHeight="true"/>
+    <row r="729" ht="14.25" customHeight="true"/>
+    <row r="730" ht="14.25" customHeight="true"/>
+    <row r="731" ht="14.25" customHeight="true"/>
+    <row r="732" ht="14.25" customHeight="true"/>
+    <row r="733" ht="14.25" customHeight="true"/>
+    <row r="734" ht="14.25" customHeight="true"/>
+    <row r="735" ht="14.25" customHeight="true"/>
+    <row r="736" ht="14.25" customHeight="true"/>
+    <row r="737" ht="14.25" customHeight="true"/>
+    <row r="738" ht="14.25" customHeight="true"/>
+    <row r="739" ht="14.25" customHeight="true"/>
+    <row r="740" ht="14.25" customHeight="true"/>
+    <row r="741" ht="14.25" customHeight="true"/>
+    <row r="742" ht="14.25" customHeight="true"/>
+    <row r="743" ht="14.25" customHeight="true"/>
+    <row r="744" ht="14.25" customHeight="true"/>
+    <row r="745" ht="14.25" customHeight="true"/>
+    <row r="746" ht="14.25" customHeight="true"/>
+    <row r="747" ht="14.25" customHeight="true"/>
+    <row r="748" ht="14.25" customHeight="true"/>
+    <row r="749" ht="14.25" customHeight="true"/>
+    <row r="750" ht="14.25" customHeight="true"/>
+    <row r="751" ht="14.25" customHeight="true"/>
+    <row r="752" ht="14.25" customHeight="true"/>
+    <row r="753" ht="14.25" customHeight="true"/>
+    <row r="754" ht="14.25" customHeight="true"/>
+    <row r="755" ht="14.25" customHeight="true"/>
+    <row r="756" ht="14.25" customHeight="true"/>
+    <row r="757" ht="14.25" customHeight="true"/>
+    <row r="758" ht="14.25" customHeight="true"/>
+    <row r="759" ht="14.25" customHeight="true"/>
+    <row r="760" ht="14.25" customHeight="true"/>
+    <row r="761" ht="14.25" customHeight="true"/>
+    <row r="762" ht="14.25" customHeight="true"/>
+    <row r="763" ht="14.25" customHeight="true"/>
+    <row r="764" ht="14.25" customHeight="true"/>
+    <row r="765" ht="14.25" customHeight="true"/>
+    <row r="766" ht="14.25" customHeight="true"/>
+    <row r="767" ht="14.25" customHeight="true"/>
+    <row r="768" ht="14.25" customHeight="true"/>
+    <row r="769" ht="14.25" customHeight="true"/>
+    <row r="770" ht="14.25" customHeight="true"/>
+    <row r="771" ht="14.25" customHeight="true"/>
+    <row r="772" ht="14.25" customHeight="true"/>
+    <row r="773" ht="14.25" customHeight="true"/>
+    <row r="774" ht="14.25" customHeight="true"/>
+    <row r="775" ht="14.25" customHeight="true"/>
+    <row r="776" ht="14.25" customHeight="true"/>
+    <row r="777" ht="14.25" customHeight="true"/>
+    <row r="778" ht="14.25" customHeight="true"/>
+    <row r="779" ht="14.25" customHeight="true"/>
+    <row r="780" ht="14.25" customHeight="true"/>
+    <row r="781" ht="14.25" customHeight="true"/>
+    <row r="782" ht="14.25" customHeight="true"/>
+    <row r="783" ht="14.25" customHeight="true"/>
+    <row r="784" ht="14.25" customHeight="true"/>
+    <row r="785" ht="14.25" customHeight="true"/>
+    <row r="786" ht="14.25" customHeight="true"/>
+    <row r="787" ht="14.25" customHeight="true"/>
+    <row r="788" ht="14.25" customHeight="true"/>
+    <row r="789" ht="14.25" customHeight="true"/>
+    <row r="790" ht="14.25" customHeight="true"/>
+    <row r="791" ht="14.25" customHeight="true"/>
+    <row r="792" ht="14.25" customHeight="true"/>
+    <row r="793" ht="14.25" customHeight="true"/>
+    <row r="794" ht="14.25" customHeight="true"/>
+    <row r="795" ht="14.25" customHeight="true"/>
+    <row r="796" ht="14.25" customHeight="true"/>
+    <row r="797" ht="14.25" customHeight="true"/>
+    <row r="798" ht="14.25" customHeight="true"/>
+    <row r="799" ht="14.25" customHeight="true"/>
+    <row r="800" ht="14.25" customHeight="true"/>
+    <row r="801" ht="14.25" customHeight="true"/>
+    <row r="802" ht="14.25" customHeight="true"/>
+    <row r="803" ht="14.25" customHeight="true"/>
+    <row r="804" ht="14.25" customHeight="true"/>
+    <row r="805" ht="14.25" customHeight="true"/>
+    <row r="806" ht="14.25" customHeight="true"/>
+    <row r="807" ht="14.25" customHeight="true"/>
+    <row r="808" ht="14.25" customHeight="true"/>
+    <row r="809" ht="14.25" customHeight="true"/>
+    <row r="810" ht="14.25" customHeight="true"/>
+    <row r="811" ht="14.25" customHeight="true"/>
+    <row r="812" ht="14.25" customHeight="true"/>
+    <row r="813" ht="14.25" customHeight="true"/>
+    <row r="814" ht="14.25" customHeight="true"/>
+    <row r="815" ht="14.25" customHeight="true"/>
+    <row r="816" ht="14.25" customHeight="true"/>
+    <row r="817" ht="14.25" customHeight="true"/>
+    <row r="818" ht="14.25" customHeight="true"/>
+    <row r="819" ht="14.25" customHeight="true"/>
+    <row r="820" ht="14.25" customHeight="true"/>
+    <row r="821" ht="14.25" customHeight="true"/>
+    <row r="822" ht="14.25" customHeight="true"/>
+    <row r="823" ht="14.25" customHeight="true"/>
+    <row r="824" ht="14.25" customHeight="true"/>
+    <row r="825" ht="14.25" customHeight="true"/>
+    <row r="826" ht="14.25" customHeight="true"/>
+    <row r="827" ht="14.25" customHeight="true"/>
+    <row r="828" ht="14.25" customHeight="true"/>
+    <row r="829" ht="14.25" customHeight="true"/>
+    <row r="830" ht="14.25" customHeight="true"/>
+    <row r="831" ht="14.25" customHeight="true"/>
+    <row r="832" ht="14.25" customHeight="true"/>
+    <row r="833" ht="14.25" customHeight="true"/>
+    <row r="834" ht="14.25" customHeight="true"/>
+    <row r="835" ht="14.25" customHeight="true"/>
+    <row r="836" ht="14.25" customHeight="true"/>
+    <row r="837" ht="14.25" customHeight="true"/>
+    <row r="838" ht="14.25" customHeight="true"/>
+    <row r="839" ht="14.25" customHeight="true"/>
+    <row r="840" ht="14.25" customHeight="true"/>
+    <row r="841" ht="14.25" customHeight="true"/>
+    <row r="842" ht="14.25" customHeight="true"/>
+    <row r="843" ht="14.25" customHeight="true"/>
+    <row r="844" ht="14.25" customHeight="true"/>
+    <row r="845" ht="14.25" customHeight="true"/>
+    <row r="846" ht="14.25" customHeight="true"/>
+    <row r="847" ht="14.25" customHeight="true"/>
+    <row r="848" ht="14.25" customHeight="true"/>
+    <row r="849" ht="14.25" customHeight="true"/>
+    <row r="850" ht="14.25" customHeight="true"/>
+    <row r="851" ht="14.25" customHeight="true"/>
+    <row r="852" ht="14.25" customHeight="true"/>
+    <row r="853" ht="14.25" customHeight="true"/>
+    <row r="854" ht="14.25" customHeight="true"/>
+    <row r="855" ht="14.25" customHeight="true"/>
+    <row r="856" ht="14.25" customHeight="true"/>
+    <row r="857" ht="14.25" customHeight="true"/>
+    <row r="858" ht="14.25" customHeight="true"/>
+    <row r="859" ht="14.25" customHeight="true"/>
+    <row r="860" ht="14.25" customHeight="true"/>
+    <row r="861" ht="14.25" customHeight="true"/>
+    <row r="862" ht="14.25" customHeight="true"/>
+    <row r="863" ht="14.25" customHeight="true"/>
+    <row r="864" ht="14.25" customHeight="true"/>
+    <row r="865" ht="14.25" customHeight="true"/>
+    <row r="866" ht="14.25" customHeight="true"/>
+    <row r="867" ht="14.25" customHeight="true"/>
+    <row r="868" ht="14.25" customHeight="true"/>
+    <row r="869" ht="14.25" customHeight="true"/>
+    <row r="870" ht="14.25" customHeight="true"/>
+    <row r="871" ht="14.25" customHeight="true"/>
+    <row r="872" ht="14.25" customHeight="true"/>
+    <row r="873" ht="14.25" customHeight="true"/>
+    <row r="874" ht="14.25" customHeight="true"/>
+    <row r="875" ht="14.25" customHeight="true"/>
+    <row r="876" ht="14.25" customHeight="true"/>
+    <row r="877" ht="14.25" customHeight="true"/>
+    <row r="878" ht="14.25" customHeight="true"/>
+    <row r="879" ht="14.25" customHeight="true"/>
+    <row r="880" ht="14.25" customHeight="true"/>
+    <row r="881" ht="14.25" customHeight="true"/>
+    <row r="882" ht="14.25" customHeight="true"/>
+    <row r="883" ht="14.25" customHeight="true"/>
+    <row r="884" ht="14.25" customHeight="true"/>
+    <row r="885" ht="14.25" customHeight="true"/>
+    <row r="886" ht="14.25" customHeight="true"/>
+    <row r="887" ht="14.25" customHeight="true"/>
+    <row r="888" ht="14.25" customHeight="true"/>
+    <row r="889" ht="14.25" customHeight="true"/>
+    <row r="890" ht="14.25" customHeight="true"/>
+    <row r="891" ht="14.25" customHeight="true"/>
+    <row r="892" ht="14.25" customHeight="true"/>
+    <row r="893" ht="14.25" customHeight="true"/>
+    <row r="894" ht="14.25" customHeight="true"/>
+    <row r="895" ht="14.25" customHeight="true"/>
+    <row r="896" ht="14.25" customHeight="true"/>
+    <row r="897" ht="14.25" customHeight="true"/>
+    <row r="898" ht="14.25" customHeight="true"/>
+    <row r="899" ht="14.25" customHeight="true"/>
+    <row r="900" ht="14.25" customHeight="true"/>
+    <row r="901" ht="14.25" customHeight="true"/>
+    <row r="902" ht="14.25" customHeight="true"/>
+    <row r="903" ht="14.25" customHeight="true"/>
+    <row r="904" ht="14.25" customHeight="true"/>
+    <row r="905" ht="14.25" customHeight="true"/>
+    <row r="906" ht="14.25" customHeight="true"/>
+    <row r="907" ht="14.25" customHeight="true"/>
+    <row r="908" ht="14.25" customHeight="true"/>
+    <row r="909" ht="14.25" customHeight="true"/>
+    <row r="910" ht="14.25" customHeight="true"/>
+    <row r="911" ht="14.25" customHeight="true"/>
+    <row r="912" ht="14.25" customHeight="true"/>
+    <row r="913" ht="14.25" customHeight="true"/>
+    <row r="914" ht="14.25" customHeight="true"/>
+    <row r="915" ht="14.25" customHeight="true"/>
+    <row r="916" ht="14.25" customHeight="true"/>
+    <row r="917" ht="14.25" customHeight="true"/>
+    <row r="918" ht="14.25" customHeight="true"/>
+    <row r="919" ht="14.25" customHeight="true"/>
+    <row r="920" ht="14.25" customHeight="true"/>
+    <row r="921" ht="14.25" customHeight="true"/>
+    <row r="922" ht="14.25" customHeight="true"/>
+    <row r="923" ht="14.25" customHeight="true"/>
+    <row r="924" ht="14.25" customHeight="true"/>
+    <row r="925" ht="14.25" customHeight="true"/>
+    <row r="926" ht="14.25" customHeight="true"/>
+    <row r="927" ht="14.25" customHeight="true"/>
+    <row r="928" ht="14.25" customHeight="true"/>
+    <row r="929" ht="14.25" customHeight="true"/>
+    <row r="930" ht="14.25" customHeight="true"/>
+    <row r="931" ht="14.25" customHeight="true"/>
+    <row r="932" ht="14.25" customHeight="true"/>
+    <row r="933" ht="14.25" customHeight="true"/>
+    <row r="934" ht="14.25" customHeight="true"/>
+    <row r="935" ht="14.25" customHeight="true"/>
+    <row r="936" ht="14.25" customHeight="true"/>
+    <row r="937" ht="14.25" customHeight="true"/>
+    <row r="938" ht="14.25" customHeight="true"/>
+    <row r="939" ht="14.25" customHeight="true"/>
+    <row r="940" ht="14.25" customHeight="true"/>
+    <row r="941" ht="14.25" customHeight="true"/>
+    <row r="942" ht="14.25" customHeight="true"/>
+    <row r="943" ht="14.25" customHeight="true"/>
+    <row r="944" ht="14.25" customHeight="true"/>
+    <row r="945" ht="14.25" customHeight="true"/>
+    <row r="946" ht="14.25" customHeight="true"/>
+    <row r="947" ht="14.25" customHeight="true"/>
+    <row r="948" ht="14.25" customHeight="true"/>
+    <row r="949" ht="14.25" customHeight="true"/>
+    <row r="950" ht="14.25" customHeight="true"/>
+    <row r="951" ht="14.25" customHeight="true"/>
+    <row r="952" ht="14.25" customHeight="true"/>
+    <row r="953" ht="14.25" customHeight="true"/>
+    <row r="954" ht="14.25" customHeight="true"/>
+    <row r="955" ht="14.25" customHeight="true"/>
+    <row r="956" ht="14.25" customHeight="true"/>
+    <row r="957" ht="14.25" customHeight="true"/>
+    <row r="958" ht="14.25" customHeight="true"/>
+    <row r="959" ht="14.25" customHeight="true"/>
+    <row r="960" ht="14.25" customHeight="true"/>
+    <row r="961" ht="14.25" customHeight="true"/>
+    <row r="962" ht="14.25" customHeight="true"/>
+    <row r="963" ht="14.25" customHeight="true"/>
+    <row r="964" ht="14.25" customHeight="true"/>
+    <row r="965" ht="14.25" customHeight="true"/>
+    <row r="966" ht="14.25" customHeight="true"/>
+    <row r="967" ht="14.25" customHeight="true"/>
+    <row r="968" ht="14.25" customHeight="true"/>
+    <row r="969" ht="14.25" customHeight="true"/>
+    <row r="970" ht="14.25" customHeight="true"/>
+    <row r="971" ht="14.25" customHeight="true"/>
+    <row r="972" ht="14.25" customHeight="true"/>
+    <row r="973" ht="14.25" customHeight="true"/>
+    <row r="974" ht="14.25" customHeight="true"/>
+    <row r="975" ht="14.25" customHeight="true"/>
+    <row r="976" ht="14.25" customHeight="true"/>
+    <row r="977" ht="14.25" customHeight="true"/>
+    <row r="978" ht="14.25" customHeight="true"/>
+    <row r="979" ht="14.25" customHeight="true"/>
+    <row r="980" ht="14.25" customHeight="true"/>
+    <row r="981" ht="14.25" customHeight="true"/>
+    <row r="982" ht="14.25" customHeight="true"/>
+    <row r="983" ht="14.25" customHeight="true"/>
+    <row r="984" ht="14.25" customHeight="true"/>
+    <row r="985" ht="14.25" customHeight="true"/>
+    <row r="986" ht="14.25" customHeight="true"/>
+    <row r="987" ht="14.25" customHeight="true"/>
+    <row r="988" ht="14.25" customHeight="true"/>
+    <row r="989" ht="14.25" customHeight="true"/>
+    <row r="990" ht="14.25" customHeight="true"/>
+    <row r="991" ht="14.25" customHeight="true"/>
+    <row r="992" ht="14.25" customHeight="true"/>
+    <row r="993" ht="14.25" customHeight="true"/>
+    <row r="994" ht="14.25" customHeight="true"/>
+    <row r="995" ht="14.25" customHeight="true"/>
+    <row r="996" ht="14.25" customHeight="true"/>
+    <row r="997" ht="14.25" customHeight="true"/>
+    <row r="998" ht="14.25" customHeight="true"/>
+    <row r="999" ht="14.25" customHeight="true"/>
+    <row r="1000" ht="14.25" customHeight="true"/>
   </sheetData>
   <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>